<commit_message>
Some suspension tires to fix tire in the ground and Linkage library
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Main/Develop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/VehicleModel/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30C082B-74F3-9D44-9799-09A7F9273786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{323979D1-431D-7A4C-BDD7-3030D0EFFB43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9060" yWindow="980" windowWidth="20480" windowHeight="19540" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8740" yWindow="800" windowWidth="16880" windowHeight="19540" firstSheet="4" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Body" sheetId="1" r:id="rId1"/>
@@ -214,9 +214,6 @@
     <t>Upright</t>
   </si>
   <si>
-    <t>sWheelCenter</t>
-  </si>
-  <si>
     <t>aToe</t>
   </si>
   <si>
@@ -526,9 +523,6 @@
     <t>TrackRod</t>
   </si>
   <si>
-    <t>which(''Hoosier_20p5x7_13_R20.tir'')</t>
-  </si>
-  <si>
     <t>xPreload</t>
   </si>
   <si>
@@ -542,6 +536,12 @@
   </si>
   <si>
     <t>Parameterized</t>
+  </si>
+  <si>
+    <t>sWheelCentre</t>
+  </si>
+  <si>
+    <t>which('Hoosier_20p5x7_13_R20.tir')</t>
   </si>
 </sst>
 </file>
@@ -3494,7 +3494,7 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -3505,7 +3505,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -3516,20 +3516,20 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="139" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B5" s="77" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="80" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="30"/>
@@ -3537,23 +3537,23 @@
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="140"/>
       <c r="B6" s="97" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C6" s="98">
         <v>52538.05</v>
       </c>
       <c r="D6" s="99" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E6" s="100"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="147"/>
       <c r="B7" s="81" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C7" s="21">
-        <v>1.559E-2</v>
+        <v>0.01</v>
       </c>
       <c r="D7" s="22" t="s">
         <v>12</v>
@@ -3562,13 +3562,13 @@
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="139" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B8" s="77" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="102" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D8" s="12"/>
       <c r="E8" s="30"/>
@@ -3576,26 +3576,26 @@
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="140"/>
       <c r="B9" s="97" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C9" s="101">
         <v>43781.708749999998</v>
       </c>
       <c r="D9" s="99" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E9" s="100"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="147"/>
       <c r="B10" s="81" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C10" s="21">
-        <v>1.3899999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E10" s="33"/>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -3669,20 +3669,20 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="139" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B5" s="77" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="80" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="30"/>
@@ -3690,72 +3690,72 @@
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="140"/>
       <c r="B6" s="97" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C6" s="98">
         <v>250000</v>
       </c>
       <c r="D6" s="99" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E6" s="100"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="140"/>
       <c r="B7" s="78" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C7" s="25">
         <v>100000</v>
       </c>
       <c r="D7" s="89" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E7" s="19"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="140"/>
       <c r="B8" s="78" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C8" s="25">
         <v>100000</v>
       </c>
       <c r="D8" s="89" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E8" s="19"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="140"/>
       <c r="B9" s="78" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C9" s="25">
         <v>150</v>
       </c>
       <c r="D9" s="89" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E9" s="19"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="140"/>
       <c r="B10" s="78" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C10" s="25">
         <v>150</v>
       </c>
       <c r="D10" s="89" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E10" s="19"/>
     </row>
     <row r="11" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="147"/>
       <c r="B11" s="81" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C11" s="27">
         <v>1E-4</v>
@@ -3767,13 +3767,13 @@
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="139" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B12" s="77" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="103" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="30"/>
@@ -3781,72 +3781,72 @@
     <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="140"/>
       <c r="B13" s="97" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C13" s="98">
         <v>250000</v>
       </c>
       <c r="D13" s="104" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E13" s="100"/>
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="140"/>
       <c r="B14" s="78" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C14" s="25">
         <v>100000</v>
       </c>
       <c r="D14" s="104" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E14" s="19"/>
     </row>
     <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="140"/>
       <c r="B15" s="78" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C15" s="25">
         <v>100000</v>
       </c>
       <c r="D15" s="104" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E15" s="19"/>
     </row>
     <row r="16" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="140"/>
       <c r="B16" s="78" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C16" s="25">
         <v>150</v>
       </c>
       <c r="D16" s="104" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E16" s="19"/>
     </row>
     <row r="17" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="140"/>
       <c r="B17" s="78" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C17" s="25">
         <v>150</v>
       </c>
       <c r="D17" s="104" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E17" s="19"/>
     </row>
     <row r="18" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="147"/>
       <c r="B18" s="81" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C18" s="27">
         <v>1E-4</v>
@@ -3902,7 +3902,7 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="105" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="105" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -3924,29 +3924,29 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="105" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="95" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B5" s="77"/>
       <c r="C5" s="124" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="D5" s="106" t="s">
+        <v>108</v>
+      </c>
+      <c r="E5" s="107" t="s">
         <v>109</v>
-      </c>
-      <c r="E5" s="107" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="95" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B6" s="77"/>
       <c r="C6" s="103">
@@ -3959,33 +3959,33 @@
     </row>
     <row r="7" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="95" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B7" s="77"/>
       <c r="C7" s="103" t="s">
+        <v>112</v>
+      </c>
+      <c r="D7" s="106" t="s">
         <v>113</v>
-      </c>
-      <c r="D7" s="106" t="s">
-        <v>114</v>
       </c>
       <c r="E7" s="30"/>
     </row>
     <row r="8" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="95" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B8" s="77"/>
       <c r="C8" s="108" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D8" s="106" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E8" s="30"/>
     </row>
     <row r="9" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="95" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B9" s="77"/>
       <c r="C9" s="103">
@@ -3996,28 +3996,28 @@
     </row>
     <row r="10" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="95" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B10" s="77"/>
       <c r="C10" s="103">
         <v>0.01</v>
       </c>
       <c r="D10" s="106" t="s">
+        <v>118</v>
+      </c>
+      <c r="E10" s="107" t="s">
         <v>119</v>
-      </c>
-      <c r="E10" s="107" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="139" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B11" s="109" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="110" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D11" s="94"/>
       <c r="E11" s="74"/>
@@ -4025,7 +4025,7 @@
     <row r="12" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="147"/>
       <c r="B12" s="111" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C12" s="112" t="s">
         <v>11</v>
@@ -4058,21 +4058,21 @@
   <sheetData>
     <row r="1" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="34" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="C1" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="D1" s="34" t="s">
         <v>125</v>
-      </c>
-      <c r="D1" s="34" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="35" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B2" s="36">
         <v>200</v>
@@ -4086,7 +4086,7 @@
     </row>
     <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="38" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B3" s="39">
         <v>-200</v>
@@ -4100,7 +4100,7 @@
     </row>
     <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="38" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B4" s="39">
         <v>11.946</v>
@@ -4114,7 +4114,7 @@
     </row>
     <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B5" s="39">
         <v>148.751</v>
@@ -4128,7 +4128,7 @@
     </row>
     <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="38" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B6" s="39">
         <v>-184.72900000000001</v>
@@ -4142,7 +4142,7 @@
     </row>
     <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="38" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B7" s="39">
         <v>-12.932</v>
@@ -4156,7 +4156,7 @@
     </row>
     <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B8" s="39">
         <v>16.193999999999999</v>
@@ -4170,7 +4170,7 @@
     </row>
     <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B9" s="39">
         <v>0</v>
@@ -4184,7 +4184,7 @@
     </row>
     <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="38" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B10" s="39">
         <v>104.241</v>
@@ -4198,7 +4198,7 @@
     </row>
     <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="38" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B11" s="39">
         <v>85.097999999999999</v>
@@ -4212,7 +4212,7 @@
     </row>
     <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B12" s="39">
         <v>11.157</v>
@@ -4226,7 +4226,7 @@
     </row>
     <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="38" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B13" s="39">
         <v>11.484999999999999</v>
@@ -4240,7 +4240,7 @@
     </row>
     <row r="14" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="38" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B14" s="39">
         <v>11.821</v>
@@ -4254,7 +4254,7 @@
     </row>
     <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="38" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B15" s="39">
         <v>11.489000000000001</v>
@@ -4268,7 +4268,7 @@
     </row>
     <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="38" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B16" s="39">
         <v>11.558</v>
@@ -4282,7 +4282,7 @@
     </row>
     <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="38" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B17" s="39">
         <v>67.965000000000003</v>
@@ -4296,7 +4296,7 @@
     </row>
     <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B18" s="39">
         <v>4</v>
@@ -4310,7 +4310,7 @@
     </row>
     <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="38" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B19" s="39">
         <v>11.526999999999999</v>
@@ -4324,7 +4324,7 @@
     </row>
     <row r="20" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="38" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B20" s="39">
         <v>104.241</v>
@@ -4338,7 +4338,7 @@
     </row>
     <row r="21" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="38" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B21" s="39">
         <v>-324.96499999999997</v>
@@ -4374,21 +4374,21 @@
   <sheetData>
     <row r="1" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="34" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="C1" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="D1" s="34" t="s">
         <v>125</v>
-      </c>
-      <c r="D1" s="34" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="35" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B2" s="36">
         <v>-1390</v>
@@ -4402,7 +4402,7 @@
     </row>
     <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="38" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B3" s="39">
         <v>-1830</v>
@@ -4416,7 +4416,7 @@
     </row>
     <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="38" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B4" s="39">
         <v>-1579.2370000000001</v>
@@ -4430,7 +4430,7 @@
     </row>
     <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B5" s="39">
         <v>-1390</v>
@@ -4444,7 +4444,7 @@
     </row>
     <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="38" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B6" s="39">
         <v>-1830</v>
@@ -4458,7 +4458,7 @@
     </row>
     <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="38" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B7" s="39">
         <v>-1569.845</v>
@@ -4472,7 +4472,7 @@
     </row>
     <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B8" s="39">
         <v>-1568.8710000000001</v>
@@ -4486,7 +4486,7 @@
     </row>
     <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B9" s="39">
         <v>-1574.5989999999999</v>
@@ -4500,7 +4500,7 @@
     </row>
     <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="38" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B10" s="39">
         <v>-1830</v>
@@ -4514,7 +4514,7 @@
     </row>
     <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="38" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B11" s="39">
         <v>-1675.904</v>
@@ -4528,7 +4528,7 @@
     </row>
     <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B12" s="39">
         <v>-1395.9760000000001</v>
@@ -4542,7 +4542,7 @@
     </row>
     <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="38" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B13" s="39">
         <v>-1579.1110000000001</v>
@@ -4556,7 +4556,7 @@
     </row>
     <row r="14" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="38" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B14" s="39">
         <v>-1597.194</v>
@@ -4570,7 +4570,7 @@
     </row>
     <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="38" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B15" s="39">
         <v>-1664.6120000000001</v>
@@ -4584,7 +4584,7 @@
     </row>
     <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="38" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B16" s="39">
         <v>-1585.771</v>
@@ -4598,7 +4598,7 @@
     </row>
     <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="38" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B17" s="39">
         <v>-1830</v>
@@ -4612,7 +4612,7 @@
     </row>
     <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="38" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B18" s="39">
         <v>-1830</v>
@@ -4626,7 +4626,7 @@
     </row>
     <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="38" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B19" s="39">
         <v>-1600.4860000000001</v>
@@ -4713,36 +4713,36 @@
       </c>
       <c r="B5" s="117"/>
       <c r="C5" s="119" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D5" s="120" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E5" s="118"/>
     </row>
     <row r="6" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B6" s="81"/>
       <c r="C6" s="88" t="s">
+        <v>65</v>
+      </c>
+      <c r="D6" s="90" t="s">
         <v>66</v>
-      </c>
-      <c r="D6" s="90" t="s">
-        <v>67</v>
       </c>
       <c r="E6" s="23"/>
     </row>
     <row r="7" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B7" s="81"/>
       <c r="C7" s="88" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D7" s="90" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E7" s="23"/>
     </row>
@@ -4965,7 +4965,7 @@
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="134"/>
       <c r="B14" s="78" t="s">
-        <v>47</v>
+        <v>155</v>
       </c>
       <c r="C14" s="25" t="str" cm="1">
         <f t="array" ref="C14">"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B9/1000,HardpointsFr!C9/1000,HardpointsFr!D9/1000)&amp;"]"</f>
@@ -4994,33 +4994,33 @@
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="137"/>
       <c r="B16" s="78" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C16" s="26">
         <v>0</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E16" s="17"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="132"/>
       <c r="B17" s="78" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C17" s="26">
         <v>-1</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E17" s="17"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="132"/>
       <c r="B18" s="78" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C18" s="115">
         <v>0.11</v>
@@ -5033,7 +5033,7 @@
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="132"/>
       <c r="B19" s="78" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C19" s="115">
         <v>0.03</v>
@@ -5046,7 +5046,7 @@
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="131"/>
       <c r="B20" s="81" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C20" s="116">
         <v>1.5</v>
@@ -5058,10 +5058,10 @@
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="130" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B21" s="77" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21" s="24" t="str" cm="1">
         <f t="array" ref="C21">"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B10/1000,HardpointsFr!C10/1000,HardpointsFr!D10/1000)&amp;"]"</f>
@@ -5105,10 +5105,10 @@
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="130" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="77" t="s">
         <v>55</v>
-      </c>
-      <c r="B24" s="77" t="s">
-        <v>56</v>
       </c>
       <c r="C24" s="24" t="str" cm="1">
         <f t="array" ref="C24">"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B12/1000,HardpointsFr!C12/1000,HardpointsFr!D12/1000)&amp;"]"</f>
@@ -5124,7 +5124,7 @@
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="132"/>
       <c r="B25" s="78" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C25" s="25" t="str" cm="1">
         <f t="array" ref="C25">"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B13/1000,HardpointsFr!C13/1000,HardpointsFr!D13/1000)&amp;"]"</f>
@@ -5140,7 +5140,7 @@
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="138"/>
       <c r="B26" s="82" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C26" s="128">
         <v>1.2</v>
@@ -5153,7 +5153,7 @@
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="131"/>
       <c r="B27" s="81" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C27" s="21">
         <v>0.8</v>
@@ -5165,10 +5165,10 @@
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="130" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" s="77" t="s">
         <v>58</v>
-      </c>
-      <c r="B28" s="77" t="s">
-        <v>59</v>
       </c>
       <c r="C28" s="28">
         <v>2.8000000000000001E-2</v>
@@ -5181,7 +5181,7 @@
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="131"/>
       <c r="B29" s="81" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C29" s="21">
         <v>-2.8000000000000001E-2</v>
@@ -5193,10 +5193,10 @@
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="130" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B30" s="91" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C30" s="24" t="str" cm="1">
         <f t="array" ref="C30">"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B15/1000,HardpointsFr!C15/1000,HardpointsFr!D15/1000)&amp;"]"</f>
@@ -5240,10 +5240,10 @@
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="130" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" s="11" t="s">
         <v>62</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>63</v>
       </c>
       <c r="C33" s="24" t="str" cm="1">
         <f t="array" ref="C33">"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B16/1000,HardpointsFr!C16/1000,HardpointsFr!D16/1000)&amp;"]"</f>
@@ -5259,7 +5259,7 @@
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="132"/>
       <c r="B34" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C34" s="25" t="str" cm="1">
         <f t="array" ref="C34">"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B19/1000,HardpointsFr!C19/1000,HardpointsFr!D19/1000)&amp;"]"</f>
@@ -5338,7 +5338,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
@@ -5360,14 +5360,14 @@
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="10"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="125" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" s="77"/>
       <c r="C6" s="24" t="str">
@@ -5383,7 +5383,7 @@
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="126" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" s="78"/>
       <c r="C7" s="25" t="str">
@@ -5415,14 +5415,14 @@
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="126" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B9" s="78"/>
       <c r="C9" s="29">
         <v>81.933000000000007</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E9" s="17"/>
     </row>
@@ -5485,7 +5485,7 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -5496,7 +5496,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -5507,21 +5507,21 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="139" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="77" t="s">
         <v>76</v>
       </c>
-      <c r="B5" s="77" t="s">
-        <v>77</v>
-      </c>
       <c r="C5" s="44" t="str">
-        <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B13/1000,HardpointsFr!C13/1000,HardpointsFr!D13/1000)&amp;"]"</f>
-        <v>[0.011485 0.317842 0.36243]</v>
+        <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B20/1000,HardpointsFr!C20/1000,HardpointsFr!D20/1000)&amp;"]"</f>
+        <v>[0.104241 0 0.171053]</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>12</v>
@@ -5546,19 +5546,19 @@
     <row r="7" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="141"/>
       <c r="B7" s="78" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C7" s="41">
         <v>50</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E7" s="16"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="142" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B8" s="78" t="s">
         <v>12</v>
@@ -5574,11 +5574,11 @@
     <row r="9" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="143"/>
       <c r="B9" s="78" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C9" s="41" t="str">
-        <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B18/1000,HardpointsFr!C18/1000,HardpointsFr!D18/1000)&amp;"]"</f>
-        <v>[0.004 0.262849 0.101519]</v>
+        <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B21/1000,HardpointsFr!C21/1000,HardpointsFr!D21/1000)&amp;"]"</f>
+        <v>[-0.324965 0 0.533792]</v>
       </c>
       <c r="D9" s="16" t="s">
         <v>12</v>
@@ -5670,23 +5670,23 @@
       </c>
       <c r="B5" s="117"/>
       <c r="C5" s="119" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D5" s="120" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E5" s="121"/>
     </row>
     <row r="6" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B6" s="81"/>
       <c r="C6" s="88" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D6" s="90" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E6" s="23"/>
     </row>
@@ -5756,7 +5756,7 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="105" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
@@ -5910,7 +5910,7 @@
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="140"/>
       <c r="B14" s="78" t="s">
-        <v>47</v>
+        <v>155</v>
       </c>
       <c r="C14" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B9/1000 +1.575,HardpointsRr!C9/1000,HardpointsRr!D9/1000)&amp;"]"</f>
@@ -5939,33 +5939,33 @@
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="140"/>
       <c r="B16" s="78" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C16" s="26">
         <v>0</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E16" s="64"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="140"/>
       <c r="B17" s="78" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C17" s="26">
         <v>-1</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E17" s="67"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="140"/>
       <c r="B18" s="78" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C18" s="115">
         <v>0.11</v>
@@ -5978,7 +5978,7 @@
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="140"/>
       <c r="B19" s="78" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C19" s="115">
         <v>0.03</v>
@@ -5991,7 +5991,7 @@
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="147"/>
       <c r="B20" s="81" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C20" s="116">
         <v>1.5</v>
@@ -6003,10 +6003,10 @@
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="139" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B21" s="77" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B10/1000 +1.575,HardpointsRr!C10/1000,HardpointsRr!D10/1000)&amp;"]"</f>
@@ -6050,10 +6050,10 @@
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="139" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="77" t="s">
         <v>55</v>
-      </c>
-      <c r="B24" s="77" t="s">
-        <v>56</v>
       </c>
       <c r="C24" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B12/1000 + 1.575,HardpointsRr!C12/1000,HardpointsRr!D12/1000)&amp;"]"</f>
@@ -6069,7 +6069,7 @@
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="140"/>
       <c r="B25" s="78" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C25" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,(HardpointsRr!B13+ 1575)/1000,HardpointsRr!C13/1000,HardpointsRr!D13/1000)&amp;"]"</f>
@@ -6085,7 +6085,7 @@
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="140"/>
       <c r="B26" s="82" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C26" s="128">
         <v>0.8</v>
@@ -6096,7 +6096,7 @@
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="147"/>
       <c r="B27" s="81" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C27" s="21">
         <v>1.2</v>
@@ -6108,10 +6108,10 @@
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="139" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" s="77" t="s">
         <v>58</v>
-      </c>
-      <c r="B28" s="77" t="s">
-        <v>59</v>
       </c>
       <c r="C28" s="28">
         <v>2.8000000000000001E-2</v>
@@ -6124,7 +6124,7 @@
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="147"/>
       <c r="B29" s="81" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C29" s="21">
         <v>-2.8000000000000001E-2</v>
@@ -6136,10 +6136,10 @@
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="144" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B30" s="91" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C30" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B14/1000 + 1.575,HardpointsRr!C14/1000,HardpointsRr!D14/1000)&amp;"]"</f>
@@ -6183,10 +6183,10 @@
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="139" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" s="11" t="s">
         <v>62</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>63</v>
       </c>
       <c r="C33" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B16/1000+ 1.575,HardpointsRr!C16/1000,HardpointsRr!D16/1000)&amp;"]"</f>
@@ -6202,7 +6202,7 @@
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="140"/>
       <c r="B34" s="14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C34" s="25" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B19/1000+ 1.575,HardpointsRr!C19/1000,HardpointsRr!D19/1000)&amp;"]"</f>
@@ -6280,7 +6280,7 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -6291,7 +6291,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -6302,14 +6302,14 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="74"/>
     </row>
     <row r="5" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="125" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B5" s="77"/>
       <c r="C5" s="24" t="str">
@@ -6317,7 +6317,7 @@
         <v>[-0.0254860000000001 0.287566 0.463988]</v>
       </c>
       <c r="D5" s="46" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E5" s="69" t="s">
         <v>42</v>
@@ -6325,7 +6325,7 @@
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="126" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" s="78"/>
       <c r="C6" s="25" t="str">
@@ -6357,14 +6357,14 @@
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="126" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B8" s="78"/>
       <c r="C8" s="31">
         <v>61.879399999999997</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E8" s="75"/>
     </row>
@@ -6425,7 +6425,7 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -6447,14 +6447,14 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="123" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B5" s="77"/>
       <c r="C5" s="24">
@@ -6465,7 +6465,7 @@
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="123" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B6" s="78"/>
       <c r="C6" s="25">
@@ -6476,37 +6476,37 @@
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="123" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B7" s="78"/>
       <c r="C7" s="25">
         <v>1.2250000000000001</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E7" s="19"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="123" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B8" s="78"/>
       <c r="C8" s="25">
         <v>1.2</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E8" s="19"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="123" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B9" s="81"/>
       <c r="C9" s="32" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>30</v>
@@ -6532,17 +6532,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009342B7EAA7728A4FA80A5CCAFE8D7EAF" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d037a5681ee6af0e7b5b5d0a2f99b20">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557458c-24b5-4c97-84ed-4c402655f54f" xmlns:ns3="72e3c584-9879-4b35-b9d8-6a248c93e240" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="966978c8b125399653e7c255ac8e342d" ns2:_="" ns3:_="">
     <xsd:import namespace="9557458c-24b5-4c97-84ed-4c402655f54f"/>
@@ -6803,6 +6792,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
   <ds:schemaRefs>
@@ -6812,17 +6812,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
-    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6839,4 +6828,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Slip Control code generated
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/VehicleModel/Scripts_Data/Data_Vehicle/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Features/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{516666C7-C43E-5B46-8624-08958B4DB664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69EA7BB-4B2D-CF4B-9859-47CE8940DE05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8740" yWindow="800" windowWidth="16880" windowHeight="19540" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8740" yWindow="800" windowWidth="16880" windowHeight="19540" firstSheet="4" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Body" sheetId="1" r:id="rId1"/>
@@ -541,10 +541,10 @@
     <t>sWheelCentre</t>
   </si>
   <si>
-    <t>which('Hoosier_20p5x7_13_R20.tir')</t>
-  </si>
-  <si>
     <t>DroplinkRod Rear</t>
+  </si>
+  <si>
+    <t>which('fsTireData.tir')</t>
   </si>
 </sst>
 </file>
@@ -3938,7 +3938,7 @@
       </c>
       <c r="B5" s="77"/>
       <c r="C5" s="124" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D5" s="106" t="s">
         <v>108</v>
@@ -6305,7 +6305,7 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="105" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="74"/>
@@ -6526,14 +6526,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6798,21 +6796,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
-    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6837,9 +6834,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
- fixed simulation sweep script to optimize ram usage - finetuned stanley driver parameters
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/VehicleModel/Scripts_Data/Data_Vehicle/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9467057-CBDC-BB46-A9BB-F089AFA0D3BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92BFAD64-F766-754D-B44D-617C0E1143D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5340" yWindow="760" windowWidth="24720" windowHeight="19840" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5320" yWindow="760" windowWidth="24720" windowHeight="19840" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Body" sheetId="1" r:id="rId1"/>
@@ -544,25 +544,25 @@
     <t>Slip</t>
   </si>
   <si>
-    <t>1 combined</t>
-  </si>
-  <si>
     <t>MFEval_Hoosier</t>
   </si>
   <si>
     <t>which('Hoosier_R20B_20p5x7_R13_7in_12psi.tir')</t>
   </si>
   <si>
-    <t>1 steady state</t>
-  </si>
-  <si>
-    <t>MFEval</t>
-  </si>
-  <si>
     <t>type</t>
   </si>
   <si>
     <t>None</t>
+  </si>
+  <si>
+    <t>2 combined+turnslip</t>
+  </si>
+  <si>
+    <t>MFMbody</t>
+  </si>
+  <si>
+    <t>3 non-linear transients</t>
   </si>
 </sst>
 </file>
@@ -2054,6 +2054,15 @@
     <xf numFmtId="49" fontId="3" fillId="4" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="71" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2086,6 +2095,12 @@
     <xf numFmtId="0" fontId="2" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="64" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2098,15 +2113,9 @@
     <xf numFmtId="49" fontId="2" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2115,15 +2124,6 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="71" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3552,7 +3552,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="139" t="s">
+      <c r="A5" s="142" t="s">
         <v>93</v>
       </c>
       <c r="B5" s="77" t="s">
@@ -3565,7 +3565,7 @@
       <c r="E5" s="30"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="140"/>
+      <c r="A6" s="143"/>
       <c r="B6" s="97" t="s">
         <v>95</v>
       </c>
@@ -3578,12 +3578,12 @@
       <c r="E6" s="100"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="147"/>
+      <c r="A7" s="152"/>
       <c r="B7" s="81" t="s">
         <v>148</v>
       </c>
       <c r="C7" s="21">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="D7" s="22" t="s">
         <v>12</v>
@@ -3591,7 +3591,7 @@
       <c r="E7" s="33"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="139" t="s">
+      <c r="A8" s="142" t="s">
         <v>97</v>
       </c>
       <c r="B8" s="77" t="s">
@@ -3604,7 +3604,7 @@
       <c r="E8" s="30"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="140"/>
+      <c r="A9" s="143"/>
       <c r="B9" s="97" t="s">
         <v>95</v>
       </c>
@@ -3617,12 +3617,12 @@
       <c r="E9" s="100"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="147"/>
+      <c r="A10" s="152"/>
       <c r="B10" s="81" t="s">
         <v>148</v>
       </c>
       <c r="C10" s="21">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="D10" s="90" t="s">
         <v>12</v>
@@ -3705,7 +3705,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="139" t="s">
+      <c r="A5" s="142" t="s">
         <v>93</v>
       </c>
       <c r="B5" s="77" t="s">
@@ -3718,7 +3718,7 @@
       <c r="E5" s="30"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="140"/>
+      <c r="A6" s="143"/>
       <c r="B6" s="97" t="s">
         <v>98</v>
       </c>
@@ -3731,7 +3731,7 @@
       <c r="E6" s="100"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="140"/>
+      <c r="A7" s="143"/>
       <c r="B7" s="78" t="s">
         <v>99</v>
       </c>
@@ -3744,7 +3744,7 @@
       <c r="E7" s="19"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="140"/>
+      <c r="A8" s="143"/>
       <c r="B8" s="78" t="s">
         <v>100</v>
       </c>
@@ -3757,7 +3757,7 @@
       <c r="E8" s="19"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="140"/>
+      <c r="A9" s="143"/>
       <c r="B9" s="78" t="s">
         <v>101</v>
       </c>
@@ -3770,7 +3770,7 @@
       <c r="E9" s="19"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="140"/>
+      <c r="A10" s="143"/>
       <c r="B10" s="78" t="s">
         <v>102</v>
       </c>
@@ -3783,7 +3783,7 @@
       <c r="E10" s="19"/>
     </row>
     <row r="11" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="147"/>
+      <c r="A11" s="152"/>
       <c r="B11" s="81" t="s">
         <v>103</v>
       </c>
@@ -3796,7 +3796,7 @@
       <c r="E11" s="33"/>
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="139" t="s">
+      <c r="A12" s="142" t="s">
         <v>97</v>
       </c>
       <c r="B12" s="77" t="s">
@@ -3809,7 +3809,7 @@
       <c r="E12" s="30"/>
     </row>
     <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="140"/>
+      <c r="A13" s="143"/>
       <c r="B13" s="97" t="s">
         <v>98</v>
       </c>
@@ -3822,7 +3822,7 @@
       <c r="E13" s="100"/>
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="140"/>
+      <c r="A14" s="143"/>
       <c r="B14" s="78" t="s">
         <v>99</v>
       </c>
@@ -3835,7 +3835,7 @@
       <c r="E14" s="19"/>
     </row>
     <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="140"/>
+      <c r="A15" s="143"/>
       <c r="B15" s="78" t="s">
         <v>100</v>
       </c>
@@ -3848,7 +3848,7 @@
       <c r="E15" s="19"/>
     </row>
     <row r="16" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="140"/>
+      <c r="A16" s="143"/>
       <c r="B16" s="78" t="s">
         <v>101</v>
       </c>
@@ -3861,7 +3861,7 @@
       <c r="E16" s="19"/>
     </row>
     <row r="17" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="140"/>
+      <c r="A17" s="143"/>
       <c r="B17" s="78" t="s">
         <v>102</v>
       </c>
@@ -3874,7 +3874,7 @@
       <c r="E17" s="19"/>
     </row>
     <row r="18" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="147"/>
+      <c r="A18" s="152"/>
       <c r="B18" s="81" t="s">
         <v>103</v>
       </c>
@@ -3943,7 +3943,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="105" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -3954,7 +3954,7 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="105" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
@@ -3965,7 +3965,7 @@
       </c>
       <c r="B5" s="77"/>
       <c r="C5" s="124" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D5" s="106" t="s">
         <v>106</v>
@@ -4040,7 +4040,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="139" t="s">
+      <c r="A11" s="142" t="s">
         <v>118</v>
       </c>
       <c r="B11" s="109" t="s">
@@ -4053,7 +4053,7 @@
       <c r="E11" s="74"/>
     </row>
     <row r="12" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="147"/>
+      <c r="A12" s="152"/>
       <c r="B12" s="111" t="s">
         <v>119</v>
       </c>
@@ -4071,7 +4071,7 @@
       </c>
       <c r="B13" s="77"/>
       <c r="C13" s="103" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D13" s="106"/>
       <c r="E13" s="30"/>
@@ -4082,7 +4082,7 @@
       </c>
       <c r="B14" s="77"/>
       <c r="C14" s="103" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D14" s="106"/>
       <c r="E14" s="107"/>
@@ -4869,7 +4869,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="133" t="s">
+      <c r="A5" s="136" t="s">
         <v>40</v>
       </c>
       <c r="B5" s="77" t="s">
@@ -4887,7 +4887,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="131"/>
+      <c r="A6" s="134"/>
       <c r="B6" s="78" t="s">
         <v>43</v>
       </c>
@@ -4903,7 +4903,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="134"/>
+      <c r="A7" s="137"/>
       <c r="B7" s="78" t="s">
         <v>44</v>
       </c>
@@ -4919,7 +4919,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="134"/>
+      <c r="A8" s="137"/>
       <c r="B8" s="81" t="s">
         <v>12</v>
       </c>
@@ -4932,7 +4932,7 @@
       <c r="E8" s="23"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="135" t="s">
+      <c r="A9" s="138" t="s">
         <v>45</v>
       </c>
       <c r="B9" s="77" t="s">
@@ -4950,7 +4950,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="132"/>
+      <c r="A10" s="135"/>
       <c r="B10" s="78" t="s">
         <v>43</v>
       </c>
@@ -4966,7 +4966,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="132"/>
+      <c r="A11" s="135"/>
       <c r="B11" s="78" t="s">
         <v>44</v>
       </c>
@@ -4982,7 +4982,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="131"/>
+      <c r="A12" s="134"/>
       <c r="B12" s="81" t="s">
         <v>12</v>
       </c>
@@ -4997,7 +4997,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="136" t="s">
+      <c r="A13" s="139" t="s">
         <v>46</v>
       </c>
       <c r="B13" s="77" t="s">
@@ -5015,7 +5015,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="134"/>
+      <c r="A14" s="137"/>
       <c r="B14" s="78" t="s">
         <v>153</v>
       </c>
@@ -5031,7 +5031,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="134"/>
+      <c r="A15" s="137"/>
       <c r="B15" s="78" t="s">
         <v>12</v>
       </c>
@@ -5044,7 +5044,7 @@
       <c r="E15" s="19"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="137"/>
+      <c r="A16" s="140"/>
       <c r="B16" s="78" t="s">
         <v>47</v>
       </c>
@@ -5057,7 +5057,7 @@
       <c r="E16" s="17"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="132"/>
+      <c r="A17" s="135"/>
       <c r="B17" s="78" t="s">
         <v>49</v>
       </c>
@@ -5070,7 +5070,7 @@
       <c r="E17" s="17"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="132"/>
+      <c r="A18" s="135"/>
       <c r="B18" s="78" t="s">
         <v>50</v>
       </c>
@@ -5083,7 +5083,7 @@
       <c r="E18" s="17"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="132"/>
+      <c r="A19" s="135"/>
       <c r="B19" s="78" t="s">
         <v>51</v>
       </c>
@@ -5096,7 +5096,7 @@
       <c r="E19" s="17"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="131"/>
+      <c r="A20" s="134"/>
       <c r="B20" s="81" t="s">
         <v>52</v>
       </c>
@@ -5109,7 +5109,7 @@
       <c r="E20" s="23"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="130" t="s">
+      <c r="A21" s="133" t="s">
         <v>147</v>
       </c>
       <c r="B21" s="77" t="s">
@@ -5127,7 +5127,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="132"/>
+      <c r="A22" s="135"/>
       <c r="B22" s="14" t="s">
         <v>44</v>
       </c>
@@ -5143,7 +5143,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="131"/>
+      <c r="A23" s="134"/>
       <c r="B23" s="20" t="s">
         <v>12</v>
       </c>
@@ -5156,7 +5156,7 @@
       <c r="E23" s="23"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="130" t="s">
+      <c r="A24" s="133" t="s">
         <v>54</v>
       </c>
       <c r="B24" s="77" t="s">
@@ -5174,7 +5174,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="132"/>
+      <c r="A25" s="135"/>
       <c r="B25" s="78" t="s">
         <v>56</v>
       </c>
@@ -5190,7 +5190,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="138"/>
+      <c r="A26" s="141"/>
       <c r="B26" s="82" t="s">
         <v>151</v>
       </c>
@@ -5203,7 +5203,7 @@
       <c r="E26" s="85"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="131"/>
+      <c r="A27" s="134"/>
       <c r="B27" s="81" t="s">
         <v>150</v>
       </c>
@@ -5216,7 +5216,7 @@
       <c r="E27" s="23"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="130" t="s">
+      <c r="A28" s="133" t="s">
         <v>57</v>
       </c>
       <c r="B28" s="77" t="s">
@@ -5231,7 +5231,7 @@
       <c r="E28" s="13"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="131"/>
+      <c r="A29" s="134"/>
       <c r="B29" s="81" t="s">
         <v>59</v>
       </c>
@@ -5244,7 +5244,7 @@
       <c r="E29" s="23"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="130" t="s">
+      <c r="A30" s="133" t="s">
         <v>60</v>
       </c>
       <c r="B30" s="91" t="s">
@@ -5262,7 +5262,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="132"/>
+      <c r="A31" s="135"/>
       <c r="B31" s="92" t="s">
         <v>44</v>
       </c>
@@ -5278,7 +5278,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="131"/>
+      <c r="A32" s="134"/>
       <c r="B32" s="93" t="s">
         <v>12</v>
       </c>
@@ -5291,7 +5291,7 @@
       <c r="E32" s="23"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="130" t="s">
+      <c r="A33" s="133" t="s">
         <v>61</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -5309,7 +5309,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="132"/>
+      <c r="A34" s="135"/>
       <c r="B34" s="14" t="s">
         <v>63</v>
       </c>
@@ -5325,7 +5325,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="131"/>
+      <c r="A35" s="134"/>
       <c r="B35" s="20" t="s">
         <v>12</v>
       </c>
@@ -5565,7 +5565,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="139" t="s">
+      <c r="A5" s="142" t="s">
         <v>75</v>
       </c>
       <c r="B5" s="77" t="s">
@@ -5583,7 +5583,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="140"/>
+      <c r="A6" s="143"/>
       <c r="B6" s="96" t="s">
         <v>12</v>
       </c>
@@ -5596,7 +5596,7 @@
       <c r="E6" s="19"/>
     </row>
     <row r="7" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="141"/>
+      <c r="A7" s="144"/>
       <c r="B7" s="78" t="s">
         <v>77</v>
       </c>
@@ -5609,7 +5609,7 @@
       <c r="E7" s="16"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="142" t="s">
+      <c r="A8" s="145" t="s">
         <v>79</v>
       </c>
       <c r="B8" s="78" t="s">
@@ -5624,7 +5624,7 @@
       <c r="E8" s="17"/>
     </row>
     <row r="9" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="143"/>
+      <c r="A9" s="146"/>
       <c r="B9" s="78" t="s">
         <v>76</v>
       </c>
@@ -5743,25 +5743,25 @@
       <c r="E6" s="23"/>
     </row>
     <row r="7" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="148" t="s">
+      <c r="A7" s="147" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="154" t="s">
-        <v>162</v>
-      </c>
-      <c r="C7" s="155" t="s">
+      <c r="B7" s="130" t="s">
+        <v>159</v>
+      </c>
+      <c r="C7" s="131" t="s">
         <v>67</v>
       </c>
       <c r="D7" s="120"/>
-      <c r="E7" s="156"/>
+      <c r="E7" s="132"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="150"/>
-      <c r="B8" s="154" t="s">
+      <c r="A8" s="148"/>
+      <c r="B8" s="130" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="119" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D8" s="120"/>
       <c r="E8" s="121"/>
@@ -5841,7 +5841,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="148" t="s">
+      <c r="A5" s="147" t="s">
         <v>40</v>
       </c>
       <c r="B5" s="77" t="s">
@@ -5859,7 +5859,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="149"/>
+      <c r="A6" s="153"/>
       <c r="B6" s="78" t="s">
         <v>43</v>
       </c>
@@ -5875,7 +5875,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="149"/>
+      <c r="A7" s="153"/>
       <c r="B7" s="78" t="s">
         <v>44</v>
       </c>
@@ -5891,7 +5891,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="150"/>
+      <c r="A8" s="148"/>
       <c r="B8" s="81" t="s">
         <v>12</v>
       </c>
@@ -5904,7 +5904,7 @@
       <c r="E8" s="60"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="151" t="s">
+      <c r="A9" s="154" t="s">
         <v>45</v>
       </c>
       <c r="B9" s="77" t="s">
@@ -5922,7 +5922,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="152"/>
+      <c r="A10" s="155"/>
       <c r="B10" s="78" t="s">
         <v>43</v>
       </c>
@@ -5938,7 +5938,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="152"/>
+      <c r="A11" s="155"/>
       <c r="B11" s="78" t="s">
         <v>44</v>
       </c>
@@ -5954,7 +5954,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="153"/>
+      <c r="A12" s="156"/>
       <c r="B12" s="81" t="s">
         <v>12</v>
       </c>
@@ -5969,7 +5969,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="139" t="s">
+      <c r="A13" s="142" t="s">
         <v>46</v>
       </c>
       <c r="B13" s="77" t="s">
@@ -5987,7 +5987,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="140"/>
+      <c r="A14" s="143"/>
       <c r="B14" s="78" t="s">
         <v>153</v>
       </c>
@@ -6003,7 +6003,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="140"/>
+      <c r="A15" s="143"/>
       <c r="B15" s="78" t="s">
         <v>12</v>
       </c>
@@ -6016,7 +6016,7 @@
       <c r="E15" s="66"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="140"/>
+      <c r="A16" s="143"/>
       <c r="B16" s="78" t="s">
         <v>47</v>
       </c>
@@ -6029,7 +6029,7 @@
       <c r="E16" s="64"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="140"/>
+      <c r="A17" s="143"/>
       <c r="B17" s="78" t="s">
         <v>49</v>
       </c>
@@ -6042,7 +6042,7 @@
       <c r="E17" s="67"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="140"/>
+      <c r="A18" s="143"/>
       <c r="B18" s="78" t="s">
         <v>50</v>
       </c>
@@ -6055,7 +6055,7 @@
       <c r="E18" s="67"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="140"/>
+      <c r="A19" s="143"/>
       <c r="B19" s="78" t="s">
         <v>51</v>
       </c>
@@ -6068,7 +6068,7 @@
       <c r="E19" s="67"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="147"/>
+      <c r="A20" s="152"/>
       <c r="B20" s="81" t="s">
         <v>52</v>
       </c>
@@ -6081,7 +6081,7 @@
       <c r="E20" s="68"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="139" t="s">
+      <c r="A21" s="142" t="s">
         <v>147</v>
       </c>
       <c r="B21" s="77" t="s">
@@ -6099,7 +6099,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="140"/>
+      <c r="A22" s="143"/>
       <c r="B22" s="14" t="s">
         <v>44</v>
       </c>
@@ -6115,7 +6115,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="147"/>
+      <c r="A23" s="152"/>
       <c r="B23" s="20" t="s">
         <v>12</v>
       </c>
@@ -6128,7 +6128,7 @@
       <c r="E23" s="70"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="139" t="s">
+      <c r="A24" s="142" t="s">
         <v>54</v>
       </c>
       <c r="B24" s="77" t="s">
@@ -6146,7 +6146,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="140"/>
+      <c r="A25" s="143"/>
       <c r="B25" s="78" t="s">
         <v>56</v>
       </c>
@@ -6162,7 +6162,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="140"/>
+      <c r="A26" s="143"/>
       <c r="B26" s="82" t="s">
         <v>150</v>
       </c>
@@ -6173,7 +6173,7 @@
       <c r="E26" s="75"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="147"/>
+      <c r="A27" s="152"/>
       <c r="B27" s="81" t="s">
         <v>151</v>
       </c>
@@ -6186,7 +6186,7 @@
       <c r="E27" s="71"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="139" t="s">
+      <c r="A28" s="142" t="s">
         <v>57</v>
       </c>
       <c r="B28" s="77" t="s">
@@ -6201,7 +6201,7 @@
       <c r="E28" s="72"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="147"/>
+      <c r="A29" s="152"/>
       <c r="B29" s="81" t="s">
         <v>59</v>
       </c>
@@ -6214,7 +6214,7 @@
       <c r="E29" s="71"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="144" t="s">
+      <c r="A30" s="149" t="s">
         <v>60</v>
       </c>
       <c r="B30" s="91" t="s">
@@ -6232,7 +6232,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="145"/>
+      <c r="A31" s="150"/>
       <c r="B31" s="92" t="s">
         <v>44</v>
       </c>
@@ -6248,7 +6248,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="146"/>
+      <c r="A32" s="151"/>
       <c r="B32" s="93" t="s">
         <v>12</v>
       </c>
@@ -6261,7 +6261,7 @@
       <c r="E32" s="73"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="139" t="s">
+      <c r="A33" s="142" t="s">
         <v>61</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -6279,7 +6279,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="140"/>
+      <c r="A34" s="143"/>
       <c r="B34" s="14" t="s">
         <v>63</v>
       </c>
@@ -6295,7 +6295,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="147"/>
+      <c r="A35" s="152"/>
       <c r="B35" s="20" t="s">
         <v>12</v>
       </c>
@@ -6602,26 +6602,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009342B7EAA7728A4FA80A5CCAFE8D7EAF" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d037a5681ee6af0e7b5b5d0a2f99b20">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557458c-24b5-4c97-84ed-4c402655f54f" xmlns:ns3="72e3c584-9879-4b35-b9d8-6a248c93e240" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="966978c8b125399653e7c255ac8e342d" ns2:_="" ns3:_="">
     <xsd:import namespace="9557458c-24b5-4c97-84ed-4c402655f54f"/>
@@ -6882,26 +6862,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
-    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6918,4 +6899,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ukf, nonlinear dampers, sweep matrics
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A2BC760-1654-E243-ACBD-98CD6C4E0CC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7450F1DA-89B1-0248-8C91-C6C607220012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23520" yWindow="1420" windowWidth="24720" windowHeight="19840" firstSheet="1" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="38400" windowHeight="22500" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Body" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
     <sheet name="HardpointsFr" sheetId="10" r:id="rId14"/>
     <sheet name="HardpointsRr" sheetId="11" r:id="rId15"/>
   </sheets>
-  <calcPr calcId="191028" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="166">
   <si>
     <t>Category</t>
   </si>
@@ -290,9 +290,6 @@
     <t>k</t>
   </si>
   <si>
-    <t>N/rad</t>
-  </si>
-  <si>
     <t>WheelDrivenRack1UJoint_Ch2_Achilles</t>
   </si>
   <si>
@@ -317,9 +314,6 @@
     <t>ARBRear</t>
   </si>
   <si>
-    <t>M</t>
-  </si>
-  <si>
     <t>Aero</t>
   </si>
   <si>
@@ -557,13 +551,25 @@
     <t>None</t>
   </si>
   <si>
-    <t>2 combined+turnslip</t>
-  </si>
-  <si>
-    <t>MFMbody</t>
-  </si>
-  <si>
-    <t>3 non-linear transients</t>
+    <t>Damper</t>
+  </si>
+  <si>
+    <t>N*m/deg</t>
+  </si>
+  <si>
+    <t>MFEval</t>
+  </si>
+  <si>
+    <t>1 steady state</t>
+  </si>
+  <si>
+    <t>1 combined</t>
+  </si>
+  <si>
+    <t>Nonlinear</t>
+  </si>
+  <si>
+    <t>TABLE</t>
   </si>
 </sst>
 </file>
@@ -574,7 +580,7 @@
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -604,6 +610,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1668,7 +1680,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="161">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2064,6 +2076,16 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="71" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3525,7 +3547,7 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -3536,7 +3558,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -3547,41 +3569,41 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="142" t="s">
-        <v>93</v>
+      <c r="A5" s="146" t="s">
+        <v>91</v>
       </c>
       <c r="B5" s="77" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="80" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="30"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="143"/>
+      <c r="A6" s="147"/>
       <c r="B6" s="97" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C6" s="98">
         <v>78807.070000000007</v>
       </c>
       <c r="D6" s="99" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E6" s="100"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="152"/>
+      <c r="A7" s="156"/>
       <c r="B7" s="81" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C7" s="21">
         <v>0</v>
@@ -3592,35 +3614,35 @@
       <c r="E7" s="33"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="142" t="s">
-        <v>97</v>
+      <c r="A8" s="146" t="s">
+        <v>95</v>
       </c>
       <c r="B8" s="77" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="102" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D8" s="12"/>
       <c r="E8" s="30"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="143"/>
+      <c r="A9" s="147"/>
       <c r="B9" s="97" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C9" s="101">
         <v>56916.22</v>
       </c>
       <c r="D9" s="99" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E9" s="100"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="152"/>
+      <c r="A10" s="156"/>
       <c r="B10" s="81" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C10" s="21">
         <v>0</v>
@@ -3677,8 +3699,8 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="8" t="s">
-        <v>91</v>
+      <c r="C2" s="105" t="s">
+        <v>159</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -3689,7 +3711,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -3700,93 +3722,95 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="142" t="s">
-        <v>93</v>
+      <c r="A5" s="146" t="s">
+        <v>91</v>
       </c>
       <c r="B5" s="77" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="80" t="s">
-        <v>94</v>
+        <v>164</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="30"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="143"/>
+      <c r="A6" s="147"/>
       <c r="B6" s="97" t="s">
-        <v>98</v>
-      </c>
-      <c r="C6" s="98">
-        <v>250000</v>
+        <v>96</v>
+      </c>
+      <c r="C6" s="134" t="s">
+        <v>96</v>
       </c>
       <c r="D6" s="99" t="s">
-        <v>96</v>
-      </c>
-      <c r="E6" s="100"/>
+        <v>94</v>
+      </c>
+      <c r="E6" s="135" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="143"/>
+      <c r="A7" s="147"/>
       <c r="B7" s="78" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C7" s="25">
         <v>100000</v>
       </c>
       <c r="D7" s="89" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E7" s="19"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="143"/>
+      <c r="A8" s="147"/>
       <c r="B8" s="78" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C8" s="25">
         <v>100000</v>
       </c>
       <c r="D8" s="89" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E8" s="19"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="143"/>
+      <c r="A9" s="147"/>
       <c r="B9" s="78" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C9" s="25">
         <v>150</v>
       </c>
       <c r="D9" s="89" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E9" s="19"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="143"/>
+      <c r="A10" s="147"/>
       <c r="B10" s="78" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C10" s="25">
         <v>150</v>
       </c>
       <c r="D10" s="89" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E10" s="19"/>
     </row>
     <row r="11" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="152"/>
+      <c r="A11" s="156"/>
       <c r="B11" s="81" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C11" s="27">
         <v>1E-4</v>
@@ -3797,87 +3821,89 @@
       <c r="E11" s="33"/>
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="142" t="s">
-        <v>97</v>
+      <c r="A12" s="146" t="s">
+        <v>95</v>
       </c>
       <c r="B12" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="103" t="s">
-        <v>94</v>
+      <c r="C12" s="80" t="s">
+        <v>164</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="30"/>
     </row>
     <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="143"/>
+      <c r="A13" s="147"/>
       <c r="B13" s="97" t="s">
-        <v>98</v>
-      </c>
-      <c r="C13" s="98">
-        <v>250000</v>
+        <v>96</v>
+      </c>
+      <c r="C13" s="134" t="s">
+        <v>96</v>
       </c>
       <c r="D13" s="104" t="s">
-        <v>96</v>
-      </c>
-      <c r="E13" s="100"/>
+        <v>94</v>
+      </c>
+      <c r="E13" s="135" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="143"/>
+      <c r="A14" s="147"/>
       <c r="B14" s="78" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C14" s="25">
         <v>100000</v>
       </c>
       <c r="D14" s="104" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E14" s="19"/>
     </row>
     <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="143"/>
+      <c r="A15" s="147"/>
       <c r="B15" s="78" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C15" s="25">
         <v>100000</v>
       </c>
       <c r="D15" s="104" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E15" s="19"/>
     </row>
     <row r="16" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="143"/>
+      <c r="A16" s="147"/>
       <c r="B16" s="78" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C16" s="25">
         <v>150</v>
       </c>
       <c r="D16" s="104" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E16" s="19"/>
     </row>
     <row r="17" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="143"/>
+      <c r="A17" s="147"/>
       <c r="B17" s="78" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C17" s="25">
         <v>150</v>
       </c>
       <c r="D17" s="104" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E17" s="19"/>
     </row>
     <row r="18" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="152"/>
+      <c r="A18" s="156"/>
       <c r="B18" s="81" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C18" s="27">
         <v>1E-4</v>
@@ -3902,9 +3928,818 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CD2A3BA-06BE-A64D-A72B-9CFCF024C1FD}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B101"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="136">
+        <v>-443.53</v>
+      </c>
+      <c r="B1" s="136">
+        <v>-3883.5949999999998</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="136">
+        <v>-433.58</v>
+      </c>
+      <c r="B2" s="136">
+        <v>-3833.1889999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="136">
+        <v>-423.97</v>
+      </c>
+      <c r="B3" s="136">
+        <v>-3778.5659999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="136">
+        <v>-415</v>
+      </c>
+      <c r="B4" s="136">
+        <v>-3715.607</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="136">
+        <v>-406.67</v>
+      </c>
+      <c r="B5" s="136">
+        <v>-3644.3130000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="136">
+        <v>-398.79</v>
+      </c>
+      <c r="B6" s="136">
+        <v>-3567.2330000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="136">
+        <v>-391.16</v>
+      </c>
+      <c r="B7" s="136">
+        <v>-3486.6219999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="136">
+        <v>-383.59</v>
+      </c>
+      <c r="B8" s="136">
+        <v>-3405.2269999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="136">
+        <v>-375.88</v>
+      </c>
+      <c r="B9" s="136">
+        <v>-3325.3029999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="136">
+        <v>-367.89</v>
+      </c>
+      <c r="B10" s="136">
+        <v>-3248.7130000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="136">
+        <v>-359.64</v>
+      </c>
+      <c r="B11" s="136">
+        <v>-3175.3589999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="136">
+        <v>-351.2</v>
+      </c>
+      <c r="B12" s="136">
+        <v>-3104.163</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" s="136">
+        <v>-342.63</v>
+      </c>
+      <c r="B13" s="136">
+        <v>-3034.5360000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" s="136">
+        <v>-334</v>
+      </c>
+      <c r="B14" s="136">
+        <v>-2965.6930000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" s="136">
+        <v>-325.38</v>
+      </c>
+      <c r="B15" s="136">
+        <v>-2896.85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="136">
+        <v>-316.77</v>
+      </c>
+      <c r="B16" s="136">
+        <v>-2827.6149999999998</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="136">
+        <v>-308.2</v>
+      </c>
+      <c r="B17" s="136">
+        <v>-2757.9879999999998</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="136">
+        <v>-299.64999999999998</v>
+      </c>
+      <c r="B18" s="136">
+        <v>-2687.9690000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="136">
+        <v>-291.14</v>
+      </c>
+      <c r="B19" s="136">
+        <v>-2617.5569999999998</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="136">
+        <v>-282.67</v>
+      </c>
+      <c r="B20" s="136">
+        <v>-2546.6550000000002</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="136">
+        <v>-274.25</v>
+      </c>
+      <c r="B21" s="136">
+        <v>-2475.1640000000002</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="136">
+        <v>-265.91000000000003</v>
+      </c>
+      <c r="B22" s="136">
+        <v>-2402.7910000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="136">
+        <v>-257.67</v>
+      </c>
+      <c r="B23" s="136">
+        <v>-2329.3389999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="136">
+        <v>-249.56</v>
+      </c>
+      <c r="B24" s="136">
+        <v>-2254.5149999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="136">
+        <v>-241.62</v>
+      </c>
+      <c r="B25" s="136">
+        <v>-2178.2190000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="136">
+        <v>-233.85</v>
+      </c>
+      <c r="B26" s="136">
+        <v>-2100.06</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="136">
+        <v>-226.23</v>
+      </c>
+      <c r="B27" s="136">
+        <v>-2020.528</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="136">
+        <v>-218.75</v>
+      </c>
+      <c r="B28" s="136">
+        <v>-1939.623</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="136">
+        <v>-211.37</v>
+      </c>
+      <c r="B29" s="136">
+        <v>-1857.934</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" s="136">
+        <v>-204.05</v>
+      </c>
+      <c r="B30" s="136">
+        <v>-1775.46</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" s="136">
+        <v>-196.78</v>
+      </c>
+      <c r="B31" s="136">
+        <v>-1692.79</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="136">
+        <v>-189.52</v>
+      </c>
+      <c r="B32" s="136">
+        <v>-1609.923</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="136">
+        <v>-182.26</v>
+      </c>
+      <c r="B33" s="136">
+        <v>-1527.155</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" s="136">
+        <v>-174.97</v>
+      </c>
+      <c r="B34" s="136">
+        <v>-1444.681</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" s="136">
+        <v>-167.65</v>
+      </c>
+      <c r="B35" s="136">
+        <v>-1362.502</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="136">
+        <v>-160.27000000000001</v>
+      </c>
+      <c r="B36" s="136">
+        <v>-1280.8119999999999</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" s="136">
+        <v>-152.82</v>
+      </c>
+      <c r="B37" s="136">
+        <v>-1199.711</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="136">
+        <v>-145.29</v>
+      </c>
+      <c r="B38" s="136">
+        <v>-1119.297</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="136">
+        <v>-137.65</v>
+      </c>
+      <c r="B39" s="136">
+        <v>-1039.7650000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="136">
+        <v>-129.9</v>
+      </c>
+      <c r="B40" s="136">
+        <v>-961.31200000000001</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="136">
+        <v>-122.02</v>
+      </c>
+      <c r="B41" s="136">
+        <v>-884.13300000000004</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="136">
+        <v>-114.01</v>
+      </c>
+      <c r="B42" s="136">
+        <v>-808.32799999999997</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="136">
+        <v>-105.84</v>
+      </c>
+      <c r="B43" s="136">
+        <v>-734.19</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" s="136">
+        <v>-97.52</v>
+      </c>
+      <c r="B44" s="136">
+        <v>-661.71799999999996</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="136">
+        <v>-89.05</v>
+      </c>
+      <c r="B45" s="136">
+        <v>-590.91399999999999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="136">
+        <v>-80.430000000000007</v>
+      </c>
+      <c r="B46" s="136">
+        <v>-521.67999999999995</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="136">
+        <v>-71.680000000000007</v>
+      </c>
+      <c r="B47" s="136">
+        <v>-454.21</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" s="136">
+        <v>-62.8</v>
+      </c>
+      <c r="B48" s="136">
+        <v>-388.113</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="136">
+        <v>-53.8</v>
+      </c>
+      <c r="B49" s="136">
+        <v>-323.68299999999999</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" s="136">
+        <v>-44.68</v>
+      </c>
+      <c r="B50" s="136">
+        <v>-260.92099999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" s="136">
+        <v>-35.409999999999997</v>
+      </c>
+      <c r="B51" s="136">
+        <v>-200.41399999999999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" s="136">
+        <v>-25.99</v>
+      </c>
+      <c r="B52" s="136">
+        <v>-142.26</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" s="136">
+        <v>-16.38</v>
+      </c>
+      <c r="B53" s="136">
+        <v>-86.950999999999993</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" s="136">
+        <v>-6.61</v>
+      </c>
+      <c r="B54" s="136">
+        <v>-34.387</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" s="136">
+        <v>0</v>
+      </c>
+      <c r="B55" s="136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" s="136">
+        <v>3.23</v>
+      </c>
+      <c r="B56" s="136">
+        <v>16.803999999999998</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" s="136">
+        <v>13.04</v>
+      </c>
+      <c r="B57" s="136">
+        <v>68.484999999999999</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" s="136">
+        <v>22.71</v>
+      </c>
+      <c r="B58" s="136">
+        <v>122.42100000000001</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" s="136">
+        <v>32.119999999999997</v>
+      </c>
+      <c r="B59" s="136">
+        <v>180.18199999999999</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" s="136">
+        <v>41.25</v>
+      </c>
+      <c r="B60" s="136">
+        <v>242.25899999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" s="136">
+        <v>50.17</v>
+      </c>
+      <c r="B61" s="136">
+        <v>307.66899999999998</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" s="136">
+        <v>58.93</v>
+      </c>
+      <c r="B62" s="136">
+        <v>375.33499999999998</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63" s="136">
+        <v>67.61</v>
+      </c>
+      <c r="B63" s="136">
+        <v>444.07900000000001</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64" s="136">
+        <v>76.28</v>
+      </c>
+      <c r="B64" s="136">
+        <v>512.92200000000003</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65" s="136">
+        <v>84.97</v>
+      </c>
+      <c r="B65" s="136">
+        <v>581.274</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66" s="136">
+        <v>93.66</v>
+      </c>
+      <c r="B66" s="136">
+        <v>649.33299999999997</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67" s="136">
+        <v>102.34</v>
+      </c>
+      <c r="B67" s="136">
+        <v>717.58699999999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" s="136">
+        <v>110.99</v>
+      </c>
+      <c r="B68" s="136">
+        <v>786.23299999999995</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" s="136">
+        <v>119.59</v>
+      </c>
+      <c r="B69" s="136">
+        <v>855.66399999999999</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" s="136">
+        <v>128.15</v>
+      </c>
+      <c r="B70" s="136">
+        <v>925.68399999999997</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" s="136">
+        <v>136.76</v>
+      </c>
+      <c r="B71" s="136">
+        <v>995.11500000000001</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72" s="136">
+        <v>145.5</v>
+      </c>
+      <c r="B72" s="136">
+        <v>1062.8789999999999</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" s="136">
+        <v>154.46</v>
+      </c>
+      <c r="B73" s="136">
+        <v>1127.6030000000001</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" s="136">
+        <v>163.72</v>
+      </c>
+      <c r="B74" s="136">
+        <v>1188.1099999999999</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" s="136">
+        <v>173.35</v>
+      </c>
+      <c r="B75" s="136">
+        <v>1243.3209999999999</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76" s="136">
+        <v>183.3</v>
+      </c>
+      <c r="B76" s="136">
+        <v>1293.0409999999999</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77" s="136">
+        <v>193.53</v>
+      </c>
+      <c r="B77" s="136">
+        <v>1336.877</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78" s="136">
+        <v>204</v>
+      </c>
+      <c r="B78" s="136">
+        <v>1374.829</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79" s="136">
+        <v>214.66</v>
+      </c>
+      <c r="B79" s="136">
+        <v>1406.7</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80" s="136">
+        <v>225.46</v>
+      </c>
+      <c r="B80" s="136">
+        <v>1433.2760000000001</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A81" s="136">
+        <v>236.35</v>
+      </c>
+      <c r="B81" s="136">
+        <v>1455.93</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A82" s="136">
+        <v>247.31</v>
+      </c>
+      <c r="B82" s="136">
+        <v>1476.0329999999999</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83" s="136">
+        <v>258.27999999999997</v>
+      </c>
+      <c r="B83" s="136">
+        <v>1494.8620000000001</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A84" s="136">
+        <v>269.26</v>
+      </c>
+      <c r="B84" s="136">
+        <v>1513.396</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A85" s="136">
+        <v>280.23</v>
+      </c>
+      <c r="B85" s="136">
+        <v>1531.8330000000001</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A86" s="136">
+        <v>291.19</v>
+      </c>
+      <c r="B86" s="136">
+        <v>1550.3679999999999</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A87" s="136">
+        <v>302.14999999999998</v>
+      </c>
+      <c r="B87" s="136">
+        <v>1569.2940000000001</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A88" s="136">
+        <v>313.10000000000002</v>
+      </c>
+      <c r="B88" s="136">
+        <v>1588.712</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A89" s="136">
+        <v>324.05</v>
+      </c>
+      <c r="B89" s="136">
+        <v>1608.325</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A90" s="136">
+        <v>335.01</v>
+      </c>
+      <c r="B90" s="136">
+        <v>1627.9380000000001</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A91" s="136">
+        <v>345.96</v>
+      </c>
+      <c r="B91" s="136">
+        <v>1647.2570000000001</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A92" s="136">
+        <v>356.92</v>
+      </c>
+      <c r="B92" s="136">
+        <v>1666.2819999999999</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A93" s="136">
+        <v>367.88</v>
+      </c>
+      <c r="B93" s="136">
+        <v>1685.6010000000001</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A94" s="136">
+        <v>378.83</v>
+      </c>
+      <c r="B94" s="136">
+        <v>1705.4110000000001</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A95" s="136">
+        <v>389.75</v>
+      </c>
+      <c r="B95" s="136">
+        <v>1726.3969999999999</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A96" s="136">
+        <v>400.65</v>
+      </c>
+      <c r="B96" s="136">
+        <v>1748.6579999999999</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A97" s="136">
+        <v>411.52</v>
+      </c>
+      <c r="B97" s="136">
+        <v>1772.39</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A98" s="136">
+        <v>422.35</v>
+      </c>
+      <c r="B98" s="136">
+        <v>1797.4949999999999</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A99" s="136">
+        <v>433.15</v>
+      </c>
+      <c r="B99" s="136">
+        <v>1823.973</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A100" s="136">
+        <v>443.91</v>
+      </c>
+      <c r="B100" s="136">
+        <v>1851.8240000000001</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A101" s="136">
+        <v>454.66</v>
+      </c>
+      <c r="B101" s="136">
+        <v>1880.3610000000001</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3942,7 +4777,7 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="105" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -3953,7 +4788,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="105" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -3964,29 +4799,29 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="105" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="95" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B5" s="77"/>
       <c r="C5" s="124" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D5" s="106" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E5" s="107" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="95" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B6" s="77"/>
       <c r="C6" s="103">
@@ -3999,33 +4834,33 @@
     </row>
     <row r="7" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="95" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B7" s="77"/>
       <c r="C7" s="103" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D7" s="106" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E7" s="30"/>
     </row>
     <row r="8" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="95" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B8" s="77"/>
       <c r="C8" s="108" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D8" s="106" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E8" s="30"/>
     </row>
     <row r="9" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="95" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B9" s="77"/>
       <c r="C9" s="103">
@@ -4036,36 +4871,36 @@
     </row>
     <row r="10" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="95" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B10" s="77"/>
       <c r="C10" s="103">
         <v>0.01</v>
       </c>
       <c r="D10" s="106" t="s">
+        <v>114</v>
+      </c>
+      <c r="E10" s="107" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="146" t="s">
         <v>116</v>
-      </c>
-      <c r="E10" s="107" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="142" t="s">
-        <v>118</v>
       </c>
       <c r="B11" s="109" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="110" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D11" s="94"/>
       <c r="E11" s="74"/>
     </row>
     <row r="12" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="152"/>
+      <c r="A12" s="156"/>
       <c r="B12" s="111" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C12" s="112" t="s">
         <v>11</v>
@@ -4077,22 +4912,22 @@
     </row>
     <row r="13" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="95" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B13" s="77"/>
       <c r="C13" s="103" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D13" s="106"/>
       <c r="E13" s="30"/>
     </row>
     <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="95" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B14" s="77"/>
       <c r="C14" s="103" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D14" s="106"/>
       <c r="E14" s="107"/>
@@ -4120,21 +4955,21 @@
   <sheetData>
     <row r="1" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="34" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="D1" s="34" t="s">
         <v>121</v>
-      </c>
-      <c r="C1" s="34" t="s">
-        <v>122</v>
-      </c>
-      <c r="D1" s="34" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="35" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B2" s="36">
         <v>200</v>
@@ -4148,7 +4983,7 @@
     </row>
     <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="38" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B3" s="39">
         <v>-200</v>
@@ -4162,7 +4997,7 @@
     </row>
     <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B4" s="39">
         <v>11.946</v>
@@ -4176,7 +5011,7 @@
     </row>
     <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B5" s="39">
         <v>148.751</v>
@@ -4190,7 +5025,7 @@
     </row>
     <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="38" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B6" s="39">
         <v>-184.72900000000001</v>
@@ -4204,7 +5039,7 @@
     </row>
     <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="38" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B7" s="39">
         <v>-12.932</v>
@@ -4218,7 +5053,7 @@
     </row>
     <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B8" s="39">
         <v>16.193999999999999</v>
@@ -4232,7 +5067,7 @@
     </row>
     <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="38" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B9" s="39">
         <v>0</v>
@@ -4246,7 +5081,7 @@
     </row>
     <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="38" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B10" s="39">
         <v>104.241</v>
@@ -4260,7 +5095,7 @@
     </row>
     <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="38" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B11" s="39">
         <v>85.097999999999999</v>
@@ -4274,7 +5109,7 @@
     </row>
     <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="38" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B12" s="39">
         <v>11.157</v>
@@ -4288,7 +5123,7 @@
     </row>
     <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B13" s="39">
         <v>11.484999999999999</v>
@@ -4302,7 +5137,7 @@
     </row>
     <row r="14" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="38" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B14" s="39">
         <v>11.821</v>
@@ -4316,7 +5151,7 @@
     </row>
     <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="38" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B15" s="39">
         <v>11.489000000000001</v>
@@ -4330,7 +5165,7 @@
     </row>
     <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="38" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B16" s="39">
         <v>11.558</v>
@@ -4344,7 +5179,7 @@
     </row>
     <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="38" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B17" s="39">
         <v>67.965000000000003</v>
@@ -4358,7 +5193,7 @@
     </row>
     <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="38" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B18" s="39">
         <v>4</v>
@@ -4372,7 +5207,7 @@
     </row>
     <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="38" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B19" s="39">
         <v>11.526999999999999</v>
@@ -4386,7 +5221,7 @@
     </row>
     <row r="20" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="38" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B20" s="39">
         <v>104.241</v>
@@ -4400,7 +5235,7 @@
     </row>
     <row r="21" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="38" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B21" s="39">
         <v>-324.96499999999997</v>
@@ -4436,21 +5271,21 @@
   <sheetData>
     <row r="1" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="34" t="s">
         <v>120</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="D1" s="34" t="s">
         <v>121</v>
-      </c>
-      <c r="C1" s="34" t="s">
-        <v>122</v>
-      </c>
-      <c r="D1" s="34" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="35" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B2" s="36">
         <v>-1390</v>
@@ -4464,7 +5299,7 @@
     </row>
     <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="38" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B3" s="39">
         <v>-1830</v>
@@ -4478,7 +5313,7 @@
     </row>
     <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B4" s="39">
         <v>-1579.2370000000001</v>
@@ -4492,7 +5327,7 @@
     </row>
     <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B5" s="39">
         <v>-1390</v>
@@ -4506,7 +5341,7 @@
     </row>
     <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="38" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B6" s="39">
         <v>-1830</v>
@@ -4520,7 +5355,7 @@
     </row>
     <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="38" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B7" s="39">
         <v>-1569.845</v>
@@ -4534,7 +5369,7 @@
     </row>
     <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B8" s="39">
         <v>-1568.8710000000001</v>
@@ -4548,7 +5383,7 @@
     </row>
     <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="38" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B9" s="39">
         <v>-1574.5989999999999</v>
@@ -4562,7 +5397,7 @@
     </row>
     <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="38" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B10" s="39">
         <v>-1830</v>
@@ -4576,7 +5411,7 @@
     </row>
     <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="38" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B11" s="39">
         <v>-1675.904</v>
@@ -4590,7 +5425,7 @@
     </row>
     <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="38" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B12" s="39">
         <v>-1395.9760000000001</v>
@@ -4604,7 +5439,7 @@
     </row>
     <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="38" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B13" s="39">
         <v>-1579.1110000000001</v>
@@ -4618,7 +5453,7 @@
     </row>
     <row r="14" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="38" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B14" s="39">
         <v>-1597.194</v>
@@ -4632,7 +5467,7 @@
     </row>
     <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="38" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B15" s="39">
         <v>-1664.6120000000001</v>
@@ -4646,7 +5481,7 @@
     </row>
     <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="38" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B16" s="39">
         <v>-1585.771</v>
@@ -4660,7 +5495,7 @@
     </row>
     <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="38" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B17" s="39">
         <v>-1830</v>
@@ -4674,7 +5509,7 @@
     </row>
     <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="38" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B18" s="39">
         <v>-1830</v>
@@ -4688,7 +5523,7 @@
     </row>
     <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="38" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B19" s="39">
         <v>-1600.4860000000001</v>
@@ -4775,7 +5610,7 @@
       </c>
       <c r="B5" s="117"/>
       <c r="C5" s="119" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D5" s="120" t="s">
         <v>66</v>
@@ -4879,7 +5714,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="136" t="s">
+      <c r="A5" s="140" t="s">
         <v>40</v>
       </c>
       <c r="B5" s="77" t="s">
@@ -4897,7 +5732,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="134"/>
+      <c r="A6" s="138"/>
       <c r="B6" s="78" t="s">
         <v>43</v>
       </c>
@@ -4913,7 +5748,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="137"/>
+      <c r="A7" s="141"/>
       <c r="B7" s="78" t="s">
         <v>44</v>
       </c>
@@ -4929,7 +5764,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="137"/>
+      <c r="A8" s="141"/>
       <c r="B8" s="81" t="s">
         <v>12</v>
       </c>
@@ -4942,7 +5777,7 @@
       <c r="E8" s="23"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="138" t="s">
+      <c r="A9" s="142" t="s">
         <v>45</v>
       </c>
       <c r="B9" s="77" t="s">
@@ -4960,7 +5795,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="135"/>
+      <c r="A10" s="139"/>
       <c r="B10" s="78" t="s">
         <v>43</v>
       </c>
@@ -4976,7 +5811,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="135"/>
+      <c r="A11" s="139"/>
       <c r="B11" s="78" t="s">
         <v>44</v>
       </c>
@@ -4992,7 +5827,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="134"/>
+      <c r="A12" s="138"/>
       <c r="B12" s="81" t="s">
         <v>12</v>
       </c>
@@ -5007,7 +5842,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="139" t="s">
+      <c r="A13" s="143" t="s">
         <v>46</v>
       </c>
       <c r="B13" s="77" t="s">
@@ -5025,9 +5860,9 @@
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="137"/>
+      <c r="A14" s="141"/>
       <c r="B14" s="78" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C14" s="25" t="str" cm="1">
         <f t="array" ref="C14">"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B9/1000,HardpointsFr!C9/1000,HardpointsFr!D9/1000)&amp;"]"</f>
@@ -5041,7 +5876,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="137"/>
+      <c r="A15" s="141"/>
       <c r="B15" s="78" t="s">
         <v>12</v>
       </c>
@@ -5054,7 +5889,7 @@
       <c r="E15" s="19"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="140"/>
+      <c r="A16" s="144"/>
       <c r="B16" s="78" t="s">
         <v>47</v>
       </c>
@@ -5067,7 +5902,7 @@
       <c r="E16" s="17"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="135"/>
+      <c r="A17" s="139"/>
       <c r="B17" s="78" t="s">
         <v>49</v>
       </c>
@@ -5080,7 +5915,7 @@
       <c r="E17" s="17"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="135"/>
+      <c r="A18" s="139"/>
       <c r="B18" s="78" t="s">
         <v>50</v>
       </c>
@@ -5093,7 +5928,7 @@
       <c r="E18" s="17"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="135"/>
+      <c r="A19" s="139"/>
       <c r="B19" s="78" t="s">
         <v>51</v>
       </c>
@@ -5106,7 +5941,7 @@
       <c r="E19" s="17"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="134"/>
+      <c r="A20" s="138"/>
       <c r="B20" s="81" t="s">
         <v>52</v>
       </c>
@@ -5119,8 +5954,8 @@
       <c r="E20" s="23"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="133" t="s">
-        <v>147</v>
+      <c r="A21" s="137" t="s">
+        <v>145</v>
       </c>
       <c r="B21" s="77" t="s">
         <v>53</v>
@@ -5137,7 +5972,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="135"/>
+      <c r="A22" s="139"/>
       <c r="B22" s="14" t="s">
         <v>44</v>
       </c>
@@ -5153,7 +5988,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="134"/>
+      <c r="A23" s="138"/>
       <c r="B23" s="20" t="s">
         <v>12</v>
       </c>
@@ -5166,7 +6001,7 @@
       <c r="E23" s="23"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="133" t="s">
+      <c r="A24" s="137" t="s">
         <v>54</v>
       </c>
       <c r="B24" s="77" t="s">
@@ -5184,7 +6019,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="135"/>
+      <c r="A25" s="139"/>
       <c r="B25" s="78" t="s">
         <v>56</v>
       </c>
@@ -5200,9 +6035,9 @@
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="141"/>
+      <c r="A26" s="145"/>
       <c r="B26" s="82" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C26" s="128">
         <v>1.2</v>
@@ -5213,9 +6048,9 @@
       <c r="E26" s="85"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="134"/>
+      <c r="A27" s="138"/>
       <c r="B27" s="81" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C27" s="21">
         <v>0.8</v>
@@ -5226,7 +6061,7 @@
       <c r="E27" s="23"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="133" t="s">
+      <c r="A28" s="137" t="s">
         <v>57</v>
       </c>
       <c r="B28" s="77" t="s">
@@ -5241,7 +6076,7 @@
       <c r="E28" s="13"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="134"/>
+      <c r="A29" s="138"/>
       <c r="B29" s="81" t="s">
         <v>59</v>
       </c>
@@ -5254,7 +6089,7 @@
       <c r="E29" s="23"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="133" t="s">
+      <c r="A30" s="137" t="s">
         <v>60</v>
       </c>
       <c r="B30" s="91" t="s">
@@ -5272,7 +6107,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="135"/>
+      <c r="A31" s="139"/>
       <c r="B31" s="92" t="s">
         <v>44</v>
       </c>
@@ -5288,7 +6123,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="134"/>
+      <c r="A32" s="138"/>
       <c r="B32" s="93" t="s">
         <v>12</v>
       </c>
@@ -5301,7 +6136,7 @@
       <c r="E32" s="23"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="133" t="s">
+      <c r="A33" s="137" t="s">
         <v>61</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -5319,7 +6154,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="135"/>
+      <c r="A34" s="139"/>
       <c r="B34" s="14" t="s">
         <v>63</v>
       </c>
@@ -5335,7 +6170,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="134"/>
+      <c r="A35" s="138"/>
       <c r="B35" s="20" t="s">
         <v>12</v>
       </c>
@@ -5483,8 +6318,8 @@
       <c r="C9" s="29">
         <v>81.933000000000007</v>
       </c>
-      <c r="D9" s="16" t="s">
-        <v>72</v>
+      <c r="D9" s="89" t="s">
+        <v>160</v>
       </c>
       <c r="E9" s="17"/>
     </row>
@@ -5558,7 +6393,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -5569,17 +6404,17 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="142" t="s">
+      <c r="A5" s="146" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="77" t="s">
         <v>75</v>
-      </c>
-      <c r="B5" s="77" t="s">
-        <v>76</v>
       </c>
       <c r="C5" s="44" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B20/1000,HardpointsFr!C20/1000,HardpointsFr!D20/1000)&amp;"]"</f>
@@ -5593,7 +6428,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="143"/>
+      <c r="A6" s="147"/>
       <c r="B6" s="96" t="s">
         <v>12</v>
       </c>
@@ -5606,21 +6441,21 @@
       <c r="E6" s="19"/>
     </row>
     <row r="7" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="144"/>
+      <c r="A7" s="148"/>
       <c r="B7" s="78" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C7" s="41">
         <v>50</v>
       </c>
       <c r="D7" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="E7" s="16"/>
+    </row>
+    <row r="8" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="149" t="s">
         <v>78</v>
-      </c>
-      <c r="E7" s="16"/>
-    </row>
-    <row r="8" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="145" t="s">
-        <v>79</v>
       </c>
       <c r="B8" s="78" t="s">
         <v>12</v>
@@ -5634,9 +6469,9 @@
       <c r="E8" s="17"/>
     </row>
     <row r="9" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="146"/>
+      <c r="A9" s="150"/>
       <c r="B9" s="78" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C9" s="41" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B21/1000,HardpointsFr!C21/1000,HardpointsFr!D21/1000)&amp;"]"</f>
@@ -5732,7 +6567,7 @@
       </c>
       <c r="B5" s="117"/>
       <c r="C5" s="119" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D5" s="120" t="s">
         <v>66</v>
@@ -5745,7 +6580,7 @@
       </c>
       <c r="B6" s="81"/>
       <c r="C6" s="88" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D6" s="90" t="s">
         <v>66</v>
@@ -5753,11 +6588,11 @@
       <c r="E6" s="23"/>
     </row>
     <row r="7" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="147" t="s">
+      <c r="A7" s="151" t="s">
         <v>67</v>
       </c>
       <c r="B7" s="130" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C7" s="131" t="s">
         <v>67</v>
@@ -5766,12 +6601,12 @@
       <c r="E7" s="132"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="148"/>
+      <c r="A8" s="152"/>
       <c r="B8" s="130" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="119" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D8" s="120"/>
       <c r="E8" s="121"/>
@@ -5845,13 +6680,13 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="105" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="147" t="s">
+      <c r="A5" s="151" t="s">
         <v>40</v>
       </c>
       <c r="B5" s="77" t="s">
@@ -5869,7 +6704,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="153"/>
+      <c r="A6" s="157"/>
       <c r="B6" s="78" t="s">
         <v>43</v>
       </c>
@@ -5885,7 +6720,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="153"/>
+      <c r="A7" s="157"/>
       <c r="B7" s="78" t="s">
         <v>44</v>
       </c>
@@ -5901,7 +6736,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="148"/>
+      <c r="A8" s="152"/>
       <c r="B8" s="81" t="s">
         <v>12</v>
       </c>
@@ -5914,7 +6749,7 @@
       <c r="E8" s="60"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="154" t="s">
+      <c r="A9" s="158" t="s">
         <v>45</v>
       </c>
       <c r="B9" s="77" t="s">
@@ -5932,7 +6767,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="155"/>
+      <c r="A10" s="159"/>
       <c r="B10" s="78" t="s">
         <v>43</v>
       </c>
@@ -5948,7 +6783,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="155"/>
+      <c r="A11" s="159"/>
       <c r="B11" s="78" t="s">
         <v>44</v>
       </c>
@@ -5964,7 +6799,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="156"/>
+      <c r="A12" s="160"/>
       <c r="B12" s="81" t="s">
         <v>12</v>
       </c>
@@ -5979,7 +6814,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="142" t="s">
+      <c r="A13" s="146" t="s">
         <v>46</v>
       </c>
       <c r="B13" s="77" t="s">
@@ -5997,9 +6832,9 @@
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="143"/>
+      <c r="A14" s="147"/>
       <c r="B14" s="78" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C14" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B9/1000 +1.575,HardpointsRr!C9/1000,HardpointsRr!D9/1000)&amp;"]"</f>
@@ -6013,7 +6848,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="143"/>
+      <c r="A15" s="147"/>
       <c r="B15" s="78" t="s">
         <v>12</v>
       </c>
@@ -6026,7 +6861,7 @@
       <c r="E15" s="66"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="143"/>
+      <c r="A16" s="147"/>
       <c r="B16" s="78" t="s">
         <v>47</v>
       </c>
@@ -6039,7 +6874,7 @@
       <c r="E16" s="64"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="143"/>
+      <c r="A17" s="147"/>
       <c r="B17" s="78" t="s">
         <v>49</v>
       </c>
@@ -6052,7 +6887,7 @@
       <c r="E17" s="67"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="143"/>
+      <c r="A18" s="147"/>
       <c r="B18" s="78" t="s">
         <v>50</v>
       </c>
@@ -6065,7 +6900,7 @@
       <c r="E18" s="67"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="143"/>
+      <c r="A19" s="147"/>
       <c r="B19" s="78" t="s">
         <v>51</v>
       </c>
@@ -6078,7 +6913,7 @@
       <c r="E19" s="67"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="152"/>
+      <c r="A20" s="156"/>
       <c r="B20" s="81" t="s">
         <v>52</v>
       </c>
@@ -6091,8 +6926,8 @@
       <c r="E20" s="68"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="142" t="s">
-        <v>147</v>
+      <c r="A21" s="146" t="s">
+        <v>145</v>
       </c>
       <c r="B21" s="77" t="s">
         <v>53</v>
@@ -6109,7 +6944,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="143"/>
+      <c r="A22" s="147"/>
       <c r="B22" s="14" t="s">
         <v>44</v>
       </c>
@@ -6125,7 +6960,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="152"/>
+      <c r="A23" s="156"/>
       <c r="B23" s="20" t="s">
         <v>12</v>
       </c>
@@ -6138,7 +6973,7 @@
       <c r="E23" s="70"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="142" t="s">
+      <c r="A24" s="146" t="s">
         <v>54</v>
       </c>
       <c r="B24" s="77" t="s">
@@ -6156,7 +6991,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="143"/>
+      <c r="A25" s="147"/>
       <c r="B25" s="78" t="s">
         <v>56</v>
       </c>
@@ -6172,9 +7007,9 @@
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="143"/>
+      <c r="A26" s="147"/>
       <c r="B26" s="82" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C26" s="128">
         <v>0.8</v>
@@ -6183,9 +7018,9 @@
       <c r="E26" s="75"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="152"/>
+      <c r="A27" s="156"/>
       <c r="B27" s="81" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C27" s="21">
         <v>1.2</v>
@@ -6196,7 +7031,7 @@
       <c r="E27" s="71"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="142" t="s">
+      <c r="A28" s="146" t="s">
         <v>57</v>
       </c>
       <c r="B28" s="77" t="s">
@@ -6211,7 +7046,7 @@
       <c r="E28" s="72"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="152"/>
+      <c r="A29" s="156"/>
       <c r="B29" s="81" t="s">
         <v>59</v>
       </c>
@@ -6224,7 +7059,7 @@
       <c r="E29" s="71"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="149" t="s">
+      <c r="A30" s="153" t="s">
         <v>60</v>
       </c>
       <c r="B30" s="91" t="s">
@@ -6242,7 +7077,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="150"/>
+      <c r="A31" s="154"/>
       <c r="B31" s="92" t="s">
         <v>44</v>
       </c>
@@ -6258,7 +7093,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="151"/>
+      <c r="A32" s="155"/>
       <c r="B32" s="93" t="s">
         <v>12</v>
       </c>
@@ -6271,7 +7106,7 @@
       <c r="E32" s="73"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="142" t="s">
+      <c r="A33" s="146" t="s">
         <v>61</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -6289,7 +7124,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="143"/>
+      <c r="A34" s="147"/>
       <c r="B34" s="14" t="s">
         <v>63</v>
       </c>
@@ -6305,7 +7140,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="152"/>
+      <c r="A35" s="156"/>
       <c r="B35" s="20" t="s">
         <v>12</v>
       </c>
@@ -6391,7 +7226,7 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="105" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="74"/>
@@ -6405,8 +7240,8 @@
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B19/1000+ 1.575,HardpointsRr!C19/1000,HardpointsRr!D19/1000)&amp;"]"</f>
         <v>[-0.0254860000000001 0.287566 0.463988]</v>
       </c>
-      <c r="D5" s="46" t="s">
-        <v>81</v>
+      <c r="D5" s="133" t="s">
+        <v>12</v>
       </c>
       <c r="E5" s="69" t="s">
         <v>42</v>
@@ -6452,8 +7287,8 @@
       <c r="C8" s="31">
         <v>61.879399999999997</v>
       </c>
-      <c r="D8" s="16" t="s">
-        <v>72</v>
+      <c r="D8" s="89" t="s">
+        <v>160</v>
       </c>
       <c r="E8" s="75"/>
     </row>
@@ -6514,7 +7349,7 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -6536,66 +7371,66 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="123" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B5" s="77"/>
       <c r="C5" s="24">
-        <v>-2.5</v>
+        <v>-2.15</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="30"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="123" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B6" s="78"/>
       <c r="C6" s="25">
-        <v>-1.5</v>
+        <v>-1</v>
       </c>
       <c r="D6" s="16"/>
       <c r="E6" s="19"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="123" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B7" s="78"/>
       <c r="C7" s="25">
         <v>1.2250000000000001</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E7" s="19"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="123" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B8" s="78"/>
       <c r="C8" s="25">
         <v>1.2</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E8" s="19"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="123" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B9" s="81"/>
       <c r="C9" s="32" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>30</v>
@@ -6612,6 +7447,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009342B7EAA7728A4FA80A5CCAFE8D7EAF" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d037a5681ee6af0e7b5b5d0a2f99b20">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557458c-24b5-4c97-84ed-4c402655f54f" xmlns:ns3="72e3c584-9879-4b35-b9d8-6a248c93e240" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="966978c8b125399653e7c255ac8e342d" ns2:_="" ns3:_="">
     <xsd:import namespace="9557458c-24b5-4c97-84ed-4c402655f54f"/>
@@ -6872,7 +7718,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -6881,18 +7727,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6911,21 +7757,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
-    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
few more fixes for the test rigs
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7450F1DA-89B1-0248-8C91-C6C607220012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C54C4FEB-37E6-4D43-A86D-3B84FC565924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="38400" windowHeight="22500" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10240" yWindow="4680" windowWidth="38400" windowHeight="22500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Body" sheetId="1" r:id="rId1"/>
@@ -7063,7 +7063,7 @@
         <v>60</v>
       </c>
       <c r="B30" s="91" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="C30" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B14/1000 + 1.575,HardpointsRr!C14/1000,HardpointsRr!D14/1000)&amp;"]"</f>
@@ -7079,7 +7079,7 @@
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="154"/>
       <c r="B31" s="92" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C31" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B15/1000 + 1.575,HardpointsRr!C15/1000,HardpointsRr!D15/1000)&amp;"]"</f>
@@ -7447,14 +7447,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7719,21 +7717,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
-    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7758,9 +7755,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
arb values added for 1deg/g config ukf parameters update
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C54C4FEB-37E6-4D43-A86D-3B84FC565924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1148AFD4-1C52-5042-B19A-BC7114E09693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10240" yWindow="4680" windowWidth="38400" windowHeight="22500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12320" yWindow="1400" windowWidth="38400" windowHeight="22500" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Body" sheetId="1" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="168">
   <si>
     <t>Category</t>
   </si>
@@ -557,28 +557,35 @@
     <t>N*m/deg</t>
   </si>
   <si>
+    <t>Nonlinear</t>
+  </si>
+  <si>
+    <t>TABLE</t>
+  </si>
+  <si>
+    <t>(1 steady state, 2 linear transients, 3 non-linear transients)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
     <t>MFEval</t>
   </si>
   <si>
+    <t>2 combined+turnslip</t>
+  </si>
+  <si>
     <t>1 steady state</t>
-  </si>
-  <si>
-    <t>1 combined</t>
-  </si>
-  <si>
-    <t>Nonlinear</t>
-  </si>
-  <si>
-    <t>TABLE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="#,##0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -1680,7 +1687,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1764,9 +1771,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2086,6 +2090,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="3" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2103,9 +2120,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="58" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2131,9 +2145,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3342,11 +3353,11 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="122" t="s">
+      <c r="A5" s="121" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="77"/>
-      <c r="C5" s="80" t="s">
+      <c r="B5" s="76"/>
+      <c r="C5" s="79" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="12" t="s">
@@ -3357,11 +3368,11 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="122" t="s">
+      <c r="A6" s="121" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="78"/>
-      <c r="C6" s="79" t="s">
+      <c r="B6" s="77"/>
+      <c r="C6" s="78" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="16" t="s">
@@ -3372,10 +3383,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="122" t="s">
+      <c r="A7" s="121" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="78"/>
+      <c r="B7" s="77"/>
       <c r="C7" s="15" t="s">
         <v>18</v>
       </c>
@@ -3385,11 +3396,11 @@
       <c r="E7" s="17"/>
     </row>
     <row r="8" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="122" t="s">
+      <c r="A8" s="121" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="78"/>
-      <c r="C8" s="79" t="s">
+      <c r="B8" s="77"/>
+      <c r="C8" s="78" t="s">
         <v>20</v>
       </c>
       <c r="D8" s="16" t="s">
@@ -3400,11 +3411,11 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="122" t="s">
+      <c r="A9" s="121" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="78"/>
-      <c r="C9" s="79" t="s">
+      <c r="B9" s="77"/>
+      <c r="C9" s="78" t="s">
         <v>23</v>
       </c>
       <c r="D9" s="16" t="s">
@@ -3415,11 +3426,11 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="122" t="s">
+      <c r="A10" s="121" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="78"/>
-      <c r="C10" s="79" t="s">
+      <c r="B10" s="77"/>
+      <c r="C10" s="78" t="s">
         <v>25</v>
       </c>
       <c r="D10" s="16" t="s">
@@ -3430,7 +3441,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="122" t="s">
+      <c r="A11" s="121" t="s">
         <v>26</v>
       </c>
       <c r="B11" s="14"/>
@@ -3446,10 +3457,10 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="122" t="s">
+      <c r="A12" s="121" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="78"/>
+      <c r="B12" s="77"/>
       <c r="C12" s="18">
         <f>HardpointsFr!C9*2/1000</f>
         <v>1.28</v>
@@ -3460,10 +3471,10 @@
       <c r="E12" s="17"/>
     </row>
     <row r="13" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="122" t="s">
+      <c r="A13" s="121" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="78"/>
+      <c r="B13" s="77"/>
       <c r="C13" s="18">
         <f>HardpointsRr!C9*2/1000</f>
         <v>1.2470640000000002</v>
@@ -3474,32 +3485,32 @@
       <c r="E13" s="19"/>
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="122" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="82"/>
-      <c r="C14" s="84">
+      <c r="A14" s="121" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="81"/>
+      <c r="C14" s="83">
         <v>259.07</v>
       </c>
-      <c r="D14" s="83" t="s">
+      <c r="D14" s="82" t="s">
         <v>30</v>
       </c>
-      <c r="E14" s="85" t="s">
+      <c r="E14" s="84" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="122" t="s">
+      <c r="A15" s="121" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="78"/>
-      <c r="C15" s="87" t="s">
+      <c r="B15" s="77"/>
+      <c r="C15" s="86" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="89" t="s">
+      <c r="D15" s="88" t="s">
         <v>34</v>
       </c>
-      <c r="E15" s="86" t="s">
+      <c r="E15" s="85" t="s">
         <v>35</v>
       </c>
     </row>
@@ -3575,34 +3586,34 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="146" t="s">
+      <c r="A5" s="139" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="77" t="s">
+      <c r="B5" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="80" t="s">
+      <c r="C5" s="79" t="s">
         <v>92</v>
       </c>
       <c r="D5" s="12"/>
-      <c r="E5" s="30"/>
+      <c r="E5" s="29"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="147"/>
-      <c r="B6" s="97" t="s">
+      <c r="A6" s="150"/>
+      <c r="B6" s="96" t="s">
         <v>93</v>
       </c>
-      <c r="C6" s="98">
+      <c r="C6" s="97">
         <v>78807.070000000007</v>
       </c>
-      <c r="D6" s="99" t="s">
+      <c r="D6" s="98" t="s">
         <v>94</v>
       </c>
-      <c r="E6" s="100"/>
+      <c r="E6" s="99"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="156"/>
-      <c r="B7" s="81" t="s">
+      <c r="A7" s="140"/>
+      <c r="B7" s="80" t="s">
         <v>146</v>
       </c>
       <c r="C7" s="21">
@@ -3611,46 +3622,46 @@
       <c r="D7" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="33"/>
+      <c r="E7" s="32"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="146" t="s">
+      <c r="A8" s="139" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="77" t="s">
+      <c r="B8" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="102" t="s">
+      <c r="C8" s="101" t="s">
         <v>92</v>
       </c>
       <c r="D8" s="12"/>
-      <c r="E8" s="30"/>
+      <c r="E8" s="29"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="147"/>
-      <c r="B9" s="97" t="s">
+      <c r="A9" s="150"/>
+      <c r="B9" s="96" t="s">
         <v>93</v>
       </c>
-      <c r="C9" s="101">
+      <c r="C9" s="100">
         <v>56916.22</v>
       </c>
-      <c r="D9" s="99" t="s">
+      <c r="D9" s="98" t="s">
         <v>94</v>
       </c>
-      <c r="E9" s="100"/>
+      <c r="E9" s="99"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="156"/>
-      <c r="B10" s="81" t="s">
+      <c r="A10" s="140"/>
+      <c r="B10" s="80" t="s">
         <v>146</v>
       </c>
       <c r="C10" s="21">
         <v>0</v>
       </c>
-      <c r="D10" s="90" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="33"/>
+      <c r="D10" s="89" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3699,7 +3710,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="105" t="s">
+      <c r="C2" s="104" t="s">
         <v>159</v>
       </c>
       <c r="D2" s="9"/>
@@ -3728,190 +3739,190 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="146" t="s">
+      <c r="A5" s="139" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="77" t="s">
+      <c r="B5" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="80" t="s">
-        <v>164</v>
+      <c r="C5" s="79" t="s">
+        <v>161</v>
       </c>
       <c r="D5" s="12"/>
-      <c r="E5" s="30"/>
+      <c r="E5" s="29"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="147"/>
-      <c r="B6" s="97" t="s">
+      <c r="A6" s="150"/>
+      <c r="B6" s="96" t="s">
         <v>96</v>
       </c>
-      <c r="C6" s="134" t="s">
+      <c r="C6" s="133" t="s">
         <v>96</v>
       </c>
-      <c r="D6" s="99" t="s">
+      <c r="D6" s="98" t="s">
         <v>94</v>
       </c>
-      <c r="E6" s="135" t="s">
-        <v>165</v>
+      <c r="E6" s="134" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="147"/>
-      <c r="B7" s="78" t="s">
+      <c r="A7" s="150"/>
+      <c r="B7" s="77" t="s">
         <v>97</v>
       </c>
       <c r="C7" s="25">
         <v>100000</v>
       </c>
-      <c r="D7" s="89" t="s">
+      <c r="D7" s="88" t="s">
         <v>94</v>
       </c>
       <c r="E7" s="19"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="147"/>
-      <c r="B8" s="78" t="s">
+      <c r="A8" s="150"/>
+      <c r="B8" s="77" t="s">
         <v>98</v>
       </c>
       <c r="C8" s="25">
         <v>100000</v>
       </c>
-      <c r="D8" s="89" t="s">
+      <c r="D8" s="88" t="s">
         <v>94</v>
       </c>
       <c r="E8" s="19"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="147"/>
-      <c r="B9" s="78" t="s">
+      <c r="A9" s="150"/>
+      <c r="B9" s="77" t="s">
         <v>99</v>
       </c>
       <c r="C9" s="25">
         <v>150</v>
       </c>
-      <c r="D9" s="89" t="s">
+      <c r="D9" s="88" t="s">
         <v>94</v>
       </c>
       <c r="E9" s="19"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="147"/>
-      <c r="B10" s="78" t="s">
+      <c r="A10" s="150"/>
+      <c r="B10" s="77" t="s">
         <v>100</v>
       </c>
       <c r="C10" s="25">
         <v>150</v>
       </c>
-      <c r="D10" s="89" t="s">
+      <c r="D10" s="88" t="s">
         <v>94</v>
       </c>
       <c r="E10" s="19"/>
     </row>
     <row r="11" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="156"/>
-      <c r="B11" s="81" t="s">
+      <c r="A11" s="140"/>
+      <c r="B11" s="80" t="s">
         <v>101</v>
       </c>
       <c r="C11" s="27">
         <v>1E-4</v>
       </c>
-      <c r="D11" s="90" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="33"/>
+      <c r="D11" s="89" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="32"/>
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="146" t="s">
+      <c r="A12" s="139" t="s">
         <v>95</v>
       </c>
-      <c r="B12" s="77" t="s">
+      <c r="B12" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="80" t="s">
-        <v>164</v>
+      <c r="C12" s="79" t="s">
+        <v>161</v>
       </c>
       <c r="D12" s="12"/>
-      <c r="E12" s="30"/>
+      <c r="E12" s="29"/>
     </row>
     <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="147"/>
-      <c r="B13" s="97" t="s">
+      <c r="A13" s="150"/>
+      <c r="B13" s="96" t="s">
         <v>96</v>
       </c>
-      <c r="C13" s="134" t="s">
+      <c r="C13" s="133" t="s">
         <v>96</v>
       </c>
-      <c r="D13" s="104" t="s">
+      <c r="D13" s="103" t="s">
         <v>94</v>
       </c>
-      <c r="E13" s="135" t="s">
-        <v>165</v>
+      <c r="E13" s="134" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="147"/>
-      <c r="B14" s="78" t="s">
+      <c r="A14" s="150"/>
+      <c r="B14" s="77" t="s">
         <v>97</v>
       </c>
       <c r="C14" s="25">
         <v>100000</v>
       </c>
-      <c r="D14" s="104" t="s">
+      <c r="D14" s="103" t="s">
         <v>94</v>
       </c>
       <c r="E14" s="19"/>
     </row>
     <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="147"/>
-      <c r="B15" s="78" t="s">
+      <c r="A15" s="150"/>
+      <c r="B15" s="77" t="s">
         <v>98</v>
       </c>
       <c r="C15" s="25">
         <v>100000</v>
       </c>
-      <c r="D15" s="104" t="s">
+      <c r="D15" s="103" t="s">
         <v>94</v>
       </c>
       <c r="E15" s="19"/>
     </row>
     <row r="16" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="147"/>
-      <c r="B16" s="78" t="s">
+      <c r="A16" s="150"/>
+      <c r="B16" s="77" t="s">
         <v>99</v>
       </c>
       <c r="C16" s="25">
         <v>150</v>
       </c>
-      <c r="D16" s="104" t="s">
+      <c r="D16" s="103" t="s">
         <v>94</v>
       </c>
       <c r="E16" s="19"/>
     </row>
     <row r="17" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="147"/>
-      <c r="B17" s="78" t="s">
+      <c r="A17" s="150"/>
+      <c r="B17" s="77" t="s">
         <v>100</v>
       </c>
       <c r="C17" s="25">
         <v>150</v>
       </c>
-      <c r="D17" s="104" t="s">
+      <c r="D17" s="103" t="s">
         <v>94</v>
       </c>
       <c r="E17" s="19"/>
     </row>
     <row r="18" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="156"/>
-      <c r="B18" s="81" t="s">
+      <c r="A18" s="140"/>
+      <c r="B18" s="80" t="s">
         <v>101</v>
       </c>
       <c r="C18" s="27">
         <v>1E-4</v>
       </c>
-      <c r="D18" s="90" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="33"/>
+      <c r="D18" s="89" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3932,810 +3943,810 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="136">
+      <c r="A1" s="135">
         <v>-443.53</v>
       </c>
-      <c r="B1" s="136">
+      <c r="B1" s="135">
         <v>-3883.5949999999998</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="136">
+      <c r="A2" s="135">
         <v>-433.58</v>
       </c>
-      <c r="B2" s="136">
+      <c r="B2" s="135">
         <v>-3833.1889999999999</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="136">
+      <c r="A3" s="135">
         <v>-423.97</v>
       </c>
-      <c r="B3" s="136">
+      <c r="B3" s="135">
         <v>-3778.5659999999998</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="136">
+      <c r="A4" s="135">
         <v>-415</v>
       </c>
-      <c r="B4" s="136">
+      <c r="B4" s="135">
         <v>-3715.607</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="136">
+      <c r="A5" s="135">
         <v>-406.67</v>
       </c>
-      <c r="B5" s="136">
+      <c r="B5" s="135">
         <v>-3644.3130000000001</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="136">
+      <c r="A6" s="135">
         <v>-398.79</v>
       </c>
-      <c r="B6" s="136">
+      <c r="B6" s="135">
         <v>-3567.2330000000002</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="136">
+      <c r="A7" s="135">
         <v>-391.16</v>
       </c>
-      <c r="B7" s="136">
+      <c r="B7" s="135">
         <v>-3486.6219999999998</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="136">
+      <c r="A8" s="135">
         <v>-383.59</v>
       </c>
-      <c r="B8" s="136">
+      <c r="B8" s="135">
         <v>-3405.2269999999999</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="136">
+      <c r="A9" s="135">
         <v>-375.88</v>
       </c>
-      <c r="B9" s="136">
+      <c r="B9" s="135">
         <v>-3325.3029999999999</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="136">
+      <c r="A10" s="135">
         <v>-367.89</v>
       </c>
-      <c r="B10" s="136">
+      <c r="B10" s="135">
         <v>-3248.7130000000002</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="136">
+      <c r="A11" s="135">
         <v>-359.64</v>
       </c>
-      <c r="B11" s="136">
+      <c r="B11" s="135">
         <v>-3175.3589999999999</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="136">
+      <c r="A12" s="135">
         <v>-351.2</v>
       </c>
-      <c r="B12" s="136">
+      <c r="B12" s="135">
         <v>-3104.163</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="136">
+      <c r="A13" s="135">
         <v>-342.63</v>
       </c>
-      <c r="B13" s="136">
+      <c r="B13" s="135">
         <v>-3034.5360000000001</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="136">
+      <c r="A14" s="135">
         <v>-334</v>
       </c>
-      <c r="B14" s="136">
+      <c r="B14" s="135">
         <v>-2965.6930000000002</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" s="136">
+      <c r="A15" s="135">
         <v>-325.38</v>
       </c>
-      <c r="B15" s="136">
+      <c r="B15" s="135">
         <v>-2896.85</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="136">
+      <c r="A16" s="135">
         <v>-316.77</v>
       </c>
-      <c r="B16" s="136">
+      <c r="B16" s="135">
         <v>-2827.6149999999998</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="136">
+      <c r="A17" s="135">
         <v>-308.2</v>
       </c>
-      <c r="B17" s="136">
+      <c r="B17" s="135">
         <v>-2757.9879999999998</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="136">
+      <c r="A18" s="135">
         <v>-299.64999999999998</v>
       </c>
-      <c r="B18" s="136">
+      <c r="B18" s="135">
         <v>-2687.9690000000001</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="136">
+      <c r="A19" s="135">
         <v>-291.14</v>
       </c>
-      <c r="B19" s="136">
+      <c r="B19" s="135">
         <v>-2617.5569999999998</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="136">
+      <c r="A20" s="135">
         <v>-282.67</v>
       </c>
-      <c r="B20" s="136">
+      <c r="B20" s="135">
         <v>-2546.6550000000002</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="136">
+      <c r="A21" s="135">
         <v>-274.25</v>
       </c>
-      <c r="B21" s="136">
+      <c r="B21" s="135">
         <v>-2475.1640000000002</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="136">
+      <c r="A22" s="135">
         <v>-265.91000000000003</v>
       </c>
-      <c r="B22" s="136">
+      <c r="B22" s="135">
         <v>-2402.7910000000002</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="136">
+      <c r="A23" s="135">
         <v>-257.67</v>
       </c>
-      <c r="B23" s="136">
+      <c r="B23" s="135">
         <v>-2329.3389999999999</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" s="136">
+      <c r="A24" s="135">
         <v>-249.56</v>
       </c>
-      <c r="B24" s="136">
+      <c r="B24" s="135">
         <v>-2254.5149999999999</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25" s="136">
+      <c r="A25" s="135">
         <v>-241.62</v>
       </c>
-      <c r="B25" s="136">
+      <c r="B25" s="135">
         <v>-2178.2190000000001</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" s="136">
+      <c r="A26" s="135">
         <v>-233.85</v>
       </c>
-      <c r="B26" s="136">
+      <c r="B26" s="135">
         <v>-2100.06</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27" s="136">
+      <c r="A27" s="135">
         <v>-226.23</v>
       </c>
-      <c r="B27" s="136">
+      <c r="B27" s="135">
         <v>-2020.528</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A28" s="136">
+      <c r="A28" s="135">
         <v>-218.75</v>
       </c>
-      <c r="B28" s="136">
+      <c r="B28" s="135">
         <v>-1939.623</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" s="136">
+      <c r="A29" s="135">
         <v>-211.37</v>
       </c>
-      <c r="B29" s="136">
+      <c r="B29" s="135">
         <v>-1857.934</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A30" s="136">
+      <c r="A30" s="135">
         <v>-204.05</v>
       </c>
-      <c r="B30" s="136">
+      <c r="B30" s="135">
         <v>-1775.46</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A31" s="136">
+      <c r="A31" s="135">
         <v>-196.78</v>
       </c>
-      <c r="B31" s="136">
+      <c r="B31" s="135">
         <v>-1692.79</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A32" s="136">
+      <c r="A32" s="135">
         <v>-189.52</v>
       </c>
-      <c r="B32" s="136">
+      <c r="B32" s="135">
         <v>-1609.923</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" s="136">
+      <c r="A33" s="135">
         <v>-182.26</v>
       </c>
-      <c r="B33" s="136">
+      <c r="B33" s="135">
         <v>-1527.155</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A34" s="136">
+      <c r="A34" s="135">
         <v>-174.97</v>
       </c>
-      <c r="B34" s="136">
+      <c r="B34" s="135">
         <v>-1444.681</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" s="136">
+      <c r="A35" s="135">
         <v>-167.65</v>
       </c>
-      <c r="B35" s="136">
+      <c r="B35" s="135">
         <v>-1362.502</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" s="136">
+      <c r="A36" s="135">
         <v>-160.27000000000001</v>
       </c>
-      <c r="B36" s="136">
+      <c r="B36" s="135">
         <v>-1280.8119999999999</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" s="136">
+      <c r="A37" s="135">
         <v>-152.82</v>
       </c>
-      <c r="B37" s="136">
+      <c r="B37" s="135">
         <v>-1199.711</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" s="136">
+      <c r="A38" s="135">
         <v>-145.29</v>
       </c>
-      <c r="B38" s="136">
+      <c r="B38" s="135">
         <v>-1119.297</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A39" s="136">
+      <c r="A39" s="135">
         <v>-137.65</v>
       </c>
-      <c r="B39" s="136">
+      <c r="B39" s="135">
         <v>-1039.7650000000001</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A40" s="136">
+      <c r="A40" s="135">
         <v>-129.9</v>
       </c>
-      <c r="B40" s="136">
+      <c r="B40" s="135">
         <v>-961.31200000000001</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A41" s="136">
+      <c r="A41" s="135">
         <v>-122.02</v>
       </c>
-      <c r="B41" s="136">
+      <c r="B41" s="135">
         <v>-884.13300000000004</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" s="136">
+      <c r="A42" s="135">
         <v>-114.01</v>
       </c>
-      <c r="B42" s="136">
+      <c r="B42" s="135">
         <v>-808.32799999999997</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A43" s="136">
+      <c r="A43" s="135">
         <v>-105.84</v>
       </c>
-      <c r="B43" s="136">
+      <c r="B43" s="135">
         <v>-734.19</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A44" s="136">
+      <c r="A44" s="135">
         <v>-97.52</v>
       </c>
-      <c r="B44" s="136">
+      <c r="B44" s="135">
         <v>-661.71799999999996</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A45" s="136">
+      <c r="A45" s="135">
         <v>-89.05</v>
       </c>
-      <c r="B45" s="136">
+      <c r="B45" s="135">
         <v>-590.91399999999999</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A46" s="136">
+      <c r="A46" s="135">
         <v>-80.430000000000007</v>
       </c>
-      <c r="B46" s="136">
+      <c r="B46" s="135">
         <v>-521.67999999999995</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A47" s="136">
+      <c r="A47" s="135">
         <v>-71.680000000000007</v>
       </c>
-      <c r="B47" s="136">
+      <c r="B47" s="135">
         <v>-454.21</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A48" s="136">
+      <c r="A48" s="135">
         <v>-62.8</v>
       </c>
-      <c r="B48" s="136">
+      <c r="B48" s="135">
         <v>-388.113</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A49" s="136">
+      <c r="A49" s="135">
         <v>-53.8</v>
       </c>
-      <c r="B49" s="136">
+      <c r="B49" s="135">
         <v>-323.68299999999999</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A50" s="136">
+      <c r="A50" s="135">
         <v>-44.68</v>
       </c>
-      <c r="B50" s="136">
+      <c r="B50" s="135">
         <v>-260.92099999999999</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A51" s="136">
+      <c r="A51" s="135">
         <v>-35.409999999999997</v>
       </c>
-      <c r="B51" s="136">
+      <c r="B51" s="135">
         <v>-200.41399999999999</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A52" s="136">
+      <c r="A52" s="135">
         <v>-25.99</v>
       </c>
-      <c r="B52" s="136">
+      <c r="B52" s="135">
         <v>-142.26</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A53" s="136">
+      <c r="A53" s="135">
         <v>-16.38</v>
       </c>
-      <c r="B53" s="136">
+      <c r="B53" s="135">
         <v>-86.950999999999993</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A54" s="136">
+      <c r="A54" s="135">
         <v>-6.61</v>
       </c>
-      <c r="B54" s="136">
+      <c r="B54" s="135">
         <v>-34.387</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A55" s="136">
+      <c r="A55" s="135">
         <v>0</v>
       </c>
-      <c r="B55" s="136">
+      <c r="B55" s="135">
         <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A56" s="136">
+      <c r="A56" s="135">
         <v>3.23</v>
       </c>
-      <c r="B56" s="136">
+      <c r="B56" s="135">
         <v>16.803999999999998</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A57" s="136">
+      <c r="A57" s="135">
         <v>13.04</v>
       </c>
-      <c r="B57" s="136">
+      <c r="B57" s="135">
         <v>68.484999999999999</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A58" s="136">
+      <c r="A58" s="135">
         <v>22.71</v>
       </c>
-      <c r="B58" s="136">
+      <c r="B58" s="135">
         <v>122.42100000000001</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A59" s="136">
+      <c r="A59" s="135">
         <v>32.119999999999997</v>
       </c>
-      <c r="B59" s="136">
+      <c r="B59" s="135">
         <v>180.18199999999999</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A60" s="136">
+      <c r="A60" s="135">
         <v>41.25</v>
       </c>
-      <c r="B60" s="136">
+      <c r="B60" s="135">
         <v>242.25899999999999</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A61" s="136">
+      <c r="A61" s="135">
         <v>50.17</v>
       </c>
-      <c r="B61" s="136">
+      <c r="B61" s="135">
         <v>307.66899999999998</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A62" s="136">
+      <c r="A62" s="135">
         <v>58.93</v>
       </c>
-      <c r="B62" s="136">
+      <c r="B62" s="135">
         <v>375.33499999999998</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A63" s="136">
+      <c r="A63" s="135">
         <v>67.61</v>
       </c>
-      <c r="B63" s="136">
+      <c r="B63" s="135">
         <v>444.07900000000001</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A64" s="136">
+      <c r="A64" s="135">
         <v>76.28</v>
       </c>
-      <c r="B64" s="136">
+      <c r="B64" s="135">
         <v>512.92200000000003</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A65" s="136">
+      <c r="A65" s="135">
         <v>84.97</v>
       </c>
-      <c r="B65" s="136">
+      <c r="B65" s="135">
         <v>581.274</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A66" s="136">
+      <c r="A66" s="135">
         <v>93.66</v>
       </c>
-      <c r="B66" s="136">
+      <c r="B66" s="135">
         <v>649.33299999999997</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A67" s="136">
+      <c r="A67" s="135">
         <v>102.34</v>
       </c>
-      <c r="B67" s="136">
+      <c r="B67" s="135">
         <v>717.58699999999999</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A68" s="136">
+      <c r="A68" s="135">
         <v>110.99</v>
       </c>
-      <c r="B68" s="136">
+      <c r="B68" s="135">
         <v>786.23299999999995</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A69" s="136">
+      <c r="A69" s="135">
         <v>119.59</v>
       </c>
-      <c r="B69" s="136">
+      <c r="B69" s="135">
         <v>855.66399999999999</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A70" s="136">
+      <c r="A70" s="135">
         <v>128.15</v>
       </c>
-      <c r="B70" s="136">
+      <c r="B70" s="135">
         <v>925.68399999999997</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A71" s="136">
+      <c r="A71" s="135">
         <v>136.76</v>
       </c>
-      <c r="B71" s="136">
+      <c r="B71" s="135">
         <v>995.11500000000001</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A72" s="136">
+      <c r="A72" s="135">
         <v>145.5</v>
       </c>
-      <c r="B72" s="136">
+      <c r="B72" s="135">
         <v>1062.8789999999999</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A73" s="136">
+      <c r="A73" s="135">
         <v>154.46</v>
       </c>
-      <c r="B73" s="136">
+      <c r="B73" s="135">
         <v>1127.6030000000001</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A74" s="136">
+      <c r="A74" s="135">
         <v>163.72</v>
       </c>
-      <c r="B74" s="136">
+      <c r="B74" s="135">
         <v>1188.1099999999999</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A75" s="136">
+      <c r="A75" s="135">
         <v>173.35</v>
       </c>
-      <c r="B75" s="136">
+      <c r="B75" s="135">
         <v>1243.3209999999999</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A76" s="136">
+      <c r="A76" s="135">
         <v>183.3</v>
       </c>
-      <c r="B76" s="136">
+      <c r="B76" s="135">
         <v>1293.0409999999999</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A77" s="136">
+      <c r="A77" s="135">
         <v>193.53</v>
       </c>
-      <c r="B77" s="136">
+      <c r="B77" s="135">
         <v>1336.877</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A78" s="136">
+      <c r="A78" s="135">
         <v>204</v>
       </c>
-      <c r="B78" s="136">
+      <c r="B78" s="135">
         <v>1374.829</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A79" s="136">
+      <c r="A79" s="135">
         <v>214.66</v>
       </c>
-      <c r="B79" s="136">
+      <c r="B79" s="135">
         <v>1406.7</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A80" s="136">
+      <c r="A80" s="135">
         <v>225.46</v>
       </c>
-      <c r="B80" s="136">
+      <c r="B80" s="135">
         <v>1433.2760000000001</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A81" s="136">
+      <c r="A81" s="135">
         <v>236.35</v>
       </c>
-      <c r="B81" s="136">
+      <c r="B81" s="135">
         <v>1455.93</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A82" s="136">
+      <c r="A82" s="135">
         <v>247.31</v>
       </c>
-      <c r="B82" s="136">
+      <c r="B82" s="135">
         <v>1476.0329999999999</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A83" s="136">
+      <c r="A83" s="135">
         <v>258.27999999999997</v>
       </c>
-      <c r="B83" s="136">
+      <c r="B83" s="135">
         <v>1494.8620000000001</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A84" s="136">
+      <c r="A84" s="135">
         <v>269.26</v>
       </c>
-      <c r="B84" s="136">
+      <c r="B84" s="135">
         <v>1513.396</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A85" s="136">
+      <c r="A85" s="135">
         <v>280.23</v>
       </c>
-      <c r="B85" s="136">
+      <c r="B85" s="135">
         <v>1531.8330000000001</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A86" s="136">
+      <c r="A86" s="135">
         <v>291.19</v>
       </c>
-      <c r="B86" s="136">
+      <c r="B86" s="135">
         <v>1550.3679999999999</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A87" s="136">
+      <c r="A87" s="135">
         <v>302.14999999999998</v>
       </c>
-      <c r="B87" s="136">
+      <c r="B87" s="135">
         <v>1569.2940000000001</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A88" s="136">
+      <c r="A88" s="135">
         <v>313.10000000000002</v>
       </c>
-      <c r="B88" s="136">
+      <c r="B88" s="135">
         <v>1588.712</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A89" s="136">
+      <c r="A89" s="135">
         <v>324.05</v>
       </c>
-      <c r="B89" s="136">
+      <c r="B89" s="135">
         <v>1608.325</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A90" s="136">
+      <c r="A90" s="135">
         <v>335.01</v>
       </c>
-      <c r="B90" s="136">
+      <c r="B90" s="135">
         <v>1627.9380000000001</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A91" s="136">
+      <c r="A91" s="135">
         <v>345.96</v>
       </c>
-      <c r="B91" s="136">
+      <c r="B91" s="135">
         <v>1647.2570000000001</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A92" s="136">
+      <c r="A92" s="135">
         <v>356.92</v>
       </c>
-      <c r="B92" s="136">
+      <c r="B92" s="135">
         <v>1666.2819999999999</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A93" s="136">
+      <c r="A93" s="135">
         <v>367.88</v>
       </c>
-      <c r="B93" s="136">
+      <c r="B93" s="135">
         <v>1685.6010000000001</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A94" s="136">
+      <c r="A94" s="135">
         <v>378.83</v>
       </c>
-      <c r="B94" s="136">
+      <c r="B94" s="135">
         <v>1705.4110000000001</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A95" s="136">
+      <c r="A95" s="135">
         <v>389.75</v>
       </c>
-      <c r="B95" s="136">
+      <c r="B95" s="135">
         <v>1726.3969999999999</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A96" s="136">
+      <c r="A96" s="135">
         <v>400.65</v>
       </c>
-      <c r="B96" s="136">
+      <c r="B96" s="135">
         <v>1748.6579999999999</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A97" s="136">
+      <c r="A97" s="135">
         <v>411.52</v>
       </c>
-      <c r="B97" s="136">
+      <c r="B97" s="135">
         <v>1772.39</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A98" s="136">
+      <c r="A98" s="135">
         <v>422.35</v>
       </c>
-      <c r="B98" s="136">
+      <c r="B98" s="135">
         <v>1797.4949999999999</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A99" s="136">
+      <c r="A99" s="135">
         <v>433.15</v>
       </c>
-      <c r="B99" s="136">
+      <c r="B99" s="135">
         <v>1823.973</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A100" s="136">
+      <c r="A100" s="135">
         <v>443.91</v>
       </c>
-      <c r="B100" s="136">
+      <c r="B100" s="135">
         <v>1851.8240000000001</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A101" s="136">
+      <c r="A101" s="135">
         <v>454.66</v>
       </c>
-      <c r="B101" s="136">
+      <c r="B101" s="135">
         <v>1880.3610000000001</v>
       </c>
     </row>
@@ -4746,14 +4757,14 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF15C171-B68F-9245-AAB8-281BA0072F89}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.33203125" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
     <col min="3" max="3" width="39.1640625" customWidth="1"/>
     <col min="4" max="4" width="12.5" customWidth="1"/>
-    <col min="5" max="5" width="37" customWidth="1"/>
+    <col min="5" max="5" width="73.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -4776,7 +4787,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="105" t="s">
+      <c r="C2" s="104" t="s">
         <v>102</v>
       </c>
       <c r="D2" s="9"/>
@@ -4787,7 +4798,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="105" t="s">
+      <c r="C3" s="104" t="s">
         <v>155</v>
       </c>
       <c r="D3" s="9"/>
@@ -4798,139 +4809,146 @@
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="105" t="s">
-        <v>161</v>
+      <c r="C4" s="104" t="s">
+        <v>165</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="95" t="s">
+      <c r="A5" s="94" t="s">
         <v>103</v>
       </c>
-      <c r="B5" s="77"/>
-      <c r="C5" s="124" t="s">
+      <c r="B5" s="76"/>
+      <c r="C5" s="123" t="s">
         <v>156</v>
       </c>
-      <c r="D5" s="106" t="s">
+      <c r="D5" s="105" t="s">
         <v>104</v>
       </c>
-      <c r="E5" s="107" t="s">
+      <c r="E5" s="106" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="95" t="s">
+      <c r="A6" s="94" t="s">
         <v>106</v>
       </c>
-      <c r="B6" s="77"/>
-      <c r="C6" s="103">
+      <c r="B6" s="76"/>
+      <c r="C6" s="102">
         <v>10</v>
       </c>
-      <c r="D6" s="106" t="s">
+      <c r="D6" s="105" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="30"/>
+      <c r="E6" s="29"/>
     </row>
     <row r="7" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="95" t="s">
+      <c r="A7" s="94" t="s">
         <v>107</v>
       </c>
-      <c r="B7" s="77"/>
-      <c r="C7" s="103" t="s">
+      <c r="B7" s="76"/>
+      <c r="C7" s="102" t="s">
         <v>108</v>
       </c>
-      <c r="D7" s="106" t="s">
+      <c r="D7" s="105" t="s">
         <v>109</v>
       </c>
-      <c r="E7" s="30"/>
+      <c r="E7" s="29"/>
     </row>
     <row r="8" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="95" t="s">
+      <c r="A8" s="94" t="s">
         <v>110</v>
       </c>
-      <c r="B8" s="77"/>
-      <c r="C8" s="108" t="s">
+      <c r="B8" s="76"/>
+      <c r="C8" s="107" t="s">
         <v>111</v>
       </c>
-      <c r="D8" s="106" t="s">
+      <c r="D8" s="105" t="s">
         <v>104</v>
       </c>
-      <c r="E8" s="30"/>
+      <c r="E8" s="29"/>
     </row>
     <row r="9" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="95" t="s">
+      <c r="A9" s="94" t="s">
         <v>112</v>
       </c>
-      <c r="B9" s="77"/>
-      <c r="C9" s="103">
+      <c r="B9" s="76"/>
+      <c r="C9" s="102">
         <v>25000</v>
       </c>
-      <c r="D9" s="106"/>
-      <c r="E9" s="30"/>
+      <c r="D9" s="105"/>
+      <c r="E9" s="29"/>
     </row>
     <row r="10" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="95" t="s">
+      <c r="A10" s="94" t="s">
         <v>113</v>
       </c>
-      <c r="B10" s="77"/>
-      <c r="C10" s="103">
+      <c r="B10" s="76"/>
+      <c r="C10" s="102">
         <v>0.01</v>
       </c>
-      <c r="D10" s="106" t="s">
+      <c r="D10" s="105" t="s">
         <v>114</v>
       </c>
-      <c r="E10" s="107" t="s">
+      <c r="E10" s="106" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="146" t="s">
+      <c r="A11" s="139" t="s">
         <v>116</v>
       </c>
-      <c r="B11" s="109" t="s">
+      <c r="B11" s="108" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="110" t="s">
+      <c r="C11" s="109" t="s">
         <v>150</v>
       </c>
-      <c r="D11" s="94"/>
-      <c r="E11" s="74"/>
+      <c r="D11" s="93"/>
+      <c r="E11" s="73"/>
     </row>
     <row r="12" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="156"/>
-      <c r="B12" s="111" t="s">
+      <c r="A12" s="140"/>
+      <c r="B12" s="110" t="s">
         <v>117</v>
       </c>
-      <c r="C12" s="112" t="s">
+      <c r="C12" s="111" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="113" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="114"/>
+      <c r="D12" s="112" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="113"/>
     </row>
     <row r="13" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="95" t="s">
+      <c r="A13" s="94" t="s">
         <v>153</v>
       </c>
-      <c r="B13" s="77"/>
-      <c r="C13" s="103" t="s">
-        <v>162</v>
-      </c>
-      <c r="D13" s="106"/>
-      <c r="E13" s="30"/>
+      <c r="B13" s="76"/>
+      <c r="C13" s="102" t="s">
+        <v>167</v>
+      </c>
+      <c r="D13" s="105"/>
+      <c r="E13" s="106" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="95" t="s">
+      <c r="A14" s="94" t="s">
         <v>154</v>
       </c>
-      <c r="B14" s="77"/>
-      <c r="C14" s="103" t="s">
-        <v>163</v>
-      </c>
-      <c r="D14" s="106"/>
-      <c r="E14" s="107"/>
+      <c r="B14" s="76"/>
+      <c r="C14" s="102" t="s">
+        <v>166</v>
+      </c>
+      <c r="D14" s="105"/>
+      <c r="E14" s="106"/>
+    </row>
+    <row r="18" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D18" s="138" t="s">
+        <v>164</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4954,296 +4972,296 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="33" t="s">
         <v>118</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="33" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="34" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="36">
+      <c r="B2" s="35">
         <v>200</v>
       </c>
-      <c r="C2" s="37">
+      <c r="C2" s="36">
         <v>203.34700000000001</v>
       </c>
-      <c r="D2" s="37">
+      <c r="D2" s="36">
         <v>126.35</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="B3" s="39">
+      <c r="B3" s="38">
         <v>-200</v>
       </c>
-      <c r="C3" s="40">
+      <c r="C3" s="39">
         <v>225</v>
       </c>
-      <c r="D3" s="40">
+      <c r="D3" s="39">
         <v>126.35</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="B4" s="39">
+      <c r="B4" s="38">
         <v>11.946</v>
       </c>
-      <c r="C4" s="40">
+      <c r="C4" s="39">
         <v>587.82100000000003</v>
       </c>
-      <c r="D4" s="40">
+      <c r="D4" s="39">
         <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="B5" s="39">
+      <c r="B5" s="38">
         <v>148.751</v>
       </c>
-      <c r="C5" s="40">
+      <c r="C5" s="39">
         <v>207.047</v>
       </c>
-      <c r="D5" s="40">
+      <c r="D5" s="39">
         <v>321.79399999999998</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="38" t="s">
+      <c r="A6" s="37" t="s">
         <v>126</v>
       </c>
-      <c r="B6" s="39">
+      <c r="B6" s="38">
         <v>-184.72900000000001</v>
       </c>
-      <c r="C6" s="40">
+      <c r="C6" s="39">
         <v>225</v>
       </c>
-      <c r="D6" s="40">
+      <c r="D6" s="39">
         <v>300.89400000000001</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="38" t="s">
+      <c r="A7" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="39">
+      <c r="B7" s="38">
         <v>-12.932</v>
       </c>
-      <c r="C7" s="40">
+      <c r="C7" s="39">
         <v>518.67999999999995</v>
       </c>
-      <c r="D7" s="40">
+      <c r="D7" s="39">
         <v>374.39299999999997</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="B8" s="39">
+      <c r="B8" s="38">
         <v>16.193999999999999</v>
       </c>
-      <c r="C8" s="40">
+      <c r="C8" s="39">
         <v>582.05899999999997</v>
       </c>
-      <c r="D8" s="40">
+      <c r="D8" s="39">
         <v>263.346</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="38" t="s">
+      <c r="A9" s="37" t="s">
         <v>129</v>
       </c>
-      <c r="B9" s="39">
+      <c r="B9" s="38">
         <v>0</v>
       </c>
-      <c r="C9" s="40">
+      <c r="C9" s="39">
         <v>640</v>
       </c>
-      <c r="D9" s="40">
+      <c r="D9" s="39">
         <v>260.36099999999999</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="38" t="s">
+      <c r="A10" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="B10" s="39">
+      <c r="B10" s="38">
         <v>104.241</v>
       </c>
-      <c r="C10" s="40">
+      <c r="C10" s="39">
         <v>250</v>
       </c>
-      <c r="D10" s="40">
+      <c r="D10" s="39">
         <v>171.053</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="38" t="s">
+      <c r="A11" s="37" t="s">
         <v>131</v>
       </c>
-      <c r="B11" s="39">
+      <c r="B11" s="38">
         <v>85.097999999999999</v>
       </c>
-      <c r="C11" s="40">
+      <c r="C11" s="39">
         <v>575.40700000000004</v>
       </c>
-      <c r="D11" s="40">
+      <c r="D11" s="39">
         <v>188.44399999999999</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="37" t="s">
         <v>132</v>
       </c>
-      <c r="B12" s="39">
+      <c r="B12" s="38">
         <v>11.157</v>
       </c>
-      <c r="C12" s="40">
+      <c r="C12" s="39">
         <v>233.131</v>
       </c>
-      <c r="D12" s="40">
+      <c r="D12" s="39">
         <v>517.55100000000004</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="38" t="s">
+      <c r="A13" s="37" t="s">
         <v>133</v>
       </c>
-      <c r="B13" s="39">
+      <c r="B13" s="38">
         <v>11.484999999999999</v>
       </c>
-      <c r="C13" s="40">
+      <c r="C13" s="39">
         <v>317.84199999999998</v>
       </c>
-      <c r="D13" s="40">
+      <c r="D13" s="39">
         <v>362.43</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="38" t="s">
+      <c r="A14" s="37" t="s">
         <v>134</v>
       </c>
-      <c r="B14" s="39">
+      <c r="B14" s="38">
         <v>11.821</v>
       </c>
-      <c r="C14" s="40">
+      <c r="C14" s="39">
         <v>550</v>
       </c>
-      <c r="D14" s="40">
+      <c r="D14" s="39">
         <v>178.70500000000001</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="38" t="s">
+      <c r="A15" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="B15" s="39">
+      <c r="B15" s="38">
         <v>11.489000000000001</v>
       </c>
-      <c r="C15" s="40">
+      <c r="C15" s="39">
         <v>351.53699999999998</v>
       </c>
-      <c r="D15" s="40">
+      <c r="D15" s="39">
         <v>360.94299999999998</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="37" t="s">
         <v>136</v>
       </c>
-      <c r="B16" s="39">
+      <c r="B16" s="38">
         <v>11.558</v>
       </c>
-      <c r="C16" s="40">
+      <c r="C16" s="39">
         <v>244.43100000000001</v>
       </c>
-      <c r="D16" s="40">
+      <c r="D16" s="39">
         <v>328.19799999999998</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="38" t="s">
+      <c r="A17" s="37" t="s">
         <v>137</v>
       </c>
-      <c r="B17" s="39">
+      <c r="B17" s="38">
         <v>67.965000000000003</v>
       </c>
-      <c r="C17" s="40">
+      <c r="C17" s="39">
         <v>262.85500000000002</v>
       </c>
-      <c r="D17" s="40">
+      <c r="D17" s="39">
         <v>101.35</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="38" t="s">
+      <c r="A18" s="37" t="s">
         <v>138</v>
       </c>
-      <c r="B18" s="39">
-        <v>4</v>
-      </c>
-      <c r="C18" s="40">
-        <v>262.84899999999999</v>
-      </c>
-      <c r="D18" s="40">
+      <c r="B18" s="38">
+        <v>-23.5</v>
+      </c>
+      <c r="C18" s="39">
+        <v>262.85500000000002</v>
+      </c>
+      <c r="D18" s="39">
         <v>101.51900000000001</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="38" t="s">
+      <c r="A19" s="37" t="s">
         <v>139</v>
       </c>
-      <c r="B19" s="39">
+      <c r="B19" s="38">
         <v>11.526999999999999</v>
       </c>
-      <c r="C19" s="40">
+      <c r="C19" s="39">
         <v>292.24599999999998</v>
       </c>
-      <c r="D19" s="40">
+      <c r="D19" s="39">
         <v>342.81599999999997</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="38" t="s">
+      <c r="A20" s="37" t="s">
         <v>140</v>
       </c>
-      <c r="B20" s="39">
+      <c r="B20" s="38">
         <v>104.241</v>
       </c>
-      <c r="C20" s="40">
+      <c r="C20" s="39">
         <v>0</v>
       </c>
-      <c r="D20" s="40">
+      <c r="D20" s="39">
         <v>171.053</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="38" t="s">
+      <c r="A21" s="37" t="s">
         <v>141</v>
       </c>
-      <c r="B21" s="39">
+      <c r="B21" s="38">
         <v>-324.96499999999997</v>
       </c>
-      <c r="C21" s="40">
+      <c r="C21" s="39">
         <v>0</v>
       </c>
-      <c r="D21" s="40">
+      <c r="D21" s="39">
         <v>533.79200000000003</v>
       </c>
     </row>
@@ -5270,268 +5288,268 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="33" t="s">
         <v>118</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="33" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="34" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="36">
+      <c r="B2" s="35">
         <v>-1390</v>
       </c>
-      <c r="C2" s="37">
+      <c r="C2" s="36">
         <v>305</v>
       </c>
-      <c r="D2" s="37">
+      <c r="D2" s="36">
         <v>126.35</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="B3" s="39">
+      <c r="B3" s="38">
         <v>-1830</v>
       </c>
-      <c r="C3" s="40">
+      <c r="C3" s="39">
         <v>270</v>
       </c>
-      <c r="D3" s="40">
+      <c r="D3" s="39">
         <v>126.35</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="B4" s="39">
+      <c r="B4" s="38">
         <v>-1579.2370000000001</v>
       </c>
-      <c r="C4" s="40">
+      <c r="C4" s="39">
         <v>573.947</v>
       </c>
-      <c r="D4" s="40">
+      <c r="D4" s="39">
         <v>137.5</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="37" t="s">
         <v>125</v>
       </c>
-      <c r="B5" s="39">
+      <c r="B5" s="38">
         <v>-1390</v>
       </c>
-      <c r="C5" s="40">
+      <c r="C5" s="39">
         <v>305</v>
       </c>
-      <c r="D5" s="40">
+      <c r="D5" s="39">
         <v>328.98099999999999</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="38" t="s">
+      <c r="A6" s="37" t="s">
         <v>126</v>
       </c>
-      <c r="B6" s="39">
+      <c r="B6" s="38">
         <v>-1830</v>
       </c>
-      <c r="C6" s="40">
+      <c r="C6" s="39">
         <v>270</v>
       </c>
-      <c r="D6" s="40">
+      <c r="D6" s="39">
         <v>354.47500000000002</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="38" t="s">
+      <c r="A7" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="B7" s="39">
+      <c r="B7" s="38">
         <v>-1569.845</v>
       </c>
-      <c r="C7" s="40">
+      <c r="C7" s="39">
         <v>506.33</v>
       </c>
-      <c r="D7" s="40">
+      <c r="D7" s="39">
         <v>382.471</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="B8" s="39">
+      <c r="B8" s="38">
         <v>-1568.8710000000001</v>
       </c>
-      <c r="C8" s="40">
+      <c r="C8" s="39">
         <v>566.64200000000005</v>
       </c>
-      <c r="D8" s="40">
+      <c r="D8" s="39">
         <v>269.14400000000001</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="38" t="s">
+      <c r="A9" s="37" t="s">
         <v>129</v>
       </c>
-      <c r="B9" s="39">
+      <c r="B9" s="38">
         <v>-1574.5989999999999</v>
       </c>
-      <c r="C9" s="40">
+      <c r="C9" s="39">
         <v>623.53200000000004</v>
       </c>
-      <c r="D9" s="40">
+      <c r="D9" s="39">
         <v>260.36099999999999</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="38" t="s">
+      <c r="A10" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="B10" s="39">
+      <c r="B10" s="38">
         <v>-1830</v>
       </c>
-      <c r="C10" s="40">
+      <c r="C10" s="39">
         <v>270</v>
       </c>
-      <c r="D10" s="40">
+      <c r="D10" s="39">
         <v>193.642</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="38" t="s">
+      <c r="A11" s="37" t="s">
         <v>131</v>
       </c>
-      <c r="B11" s="39">
+      <c r="B11" s="38">
         <v>-1675.904</v>
       </c>
-      <c r="C11" s="40">
+      <c r="C11" s="39">
         <v>576.73500000000001</v>
       </c>
-      <c r="D11" s="40">
+      <c r="D11" s="39">
         <v>225.33099999999999</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="37" t="s">
         <v>132</v>
       </c>
-      <c r="B12" s="39">
+      <c r="B12" s="38">
         <v>-1395.9760000000001</v>
       </c>
-      <c r="C12" s="40">
+      <c r="C12" s="39">
         <v>283.399</v>
       </c>
-      <c r="D12" s="40">
+      <c r="D12" s="39">
         <v>436.10300000000001</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="38" t="s">
+      <c r="A13" s="37" t="s">
         <v>133</v>
       </c>
-      <c r="B13" s="39">
+      <c r="B13" s="38">
         <v>-1579.1110000000001</v>
       </c>
-      <c r="C13" s="40">
+      <c r="C13" s="39">
         <v>267.07299999999998</v>
       </c>
-      <c r="D13" s="40">
+      <c r="D13" s="39">
         <v>484.01</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="38" t="s">
+      <c r="A14" s="37" t="s">
         <v>134</v>
       </c>
-      <c r="B14" s="39">
+      <c r="B14" s="38">
         <v>-1597.194</v>
       </c>
-      <c r="C14" s="40">
+      <c r="C14" s="39">
         <v>526.39499999999998</v>
       </c>
-      <c r="D14" s="40">
+      <c r="D14" s="39">
         <v>155.28700000000001</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="38" t="s">
+      <c r="A15" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="B15" s="39">
+      <c r="B15" s="38">
         <v>-1664.6120000000001</v>
       </c>
-      <c r="C15" s="40">
+      <c r="C15" s="39">
         <v>349.04700000000003</v>
       </c>
-      <c r="D15" s="40">
+      <c r="D15" s="39">
         <v>403.92399999999998</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="37" t="s">
         <v>136</v>
       </c>
-      <c r="B16" s="39">
+      <c r="B16" s="38">
         <v>-1585.771</v>
       </c>
-      <c r="C16" s="40">
+      <c r="C16" s="39">
         <v>318.42700000000002</v>
       </c>
-      <c r="D16" s="40">
+      <c r="D16" s="39">
         <v>426.35</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="38" t="s">
+      <c r="A17" s="37" t="s">
         <v>137</v>
       </c>
-      <c r="B17" s="39">
+      <c r="B17" s="38">
         <v>-1830</v>
       </c>
-      <c r="C17" s="40">
+      <c r="C17" s="39">
         <v>305</v>
       </c>
-      <c r="D17" s="40">
+      <c r="D17" s="39">
         <v>401.35</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="38" t="s">
+      <c r="A18" s="37" t="s">
         <v>138</v>
       </c>
-      <c r="B18" s="39">
+      <c r="B18" s="38">
         <v>-1830</v>
       </c>
-      <c r="C18" s="40">
+      <c r="C18" s="39">
         <v>305</v>
       </c>
-      <c r="D18" s="40">
-        <v>465.35</v>
+      <c r="D18" s="39">
+        <v>448.35</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="38" t="s">
+      <c r="A19" s="37" t="s">
         <v>139</v>
       </c>
-      <c r="B19" s="39">
+      <c r="B19" s="38">
         <v>-1600.4860000000001</v>
       </c>
-      <c r="C19" s="40">
+      <c r="C19" s="39">
         <v>287.56599999999997</v>
       </c>
-      <c r="D19" s="40">
+      <c r="D19" s="39">
         <v>463.988</v>
       </c>
     </row>
@@ -5608,24 +5626,24 @@
       <c r="A5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="117"/>
-      <c r="C5" s="119" t="s">
+      <c r="B5" s="116"/>
+      <c r="C5" s="118" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="120" t="s">
+      <c r="D5" s="119" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="118"/>
+      <c r="E5" s="117"/>
     </row>
     <row r="6" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B6" s="81"/>
-      <c r="C6" s="88" t="s">
+      <c r="B6" s="80"/>
+      <c r="C6" s="87" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="90" t="s">
+      <c r="D6" s="89" t="s">
         <v>66</v>
       </c>
       <c r="E6" s="23"/>
@@ -5634,11 +5652,11 @@
       <c r="A7" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="81"/>
-      <c r="C7" s="88" t="s">
+      <c r="B7" s="80"/>
+      <c r="C7" s="87" t="s">
         <v>67</v>
       </c>
-      <c r="D7" s="90" t="s">
+      <c r="D7" s="89" t="s">
         <v>66</v>
       </c>
       <c r="E7" s="23"/>
@@ -5685,7 +5703,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="105" t="s">
+      <c r="C2" s="104" t="s">
         <v>37</v>
       </c>
       <c r="D2" s="9"/>
@@ -5696,7 +5714,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="105" t="s">
+      <c r="C3" s="104" t="s">
         <v>38</v>
       </c>
       <c r="D3" s="9"/>
@@ -5707,17 +5725,17 @@
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="105" t="s">
+      <c r="C4" s="104" t="s">
         <v>39</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="140" t="s">
+      <c r="A5" s="144" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="77" t="s">
+      <c r="B5" s="76" t="s">
         <v>41</v>
       </c>
       <c r="C5" s="24" t="str">
@@ -5732,8 +5750,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="138"/>
-      <c r="B6" s="78" t="s">
+      <c r="A6" s="142"/>
+      <c r="B6" s="77" t="s">
         <v>43</v>
       </c>
       <c r="C6" s="25" t="str" cm="1">
@@ -5748,8 +5766,8 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="141"/>
-      <c r="B7" s="78" t="s">
+      <c r="A7" s="145"/>
+      <c r="B7" s="77" t="s">
         <v>44</v>
       </c>
       <c r="C7" s="25" t="str" cm="1">
@@ -5764,8 +5782,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="141"/>
-      <c r="B8" s="81" t="s">
+      <c r="A8" s="145"/>
+      <c r="B8" s="80" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="21">
@@ -5777,10 +5795,10 @@
       <c r="E8" s="23"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="142" t="s">
+      <c r="A9" s="146" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="77" t="s">
+      <c r="B9" s="76" t="s">
         <v>41</v>
       </c>
       <c r="C9" s="24" t="str" cm="1">
@@ -5795,8 +5813,8 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="139"/>
-      <c r="B10" s="78" t="s">
+      <c r="A10" s="143"/>
+      <c r="B10" s="77" t="s">
         <v>43</v>
       </c>
       <c r="C10" s="25" t="str" cm="1">
@@ -5811,8 +5829,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="139"/>
-      <c r="B11" s="78" t="s">
+      <c r="A11" s="143"/>
+      <c r="B11" s="77" t="s">
         <v>44</v>
       </c>
       <c r="C11" s="25" t="str" cm="1">
@@ -5827,8 +5845,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="138"/>
-      <c r="B12" s="81" t="s">
+      <c r="A12" s="142"/>
+      <c r="B12" s="80" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="21">
@@ -5842,10 +5860,10 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="143" t="s">
+      <c r="A13" s="147" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="77" t="s">
+      <c r="B13" s="76" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="24" t="str" cm="1">
@@ -5860,8 +5878,8 @@
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="141"/>
-      <c r="B14" s="78" t="s">
+      <c r="A14" s="145"/>
+      <c r="B14" s="77" t="s">
         <v>151</v>
       </c>
       <c r="C14" s="25" t="str" cm="1">
@@ -5876,8 +5894,8 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="141"/>
-      <c r="B15" s="78" t="s">
+      <c r="A15" s="145"/>
+      <c r="B15" s="77" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="26">
@@ -5889,8 +5907,8 @@
       <c r="E15" s="19"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="144"/>
-      <c r="B16" s="78" t="s">
+      <c r="A16" s="148"/>
+      <c r="B16" s="77" t="s">
         <v>47</v>
       </c>
       <c r="C16" s="26">
@@ -5902,8 +5920,8 @@
       <c r="E16" s="17"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="139"/>
-      <c r="B17" s="78" t="s">
+      <c r="A17" s="143"/>
+      <c r="B17" s="77" t="s">
         <v>49</v>
       </c>
       <c r="C17" s="26">
@@ -5915,11 +5933,11 @@
       <c r="E17" s="17"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="139"/>
-      <c r="B18" s="78" t="s">
+      <c r="A18" s="143"/>
+      <c r="B18" s="77" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="115">
+      <c r="C18" s="114">
         <v>0.11</v>
       </c>
       <c r="D18" s="16" t="s">
@@ -5928,11 +5946,11 @@
       <c r="E18" s="17"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="139"/>
-      <c r="B19" s="78" t="s">
+      <c r="A19" s="143"/>
+      <c r="B19" s="77" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="115">
+      <c r="C19" s="114">
         <v>0.03</v>
       </c>
       <c r="D19" s="16" t="s">
@@ -5941,11 +5959,11 @@
       <c r="E19" s="17"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="138"/>
-      <c r="B20" s="81" t="s">
+      <c r="A20" s="142"/>
+      <c r="B20" s="80" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="116">
+      <c r="C20" s="115">
         <v>1.5</v>
       </c>
       <c r="D20" s="22" t="s">
@@ -5954,10 +5972,10 @@
       <c r="E20" s="23"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="137" t="s">
+      <c r="A21" s="141" t="s">
         <v>145</v>
       </c>
-      <c r="B21" s="77" t="s">
+      <c r="B21" s="76" t="s">
         <v>53</v>
       </c>
       <c r="C21" s="24" t="str" cm="1">
@@ -5972,7 +5990,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="139"/>
+      <c r="A22" s="143"/>
       <c r="B22" s="14" t="s">
         <v>44</v>
       </c>
@@ -5988,7 +6006,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="138"/>
+      <c r="A23" s="142"/>
       <c r="B23" s="20" t="s">
         <v>12</v>
       </c>
@@ -6001,10 +6019,10 @@
       <c r="E23" s="23"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="137" t="s">
+      <c r="A24" s="141" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="77" t="s">
+      <c r="B24" s="76" t="s">
         <v>55</v>
       </c>
       <c r="C24" s="24" t="str" cm="1">
@@ -6019,8 +6037,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="139"/>
-      <c r="B25" s="78" t="s">
+      <c r="A25" s="143"/>
+      <c r="B25" s="77" t="s">
         <v>56</v>
       </c>
       <c r="C25" s="25" t="str" cm="1">
@@ -6035,21 +6053,21 @@
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="145"/>
-      <c r="B26" s="82" t="s">
+      <c r="A26" s="149"/>
+      <c r="B26" s="81" t="s">
         <v>149</v>
       </c>
-      <c r="C26" s="128">
+      <c r="C26" s="127">
         <v>1.2</v>
       </c>
-      <c r="D26" s="129" t="s">
+      <c r="D26" s="128" t="s">
         <v>30</v>
       </c>
-      <c r="E26" s="85"/>
+      <c r="E26" s="84"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="138"/>
-      <c r="B27" s="81" t="s">
+      <c r="A27" s="142"/>
+      <c r="B27" s="80" t="s">
         <v>148</v>
       </c>
       <c r="C27" s="21">
@@ -6061,10 +6079,10 @@
       <c r="E27" s="23"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="137" t="s">
+      <c r="A28" s="141" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="77" t="s">
+      <c r="B28" s="76" t="s">
         <v>58</v>
       </c>
       <c r="C28" s="28">
@@ -6076,8 +6094,8 @@
       <c r="E28" s="13"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="138"/>
-      <c r="B29" s="81" t="s">
+      <c r="A29" s="142"/>
+      <c r="B29" s="80" t="s">
         <v>59</v>
       </c>
       <c r="C29" s="21">
@@ -6089,10 +6107,10 @@
       <c r="E29" s="23"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="137" t="s">
+      <c r="A30" s="141" t="s">
         <v>60</v>
       </c>
-      <c r="B30" s="91" t="s">
+      <c r="B30" s="90" t="s">
         <v>53</v>
       </c>
       <c r="C30" s="24" t="str" cm="1">
@@ -6107,8 +6125,8 @@
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="139"/>
-      <c r="B31" s="92" t="s">
+      <c r="A31" s="143"/>
+      <c r="B31" s="91" t="s">
         <v>44</v>
       </c>
       <c r="C31" s="25" t="str" cm="1">
@@ -6123,8 +6141,8 @@
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="138"/>
-      <c r="B32" s="93" t="s">
+      <c r="A32" s="142"/>
+      <c r="B32" s="92" t="s">
         <v>12</v>
       </c>
       <c r="C32" s="21">
@@ -6136,7 +6154,7 @@
       <c r="E32" s="23"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="137" t="s">
+      <c r="A33" s="141" t="s">
         <v>61</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -6154,7 +6172,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="139"/>
+      <c r="A34" s="143"/>
       <c r="B34" s="14" t="s">
         <v>63</v>
       </c>
@@ -6170,7 +6188,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="138"/>
+      <c r="A35" s="142"/>
       <c r="B35" s="20" t="s">
         <v>12</v>
       </c>
@@ -6263,10 +6281,10 @@
       <c r="E5" s="10"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="125" t="s">
+      <c r="A6" s="124" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="77"/>
+      <c r="B6" s="76"/>
       <c r="C6" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B19/1000,HardpointsFr!C19/1000,HardpointsFr!D19/1000)&amp;"]"</f>
         <v>[0.011527 0.292246 0.342816]</v>
@@ -6279,10 +6297,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="126" t="s">
+      <c r="A7" s="125" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="78"/>
+      <c r="B7" s="77"/>
       <c r="C7" s="25" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B17/1000,HardpointsFr!C17/1000,HardpointsFr!D17/1000)&amp;"]"</f>
         <v>[0.067965 0.262855 0.10135]</v>
@@ -6295,13 +6313,13 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="126" t="s">
+      <c r="A8" s="125" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="78"/>
+      <c r="B8" s="77"/>
       <c r="C8" s="25" t="str" cm="1">
         <f t="array" ref="C8">"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B18/1000,HardpointsFr!C18/1000,HardpointsFr!D18/1000)&amp;"]"</f>
-        <v>[0.004 0.262849 0.101519]</v>
+        <v>[-0.0235 0.262855 0.101519]</v>
       </c>
       <c r="D8" s="16" t="s">
         <v>12</v>
@@ -6311,24 +6329,25 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="126" t="s">
+      <c r="A9" s="125" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="78"/>
-      <c r="C9" s="29">
-        <v>81.933000000000007</v>
-      </c>
-      <c r="D9" s="89" t="s">
+      <c r="B9" s="77"/>
+      <c r="C9" s="136">
+        <f>2.2813*2</f>
+        <v>4.5625999999999998</v>
+      </c>
+      <c r="D9" s="88" t="s">
         <v>160</v>
       </c>
       <c r="E9" s="17"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="127" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="81"/>
-      <c r="C10" s="21">
+      <c r="A10" s="126" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="80"/>
+      <c r="C10" s="137">
         <v>0.7</v>
       </c>
       <c r="D10" s="22" t="s">
@@ -6410,13 +6429,13 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="146" t="s">
+      <c r="A5" s="139" t="s">
         <v>74</v>
       </c>
-      <c r="B5" s="77" t="s">
+      <c r="B5" s="76" t="s">
         <v>75</v>
       </c>
-      <c r="C5" s="44" t="str">
+      <c r="C5" s="43" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B20/1000,HardpointsFr!C20/1000,HardpointsFr!D20/1000)&amp;"]"</f>
         <v>[0.104241 0 0.171053]</v>
       </c>
@@ -6428,24 +6447,24 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="147"/>
-      <c r="B6" s="96" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="42">
+      <c r="A6" s="150"/>
+      <c r="B6" s="95" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="41">
         <v>0.87</v>
       </c>
-      <c r="D6" s="43" t="s">
+      <c r="D6" s="42" t="s">
         <v>30</v>
       </c>
       <c r="E6" s="19"/>
     </row>
     <row r="7" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="148"/>
-      <c r="B7" s="78" t="s">
+      <c r="A7" s="151"/>
+      <c r="B7" s="77" t="s">
         <v>76</v>
       </c>
-      <c r="C7" s="41">
+      <c r="C7" s="40">
         <v>50</v>
       </c>
       <c r="D7" s="16" t="s">
@@ -6454,26 +6473,26 @@
       <c r="E7" s="16"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="149" t="s">
+      <c r="A8" s="152" t="s">
         <v>78</v>
       </c>
-      <c r="B8" s="78" t="s">
+      <c r="B8" s="77" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="25">
         <v>0.5</v>
       </c>
-      <c r="D8" s="89" t="s">
+      <c r="D8" s="88" t="s">
         <v>30</v>
       </c>
       <c r="E8" s="17"/>
     </row>
     <row r="9" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="150"/>
-      <c r="B9" s="78" t="s">
+      <c r="A9" s="153"/>
+      <c r="B9" s="77" t="s">
         <v>75</v>
       </c>
-      <c r="C9" s="41" t="str">
+      <c r="C9" s="40" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B21/1000,HardpointsFr!C21/1000,HardpointsFr!D21/1000)&amp;"]"</f>
         <v>[-0.324965 0 0.533792]</v>
       </c>
@@ -6537,7 +6556,7 @@
         <v>37</v>
       </c>
       <c r="D2" s="9"/>
-      <c r="E2" s="56"/>
+      <c r="E2" s="55"/>
     </row>
     <row r="3" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -6548,68 +6567,68 @@
         <v>38</v>
       </c>
       <c r="D3" s="9"/>
-      <c r="E3" s="56"/>
+      <c r="E3" s="55"/>
     </row>
     <row r="4" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="105" t="s">
+      <c r="C4" s="104" t="s">
         <v>37</v>
       </c>
       <c r="D4" s="9"/>
-      <c r="E4" s="56"/>
+      <c r="E4" s="55"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="117"/>
-      <c r="C5" s="119" t="s">
+      <c r="B5" s="116"/>
+      <c r="C5" s="118" t="s">
         <v>144</v>
       </c>
-      <c r="D5" s="120" t="s">
+      <c r="D5" s="119" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="121"/>
+      <c r="E5" s="120"/>
     </row>
     <row r="6" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B6" s="81"/>
-      <c r="C6" s="88" t="s">
+      <c r="B6" s="80"/>
+      <c r="C6" s="87" t="s">
         <v>79</v>
       </c>
-      <c r="D6" s="90" t="s">
+      <c r="D6" s="89" t="s">
         <v>66</v>
       </c>
       <c r="E6" s="23"/>
     </row>
     <row r="7" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="151" t="s">
+      <c r="A7" s="154" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="130" t="s">
+      <c r="B7" s="129" t="s">
         <v>157</v>
       </c>
-      <c r="C7" s="131" t="s">
+      <c r="C7" s="130" t="s">
         <v>67</v>
       </c>
-      <c r="D7" s="120"/>
-      <c r="E7" s="132"/>
+      <c r="D7" s="119"/>
+      <c r="E7" s="131"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="152"/>
-      <c r="B8" s="130" t="s">
+      <c r="A8" s="155"/>
+      <c r="B8" s="129" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="119" t="s">
+      <c r="C8" s="118" t="s">
         <v>158</v>
       </c>
-      <c r="D8" s="120"/>
-      <c r="E8" s="121"/>
+      <c r="D8" s="119"/>
+      <c r="E8" s="120"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6657,7 +6676,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="105" t="s">
+      <c r="C2" s="104" t="s">
         <v>37</v>
       </c>
       <c r="D2" s="9"/>
@@ -6668,7 +6687,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="105" t="s">
+      <c r="C3" s="104" t="s">
         <v>38</v>
       </c>
       <c r="D3" s="9"/>
@@ -6679,17 +6698,17 @@
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="105" t="s">
+      <c r="C4" s="104" t="s">
         <v>143</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="151" t="s">
+      <c r="A5" s="154" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="77" t="s">
+      <c r="B5" s="76" t="s">
         <v>41</v>
       </c>
       <c r="C5" s="24" t="str">
@@ -6699,125 +6718,125 @@
       <c r="D5" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="57" t="s">
+      <c r="E5" s="56" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="157"/>
-      <c r="B6" s="78" t="s">
+      <c r="A6" s="159"/>
+      <c r="B6" s="77" t="s">
         <v>43</v>
       </c>
       <c r="C6" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B3/1000 +1.575,HardpointsRr!C3/1000,HardpointsRr!D3/1000)&amp;"]"</f>
         <v>[-0.255 0.27 0.12635]</v>
       </c>
-      <c r="D6" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="58" t="s">
+      <c r="D6" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="57" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="157"/>
-      <c r="B7" s="78" t="s">
+      <c r="A7" s="159"/>
+      <c r="B7" s="77" t="s">
         <v>44</v>
       </c>
       <c r="C7" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B4/1000 +1.575,HardpointsRr!C4/1000,HardpointsRr!D4/1000)&amp;"]"</f>
         <v>[-0.00423700000000005 0.573947 0.1375]</v>
       </c>
-      <c r="D7" s="49" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="59" t="s">
+      <c r="D7" s="48" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="58" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="152"/>
-      <c r="B8" s="81" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="51">
+      <c r="A8" s="155"/>
+      <c r="B8" s="80" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="50">
         <v>0.16500000000000001</v>
       </c>
-      <c r="D8" s="50" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="60"/>
+      <c r="D8" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="59"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="158" t="s">
+      <c r="A9" s="160" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="77" t="s">
+      <c r="B9" s="76" t="s">
         <v>41</v>
       </c>
       <c r="C9" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B5/1000 +1.575,HardpointsRr!C5/1000,HardpointsRr!D5/1000)&amp;"]"</f>
         <v>[0.185 0.305 0.328981]</v>
       </c>
-      <c r="D9" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="61" t="s">
+      <c r="D9" s="51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="60" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="159"/>
-      <c r="B10" s="78" t="s">
+      <c r="A10" s="161"/>
+      <c r="B10" s="77" t="s">
         <v>43</v>
       </c>
       <c r="C10" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B6/1000 +1.575,HardpointsRr!C6/1000,HardpointsRr!D6/1000)&amp;"]"</f>
         <v>[-0.255 0.27 0.354475]</v>
       </c>
-      <c r="D10" s="55" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="62" t="s">
+      <c r="D10" s="54" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="61" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="159"/>
-      <c r="B11" s="78" t="s">
+      <c r="A11" s="161"/>
+      <c r="B11" s="77" t="s">
         <v>44</v>
       </c>
       <c r="C11" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B7/1000 +1.575,HardpointsRr!C7/1000,HardpointsRr!D7/1000)&amp;"]"</f>
         <v>[0.00515500000000002 0.50633 0.382471]</v>
       </c>
-      <c r="D11" s="53" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="63" t="s">
+      <c r="D11" s="52" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="62" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="160"/>
-      <c r="B12" s="81" t="s">
+      <c r="A12" s="162"/>
+      <c r="B12" s="80" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="21">
         <v>0.12</v>
       </c>
-      <c r="D12" s="54" t="s">
+      <c r="D12" s="53" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="64" t="s">
+      <c r="E12" s="63" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="146" t="s">
+      <c r="A13" s="139" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="77" t="s">
+      <c r="B13" s="76" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="24" t="str">
@@ -6827,42 +6846,42 @@
       <c r="D13" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="57" t="s">
+      <c r="E13" s="56" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="147"/>
-      <c r="B14" s="78" t="s">
+      <c r="A14" s="150"/>
+      <c r="B14" s="77" t="s">
         <v>151</v>
       </c>
       <c r="C14" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B9/1000 +1.575,HardpointsRr!C9/1000,HardpointsRr!D9/1000)&amp;"]"</f>
         <v>[0.000401000000000096 0.623532 0.260361]</v>
       </c>
-      <c r="D14" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="65" t="s">
+      <c r="D14" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="64" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="147"/>
-      <c r="B15" s="78" t="s">
+      <c r="A15" s="150"/>
+      <c r="B15" s="77" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="26">
         <v>1</v>
       </c>
-      <c r="D15" s="45" t="s">
+      <c r="D15" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="66"/>
+      <c r="E15" s="65"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="147"/>
-      <c r="B16" s="78" t="s">
+      <c r="A16" s="150"/>
+      <c r="B16" s="77" t="s">
         <v>47</v>
       </c>
       <c r="C16" s="26">
@@ -6871,11 +6890,11 @@
       <c r="D16" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="64"/>
+      <c r="E16" s="63"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="147"/>
-      <c r="B17" s="78" t="s">
+      <c r="A17" s="150"/>
+      <c r="B17" s="77" t="s">
         <v>49</v>
       </c>
       <c r="C17" s="26">
@@ -6884,67 +6903,67 @@
       <c r="D17" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="E17" s="67"/>
+      <c r="E17" s="66"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="147"/>
-      <c r="B18" s="78" t="s">
+      <c r="A18" s="150"/>
+      <c r="B18" s="77" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="115">
+      <c r="C18" s="114">
         <v>0.11</v>
       </c>
       <c r="D18" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="67"/>
+      <c r="E18" s="66"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="147"/>
-      <c r="B19" s="78" t="s">
+      <c r="A19" s="150"/>
+      <c r="B19" s="77" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="115">
+      <c r="C19" s="114">
         <v>0.03</v>
       </c>
       <c r="D19" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="67"/>
+      <c r="E19" s="66"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="156"/>
-      <c r="B20" s="81" t="s">
+      <c r="A20" s="140"/>
+      <c r="B20" s="80" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="116">
+      <c r="C20" s="115">
         <v>1.5</v>
       </c>
       <c r="D20" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="E20" s="68"/>
+      <c r="E20" s="67"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="146" t="s">
+      <c r="A21" s="139" t="s">
         <v>145</v>
       </c>
-      <c r="B21" s="77" t="s">
+      <c r="B21" s="76" t="s">
         <v>53</v>
       </c>
       <c r="C21" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B10/1000 +1.575,HardpointsRr!C10/1000,HardpointsRr!D10/1000)&amp;"]"</f>
         <v>[-0.255 0.27 0.193642]</v>
       </c>
-      <c r="D21" s="46" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" s="69" t="s">
+      <c r="D21" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="68" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="147"/>
+      <c r="A22" s="150"/>
       <c r="B22" s="14" t="s">
         <v>44</v>
       </c>
@@ -6952,15 +6971,15 @@
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B11/1000 +1.575,HardpointsRr!C11/1000,HardpointsRr!D11/1000)&amp;"]"</f>
         <v>[-0.100904 0.576735 0.225331]</v>
       </c>
-      <c r="D22" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="E22" s="62" t="s">
+      <c r="D22" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" s="61" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="156"/>
+      <c r="A23" s="140"/>
       <c r="B23" s="20" t="s">
         <v>12</v>
       </c>
@@ -6970,29 +6989,29 @@
       <c r="D23" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="E23" s="70"/>
+      <c r="E23" s="69"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="146" t="s">
+      <c r="A24" s="139" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="77" t="s">
+      <c r="B24" s="76" t="s">
         <v>55</v>
       </c>
       <c r="C24" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B12/1000 + 1.575,HardpointsRr!C12/1000,HardpointsRr!D12/1000)&amp;"]"</f>
         <v>[0.179024 0.283399 0.436103]</v>
       </c>
-      <c r="D24" s="46" t="s">
-        <v>12</v>
-      </c>
-      <c r="E24" s="63" t="s">
+      <c r="D24" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="62" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="147"/>
-      <c r="B25" s="78" t="s">
+      <c r="A25" s="150"/>
+      <c r="B25" s="77" t="s">
         <v>56</v>
       </c>
       <c r="C25" s="24" t="str">
@@ -7002,24 +7021,24 @@
       <c r="D25" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E25" s="64" t="s">
+      <c r="E25" s="63" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="147"/>
-      <c r="B26" s="82" t="s">
+      <c r="A26" s="150"/>
+      <c r="B26" s="81" t="s">
         <v>148</v>
       </c>
-      <c r="C26" s="128">
+      <c r="C26" s="127">
         <v>0.8</v>
       </c>
-      <c r="D26" s="83"/>
-      <c r="E26" s="75"/>
+      <c r="D26" s="82"/>
+      <c r="E26" s="74"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="156"/>
-      <c r="B27" s="81" t="s">
+      <c r="A27" s="140"/>
+      <c r="B27" s="80" t="s">
         <v>149</v>
       </c>
       <c r="C27" s="21">
@@ -7028,13 +7047,13 @@
       <c r="D27" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="E27" s="71"/>
+      <c r="E27" s="70"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="146" t="s">
+      <c r="A28" s="139" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="77" t="s">
+      <c r="B28" s="76" t="s">
         <v>58</v>
       </c>
       <c r="C28" s="28">
@@ -7043,11 +7062,11 @@
       <c r="D28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E28" s="72"/>
+      <c r="E28" s="71"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="156"/>
-      <c r="B29" s="81" t="s">
+      <c r="A29" s="140"/>
+      <c r="B29" s="80" t="s">
         <v>59</v>
       </c>
       <c r="C29" s="21">
@@ -7056,13 +7075,13 @@
       <c r="D29" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="E29" s="71"/>
+      <c r="E29" s="70"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="153" t="s">
+      <c r="A30" s="156" t="s">
         <v>60</v>
       </c>
-      <c r="B30" s="91" t="s">
+      <c r="B30" s="90" t="s">
         <v>44</v>
       </c>
       <c r="C30" s="24" t="str">
@@ -7072,29 +7091,29 @@
       <c r="D30" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E30" s="57" t="s">
+      <c r="E30" s="56" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="154"/>
-      <c r="B31" s="92" t="s">
+      <c r="A31" s="157"/>
+      <c r="B31" s="91" t="s">
         <v>53</v>
       </c>
       <c r="C31" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B15/1000 + 1.575,HardpointsRr!C15/1000,HardpointsRr!D15/1000)&amp;"]"</f>
         <v>[-0.089612 0.349047 0.403924]</v>
       </c>
-      <c r="D31" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="E31" s="62" t="s">
+      <c r="D31" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" s="61" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="155"/>
-      <c r="B32" s="93" t="s">
+      <c r="A32" s="158"/>
+      <c r="B32" s="92" t="s">
         <v>12</v>
       </c>
       <c r="C32" s="21">
@@ -7103,10 +7122,10 @@
       <c r="D32" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="E32" s="73"/>
+      <c r="E32" s="72"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="146" t="s">
+      <c r="A33" s="139" t="s">
         <v>61</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -7119,12 +7138,12 @@
       <c r="D33" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E33" s="57" t="s">
+      <c r="E33" s="56" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="147"/>
+      <c r="A34" s="150"/>
       <c r="B34" s="14" t="s">
         <v>63</v>
       </c>
@@ -7132,15 +7151,15 @@
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B19/1000+ 1.575,HardpointsRr!C19/1000,HardpointsRr!D19/1000)&amp;"]"</f>
         <v>[-0.0254860000000001 0.287566 0.463988]</v>
       </c>
-      <c r="D34" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="E34" s="62" t="s">
+      <c r="D34" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" s="61" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="156"/>
+      <c r="A35" s="140"/>
       <c r="B35" s="20" t="s">
         <v>12</v>
       </c>
@@ -7150,7 +7169,7 @@
       <c r="D35" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="E35" s="73"/>
+      <c r="E35" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -7225,85 +7244,86 @@
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="105" t="s">
+      <c r="C4" s="104" t="s">
         <v>152</v>
       </c>
       <c r="D4" s="9"/>
-      <c r="E4" s="74"/>
+      <c r="E4" s="73"/>
     </row>
     <row r="5" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="125" t="s">
+      <c r="A5" s="124" t="s">
         <v>70</v>
       </c>
-      <c r="B5" s="77"/>
+      <c r="B5" s="76"/>
       <c r="C5" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B19/1000+ 1.575,HardpointsRr!C19/1000,HardpointsRr!D19/1000)&amp;"]"</f>
         <v>[-0.0254860000000001 0.287566 0.463988]</v>
       </c>
-      <c r="D5" s="133" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="69" t="s">
+      <c r="D5" s="132" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="68" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="126" t="s">
+      <c r="A6" s="125" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="78"/>
+      <c r="B6" s="77"/>
       <c r="C6" s="25" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B17/1000+ 1.575,HardpointsRr!C17/1000,HardpointsRr!D17/1000)&amp;"]"</f>
         <v>[-0.255 0.305 0.40135]</v>
       </c>
-      <c r="D6" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="58" t="s">
+      <c r="D6" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="57" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="126" t="s">
+      <c r="A7" s="125" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="78"/>
+      <c r="B7" s="77"/>
       <c r="C7" s="25" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B18/1000 + 1.575,HardpointsRr!C18/1000,HardpointsRr!D18/1000)&amp;"]"</f>
-        <v>[-0.255 0.305 0.46535]</v>
-      </c>
-      <c r="D7" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="62" t="s">
+        <v>[-0.255 0.305 0.44835]</v>
+      </c>
+      <c r="D7" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="61" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="126" t="s">
+      <c r="A8" s="125" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="78"/>
-      <c r="C8" s="31">
-        <v>61.879399999999997</v>
-      </c>
-      <c r="D8" s="89" t="s">
+      <c r="B8" s="77"/>
+      <c r="C8" s="30">
+        <f>1.979*2</f>
+        <v>3.9580000000000002</v>
+      </c>
+      <c r="D8" s="88" t="s">
         <v>160</v>
       </c>
-      <c r="E8" s="75"/>
+      <c r="E8" s="74"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="127" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="81"/>
+      <c r="A9" s="126" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="80"/>
       <c r="C9" s="21">
         <v>0.7</v>
       </c>
-      <c r="D9" s="47" t="s">
+      <c r="D9" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="76"/>
+      <c r="E9" s="75"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7377,21 +7397,21 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="123" t="s">
+      <c r="A5" s="122" t="s">
         <v>82</v>
       </c>
-      <c r="B5" s="77"/>
+      <c r="B5" s="76"/>
       <c r="C5" s="24">
         <v>-2.15</v>
       </c>
       <c r="D5" s="12"/>
-      <c r="E5" s="30"/>
+      <c r="E5" s="29"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="123" t="s">
+      <c r="A6" s="122" t="s">
         <v>83</v>
       </c>
-      <c r="B6" s="78"/>
+      <c r="B6" s="77"/>
       <c r="C6" s="25">
         <v>-1</v>
       </c>
@@ -7399,10 +7419,10 @@
       <c r="E6" s="19"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="123" t="s">
+      <c r="A7" s="122" t="s">
         <v>84</v>
       </c>
-      <c r="B7" s="78"/>
+      <c r="B7" s="77"/>
       <c r="C7" s="25">
         <v>1.2250000000000001</v>
       </c>
@@ -7412,10 +7432,10 @@
       <c r="E7" s="19"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="123" t="s">
+      <c r="A8" s="122" t="s">
         <v>147</v>
       </c>
-      <c r="B8" s="78"/>
+      <c r="B8" s="77"/>
       <c r="C8" s="25">
         <v>1.2</v>
       </c>
@@ -7425,11 +7445,11 @@
       <c r="E8" s="19"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="123" t="s">
+      <c r="A9" s="122" t="s">
         <v>87</v>
       </c>
-      <c r="B9" s="81"/>
-      <c r="C9" s="32" t="s">
+      <c r="B9" s="80"/>
+      <c r="C9" s="31" t="s">
         <v>88</v>
       </c>
       <c r="D9" s="22" t="s">
@@ -7447,15 +7467,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009342B7EAA7728A4FA80A5CCAFE8D7EAF" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d037a5681ee6af0e7b5b5d0a2f99b20">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557458c-24b5-4c97-84ed-4c402655f54f" xmlns:ns3="72e3c584-9879-4b35-b9d8-6a248c93e240" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="966978c8b125399653e7c255ac8e342d" ns2:_="" ns3:_="">
     <xsd:import namespace="9557458c-24b5-4c97-84ed-4c402655f54f"/>
@@ -7716,7 +7727,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
@@ -7727,15 +7738,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7754,7 +7766,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -7763,4 +7775,12 @@
     <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
commented UKF for efficiency
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1148AFD4-1C52-5042-B19A-BC7114E09693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86D21592-9E60-3244-BA9E-11F6B78BE2CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12320" yWindow="1400" windowWidth="38400" windowHeight="22500" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -575,7 +575,7 @@
     <t>2 combined+turnslip</t>
   </si>
   <si>
-    <t>1 steady state</t>
+    <t>3 non-linear transients</t>
   </si>
 </sst>
 </file>
@@ -7467,6 +7467,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009342B7EAA7728A4FA80A5CCAFE8D7EAF" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d037a5681ee6af0e7b5b5d0a2f99b20">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557458c-24b5-4c97-84ed-4c402655f54f" xmlns:ns3="72e3c584-9879-4b35-b9d8-6a248c93e240" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="966978c8b125399653e7c255ac8e342d" ns2:_="" ns3:_="">
     <xsd:import namespace="9557458c-24b5-4c97-84ed-4c402655f54f"/>
@@ -7727,27 +7747,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7764,23 +7783,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
-    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Changed driver for improved performace and path following Added plots for tire usage, grip balance and understeer gradient Added new version of slip control with PID controller
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86D21592-9E60-3244-BA9E-11F6B78BE2CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B04CC85-8DBA-704A-BA6D-55A574C2F0E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12320" yWindow="1400" windowWidth="38400" windowHeight="22500" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="38400" windowHeight="22380" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Body" sheetId="1" r:id="rId1"/>
@@ -572,10 +572,10 @@
     <t>MFEval</t>
   </si>
   <si>
-    <t>2 combined+turnslip</t>
-  </si>
-  <si>
-    <t>3 non-linear transients</t>
+    <t>1 steady state</t>
+  </si>
+  <si>
+    <t>1 combined</t>
   </si>
 </sst>
 </file>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="B13" s="76"/>
       <c r="C13" s="102" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D13" s="105"/>
       <c r="E13" s="106" t="s">
@@ -4940,7 +4940,7 @@
       </c>
       <c r="B14" s="76"/>
       <c r="C14" s="102" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D14" s="105"/>
       <c r="E14" s="106"/>
@@ -7467,26 +7467,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009342B7EAA7728A4FA80A5CCAFE8D7EAF" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d037a5681ee6af0e7b5b5d0a2f99b20">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557458c-24b5-4c97-84ed-4c402655f54f" xmlns:ns3="72e3c584-9879-4b35-b9d8-6a248c93e240" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="966978c8b125399653e7c255ac8e342d" ns2:_="" ns3:_="">
     <xsd:import namespace="9557458c-24b5-4c97-84ed-4c402655f54f"/>
@@ -7747,10 +7727,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7767,20 +7778,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
-    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
bug fix of unadded path files
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48625C90-9D53-F04F-A63C-A81501038C95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E6E63F5-D62B-3F4F-8E03-7C0B9806B7D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="38400" windowHeight="22380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10580" yWindow="1880" windowWidth="38400" windowHeight="22380" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Body" sheetId="1" r:id="rId1"/>
@@ -1771,9 +1771,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2155,6 +2152,9 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3350,11 +3350,11 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="120" t="s">
+      <c r="A5" s="119" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="78" t="s">
+      <c r="B5" s="74"/>
+      <c r="C5" s="77" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="12" t="s">
@@ -3365,11 +3365,11 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="120" t="s">
+      <c r="A6" s="119" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="76"/>
-      <c r="C6" s="77" t="s">
+      <c r="B6" s="75"/>
+      <c r="C6" s="76" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="15" t="s">
@@ -3380,11 +3380,11 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="119" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="76"/>
-      <c r="C7" s="77" t="s">
+      <c r="B7" s="75"/>
+      <c r="C7" s="76" t="s">
         <v>167</v>
       </c>
       <c r="D7" s="15" t="s">
@@ -3393,11 +3393,11 @@
       <c r="E7" s="16"/>
     </row>
     <row r="8" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="120" t="s">
+      <c r="A8" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="76"/>
-      <c r="C8" s="77" t="s">
+      <c r="B8" s="75"/>
+      <c r="C8" s="76" t="s">
         <v>19</v>
       </c>
       <c r="D8" s="15" t="s">
@@ -3408,11 +3408,11 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="120" t="s">
+      <c r="A9" s="119" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="76"/>
-      <c r="C9" s="77" t="s">
+      <c r="B9" s="75"/>
+      <c r="C9" s="76" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="15" t="s">
@@ -3423,11 +3423,11 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="120" t="s">
+      <c r="A10" s="119" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="76"/>
-      <c r="C10" s="77" t="s">
+      <c r="B10" s="75"/>
+      <c r="C10" s="76" t="s">
         <v>24</v>
       </c>
       <c r="D10" s="15" t="s">
@@ -3438,7 +3438,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="120" t="s">
+      <c r="A11" s="119" t="s">
         <v>25</v>
       </c>
       <c r="B11" s="14"/>
@@ -3454,10 +3454,10 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="120" t="s">
+      <c r="A12" s="119" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="76"/>
+      <c r="B12" s="75"/>
       <c r="C12" s="17">
         <f>HardpointsFr!C9*2/1000</f>
         <v>1.28</v>
@@ -3468,10 +3468,10 @@
       <c r="E12" s="16"/>
     </row>
     <row r="13" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="120" t="s">
+      <c r="A13" s="119" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="76"/>
+      <c r="B13" s="75"/>
       <c r="C13" s="17">
         <f>HardpointsRr!C9*2/1000</f>
         <v>1.2470640000000002</v>
@@ -3482,32 +3482,32 @@
       <c r="E13" s="18"/>
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="120" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="80"/>
-      <c r="C14" s="82">
+      <c r="A14" s="119" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="79"/>
+      <c r="C14" s="81">
         <v>255.07</v>
       </c>
-      <c r="D14" s="81" t="s">
+      <c r="D14" s="80" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="83" t="s">
+      <c r="E14" s="82" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="120" t="s">
+      <c r="A15" s="119" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="76"/>
-      <c r="C15" s="85" t="s">
+      <c r="B15" s="75"/>
+      <c r="C15" s="84" t="s">
         <v>166</v>
       </c>
-      <c r="D15" s="87" t="s">
+      <c r="D15" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="84" t="s">
+      <c r="E15" s="83" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3583,34 +3583,34 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="147" t="s">
+      <c r="A5" s="146" t="s">
         <v>89</v>
       </c>
-      <c r="B5" s="75" t="s">
+      <c r="B5" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="78" t="s">
+      <c r="C5" s="77" t="s">
         <v>90</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="148"/>
-      <c r="B6" s="95" t="s">
+      <c r="A6" s="147"/>
+      <c r="B6" s="94" t="s">
         <v>91</v>
       </c>
-      <c r="C6" s="96">
+      <c r="C6" s="95">
         <v>78807.070000000007</v>
       </c>
-      <c r="D6" s="97" t="s">
+      <c r="D6" s="96" t="s">
         <v>92</v>
       </c>
-      <c r="E6" s="98"/>
+      <c r="E6" s="97"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="157"/>
-      <c r="B7" s="79" t="s">
+      <c r="A7" s="156"/>
+      <c r="B7" s="78" t="s">
         <v>144</v>
       </c>
       <c r="C7" s="20">
@@ -3619,46 +3619,46 @@
       <c r="D7" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="31"/>
+      <c r="E7" s="30"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="147" t="s">
+      <c r="A8" s="146" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="75" t="s">
+      <c r="B8" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="100" t="s">
+      <c r="C8" s="99" t="s">
         <v>90</v>
       </c>
       <c r="D8" s="12"/>
       <c r="E8" s="28"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="148"/>
-      <c r="B9" s="95" t="s">
+      <c r="A9" s="147"/>
+      <c r="B9" s="94" t="s">
         <v>91</v>
       </c>
-      <c r="C9" s="99">
+      <c r="C9" s="98">
         <v>56916.22</v>
       </c>
-      <c r="D9" s="97" t="s">
+      <c r="D9" s="96" t="s">
         <v>92</v>
       </c>
-      <c r="E9" s="98"/>
+      <c r="E9" s="97"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="157"/>
-      <c r="B10" s="79" t="s">
+      <c r="A10" s="156"/>
+      <c r="B10" s="78" t="s">
         <v>144</v>
       </c>
       <c r="C10" s="20">
         <v>0</v>
       </c>
-      <c r="D10" s="88" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="31"/>
+      <c r="D10" s="87" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3707,7 +3707,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="103" t="s">
+      <c r="C2" s="102" t="s">
         <v>157</v>
       </c>
       <c r="D2" s="9"/>
@@ -3736,190 +3736,190 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="147" t="s">
+      <c r="A5" s="146" t="s">
         <v>89</v>
       </c>
-      <c r="B5" s="75" t="s">
+      <c r="B5" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="78" t="s">
+      <c r="C5" s="77" t="s">
         <v>159</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="148"/>
-      <c r="B6" s="95" t="s">
+      <c r="A6" s="147"/>
+      <c r="B6" s="94" t="s">
         <v>94</v>
       </c>
-      <c r="C6" s="132" t="s">
+      <c r="C6" s="131" t="s">
         <v>94</v>
       </c>
-      <c r="D6" s="97" t="s">
+      <c r="D6" s="96" t="s">
         <v>92</v>
       </c>
-      <c r="E6" s="133" t="s">
+      <c r="E6" s="132" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="148"/>
-      <c r="B7" s="76" t="s">
+      <c r="A7" s="147"/>
+      <c r="B7" s="75" t="s">
         <v>95</v>
       </c>
       <c r="C7" s="24">
         <v>100000</v>
       </c>
-      <c r="D7" s="87" t="s">
+      <c r="D7" s="86" t="s">
         <v>92</v>
       </c>
       <c r="E7" s="18"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="148"/>
-      <c r="B8" s="76" t="s">
+      <c r="A8" s="147"/>
+      <c r="B8" s="75" t="s">
         <v>96</v>
       </c>
       <c r="C8" s="24">
         <v>100000</v>
       </c>
-      <c r="D8" s="87" t="s">
+      <c r="D8" s="86" t="s">
         <v>92</v>
       </c>
       <c r="E8" s="18"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="148"/>
-      <c r="B9" s="76" t="s">
+      <c r="A9" s="147"/>
+      <c r="B9" s="75" t="s">
         <v>97</v>
       </c>
       <c r="C9" s="24">
         <v>150</v>
       </c>
-      <c r="D9" s="87" t="s">
+      <c r="D9" s="86" t="s">
         <v>92</v>
       </c>
       <c r="E9" s="18"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="148"/>
-      <c r="B10" s="76" t="s">
+      <c r="A10" s="147"/>
+      <c r="B10" s="75" t="s">
         <v>98</v>
       </c>
       <c r="C10" s="24">
         <v>150</v>
       </c>
-      <c r="D10" s="87" t="s">
+      <c r="D10" s="86" t="s">
         <v>92</v>
       </c>
       <c r="E10" s="18"/>
     </row>
     <row r="11" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="157"/>
-      <c r="B11" s="79" t="s">
+      <c r="A11" s="156"/>
+      <c r="B11" s="78" t="s">
         <v>99</v>
       </c>
       <c r="C11" s="26">
         <v>1E-4</v>
       </c>
-      <c r="D11" s="88" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="31"/>
+      <c r="D11" s="87" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="30"/>
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="147" t="s">
+      <c r="A12" s="146" t="s">
         <v>93</v>
       </c>
-      <c r="B12" s="75" t="s">
+      <c r="B12" s="74" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="78" t="s">
+      <c r="C12" s="77" t="s">
         <v>159</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="28"/>
     </row>
     <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="148"/>
-      <c r="B13" s="95" t="s">
+      <c r="A13" s="147"/>
+      <c r="B13" s="94" t="s">
         <v>94</v>
       </c>
-      <c r="C13" s="132" t="s">
+      <c r="C13" s="131" t="s">
         <v>94</v>
       </c>
-      <c r="D13" s="102" t="s">
+      <c r="D13" s="101" t="s">
         <v>92</v>
       </c>
-      <c r="E13" s="133" t="s">
+      <c r="E13" s="132" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="148"/>
-      <c r="B14" s="76" t="s">
+      <c r="A14" s="147"/>
+      <c r="B14" s="75" t="s">
         <v>95</v>
       </c>
       <c r="C14" s="24">
         <v>100000</v>
       </c>
-      <c r="D14" s="102" t="s">
+      <c r="D14" s="101" t="s">
         <v>92</v>
       </c>
       <c r="E14" s="18"/>
     </row>
     <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="148"/>
-      <c r="B15" s="76" t="s">
+      <c r="A15" s="147"/>
+      <c r="B15" s="75" t="s">
         <v>96</v>
       </c>
       <c r="C15" s="24">
         <v>100000</v>
       </c>
-      <c r="D15" s="102" t="s">
+      <c r="D15" s="101" t="s">
         <v>92</v>
       </c>
       <c r="E15" s="18"/>
     </row>
     <row r="16" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="148"/>
-      <c r="B16" s="76" t="s">
+      <c r="A16" s="147"/>
+      <c r="B16" s="75" t="s">
         <v>97</v>
       </c>
       <c r="C16" s="24">
         <v>150</v>
       </c>
-      <c r="D16" s="102" t="s">
+      <c r="D16" s="101" t="s">
         <v>92</v>
       </c>
       <c r="E16" s="18"/>
     </row>
     <row r="17" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="148"/>
-      <c r="B17" s="76" t="s">
+      <c r="A17" s="147"/>
+      <c r="B17" s="75" t="s">
         <v>98</v>
       </c>
       <c r="C17" s="24">
         <v>150</v>
       </c>
-      <c r="D17" s="102" t="s">
+      <c r="D17" s="101" t="s">
         <v>92</v>
       </c>
       <c r="E17" s="18"/>
     </row>
     <row r="18" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="157"/>
-      <c r="B18" s="79" t="s">
+      <c r="A18" s="156"/>
+      <c r="B18" s="78" t="s">
         <v>99</v>
       </c>
       <c r="C18" s="26">
         <v>1E-4</v>
       </c>
-      <c r="D18" s="88" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="31"/>
+      <c r="D18" s="87" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3940,810 +3940,810 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="134">
+      <c r="A1" s="133">
         <v>-443.53</v>
       </c>
-      <c r="B1" s="134">
+      <c r="B1" s="133">
         <v>-3883.5949999999998</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="134">
+      <c r="A2" s="133">
         <v>-433.58</v>
       </c>
-      <c r="B2" s="134">
+      <c r="B2" s="133">
         <v>-3833.1889999999999</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="134">
+      <c r="A3" s="133">
         <v>-423.97</v>
       </c>
-      <c r="B3" s="134">
+      <c r="B3" s="133">
         <v>-3778.5659999999998</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="134">
+      <c r="A4" s="133">
         <v>-415</v>
       </c>
-      <c r="B4" s="134">
+      <c r="B4" s="133">
         <v>-3715.607</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="134">
+      <c r="A5" s="133">
         <v>-406.67</v>
       </c>
-      <c r="B5" s="134">
+      <c r="B5" s="133">
         <v>-3644.3130000000001</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="134">
+      <c r="A6" s="133">
         <v>-398.79</v>
       </c>
-      <c r="B6" s="134">
+      <c r="B6" s="133">
         <v>-3567.2330000000002</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="134">
+      <c r="A7" s="133">
         <v>-391.16</v>
       </c>
-      <c r="B7" s="134">
+      <c r="B7" s="133">
         <v>-3486.6219999999998</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="134">
+      <c r="A8" s="133">
         <v>-383.59</v>
       </c>
-      <c r="B8" s="134">
+      <c r="B8" s="133">
         <v>-3405.2269999999999</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="134">
+      <c r="A9" s="133">
         <v>-375.88</v>
       </c>
-      <c r="B9" s="134">
+      <c r="B9" s="133">
         <v>-3325.3029999999999</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="134">
+      <c r="A10" s="133">
         <v>-367.89</v>
       </c>
-      <c r="B10" s="134">
+      <c r="B10" s="133">
         <v>-3248.7130000000002</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="134">
+      <c r="A11" s="133">
         <v>-359.64</v>
       </c>
-      <c r="B11" s="134">
+      <c r="B11" s="133">
         <v>-3175.3589999999999</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="134">
+      <c r="A12" s="133">
         <v>-351.2</v>
       </c>
-      <c r="B12" s="134">
+      <c r="B12" s="133">
         <v>-3104.163</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="134">
+      <c r="A13" s="133">
         <v>-342.63</v>
       </c>
-      <c r="B13" s="134">
+      <c r="B13" s="133">
         <v>-3034.5360000000001</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="134">
+      <c r="A14" s="133">
         <v>-334</v>
       </c>
-      <c r="B14" s="134">
+      <c r="B14" s="133">
         <v>-2965.6930000000002</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" s="134">
+      <c r="A15" s="133">
         <v>-325.38</v>
       </c>
-      <c r="B15" s="134">
+      <c r="B15" s="133">
         <v>-2896.85</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="134">
+      <c r="A16" s="133">
         <v>-316.77</v>
       </c>
-      <c r="B16" s="134">
+      <c r="B16" s="133">
         <v>-2827.6149999999998</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="134">
+      <c r="A17" s="133">
         <v>-308.2</v>
       </c>
-      <c r="B17" s="134">
+      <c r="B17" s="133">
         <v>-2757.9879999999998</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="134">
+      <c r="A18" s="133">
         <v>-299.64999999999998</v>
       </c>
-      <c r="B18" s="134">
+      <c r="B18" s="133">
         <v>-2687.9690000000001</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="134">
+      <c r="A19" s="133">
         <v>-291.14</v>
       </c>
-      <c r="B19" s="134">
+      <c r="B19" s="133">
         <v>-2617.5569999999998</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="134">
+      <c r="A20" s="133">
         <v>-282.67</v>
       </c>
-      <c r="B20" s="134">
+      <c r="B20" s="133">
         <v>-2546.6550000000002</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="134">
+      <c r="A21" s="133">
         <v>-274.25</v>
       </c>
-      <c r="B21" s="134">
+      <c r="B21" s="133">
         <v>-2475.1640000000002</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="134">
+      <c r="A22" s="133">
         <v>-265.91000000000003</v>
       </c>
-      <c r="B22" s="134">
+      <c r="B22" s="133">
         <v>-2402.7910000000002</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="134">
+      <c r="A23" s="133">
         <v>-257.67</v>
       </c>
-      <c r="B23" s="134">
+      <c r="B23" s="133">
         <v>-2329.3389999999999</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" s="134">
+      <c r="A24" s="133">
         <v>-249.56</v>
       </c>
-      <c r="B24" s="134">
+      <c r="B24" s="133">
         <v>-2254.5149999999999</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25" s="134">
+      <c r="A25" s="133">
         <v>-241.62</v>
       </c>
-      <c r="B25" s="134">
+      <c r="B25" s="133">
         <v>-2178.2190000000001</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" s="134">
+      <c r="A26" s="133">
         <v>-233.85</v>
       </c>
-      <c r="B26" s="134">
+      <c r="B26" s="133">
         <v>-2100.06</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27" s="134">
+      <c r="A27" s="133">
         <v>-226.23</v>
       </c>
-      <c r="B27" s="134">
+      <c r="B27" s="133">
         <v>-2020.528</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A28" s="134">
+      <c r="A28" s="133">
         <v>-218.75</v>
       </c>
-      <c r="B28" s="134">
+      <c r="B28" s="133">
         <v>-1939.623</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" s="134">
+      <c r="A29" s="133">
         <v>-211.37</v>
       </c>
-      <c r="B29" s="134">
+      <c r="B29" s="133">
         <v>-1857.934</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A30" s="134">
+      <c r="A30" s="133">
         <v>-204.05</v>
       </c>
-      <c r="B30" s="134">
+      <c r="B30" s="133">
         <v>-1775.46</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A31" s="134">
+      <c r="A31" s="133">
         <v>-196.78</v>
       </c>
-      <c r="B31" s="134">
+      <c r="B31" s="133">
         <v>-1692.79</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A32" s="134">
+      <c r="A32" s="133">
         <v>-189.52</v>
       </c>
-      <c r="B32" s="134">
+      <c r="B32" s="133">
         <v>-1609.923</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" s="134">
+      <c r="A33" s="133">
         <v>-182.26</v>
       </c>
-      <c r="B33" s="134">
+      <c r="B33" s="133">
         <v>-1527.155</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A34" s="134">
+      <c r="A34" s="133">
         <v>-174.97</v>
       </c>
-      <c r="B34" s="134">
+      <c r="B34" s="133">
         <v>-1444.681</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" s="134">
+      <c r="A35" s="133">
         <v>-167.65</v>
       </c>
-      <c r="B35" s="134">
+      <c r="B35" s="133">
         <v>-1362.502</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" s="134">
+      <c r="A36" s="133">
         <v>-160.27000000000001</v>
       </c>
-      <c r="B36" s="134">
+      <c r="B36" s="133">
         <v>-1280.8119999999999</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" s="134">
+      <c r="A37" s="133">
         <v>-152.82</v>
       </c>
-      <c r="B37" s="134">
+      <c r="B37" s="133">
         <v>-1199.711</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" s="134">
+      <c r="A38" s="133">
         <v>-145.29</v>
       </c>
-      <c r="B38" s="134">
+      <c r="B38" s="133">
         <v>-1119.297</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A39" s="134">
+      <c r="A39" s="133">
         <v>-137.65</v>
       </c>
-      <c r="B39" s="134">
+      <c r="B39" s="133">
         <v>-1039.7650000000001</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A40" s="134">
+      <c r="A40" s="133">
         <v>-129.9</v>
       </c>
-      <c r="B40" s="134">
+      <c r="B40" s="133">
         <v>-961.31200000000001</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A41" s="134">
+      <c r="A41" s="133">
         <v>-122.02</v>
       </c>
-      <c r="B41" s="134">
+      <c r="B41" s="133">
         <v>-884.13300000000004</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" s="134">
+      <c r="A42" s="133">
         <v>-114.01</v>
       </c>
-      <c r="B42" s="134">
+      <c r="B42" s="133">
         <v>-808.32799999999997</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A43" s="134">
+      <c r="A43" s="133">
         <v>-105.84</v>
       </c>
-      <c r="B43" s="134">
+      <c r="B43" s="133">
         <v>-734.19</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A44" s="134">
+      <c r="A44" s="133">
         <v>-97.52</v>
       </c>
-      <c r="B44" s="134">
+      <c r="B44" s="133">
         <v>-661.71799999999996</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A45" s="134">
+      <c r="A45" s="133">
         <v>-89.05</v>
       </c>
-      <c r="B45" s="134">
+      <c r="B45" s="133">
         <v>-590.91399999999999</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A46" s="134">
+      <c r="A46" s="133">
         <v>-80.430000000000007</v>
       </c>
-      <c r="B46" s="134">
+      <c r="B46" s="133">
         <v>-521.67999999999995</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A47" s="134">
+      <c r="A47" s="133">
         <v>-71.680000000000007</v>
       </c>
-      <c r="B47" s="134">
+      <c r="B47" s="133">
         <v>-454.21</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A48" s="134">
+      <c r="A48" s="133">
         <v>-62.8</v>
       </c>
-      <c r="B48" s="134">
+      <c r="B48" s="133">
         <v>-388.113</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A49" s="134">
+      <c r="A49" s="133">
         <v>-53.8</v>
       </c>
-      <c r="B49" s="134">
+      <c r="B49" s="133">
         <v>-323.68299999999999</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A50" s="134">
+      <c r="A50" s="133">
         <v>-44.68</v>
       </c>
-      <c r="B50" s="134">
+      <c r="B50" s="133">
         <v>-260.92099999999999</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A51" s="134">
+      <c r="A51" s="133">
         <v>-35.409999999999997</v>
       </c>
-      <c r="B51" s="134">
+      <c r="B51" s="133">
         <v>-200.41399999999999</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A52" s="134">
+      <c r="A52" s="133">
         <v>-25.99</v>
       </c>
-      <c r="B52" s="134">
+      <c r="B52" s="133">
         <v>-142.26</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A53" s="134">
+      <c r="A53" s="133">
         <v>-16.38</v>
       </c>
-      <c r="B53" s="134">
+      <c r="B53" s="133">
         <v>-86.950999999999993</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A54" s="134">
+      <c r="A54" s="133">
         <v>-6.61</v>
       </c>
-      <c r="B54" s="134">
+      <c r="B54" s="133">
         <v>-34.387</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A55" s="134">
+      <c r="A55" s="133">
         <v>0</v>
       </c>
-      <c r="B55" s="134">
+      <c r="B55" s="133">
         <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A56" s="134">
+      <c r="A56" s="133">
         <v>3.23</v>
       </c>
-      <c r="B56" s="134">
+      <c r="B56" s="133">
         <v>16.803999999999998</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A57" s="134">
+      <c r="A57" s="133">
         <v>13.04</v>
       </c>
-      <c r="B57" s="134">
+      <c r="B57" s="133">
         <v>68.484999999999999</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A58" s="134">
+      <c r="A58" s="133">
         <v>22.71</v>
       </c>
-      <c r="B58" s="134">
+      <c r="B58" s="133">
         <v>122.42100000000001</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A59" s="134">
+      <c r="A59" s="133">
         <v>32.119999999999997</v>
       </c>
-      <c r="B59" s="134">
+      <c r="B59" s="133">
         <v>180.18199999999999</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A60" s="134">
+      <c r="A60" s="133">
         <v>41.25</v>
       </c>
-      <c r="B60" s="134">
+      <c r="B60" s="133">
         <v>242.25899999999999</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A61" s="134">
+      <c r="A61" s="133">
         <v>50.17</v>
       </c>
-      <c r="B61" s="134">
+      <c r="B61" s="133">
         <v>307.66899999999998</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A62" s="134">
+      <c r="A62" s="133">
         <v>58.93</v>
       </c>
-      <c r="B62" s="134">
+      <c r="B62" s="133">
         <v>375.33499999999998</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A63" s="134">
+      <c r="A63" s="133">
         <v>67.61</v>
       </c>
-      <c r="B63" s="134">
+      <c r="B63" s="133">
         <v>444.07900000000001</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A64" s="134">
+      <c r="A64" s="133">
         <v>76.28</v>
       </c>
-      <c r="B64" s="134">
+      <c r="B64" s="133">
         <v>512.92200000000003</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A65" s="134">
+      <c r="A65" s="133">
         <v>84.97</v>
       </c>
-      <c r="B65" s="134">
+      <c r="B65" s="133">
         <v>581.274</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A66" s="134">
+      <c r="A66" s="133">
         <v>93.66</v>
       </c>
-      <c r="B66" s="134">
+      <c r="B66" s="133">
         <v>649.33299999999997</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A67" s="134">
+      <c r="A67" s="133">
         <v>102.34</v>
       </c>
-      <c r="B67" s="134">
+      <c r="B67" s="133">
         <v>717.58699999999999</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A68" s="134">
+      <c r="A68" s="133">
         <v>110.99</v>
       </c>
-      <c r="B68" s="134">
+      <c r="B68" s="133">
         <v>786.23299999999995</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A69" s="134">
+      <c r="A69" s="133">
         <v>119.59</v>
       </c>
-      <c r="B69" s="134">
+      <c r="B69" s="133">
         <v>855.66399999999999</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A70" s="134">
+      <c r="A70" s="133">
         <v>128.15</v>
       </c>
-      <c r="B70" s="134">
+      <c r="B70" s="133">
         <v>925.68399999999997</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A71" s="134">
+      <c r="A71" s="133">
         <v>136.76</v>
       </c>
-      <c r="B71" s="134">
+      <c r="B71" s="133">
         <v>995.11500000000001</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A72" s="134">
+      <c r="A72" s="133">
         <v>145.5</v>
       </c>
-      <c r="B72" s="134">
+      <c r="B72" s="133">
         <v>1062.8789999999999</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A73" s="134">
+      <c r="A73" s="133">
         <v>154.46</v>
       </c>
-      <c r="B73" s="134">
+      <c r="B73" s="133">
         <v>1127.6030000000001</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A74" s="134">
+      <c r="A74" s="133">
         <v>163.72</v>
       </c>
-      <c r="B74" s="134">
+      <c r="B74" s="133">
         <v>1188.1099999999999</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A75" s="134">
+      <c r="A75" s="133">
         <v>173.35</v>
       </c>
-      <c r="B75" s="134">
+      <c r="B75" s="133">
         <v>1243.3209999999999</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A76" s="134">
+      <c r="A76" s="133">
         <v>183.3</v>
       </c>
-      <c r="B76" s="134">
+      <c r="B76" s="133">
         <v>1293.0409999999999</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A77" s="134">
+      <c r="A77" s="133">
         <v>193.53</v>
       </c>
-      <c r="B77" s="134">
+      <c r="B77" s="133">
         <v>1336.877</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A78" s="134">
+      <c r="A78" s="133">
         <v>204</v>
       </c>
-      <c r="B78" s="134">
+      <c r="B78" s="133">
         <v>1374.829</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A79" s="134">
+      <c r="A79" s="133">
         <v>214.66</v>
       </c>
-      <c r="B79" s="134">
+      <c r="B79" s="133">
         <v>1406.7</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A80" s="134">
+      <c r="A80" s="133">
         <v>225.46</v>
       </c>
-      <c r="B80" s="134">
+      <c r="B80" s="133">
         <v>1433.2760000000001</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A81" s="134">
+      <c r="A81" s="133">
         <v>236.35</v>
       </c>
-      <c r="B81" s="134">
+      <c r="B81" s="133">
         <v>1455.93</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A82" s="134">
+      <c r="A82" s="133">
         <v>247.31</v>
       </c>
-      <c r="B82" s="134">
+      <c r="B82" s="133">
         <v>1476.0329999999999</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A83" s="134">
+      <c r="A83" s="133">
         <v>258.27999999999997</v>
       </c>
-      <c r="B83" s="134">
+      <c r="B83" s="133">
         <v>1494.8620000000001</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A84" s="134">
+      <c r="A84" s="133">
         <v>269.26</v>
       </c>
-      <c r="B84" s="134">
+      <c r="B84" s="133">
         <v>1513.396</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A85" s="134">
+      <c r="A85" s="133">
         <v>280.23</v>
       </c>
-      <c r="B85" s="134">
+      <c r="B85" s="133">
         <v>1531.8330000000001</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A86" s="134">
+      <c r="A86" s="133">
         <v>291.19</v>
       </c>
-      <c r="B86" s="134">
+      <c r="B86" s="133">
         <v>1550.3679999999999</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A87" s="134">
+      <c r="A87" s="133">
         <v>302.14999999999998</v>
       </c>
-      <c r="B87" s="134">
+      <c r="B87" s="133">
         <v>1569.2940000000001</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A88" s="134">
+      <c r="A88" s="133">
         <v>313.10000000000002</v>
       </c>
-      <c r="B88" s="134">
+      <c r="B88" s="133">
         <v>1588.712</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A89" s="134">
+      <c r="A89" s="133">
         <v>324.05</v>
       </c>
-      <c r="B89" s="134">
+      <c r="B89" s="133">
         <v>1608.325</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A90" s="134">
+      <c r="A90" s="133">
         <v>335.01</v>
       </c>
-      <c r="B90" s="134">
+      <c r="B90" s="133">
         <v>1627.9380000000001</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A91" s="134">
+      <c r="A91" s="133">
         <v>345.96</v>
       </c>
-      <c r="B91" s="134">
+      <c r="B91" s="133">
         <v>1647.2570000000001</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A92" s="134">
+      <c r="A92" s="133">
         <v>356.92</v>
       </c>
-      <c r="B92" s="134">
+      <c r="B92" s="133">
         <v>1666.2819999999999</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A93" s="134">
+      <c r="A93" s="133">
         <v>367.88</v>
       </c>
-      <c r="B93" s="134">
+      <c r="B93" s="133">
         <v>1685.6010000000001</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A94" s="134">
+      <c r="A94" s="133">
         <v>378.83</v>
       </c>
-      <c r="B94" s="134">
+      <c r="B94" s="133">
         <v>1705.4110000000001</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A95" s="134">
+      <c r="A95" s="133">
         <v>389.75</v>
       </c>
-      <c r="B95" s="134">
+      <c r="B95" s="133">
         <v>1726.3969999999999</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A96" s="134">
+      <c r="A96" s="133">
         <v>400.65</v>
       </c>
-      <c r="B96" s="134">
+      <c r="B96" s="133">
         <v>1748.6579999999999</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A97" s="134">
+      <c r="A97" s="133">
         <v>411.52</v>
       </c>
-      <c r="B97" s="134">
+      <c r="B97" s="133">
         <v>1772.39</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A98" s="134">
+      <c r="A98" s="133">
         <v>422.35</v>
       </c>
-      <c r="B98" s="134">
+      <c r="B98" s="133">
         <v>1797.4949999999999</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A99" s="134">
+      <c r="A99" s="133">
         <v>433.15</v>
       </c>
-      <c r="B99" s="134">
+      <c r="B99" s="133">
         <v>1823.973</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A100" s="134">
+      <c r="A100" s="133">
         <v>443.91</v>
       </c>
-      <c r="B100" s="134">
+      <c r="B100" s="133">
         <v>1851.8240000000001</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A101" s="134">
+      <c r="A101" s="133">
         <v>454.66</v>
       </c>
-      <c r="B101" s="134">
+      <c r="B101" s="133">
         <v>1880.3610000000001</v>
       </c>
     </row>
@@ -4784,7 +4784,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="103" t="s">
+      <c r="C2" s="102" t="s">
         <v>100</v>
       </c>
       <c r="D2" s="9"/>
@@ -4795,7 +4795,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="103" t="s">
+      <c r="C3" s="102" t="s">
         <v>153</v>
       </c>
       <c r="D3" s="9"/>
@@ -4806,144 +4806,144 @@
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="103" t="s">
+      <c r="C4" s="102" t="s">
         <v>163</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="93" t="s">
+      <c r="A5" s="92" t="s">
         <v>101</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="122" t="s">
+      <c r="B5" s="74"/>
+      <c r="C5" s="121" t="s">
         <v>154</v>
       </c>
-      <c r="D5" s="104" t="s">
+      <c r="D5" s="103" t="s">
         <v>102</v>
       </c>
-      <c r="E5" s="105" t="s">
+      <c r="E5" s="104" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="93" t="s">
+      <c r="A6" s="92" t="s">
         <v>104</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="101">
+      <c r="B6" s="74"/>
+      <c r="C6" s="100">
         <v>10</v>
       </c>
-      <c r="D6" s="104" t="s">
+      <c r="D6" s="103" t="s">
         <v>29</v>
       </c>
       <c r="E6" s="28"/>
     </row>
     <row r="7" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="93" t="s">
+      <c r="A7" s="92" t="s">
         <v>105</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="101" t="s">
+      <c r="B7" s="74"/>
+      <c r="C7" s="100" t="s">
         <v>106</v>
       </c>
-      <c r="D7" s="104" t="s">
+      <c r="D7" s="103" t="s">
         <v>107</v>
       </c>
       <c r="E7" s="28"/>
     </row>
     <row r="8" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="93" t="s">
+      <c r="A8" s="92" t="s">
         <v>108</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="106" t="s">
+      <c r="B8" s="74"/>
+      <c r="C8" s="105" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="104" t="s">
+      <c r="D8" s="103" t="s">
         <v>102</v>
       </c>
       <c r="E8" s="28"/>
     </row>
     <row r="9" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="93" t="s">
+      <c r="A9" s="92" t="s">
         <v>110</v>
       </c>
-      <c r="B9" s="75"/>
-      <c r="C9" s="101">
+      <c r="B9" s="74"/>
+      <c r="C9" s="100">
         <v>25000</v>
       </c>
-      <c r="D9" s="104"/>
+      <c r="D9" s="103"/>
       <c r="E9" s="28"/>
     </row>
     <row r="10" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="93" t="s">
+      <c r="A10" s="92" t="s">
         <v>111</v>
       </c>
-      <c r="B10" s="75"/>
-      <c r="C10" s="101">
+      <c r="B10" s="74"/>
+      <c r="C10" s="100">
         <v>0.01</v>
       </c>
-      <c r="D10" s="104" t="s">
+      <c r="D10" s="103" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="105" t="s">
+      <c r="E10" s="104" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="147" t="s">
+      <c r="A11" s="146" t="s">
         <v>114</v>
       </c>
-      <c r="B11" s="107" t="s">
+      <c r="B11" s="106" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="108" t="s">
+      <c r="C11" s="107" t="s">
         <v>148</v>
       </c>
-      <c r="D11" s="92"/>
-      <c r="E11" s="72"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="71"/>
     </row>
     <row r="12" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="157"/>
-      <c r="B12" s="109" t="s">
+      <c r="A12" s="156"/>
+      <c r="B12" s="108" t="s">
         <v>115</v>
       </c>
-      <c r="C12" s="110" t="s">
+      <c r="C12" s="109" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="111" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="112"/>
+      <c r="D12" s="110" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="111"/>
     </row>
     <row r="13" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="93" t="s">
+      <c r="A13" s="92" t="s">
         <v>151</v>
       </c>
-      <c r="B13" s="75"/>
-      <c r="C13" s="101" t="s">
+      <c r="B13" s="74"/>
+      <c r="C13" s="100" t="s">
         <v>164</v>
       </c>
-      <c r="D13" s="104"/>
-      <c r="E13" s="105" t="s">
+      <c r="D13" s="103"/>
+      <c r="E13" s="104" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="93" t="s">
+      <c r="A14" s="92" t="s">
         <v>152</v>
       </c>
-      <c r="B14" s="75"/>
-      <c r="C14" s="101" t="s">
+      <c r="B14" s="74"/>
+      <c r="C14" s="100" t="s">
         <v>165</v>
       </c>
-      <c r="D14" s="104"/>
-      <c r="E14" s="105"/>
+      <c r="D14" s="103"/>
+      <c r="E14" s="104"/>
     </row>
     <row r="18" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D18" s="137" t="s">
+      <c r="D18" s="136" t="s">
         <v>162</v>
       </c>
     </row>
@@ -4969,296 +4969,296 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="31" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="31" t="s">
         <v>117</v>
       </c>
-      <c r="C1" s="32" t="s">
+      <c r="C1" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="31" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="B2" s="34">
+      <c r="B2" s="33">
         <v>200</v>
       </c>
-      <c r="C2" s="35">
+      <c r="C2" s="34">
         <v>203.34700000000001</v>
       </c>
-      <c r="D2" s="35">
+      <c r="D2" s="34">
         <v>126.35</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="B3" s="37">
+      <c r="B3" s="36">
         <v>-200</v>
       </c>
-      <c r="C3" s="38">
+      <c r="C3" s="37">
         <v>225</v>
       </c>
-      <c r="D3" s="38">
+      <c r="D3" s="37">
         <v>126.35</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="35" t="s">
         <v>122</v>
       </c>
-      <c r="B4" s="37">
+      <c r="B4" s="36">
         <v>11.946</v>
       </c>
-      <c r="C4" s="38">
+      <c r="C4" s="37">
         <v>587.82100000000003</v>
       </c>
-      <c r="D4" s="38">
+      <c r="D4" s="37">
         <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="35" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="37">
+      <c r="B5" s="36">
         <v>148.751</v>
       </c>
-      <c r="C5" s="38">
+      <c r="C5" s="37">
         <v>207.047</v>
       </c>
-      <c r="D5" s="38">
+      <c r="D5" s="37">
         <v>321.79399999999998</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="35" t="s">
         <v>124</v>
       </c>
-      <c r="B6" s="37">
+      <c r="B6" s="36">
         <v>-184.72900000000001</v>
       </c>
-      <c r="C6" s="38">
+      <c r="C6" s="37">
         <v>225</v>
       </c>
-      <c r="D6" s="38">
+      <c r="D6" s="37">
         <v>300.89400000000001</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="35" t="s">
         <v>125</v>
       </c>
-      <c r="B7" s="37">
+      <c r="B7" s="36">
         <v>-12.932</v>
       </c>
-      <c r="C7" s="38">
+      <c r="C7" s="37">
         <v>518.67999999999995</v>
       </c>
-      <c r="D7" s="38">
+      <c r="D7" s="37">
         <v>374.39299999999997</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="B8" s="37">
+      <c r="B8" s="36">
         <v>16.193999999999999</v>
       </c>
-      <c r="C8" s="38">
+      <c r="C8" s="37">
         <v>582.05899999999997</v>
       </c>
-      <c r="D8" s="38">
+      <c r="D8" s="37">
         <v>263.346</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="35" t="s">
         <v>127</v>
       </c>
-      <c r="B9" s="37">
+      <c r="B9" s="36">
         <v>0</v>
       </c>
-      <c r="C9" s="38">
+      <c r="C9" s="37">
         <v>640</v>
       </c>
-      <c r="D9" s="38">
+      <c r="D9" s="37">
         <v>260.36099999999999</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="35" t="s">
         <v>128</v>
       </c>
-      <c r="B10" s="37">
+      <c r="B10" s="36">
         <v>104.241</v>
       </c>
-      <c r="C10" s="38">
+      <c r="C10" s="37">
         <v>250</v>
       </c>
-      <c r="D10" s="38">
+      <c r="D10" s="37">
         <v>171.053</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="36" t="s">
+      <c r="A11" s="35" t="s">
         <v>129</v>
       </c>
-      <c r="B11" s="37">
+      <c r="B11" s="36">
         <v>85.097999999999999</v>
       </c>
-      <c r="C11" s="38">
+      <c r="C11" s="37">
         <v>575.40700000000004</v>
       </c>
-      <c r="D11" s="38">
+      <c r="D11" s="37">
         <v>188.44399999999999</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="36" t="s">
+      <c r="A12" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="B12" s="37">
+      <c r="B12" s="36">
         <v>11.157</v>
       </c>
-      <c r="C12" s="38">
+      <c r="C12" s="37">
         <v>233.131</v>
       </c>
-      <c r="D12" s="38">
+      <c r="D12" s="37">
         <v>517.55100000000004</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="36" t="s">
+      <c r="A13" s="35" t="s">
         <v>131</v>
       </c>
-      <c r="B13" s="37">
+      <c r="B13" s="36">
         <v>11.484999999999999</v>
       </c>
-      <c r="C13" s="38">
+      <c r="C13" s="37">
         <v>317.84199999999998</v>
       </c>
-      <c r="D13" s="38">
+      <c r="D13" s="37">
         <v>362.43</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="35" t="s">
         <v>132</v>
       </c>
-      <c r="B14" s="37">
+      <c r="B14" s="36">
         <v>11.821</v>
       </c>
-      <c r="C14" s="38">
+      <c r="C14" s="37">
         <v>550</v>
       </c>
-      <c r="D14" s="38">
+      <c r="D14" s="37">
         <v>178.70500000000001</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="36" t="s">
+      <c r="A15" s="35" t="s">
         <v>133</v>
       </c>
-      <c r="B15" s="37">
+      <c r="B15" s="36">
         <v>11.489000000000001</v>
       </c>
-      <c r="C15" s="38">
+      <c r="C15" s="37">
         <v>351.53699999999998</v>
       </c>
-      <c r="D15" s="38">
+      <c r="D15" s="37">
         <v>360.94299999999998</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="36" t="s">
+      <c r="A16" s="35" t="s">
         <v>134</v>
       </c>
-      <c r="B16" s="37">
+      <c r="B16" s="36">
         <v>11.558</v>
       </c>
-      <c r="C16" s="38">
+      <c r="C16" s="37">
         <v>244.43100000000001</v>
       </c>
-      <c r="D16" s="38">
+      <c r="D16" s="37">
         <v>328.19799999999998</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="B17" s="37">
-        <v>67.965000000000003</v>
-      </c>
-      <c r="C17" s="38">
+      <c r="B17" s="36">
+        <v>20.965</v>
+      </c>
+      <c r="C17" s="37">
         <v>262.85500000000002</v>
       </c>
-      <c r="D17" s="38">
+      <c r="D17" s="37">
         <v>101.35</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="36" t="s">
+      <c r="A18" s="35" t="s">
         <v>136</v>
       </c>
-      <c r="B18" s="37">
+      <c r="B18" s="36">
         <v>-23.5</v>
       </c>
-      <c r="C18" s="38">
+      <c r="C18" s="37">
         <v>262.85500000000002</v>
       </c>
-      <c r="D18" s="38">
+      <c r="D18" s="37">
         <v>101.51900000000001</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="35" t="s">
         <v>137</v>
       </c>
-      <c r="B19" s="37">
+      <c r="B19" s="36">
         <v>11.526999999999999</v>
       </c>
-      <c r="C19" s="38">
+      <c r="C19" s="37">
         <v>292.24599999999998</v>
       </c>
-      <c r="D19" s="38">
+      <c r="D19" s="37">
         <v>342.81599999999997</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="36" t="s">
+      <c r="A20" s="35" t="s">
         <v>138</v>
       </c>
-      <c r="B20" s="37">
+      <c r="B20" s="36">
         <v>104.241</v>
       </c>
-      <c r="C20" s="38">
+      <c r="C20" s="37">
         <v>0</v>
       </c>
-      <c r="D20" s="38">
+      <c r="D20" s="37">
         <v>171.053</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="35" t="s">
         <v>139</v>
       </c>
-      <c r="B21" s="37">
+      <c r="B21" s="36">
         <v>-324.96499999999997</v>
       </c>
-      <c r="C21" s="38">
+      <c r="C21" s="37">
         <v>0</v>
       </c>
-      <c r="D21" s="38">
+      <c r="D21" s="37">
         <v>533.79200000000003</v>
       </c>
     </row>
@@ -5285,268 +5285,268 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="31" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="31" t="s">
         <v>117</v>
       </c>
-      <c r="C1" s="32" t="s">
+      <c r="C1" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="31" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="B2" s="34">
+      <c r="B2" s="33">
         <v>-1390</v>
       </c>
-      <c r="C2" s="35">
+      <c r="C2" s="34">
         <v>305</v>
       </c>
-      <c r="D2" s="35">
+      <c r="D2" s="34">
         <v>126.35</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="B3" s="37">
+      <c r="B3" s="36">
         <v>-1830</v>
       </c>
-      <c r="C3" s="38">
+      <c r="C3" s="37">
         <v>270</v>
       </c>
-      <c r="D3" s="38">
+      <c r="D3" s="37">
         <v>126.35</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="35" t="s">
         <v>122</v>
       </c>
-      <c r="B4" s="37">
+      <c r="B4" s="36">
         <v>-1579.2370000000001</v>
       </c>
-      <c r="C4" s="38">
+      <c r="C4" s="37">
         <v>573.947</v>
       </c>
-      <c r="D4" s="38">
+      <c r="D4" s="37">
         <v>137.5</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="35" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="37">
+      <c r="B5" s="36">
         <v>-1390</v>
       </c>
-      <c r="C5" s="38">
+      <c r="C5" s="37">
         <v>305</v>
       </c>
-      <c r="D5" s="38">
+      <c r="D5" s="37">
         <v>328.98099999999999</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="35" t="s">
         <v>124</v>
       </c>
-      <c r="B6" s="37">
+      <c r="B6" s="36">
         <v>-1830</v>
       </c>
-      <c r="C6" s="38">
+      <c r="C6" s="37">
         <v>270</v>
       </c>
-      <c r="D6" s="38">
+      <c r="D6" s="37">
         <v>354.47500000000002</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="35" t="s">
         <v>125</v>
       </c>
-      <c r="B7" s="37">
+      <c r="B7" s="36">
         <v>-1569.845</v>
       </c>
-      <c r="C7" s="38">
+      <c r="C7" s="37">
         <v>506.33</v>
       </c>
-      <c r="D7" s="38">
+      <c r="D7" s="37">
         <v>382.471</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="B8" s="37">
+      <c r="B8" s="36">
         <v>-1568.8710000000001</v>
       </c>
-      <c r="C8" s="38">
+      <c r="C8" s="37">
         <v>566.64200000000005</v>
       </c>
-      <c r="D8" s="38">
+      <c r="D8" s="37">
         <v>269.14400000000001</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="35" t="s">
         <v>127</v>
       </c>
-      <c r="B9" s="37">
+      <c r="B9" s="36">
         <v>-1574.5989999999999</v>
       </c>
-      <c r="C9" s="38">
+      <c r="C9" s="37">
         <v>623.53200000000004</v>
       </c>
-      <c r="D9" s="38">
+      <c r="D9" s="37">
         <v>260.36099999999999</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="35" t="s">
         <v>128</v>
       </c>
-      <c r="B10" s="37">
+      <c r="B10" s="36">
         <v>-1830</v>
       </c>
-      <c r="C10" s="38">
+      <c r="C10" s="37">
         <v>270</v>
       </c>
-      <c r="D10" s="38">
+      <c r="D10" s="37">
         <v>193.642</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="36" t="s">
+      <c r="A11" s="35" t="s">
         <v>129</v>
       </c>
-      <c r="B11" s="37">
+      <c r="B11" s="36">
         <v>-1675.904</v>
       </c>
-      <c r="C11" s="38">
+      <c r="C11" s="37">
         <v>576.73500000000001</v>
       </c>
-      <c r="D11" s="38">
+      <c r="D11" s="37">
         <v>225.33099999999999</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="36" t="s">
+      <c r="A12" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="B12" s="37">
+      <c r="B12" s="36">
         <v>-1395.9760000000001</v>
       </c>
-      <c r="C12" s="38">
+      <c r="C12" s="37">
         <v>283.399</v>
       </c>
-      <c r="D12" s="38">
+      <c r="D12" s="37">
         <v>436.10300000000001</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="36" t="s">
+      <c r="A13" s="35" t="s">
         <v>131</v>
       </c>
-      <c r="B13" s="37">
+      <c r="B13" s="36">
         <v>-1579.1110000000001</v>
       </c>
-      <c r="C13" s="38">
+      <c r="C13" s="37">
         <v>267.07299999999998</v>
       </c>
-      <c r="D13" s="38">
+      <c r="D13" s="37">
         <v>484.01</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="35" t="s">
         <v>132</v>
       </c>
-      <c r="B14" s="37">
+      <c r="B14" s="36">
         <v>-1597.194</v>
       </c>
-      <c r="C14" s="38">
+      <c r="C14" s="37">
         <v>526.39499999999998</v>
       </c>
-      <c r="D14" s="38">
+      <c r="D14" s="37">
         <v>155.28700000000001</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="36" t="s">
+      <c r="A15" s="35" t="s">
         <v>133</v>
       </c>
-      <c r="B15" s="37">
+      <c r="B15" s="36">
         <v>-1664.6120000000001</v>
       </c>
-      <c r="C15" s="38">
+      <c r="C15" s="37">
         <v>349.04700000000003</v>
       </c>
-      <c r="D15" s="38">
+      <c r="D15" s="37">
         <v>403.92399999999998</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="36" t="s">
+      <c r="A16" s="35" t="s">
         <v>134</v>
       </c>
-      <c r="B16" s="37">
+      <c r="B16" s="36">
         <v>-1585.771</v>
       </c>
-      <c r="C16" s="38">
+      <c r="C16" s="37">
         <v>318.42700000000002</v>
       </c>
-      <c r="D16" s="38">
+      <c r="D16" s="37">
         <v>426.35</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="35" t="s">
         <v>135</v>
       </c>
-      <c r="B17" s="37">
+      <c r="B17" s="36">
         <v>-1830</v>
       </c>
-      <c r="C17" s="38">
+      <c r="C17" s="37">
         <v>305</v>
       </c>
-      <c r="D17" s="38">
+      <c r="D17" s="37">
         <v>401.35</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="36" t="s">
+      <c r="A18" s="35" t="s">
         <v>136</v>
       </c>
-      <c r="B18" s="37">
+      <c r="B18" s="36">
         <v>-1830</v>
       </c>
-      <c r="C18" s="38">
+      <c r="C18" s="37">
         <v>305</v>
       </c>
-      <c r="D18" s="38">
+      <c r="D18" s="37">
         <v>448.35</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="35" t="s">
         <v>137</v>
       </c>
-      <c r="B19" s="37">
+      <c r="B19" s="36">
         <v>-1600.4860000000001</v>
       </c>
-      <c r="C19" s="38">
+      <c r="C19" s="37">
         <v>287.56599999999997</v>
       </c>
-      <c r="D19" s="38">
+      <c r="D19" s="37">
         <v>463.988</v>
       </c>
     </row>
@@ -5623,24 +5623,24 @@
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="115"/>
-      <c r="C5" s="117" t="s">
+      <c r="B5" s="114"/>
+      <c r="C5" s="116" t="s">
         <v>140</v>
       </c>
-      <c r="D5" s="118" t="s">
+      <c r="D5" s="117" t="s">
         <v>64</v>
       </c>
-      <c r="E5" s="116"/>
+      <c r="E5" s="115"/>
     </row>
     <row r="6" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="79"/>
-      <c r="C6" s="86" t="s">
+      <c r="B6" s="78"/>
+      <c r="C6" s="85" t="s">
         <v>63</v>
       </c>
-      <c r="D6" s="88" t="s">
+      <c r="D6" s="87" t="s">
         <v>64</v>
       </c>
       <c r="E6" s="22"/>
@@ -5649,11 +5649,11 @@
       <c r="A7" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B7" s="79"/>
-      <c r="C7" s="86" t="s">
+      <c r="B7" s="78"/>
+      <c r="C7" s="85" t="s">
         <v>65</v>
       </c>
-      <c r="D7" s="88" t="s">
+      <c r="D7" s="87" t="s">
         <v>64</v>
       </c>
       <c r="E7" s="22"/>
@@ -5700,7 +5700,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="103" t="s">
+      <c r="C2" s="102" t="s">
         <v>35</v>
       </c>
       <c r="D2" s="9"/>
@@ -5711,7 +5711,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="103" t="s">
+      <c r="C3" s="102" t="s">
         <v>36</v>
       </c>
       <c r="D3" s="9"/>
@@ -5722,17 +5722,17 @@
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="103" t="s">
+      <c r="C4" s="102" t="s">
         <v>37</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="141" t="s">
+      <c r="A5" s="140" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="75" t="s">
+      <c r="B5" s="74" t="s">
         <v>39</v>
       </c>
       <c r="C5" s="23" t="str">
@@ -5747,8 +5747,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="139"/>
-      <c r="B6" s="76" t="s">
+      <c r="A6" s="138"/>
+      <c r="B6" s="75" t="s">
         <v>41</v>
       </c>
       <c r="C6" s="24" t="str" cm="1">
@@ -5763,8 +5763,8 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="142"/>
-      <c r="B7" s="76" t="s">
+      <c r="A7" s="141"/>
+      <c r="B7" s="75" t="s">
         <v>42</v>
       </c>
       <c r="C7" s="24" t="str" cm="1">
@@ -5779,8 +5779,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="142"/>
-      <c r="B8" s="79" t="s">
+      <c r="A8" s="141"/>
+      <c r="B8" s="78" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="20">
@@ -5792,10 +5792,10 @@
       <c r="E8" s="22"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="143" t="s">
+      <c r="A9" s="142" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="75" t="s">
+      <c r="B9" s="74" t="s">
         <v>39</v>
       </c>
       <c r="C9" s="23" t="str" cm="1">
@@ -5810,8 +5810,8 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="140"/>
-      <c r="B10" s="76" t="s">
+      <c r="A10" s="139"/>
+      <c r="B10" s="75" t="s">
         <v>41</v>
       </c>
       <c r="C10" s="24" t="str" cm="1">
@@ -5826,8 +5826,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="140"/>
-      <c r="B11" s="76" t="s">
+      <c r="A11" s="139"/>
+      <c r="B11" s="75" t="s">
         <v>42</v>
       </c>
       <c r="C11" s="24" t="str" cm="1">
@@ -5842,8 +5842,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="139"/>
-      <c r="B12" s="79" t="s">
+      <c r="A12" s="138"/>
+      <c r="B12" s="78" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="20">
@@ -5857,10 +5857,10 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="144" t="s">
+      <c r="A13" s="143" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="75" t="s">
+      <c r="B13" s="74" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="23" t="str" cm="1">
@@ -5875,8 +5875,8 @@
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="142"/>
-      <c r="B14" s="76" t="s">
+      <c r="A14" s="141"/>
+      <c r="B14" s="75" t="s">
         <v>149</v>
       </c>
       <c r="C14" s="24" t="str" cm="1">
@@ -5891,8 +5891,8 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="142"/>
-      <c r="B15" s="76" t="s">
+      <c r="A15" s="141"/>
+      <c r="B15" s="75" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="25">
@@ -5904,12 +5904,12 @@
       <c r="E15" s="18"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="145"/>
-      <c r="B16" s="76" t="s">
+      <c r="A16" s="144"/>
+      <c r="B16" s="75" t="s">
         <v>45</v>
       </c>
       <c r="C16" s="25">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>46</v>
@@ -5917,8 +5917,8 @@
       <c r="E16" s="16"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="140"/>
-      <c r="B17" s="76" t="s">
+      <c r="A17" s="139"/>
+      <c r="B17" s="75" t="s">
         <v>47</v>
       </c>
       <c r="C17" s="25">
@@ -5930,11 +5930,11 @@
       <c r="E17" s="16"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="140"/>
-      <c r="B18" s="76" t="s">
+      <c r="A18" s="139"/>
+      <c r="B18" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="113">
+      <c r="C18" s="112">
         <v>0.11</v>
       </c>
       <c r="D18" s="15" t="s">
@@ -5943,11 +5943,11 @@
       <c r="E18" s="16"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="140"/>
-      <c r="B19" s="76" t="s">
+      <c r="A19" s="139"/>
+      <c r="B19" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="113">
+      <c r="C19" s="112">
         <v>0.03</v>
       </c>
       <c r="D19" s="15" t="s">
@@ -5956,11 +5956,11 @@
       <c r="E19" s="16"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="139"/>
-      <c r="B20" s="79" t="s">
+      <c r="A20" s="138"/>
+      <c r="B20" s="78" t="s">
         <v>50</v>
       </c>
-      <c r="C20" s="114">
+      <c r="C20" s="113">
         <v>1.5</v>
       </c>
       <c r="D20" s="21" t="s">
@@ -5969,10 +5969,10 @@
       <c r="E20" s="22"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="138" t="s">
+      <c r="A21" s="137" t="s">
         <v>143</v>
       </c>
-      <c r="B21" s="75" t="s">
+      <c r="B21" s="74" t="s">
         <v>51</v>
       </c>
       <c r="C21" s="23" t="str" cm="1">
@@ -5987,7 +5987,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="140"/>
+      <c r="A22" s="139"/>
       <c r="B22" s="14" t="s">
         <v>42</v>
       </c>
@@ -6003,7 +6003,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="139"/>
+      <c r="A23" s="138"/>
       <c r="B23" s="19" t="s">
         <v>12</v>
       </c>
@@ -6016,10 +6016,10 @@
       <c r="E23" s="22"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="138" t="s">
+      <c r="A24" s="137" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="75" t="s">
+      <c r="B24" s="74" t="s">
         <v>53</v>
       </c>
       <c r="C24" s="23" t="str" cm="1">
@@ -6034,8 +6034,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="140"/>
-      <c r="B25" s="76" t="s">
+      <c r="A25" s="139"/>
+      <c r="B25" s="75" t="s">
         <v>54</v>
       </c>
       <c r="C25" s="24" t="str" cm="1">
@@ -6050,21 +6050,21 @@
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="146"/>
-      <c r="B26" s="80" t="s">
+      <c r="A26" s="145"/>
+      <c r="B26" s="79" t="s">
         <v>147</v>
       </c>
-      <c r="C26" s="126">
+      <c r="C26" s="125">
         <v>1.2</v>
       </c>
-      <c r="D26" s="127" t="s">
+      <c r="D26" s="126" t="s">
         <v>29</v>
       </c>
-      <c r="E26" s="83"/>
+      <c r="E26" s="82"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="139"/>
-      <c r="B27" s="79" t="s">
+      <c r="A27" s="138"/>
+      <c r="B27" s="78" t="s">
         <v>146</v>
       </c>
       <c r="C27" s="20">
@@ -6076,10 +6076,10 @@
       <c r="E27" s="22"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="138" t="s">
+      <c r="A28" s="137" t="s">
         <v>55</v>
       </c>
-      <c r="B28" s="75" t="s">
+      <c r="B28" s="74" t="s">
         <v>56</v>
       </c>
       <c r="C28" s="27">
@@ -6091,8 +6091,8 @@
       <c r="E28" s="13"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="139"/>
-      <c r="B29" s="79" t="s">
+      <c r="A29" s="138"/>
+      <c r="B29" s="78" t="s">
         <v>57</v>
       </c>
       <c r="C29" s="20">
@@ -6104,10 +6104,10 @@
       <c r="E29" s="22"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="138" t="s">
+      <c r="A30" s="137" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="89" t="s">
+      <c r="B30" s="88" t="s">
         <v>51</v>
       </c>
       <c r="C30" s="23" t="str" cm="1">
@@ -6122,8 +6122,8 @@
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="140"/>
-      <c r="B31" s="90" t="s">
+      <c r="A31" s="139"/>
+      <c r="B31" s="89" t="s">
         <v>42</v>
       </c>
       <c r="C31" s="24" t="str" cm="1">
@@ -6138,8 +6138,8 @@
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="139"/>
-      <c r="B32" s="91" t="s">
+      <c r="A32" s="138"/>
+      <c r="B32" s="90" t="s">
         <v>12</v>
       </c>
       <c r="C32" s="20">
@@ -6151,7 +6151,7 @@
       <c r="E32" s="22"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="138" t="s">
+      <c r="A33" s="137" t="s">
         <v>59</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -6169,7 +6169,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="140"/>
+      <c r="A34" s="139"/>
       <c r="B34" s="14" t="s">
         <v>61</v>
       </c>
@@ -6185,7 +6185,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="139"/>
+      <c r="A35" s="138"/>
       <c r="B35" s="19" t="s">
         <v>12</v>
       </c>
@@ -6278,10 +6278,10 @@
       <c r="E5" s="10"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="123" t="s">
+      <c r="A6" s="122" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="75"/>
+      <c r="B6" s="74"/>
       <c r="C6" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B19/1000,HardpointsFr!C19/1000,HardpointsFr!D19/1000)&amp;"]"</f>
         <v>[0.011527 0.292246 0.342816]</v>
@@ -6294,13 +6294,13 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="124" t="s">
+      <c r="A7" s="123" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="76"/>
+      <c r="B7" s="75"/>
       <c r="C7" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B17/1000,HardpointsFr!C17/1000,HardpointsFr!D17/1000)&amp;"]"</f>
-        <v>[0.067965 0.262855 0.10135]</v>
+        <v>[0.020965 0.262855 0.10135]</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>12</v>
@@ -6310,10 +6310,10 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="124" t="s">
+      <c r="A8" s="123" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="76"/>
+      <c r="B8" s="75"/>
       <c r="C8" s="24" t="str" cm="1">
         <f t="array" ref="C8">"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B18/1000,HardpointsFr!C18/1000,HardpointsFr!D18/1000)&amp;"]"</f>
         <v>[-0.0235 0.262855 0.101519]</v>
@@ -6326,25 +6326,25 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="124" t="s">
+      <c r="A9" s="123" t="s">
         <v>69</v>
       </c>
-      <c r="B9" s="76"/>
-      <c r="C9" s="135">
+      <c r="B9" s="75"/>
+      <c r="C9" s="134">
         <f>2.2813*2</f>
         <v>4.5625999999999998</v>
       </c>
-      <c r="D9" s="87" t="s">
+      <c r="D9" s="86" t="s">
         <v>158</v>
       </c>
       <c r="E9" s="16"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="125" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="79"/>
-      <c r="C10" s="136">
+      <c r="A10" s="124" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="78"/>
+      <c r="C10" s="135">
         <v>0.7</v>
       </c>
       <c r="D10" s="21" t="s">
@@ -6426,13 +6426,13 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="147" t="s">
+      <c r="A5" s="146" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="75" t="s">
+      <c r="B5" s="74" t="s">
         <v>73</v>
       </c>
-      <c r="C5" s="42" t="str">
+      <c r="C5" s="41" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B20/1000,HardpointsFr!C20/1000,HardpointsFr!D20/1000)&amp;"]"</f>
         <v>[0.104241 0 0.171053]</v>
       </c>
@@ -6444,24 +6444,24 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="148"/>
-      <c r="B6" s="94" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="40">
+      <c r="A6" s="147"/>
+      <c r="B6" s="93" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="39">
         <v>0.87</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="40" t="s">
         <v>29</v>
       </c>
       <c r="E6" s="18"/>
     </row>
     <row r="7" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="149"/>
-      <c r="B7" s="76" t="s">
+      <c r="A7" s="148"/>
+      <c r="B7" s="75" t="s">
         <v>74</v>
       </c>
-      <c r="C7" s="39">
+      <c r="C7" s="38">
         <v>50</v>
       </c>
       <c r="D7" s="15" t="s">
@@ -6470,26 +6470,26 @@
       <c r="E7" s="15"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="150" t="s">
+      <c r="A8" s="149" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="76" t="s">
+      <c r="B8" s="75" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="24">
         <v>0.5</v>
       </c>
-      <c r="D8" s="87" t="s">
+      <c r="D8" s="86" t="s">
         <v>29</v>
       </c>
       <c r="E8" s="16"/>
     </row>
     <row r="9" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="151"/>
-      <c r="B9" s="76" t="s">
+      <c r="A9" s="150"/>
+      <c r="B9" s="75" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="39" t="str">
+      <c r="C9" s="38" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B21/1000,HardpointsFr!C21/1000,HardpointsFr!D21/1000)&amp;"]"</f>
         <v>[-0.324965 0 0.533792]</v>
       </c>
@@ -6553,7 +6553,7 @@
         <v>35</v>
       </c>
       <c r="D2" s="9"/>
-      <c r="E2" s="54"/>
+      <c r="E2" s="53"/>
     </row>
     <row r="3" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -6564,68 +6564,68 @@
         <v>36</v>
       </c>
       <c r="D3" s="9"/>
-      <c r="E3" s="54"/>
+      <c r="E3" s="53"/>
     </row>
     <row r="4" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="103" t="s">
+      <c r="C4" s="102" t="s">
         <v>35</v>
       </c>
       <c r="D4" s="9"/>
-      <c r="E4" s="54"/>
+      <c r="E4" s="53"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="115"/>
-      <c r="C5" s="117" t="s">
+      <c r="B5" s="114"/>
+      <c r="C5" s="116" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="118" t="s">
+      <c r="D5" s="117" t="s">
         <v>64</v>
       </c>
-      <c r="E5" s="119"/>
+      <c r="E5" s="118"/>
     </row>
     <row r="6" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="79"/>
-      <c r="C6" s="86" t="s">
+      <c r="B6" s="78"/>
+      <c r="C6" s="85" t="s">
         <v>77</v>
       </c>
-      <c r="D6" s="88" t="s">
+      <c r="D6" s="87" t="s">
         <v>64</v>
       </c>
       <c r="E6" s="22"/>
     </row>
     <row r="7" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="152" t="s">
+      <c r="A7" s="151" t="s">
         <v>65</v>
       </c>
-      <c r="B7" s="128" t="s">
+      <c r="B7" s="127" t="s">
         <v>155</v>
       </c>
-      <c r="C7" s="129" t="s">
+      <c r="C7" s="128" t="s">
         <v>65</v>
       </c>
-      <c r="D7" s="118"/>
-      <c r="E7" s="130"/>
+      <c r="D7" s="117"/>
+      <c r="E7" s="129"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="153"/>
-      <c r="B8" s="128" t="s">
+      <c r="A8" s="152"/>
+      <c r="B8" s="127" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="117" t="s">
+      <c r="C8" s="116" t="s">
         <v>156</v>
       </c>
-      <c r="D8" s="118"/>
-      <c r="E8" s="119"/>
+      <c r="D8" s="117"/>
+      <c r="E8" s="118"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6673,7 +6673,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="103" t="s">
+      <c r="C2" s="102" t="s">
         <v>35</v>
       </c>
       <c r="D2" s="9"/>
@@ -6684,7 +6684,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="103" t="s">
+      <c r="C3" s="102" t="s">
         <v>36</v>
       </c>
       <c r="D3" s="9"/>
@@ -6695,17 +6695,17 @@
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="103" t="s">
+      <c r="C4" s="102" t="s">
         <v>141</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="152" t="s">
+      <c r="A5" s="151" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="75" t="s">
+      <c r="B5" s="74" t="s">
         <v>39</v>
       </c>
       <c r="C5" s="23" t="str">
@@ -6715,125 +6715,125 @@
       <c r="D5" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="55" t="s">
+      <c r="E5" s="54" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="158"/>
-      <c r="B6" s="76" t="s">
+      <c r="A6" s="157"/>
+      <c r="B6" s="75" t="s">
         <v>41</v>
       </c>
       <c r="C6" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B3/1000 +1.575,HardpointsRr!C3/1000,HardpointsRr!D3/1000)&amp;"]"</f>
         <v>[-0.255 0.27 0.12635]</v>
       </c>
-      <c r="D6" s="46" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="56" t="s">
+      <c r="D6" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="55" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="158"/>
-      <c r="B7" s="76" t="s">
+      <c r="A7" s="157"/>
+      <c r="B7" s="75" t="s">
         <v>42</v>
       </c>
       <c r="C7" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B4/1000 +1.575,HardpointsRr!C4/1000,HardpointsRr!D4/1000)&amp;"]"</f>
         <v>[-0.00423700000000005 0.573947 0.1375]</v>
       </c>
-      <c r="D7" s="47" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="57" t="s">
+      <c r="D7" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="56" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="153"/>
-      <c r="B8" s="79" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="49">
+      <c r="A8" s="152"/>
+      <c r="B8" s="78" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="48">
         <v>0.16500000000000001</v>
       </c>
-      <c r="D8" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="58"/>
+      <c r="D8" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="57"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="159" t="s">
+      <c r="A9" s="158" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="75" t="s">
+      <c r="B9" s="74" t="s">
         <v>39</v>
       </c>
       <c r="C9" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B5/1000 +1.575,HardpointsRr!C5/1000,HardpointsRr!D5/1000)&amp;"]"</f>
         <v>[0.185 0.305 0.328981]</v>
       </c>
-      <c r="D9" s="50" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="59" t="s">
+      <c r="D9" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="58" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="160"/>
-      <c r="B10" s="76" t="s">
+      <c r="A10" s="159"/>
+      <c r="B10" s="75" t="s">
         <v>41</v>
       </c>
       <c r="C10" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B6/1000 +1.575,HardpointsRr!C6/1000,HardpointsRr!D6/1000)&amp;"]"</f>
         <v>[-0.255 0.27 0.354475]</v>
       </c>
-      <c r="D10" s="53" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="60" t="s">
+      <c r="D10" s="52" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="59" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="160"/>
-      <c r="B11" s="76" t="s">
+      <c r="A11" s="159"/>
+      <c r="B11" s="75" t="s">
         <v>42</v>
       </c>
       <c r="C11" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B7/1000 +1.575,HardpointsRr!C7/1000,HardpointsRr!D7/1000)&amp;"]"</f>
         <v>[0.00515500000000002 0.50633 0.382471]</v>
       </c>
-      <c r="D11" s="51" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="61" t="s">
+      <c r="D11" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="60" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="161"/>
-      <c r="B12" s="79" t="s">
+      <c r="A12" s="160"/>
+      <c r="B12" s="78" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="20">
         <v>0.12</v>
       </c>
-      <c r="D12" s="52" t="s">
+      <c r="D12" s="51" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="62" t="s">
+      <c r="E12" s="61" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="147" t="s">
+      <c r="A13" s="146" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="75" t="s">
+      <c r="B13" s="74" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="23" t="str">
@@ -6843,55 +6843,55 @@
       <c r="D13" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="55" t="s">
+      <c r="E13" s="54" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="148"/>
-      <c r="B14" s="76" t="s">
+      <c r="A14" s="147"/>
+      <c r="B14" s="75" t="s">
         <v>149</v>
       </c>
       <c r="C14" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B9/1000 +1.575,HardpointsRr!C9/1000,HardpointsRr!D9/1000)&amp;"]"</f>
         <v>[0.000401000000000096 0.623532 0.260361]</v>
       </c>
-      <c r="D14" s="43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="63" t="s">
+      <c r="D14" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="62" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="148"/>
-      <c r="B15" s="76" t="s">
+      <c r="A15" s="147"/>
+      <c r="B15" s="75" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="25">
         <v>1</v>
       </c>
-      <c r="D15" s="43" t="s">
+      <c r="D15" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="64"/>
+      <c r="E15" s="63"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="148"/>
-      <c r="B16" s="76" t="s">
+      <c r="A16" s="147"/>
+      <c r="B16" s="75" t="s">
         <v>45</v>
       </c>
       <c r="C16" s="25">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="62"/>
+      <c r="E16" s="61"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="148"/>
-      <c r="B17" s="76" t="s">
+      <c r="A17" s="147"/>
+      <c r="B17" s="75" t="s">
         <v>47</v>
       </c>
       <c r="C17" s="25">
@@ -6900,67 +6900,67 @@
       <c r="D17" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="65"/>
+      <c r="E17" s="64"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="148"/>
-      <c r="B18" s="76" t="s">
+      <c r="A18" s="147"/>
+      <c r="B18" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="113">
+      <c r="C18" s="112">
         <v>0.11</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="65"/>
+      <c r="E18" s="64"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="148"/>
-      <c r="B19" s="76" t="s">
+      <c r="A19" s="147"/>
+      <c r="B19" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="113">
+      <c r="C19" s="112">
         <v>0.03</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="65"/>
+      <c r="E19" s="64"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="157"/>
-      <c r="B20" s="79" t="s">
+      <c r="A20" s="156"/>
+      <c r="B20" s="78" t="s">
         <v>50</v>
       </c>
-      <c r="C20" s="114">
+      <c r="C20" s="113">
         <v>1.5</v>
       </c>
       <c r="D20" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="66"/>
+      <c r="E20" s="65"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="147" t="s">
+      <c r="A21" s="146" t="s">
         <v>143</v>
       </c>
-      <c r="B21" s="75" t="s">
+      <c r="B21" s="74" t="s">
         <v>51</v>
       </c>
       <c r="C21" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B10/1000 +1.575,HardpointsRr!C10/1000,HardpointsRr!D10/1000)&amp;"]"</f>
         <v>[-0.255 0.27 0.193642]</v>
       </c>
-      <c r="D21" s="44" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" s="67" t="s">
+      <c r="D21" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="66" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="148"/>
+      <c r="A22" s="147"/>
       <c r="B22" s="14" t="s">
         <v>42</v>
       </c>
@@ -6968,15 +6968,15 @@
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B11/1000 +1.575,HardpointsRr!C11/1000,HardpointsRr!D11/1000)&amp;"]"</f>
         <v>[-0.100904 0.576735 0.225331]</v>
       </c>
-      <c r="D22" s="43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E22" s="60" t="s">
+      <c r="D22" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" s="59" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="157"/>
+      <c r="A23" s="156"/>
       <c r="B23" s="19" t="s">
         <v>12</v>
       </c>
@@ -6986,29 +6986,29 @@
       <c r="D23" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E23" s="68"/>
+      <c r="E23" s="67"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="147" t="s">
+      <c r="A24" s="146" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="75" t="s">
+      <c r="B24" s="74" t="s">
         <v>53</v>
       </c>
       <c r="C24" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B12/1000 + 1.575,HardpointsRr!C12/1000,HardpointsRr!D12/1000)&amp;"]"</f>
         <v>[0.179024 0.283399 0.436103]</v>
       </c>
-      <c r="D24" s="44" t="s">
-        <v>12</v>
-      </c>
-      <c r="E24" s="61" t="s">
+      <c r="D24" s="43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="60" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="148"/>
-      <c r="B25" s="76" t="s">
+      <c r="A25" s="147"/>
+      <c r="B25" s="75" t="s">
         <v>54</v>
       </c>
       <c r="C25" s="23" t="str">
@@ -7018,24 +7018,24 @@
       <c r="D25" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E25" s="62" t="s">
+      <c r="E25" s="61" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="148"/>
-      <c r="B26" s="80" t="s">
+      <c r="A26" s="147"/>
+      <c r="B26" s="79" t="s">
         <v>146</v>
       </c>
-      <c r="C26" s="126">
+      <c r="C26" s="125">
         <v>0.8</v>
       </c>
-      <c r="D26" s="81"/>
-      <c r="E26" s="73"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="72"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="157"/>
-      <c r="B27" s="79" t="s">
+      <c r="A27" s="156"/>
+      <c r="B27" s="78" t="s">
         <v>147</v>
       </c>
       <c r="C27" s="20">
@@ -7044,13 +7044,13 @@
       <c r="D27" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E27" s="69"/>
+      <c r="E27" s="68"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="147" t="s">
+      <c r="A28" s="146" t="s">
         <v>55</v>
       </c>
-      <c r="B28" s="75" t="s">
+      <c r="B28" s="74" t="s">
         <v>56</v>
       </c>
       <c r="C28" s="27">
@@ -7059,11 +7059,11 @@
       <c r="D28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E28" s="70"/>
+      <c r="E28" s="69"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="157"/>
-      <c r="B29" s="79" t="s">
+      <c r="A29" s="156"/>
+      <c r="B29" s="78" t="s">
         <v>57</v>
       </c>
       <c r="C29" s="20">
@@ -7072,13 +7072,13 @@
       <c r="D29" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="E29" s="69"/>
+      <c r="E29" s="68"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="154" t="s">
+      <c r="A30" s="153" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="89" t="s">
+      <c r="B30" s="88" t="s">
         <v>42</v>
       </c>
       <c r="C30" s="23" t="str">
@@ -7088,29 +7088,29 @@
       <c r="D30" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E30" s="55" t="s">
+      <c r="E30" s="54" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="155"/>
-      <c r="B31" s="90" t="s">
+      <c r="A31" s="154"/>
+      <c r="B31" s="89" t="s">
         <v>51</v>
       </c>
       <c r="C31" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B15/1000 + 1.575,HardpointsRr!C15/1000,HardpointsRr!D15/1000)&amp;"]"</f>
         <v>[-0.089612 0.349047 0.403924]</v>
       </c>
-      <c r="D31" s="43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E31" s="60" t="s">
+      <c r="D31" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" s="59" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="156"/>
-      <c r="B32" s="91" t="s">
+      <c r="A32" s="155"/>
+      <c r="B32" s="90" t="s">
         <v>12</v>
       </c>
       <c r="C32" s="20">
@@ -7119,10 +7119,10 @@
       <c r="D32" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E32" s="71"/>
+      <c r="E32" s="70"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="147" t="s">
+      <c r="A33" s="146" t="s">
         <v>59</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -7135,12 +7135,12 @@
       <c r="D33" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E33" s="55" t="s">
+      <c r="E33" s="54" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="148"/>
+      <c r="A34" s="147"/>
       <c r="B34" s="14" t="s">
         <v>61</v>
       </c>
@@ -7148,15 +7148,15 @@
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B19/1000+ 1.575,HardpointsRr!C19/1000,HardpointsRr!D19/1000)&amp;"]"</f>
         <v>[-0.0254860000000001 0.287566 0.463988]</v>
       </c>
-      <c r="D34" s="43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E34" s="60" t="s">
+      <c r="D34" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" s="59" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="157"/>
+      <c r="A35" s="156"/>
       <c r="B35" s="19" t="s">
         <v>12</v>
       </c>
@@ -7166,7 +7166,7 @@
       <c r="D35" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E35" s="71"/>
+      <c r="E35" s="70"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -7241,86 +7241,86 @@
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="103" t="s">
+      <c r="C4" s="102" t="s">
         <v>150</v>
       </c>
       <c r="D4" s="9"/>
-      <c r="E4" s="72"/>
+      <c r="E4" s="71"/>
     </row>
     <row r="5" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="123" t="s">
+      <c r="A5" s="122" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="75"/>
+      <c r="B5" s="74"/>
       <c r="C5" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B19/1000+ 1.575,HardpointsRr!C19/1000,HardpointsRr!D19/1000)&amp;"]"</f>
         <v>[-0.0254860000000001 0.287566 0.463988]</v>
       </c>
-      <c r="D5" s="131" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="67" t="s">
+      <c r="D5" s="130" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="66" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="124" t="s">
+      <c r="A6" s="123" t="s">
         <v>51</v>
       </c>
-      <c r="B6" s="76"/>
+      <c r="B6" s="75"/>
       <c r="C6" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B17/1000+ 1.575,HardpointsRr!C17/1000,HardpointsRr!D17/1000)&amp;"]"</f>
         <v>[-0.255 0.305 0.40135]</v>
       </c>
-      <c r="D6" s="43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="56" t="s">
+      <c r="D6" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="55" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="124" t="s">
+      <c r="A7" s="123" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="76"/>
+      <c r="B7" s="75"/>
       <c r="C7" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B18/1000 + 1.575,HardpointsRr!C18/1000,HardpointsRr!D18/1000)&amp;"]"</f>
         <v>[-0.255 0.305 0.44835]</v>
       </c>
-      <c r="D7" s="43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="60" t="s">
+      <c r="D7" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="59" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="124" t="s">
+      <c r="A8" s="123" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="76"/>
-      <c r="C8" s="29">
+      <c r="B8" s="75"/>
+      <c r="C8" s="161">
         <f>1.979*2</f>
         <v>3.9580000000000002</v>
       </c>
-      <c r="D8" s="87" t="s">
+      <c r="D8" s="86" t="s">
         <v>158</v>
       </c>
-      <c r="E8" s="73"/>
+      <c r="E8" s="72"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="125" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="79"/>
+      <c r="A9" s="124" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="78"/>
       <c r="C9" s="20">
         <v>0.7</v>
       </c>
-      <c r="D9" s="45" t="s">
+      <c r="D9" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="74"/>
+      <c r="E9" s="73"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7394,10 +7394,10 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="121" t="s">
+      <c r="A5" s="120" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="75"/>
+      <c r="B5" s="74"/>
       <c r="C5" s="23">
         <v>-2.15</v>
       </c>
@@ -7405,10 +7405,10 @@
       <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="121" t="s">
+      <c r="A6" s="120" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="76"/>
+      <c r="B6" s="75"/>
       <c r="C6" s="24">
         <v>-1</v>
       </c>
@@ -7416,10 +7416,10 @@
       <c r="E6" s="18"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="121" t="s">
+      <c r="A7" s="120" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="76"/>
+      <c r="B7" s="75"/>
       <c r="C7" s="24">
         <v>1.2250000000000001</v>
       </c>
@@ -7429,10 +7429,10 @@
       <c r="E7" s="18"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="121" t="s">
+      <c r="A8" s="120" t="s">
         <v>145</v>
       </c>
-      <c r="B8" s="76"/>
+      <c r="B8" s="75"/>
       <c r="C8" s="24">
         <v>1.2</v>
       </c>
@@ -7442,11 +7442,11 @@
       <c r="E8" s="18"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="121" t="s">
+      <c r="A9" s="120" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="79"/>
-      <c r="C9" s="30" t="s">
+      <c r="B9" s="78"/>
+      <c r="C9" s="29" t="s">
         <v>86</v>
       </c>
       <c r="D9" s="21" t="s">
@@ -7464,26 +7464,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009342B7EAA7728A4FA80A5CCAFE8D7EAF" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d037a5681ee6af0e7b5b5d0a2f99b20">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557458c-24b5-4c97-84ed-4c402655f54f" xmlns:ns3="72e3c584-9879-4b35-b9d8-6a248c93e240" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="966978c8b125399653e7c255ac8e342d" ns2:_="" ns3:_="">
     <xsd:import namespace="9557458c-24b5-4c97-84ed-4c402655f54f"/>
@@ -7744,10 +7724,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7764,20 +7775,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
-    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
UKF code gen added
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E6E63F5-D62B-3F4F-8E03-7C0B9806B7D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC91F7D0-38BA-B946-A86E-9C35B31B7FC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10580" yWindow="1880" windowWidth="38400" windowHeight="22380" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="23260" windowHeight="12460" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Body" sheetId="1" r:id="rId1"/>
@@ -2091,6 +2091,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2108,12 +2120,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="58" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="63" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2138,9 +2144,6 @@
     <xf numFmtId="49" fontId="2" fillId="7" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2152,9 +2155,6 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3583,7 +3583,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="146" t="s">
+      <c r="A5" s="138" t="s">
         <v>89</v>
       </c>
       <c r="B5" s="74" t="s">
@@ -3596,7 +3596,7 @@
       <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="147"/>
+      <c r="A6" s="139"/>
       <c r="B6" s="94" t="s">
         <v>91</v>
       </c>
@@ -3609,12 +3609,12 @@
       <c r="E6" s="97"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="156"/>
+      <c r="A7" s="140"/>
       <c r="B7" s="78" t="s">
         <v>144</v>
       </c>
       <c r="C7" s="20">
-        <v>0</v>
+        <v>1.6E-2</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>12</v>
@@ -3622,7 +3622,7 @@
       <c r="E7" s="30"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="146" t="s">
+      <c r="A8" s="138" t="s">
         <v>93</v>
       </c>
       <c r="B8" s="74" t="s">
@@ -3635,7 +3635,7 @@
       <c r="E8" s="28"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="147"/>
+      <c r="A9" s="139"/>
       <c r="B9" s="94" t="s">
         <v>91</v>
       </c>
@@ -3648,12 +3648,12 @@
       <c r="E9" s="97"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="156"/>
+      <c r="A10" s="140"/>
       <c r="B10" s="78" t="s">
         <v>144</v>
       </c>
       <c r="C10" s="20">
-        <v>0</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="D10" s="87" t="s">
         <v>12</v>
@@ -3736,7 +3736,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="146" t="s">
+      <c r="A5" s="138" t="s">
         <v>89</v>
       </c>
       <c r="B5" s="74" t="s">
@@ -3749,7 +3749,7 @@
       <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="147"/>
+      <c r="A6" s="139"/>
       <c r="B6" s="94" t="s">
         <v>94</v>
       </c>
@@ -3764,7 +3764,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="147"/>
+      <c r="A7" s="139"/>
       <c r="B7" s="75" t="s">
         <v>95</v>
       </c>
@@ -3777,7 +3777,7 @@
       <c r="E7" s="18"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="147"/>
+      <c r="A8" s="139"/>
       <c r="B8" s="75" t="s">
         <v>96</v>
       </c>
@@ -3790,7 +3790,7 @@
       <c r="E8" s="18"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="147"/>
+      <c r="A9" s="139"/>
       <c r="B9" s="75" t="s">
         <v>97</v>
       </c>
@@ -3803,7 +3803,7 @@
       <c r="E9" s="18"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="147"/>
+      <c r="A10" s="139"/>
       <c r="B10" s="75" t="s">
         <v>98</v>
       </c>
@@ -3816,7 +3816,7 @@
       <c r="E10" s="18"/>
     </row>
     <row r="11" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="156"/>
+      <c r="A11" s="140"/>
       <c r="B11" s="78" t="s">
         <v>99</v>
       </c>
@@ -3829,7 +3829,7 @@
       <c r="E11" s="30"/>
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="146" t="s">
+      <c r="A12" s="138" t="s">
         <v>93</v>
       </c>
       <c r="B12" s="74" t="s">
@@ -3842,7 +3842,7 @@
       <c r="E12" s="28"/>
     </row>
     <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="147"/>
+      <c r="A13" s="139"/>
       <c r="B13" s="94" t="s">
         <v>94</v>
       </c>
@@ -3857,7 +3857,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="147"/>
+      <c r="A14" s="139"/>
       <c r="B14" s="75" t="s">
         <v>95</v>
       </c>
@@ -3870,7 +3870,7 @@
       <c r="E14" s="18"/>
     </row>
     <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="147"/>
+      <c r="A15" s="139"/>
       <c r="B15" s="75" t="s">
         <v>96</v>
       </c>
@@ -3883,7 +3883,7 @@
       <c r="E15" s="18"/>
     </row>
     <row r="16" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="147"/>
+      <c r="A16" s="139"/>
       <c r="B16" s="75" t="s">
         <v>97</v>
       </c>
@@ -3896,7 +3896,7 @@
       <c r="E16" s="18"/>
     </row>
     <row r="17" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="147"/>
+      <c r="A17" s="139"/>
       <c r="B17" s="75" t="s">
         <v>98</v>
       </c>
@@ -3909,7 +3909,7 @@
       <c r="E17" s="18"/>
     </row>
     <row r="18" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="156"/>
+      <c r="A18" s="140"/>
       <c r="B18" s="78" t="s">
         <v>99</v>
       </c>
@@ -3937,7 +3937,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CD2A3BA-06BE-A64D-A72B-9CFCF024C1FD}">
   <dimension ref="A1:B101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="133">
@@ -4893,7 +4893,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="146" t="s">
+      <c r="A11" s="138" t="s">
         <v>114</v>
       </c>
       <c r="B11" s="106" t="s">
@@ -4906,7 +4906,7 @@
       <c r="E11" s="71"/>
     </row>
     <row r="12" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="156"/>
+      <c r="A12" s="140"/>
       <c r="B12" s="108" t="s">
         <v>115</v>
       </c>
@@ -5337,7 +5337,7 @@
         <v>573.947</v>
       </c>
       <c r="D4" s="37">
-        <v>137.5</v>
+        <v>163.18</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
@@ -5379,7 +5379,7 @@
         <v>506.33</v>
       </c>
       <c r="D7" s="37">
-        <v>382.471</v>
+        <v>408.15100000000001</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
@@ -5393,7 +5393,7 @@
         <v>566.64200000000005</v>
       </c>
       <c r="D8" s="37">
-        <v>269.14400000000001</v>
+        <v>294.82</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
@@ -5407,7 +5407,7 @@
         <v>623.53200000000004</v>
       </c>
       <c r="D9" s="37">
-        <v>260.36099999999999</v>
+        <v>286.04000000000002</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
@@ -5435,7 +5435,7 @@
         <v>576.73500000000001</v>
       </c>
       <c r="D11" s="37">
-        <v>225.33099999999999</v>
+        <v>251.011</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
@@ -5477,7 +5477,7 @@
         <v>526.39499999999998</v>
       </c>
       <c r="D14" s="37">
-        <v>155.28700000000001</v>
+        <v>180.96700000000001</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
@@ -5670,7 +5670,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23B3B35C-CB70-D641-97B1-CD6FD7CCE140}">
   <dimension ref="A1:E35"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="33.6640625" bestFit="1" customWidth="1"/>
@@ -5729,7 +5729,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="140" t="s">
+      <c r="A5" s="144" t="s">
         <v>38</v>
       </c>
       <c r="B5" s="74" t="s">
@@ -5747,7 +5747,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="138"/>
+      <c r="A6" s="142"/>
       <c r="B6" s="75" t="s">
         <v>41</v>
       </c>
@@ -5763,7 +5763,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="141"/>
+      <c r="A7" s="145"/>
       <c r="B7" s="75" t="s">
         <v>42</v>
       </c>
@@ -5779,7 +5779,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="141"/>
+      <c r="A8" s="145"/>
       <c r="B8" s="78" t="s">
         <v>12</v>
       </c>
@@ -5792,7 +5792,7 @@
       <c r="E8" s="22"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="142" t="s">
+      <c r="A9" s="146" t="s">
         <v>43</v>
       </c>
       <c r="B9" s="74" t="s">
@@ -5810,7 +5810,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="139"/>
+      <c r="A10" s="143"/>
       <c r="B10" s="75" t="s">
         <v>41</v>
       </c>
@@ -5826,7 +5826,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="139"/>
+      <c r="A11" s="143"/>
       <c r="B11" s="75" t="s">
         <v>42</v>
       </c>
@@ -5842,7 +5842,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="138"/>
+      <c r="A12" s="142"/>
       <c r="B12" s="78" t="s">
         <v>12</v>
       </c>
@@ -5857,7 +5857,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="143" t="s">
+      <c r="A13" s="147" t="s">
         <v>44</v>
       </c>
       <c r="B13" s="74" t="s">
@@ -5875,7 +5875,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="141"/>
+      <c r="A14" s="145"/>
       <c r="B14" s="75" t="s">
         <v>149</v>
       </c>
@@ -5891,7 +5891,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="141"/>
+      <c r="A15" s="145"/>
       <c r="B15" s="75" t="s">
         <v>12</v>
       </c>
@@ -5904,7 +5904,7 @@
       <c r="E15" s="18"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="144"/>
+      <c r="A16" s="148"/>
       <c r="B16" s="75" t="s">
         <v>45</v>
       </c>
@@ -5917,7 +5917,7 @@
       <c r="E16" s="16"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="139"/>
+      <c r="A17" s="143"/>
       <c r="B17" s="75" t="s">
         <v>47</v>
       </c>
@@ -5930,7 +5930,7 @@
       <c r="E17" s="16"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="139"/>
+      <c r="A18" s="143"/>
       <c r="B18" s="75" t="s">
         <v>48</v>
       </c>
@@ -5943,7 +5943,7 @@
       <c r="E18" s="16"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="139"/>
+      <c r="A19" s="143"/>
       <c r="B19" s="75" t="s">
         <v>49</v>
       </c>
@@ -5956,7 +5956,7 @@
       <c r="E19" s="16"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="138"/>
+      <c r="A20" s="142"/>
       <c r="B20" s="78" t="s">
         <v>50</v>
       </c>
@@ -5969,7 +5969,7 @@
       <c r="E20" s="22"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="137" t="s">
+      <c r="A21" s="141" t="s">
         <v>143</v>
       </c>
       <c r="B21" s="74" t="s">
@@ -5987,7 +5987,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="139"/>
+      <c r="A22" s="143"/>
       <c r="B22" s="14" t="s">
         <v>42</v>
       </c>
@@ -6003,7 +6003,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="138"/>
+      <c r="A23" s="142"/>
       <c r="B23" s="19" t="s">
         <v>12</v>
       </c>
@@ -6016,7 +6016,7 @@
       <c r="E23" s="22"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="137" t="s">
+      <c r="A24" s="141" t="s">
         <v>52</v>
       </c>
       <c r="B24" s="74" t="s">
@@ -6034,7 +6034,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="139"/>
+      <c r="A25" s="143"/>
       <c r="B25" s="75" t="s">
         <v>54</v>
       </c>
@@ -6050,7 +6050,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="145"/>
+      <c r="A26" s="149"/>
       <c r="B26" s="79" t="s">
         <v>147</v>
       </c>
@@ -6063,7 +6063,7 @@
       <c r="E26" s="82"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="138"/>
+      <c r="A27" s="142"/>
       <c r="B27" s="78" t="s">
         <v>146</v>
       </c>
@@ -6076,7 +6076,7 @@
       <c r="E27" s="22"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="137" t="s">
+      <c r="A28" s="141" t="s">
         <v>55</v>
       </c>
       <c r="B28" s="74" t="s">
@@ -6091,7 +6091,7 @@
       <c r="E28" s="13"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="138"/>
+      <c r="A29" s="142"/>
       <c r="B29" s="78" t="s">
         <v>57</v>
       </c>
@@ -6104,7 +6104,7 @@
       <c r="E29" s="22"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="137" t="s">
+      <c r="A30" s="141" t="s">
         <v>58</v>
       </c>
       <c r="B30" s="88" t="s">
@@ -6122,7 +6122,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="139"/>
+      <c r="A31" s="143"/>
       <c r="B31" s="89" t="s">
         <v>42</v>
       </c>
@@ -6138,7 +6138,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="138"/>
+      <c r="A32" s="142"/>
       <c r="B32" s="90" t="s">
         <v>12</v>
       </c>
@@ -6151,7 +6151,7 @@
       <c r="E32" s="22"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="137" t="s">
+      <c r="A33" s="141" t="s">
         <v>59</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -6169,7 +6169,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="139"/>
+      <c r="A34" s="143"/>
       <c r="B34" s="14" t="s">
         <v>61</v>
       </c>
@@ -6185,7 +6185,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="138"/>
+      <c r="A35" s="142"/>
       <c r="B35" s="19" t="s">
         <v>12</v>
       </c>
@@ -6426,7 +6426,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="146" t="s">
+      <c r="A5" s="138" t="s">
         <v>72</v>
       </c>
       <c r="B5" s="74" t="s">
@@ -6444,7 +6444,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="147"/>
+      <c r="A6" s="139"/>
       <c r="B6" s="93" t="s">
         <v>12</v>
       </c>
@@ -6457,7 +6457,7 @@
       <c r="E6" s="18"/>
     </row>
     <row r="7" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="148"/>
+      <c r="A7" s="150"/>
       <c r="B7" s="75" t="s">
         <v>74</v>
       </c>
@@ -6470,7 +6470,7 @@
       <c r="E7" s="15"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="149" t="s">
+      <c r="A8" s="151" t="s">
         <v>76</v>
       </c>
       <c r="B8" s="75" t="s">
@@ -6485,7 +6485,7 @@
       <c r="E8" s="16"/>
     </row>
     <row r="9" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="150"/>
+      <c r="A9" s="152"/>
       <c r="B9" s="75" t="s">
         <v>73</v>
       </c>
@@ -6604,7 +6604,7 @@
       <c r="E6" s="22"/>
     </row>
     <row r="7" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="151" t="s">
+      <c r="A7" s="153" t="s">
         <v>65</v>
       </c>
       <c r="B7" s="127" t="s">
@@ -6617,7 +6617,7 @@
       <c r="E7" s="129"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="152"/>
+      <c r="A8" s="154"/>
       <c r="B8" s="127" t="s">
         <v>8</v>
       </c>
@@ -6642,7 +6642,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E45A869-B0F3-7240-9246-177BC72F43B2}">
   <dimension ref="A1:E35"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
@@ -6702,7 +6702,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="151" t="s">
+      <c r="A5" s="153" t="s">
         <v>38</v>
       </c>
       <c r="B5" s="74" t="s">
@@ -6720,7 +6720,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="157"/>
+      <c r="A6" s="158"/>
       <c r="B6" s="75" t="s">
         <v>41</v>
       </c>
@@ -6736,13 +6736,13 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="157"/>
+      <c r="A7" s="158"/>
       <c r="B7" s="75" t="s">
         <v>42</v>
       </c>
       <c r="C7" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B4/1000 +1.575,HardpointsRr!C4/1000,HardpointsRr!D4/1000)&amp;"]"</f>
-        <v>[-0.00423700000000005 0.573947 0.1375]</v>
+        <v>[-0.00423700000000005 0.573947 0.16318]</v>
       </c>
       <c r="D7" s="46" t="s">
         <v>12</v>
@@ -6752,7 +6752,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="152"/>
+      <c r="A8" s="154"/>
       <c r="B8" s="78" t="s">
         <v>12</v>
       </c>
@@ -6765,7 +6765,7 @@
       <c r="E8" s="57"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="158" t="s">
+      <c r="A9" s="159" t="s">
         <v>43</v>
       </c>
       <c r="B9" s="74" t="s">
@@ -6783,7 +6783,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="159"/>
+      <c r="A10" s="160"/>
       <c r="B10" s="75" t="s">
         <v>41</v>
       </c>
@@ -6799,13 +6799,13 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="159"/>
+      <c r="A11" s="160"/>
       <c r="B11" s="75" t="s">
         <v>42</v>
       </c>
       <c r="C11" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B7/1000 +1.575,HardpointsRr!C7/1000,HardpointsRr!D7/1000)&amp;"]"</f>
-        <v>[0.00515500000000002 0.50633 0.382471]</v>
+        <v>[0.00515500000000002 0.50633 0.408151]</v>
       </c>
       <c r="D11" s="50" t="s">
         <v>12</v>
@@ -6815,7 +6815,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="160"/>
+      <c r="A12" s="161"/>
       <c r="B12" s="78" t="s">
         <v>12</v>
       </c>
@@ -6830,7 +6830,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="146" t="s">
+      <c r="A13" s="138" t="s">
         <v>44</v>
       </c>
       <c r="B13" s="74" t="s">
@@ -6838,7 +6838,7 @@
       </c>
       <c r="C13" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B8/1000 +1.575,HardpointsRr!C8/1000,HardpointsRr!D8/1000)&amp;"]"</f>
-        <v>[0.00612899999999983 0.566642 0.269144]</v>
+        <v>[0.00612899999999983 0.566642 0.29482]</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>12</v>
@@ -6848,13 +6848,13 @@
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="147"/>
+      <c r="A14" s="139"/>
       <c r="B14" s="75" t="s">
         <v>149</v>
       </c>
       <c r="C14" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B9/1000 +1.575,HardpointsRr!C9/1000,HardpointsRr!D9/1000)&amp;"]"</f>
-        <v>[0.000401000000000096 0.623532 0.260361]</v>
+        <v>[0.000401000000000096 0.623532 0.28604]</v>
       </c>
       <c r="D14" s="42" t="s">
         <v>12</v>
@@ -6864,7 +6864,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="147"/>
+      <c r="A15" s="139"/>
       <c r="B15" s="75" t="s">
         <v>12</v>
       </c>
@@ -6877,7 +6877,7 @@
       <c r="E15" s="63"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="147"/>
+      <c r="A16" s="139"/>
       <c r="B16" s="75" t="s">
         <v>45</v>
       </c>
@@ -6890,7 +6890,7 @@
       <c r="E16" s="61"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="147"/>
+      <c r="A17" s="139"/>
       <c r="B17" s="75" t="s">
         <v>47</v>
       </c>
@@ -6903,7 +6903,7 @@
       <c r="E17" s="64"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="147"/>
+      <c r="A18" s="139"/>
       <c r="B18" s="75" t="s">
         <v>48</v>
       </c>
@@ -6916,7 +6916,7 @@
       <c r="E18" s="64"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="147"/>
+      <c r="A19" s="139"/>
       <c r="B19" s="75" t="s">
         <v>49</v>
       </c>
@@ -6929,7 +6929,7 @@
       <c r="E19" s="64"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="156"/>
+      <c r="A20" s="140"/>
       <c r="B20" s="78" t="s">
         <v>50</v>
       </c>
@@ -6942,7 +6942,7 @@
       <c r="E20" s="65"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="146" t="s">
+      <c r="A21" s="138" t="s">
         <v>143</v>
       </c>
       <c r="B21" s="74" t="s">
@@ -6960,13 +6960,13 @@
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="147"/>
+      <c r="A22" s="139"/>
       <c r="B22" s="14" t="s">
         <v>42</v>
       </c>
       <c r="C22" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B11/1000 +1.575,HardpointsRr!C11/1000,HardpointsRr!D11/1000)&amp;"]"</f>
-        <v>[-0.100904 0.576735 0.225331]</v>
+        <v>[-0.100904 0.576735 0.251011]</v>
       </c>
       <c r="D22" s="42" t="s">
         <v>12</v>
@@ -6976,7 +6976,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="156"/>
+      <c r="A23" s="140"/>
       <c r="B23" s="19" t="s">
         <v>12</v>
       </c>
@@ -6989,7 +6989,7 @@
       <c r="E23" s="67"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="146" t="s">
+      <c r="A24" s="138" t="s">
         <v>52</v>
       </c>
       <c r="B24" s="74" t="s">
@@ -7007,7 +7007,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="147"/>
+      <c r="A25" s="139"/>
       <c r="B25" s="75" t="s">
         <v>54</v>
       </c>
@@ -7023,7 +7023,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="147"/>
+      <c r="A26" s="139"/>
       <c r="B26" s="79" t="s">
         <v>146</v>
       </c>
@@ -7034,7 +7034,7 @@
       <c r="E26" s="72"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="156"/>
+      <c r="A27" s="140"/>
       <c r="B27" s="78" t="s">
         <v>147</v>
       </c>
@@ -7047,7 +7047,7 @@
       <c r="E27" s="68"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="146" t="s">
+      <c r="A28" s="138" t="s">
         <v>55</v>
       </c>
       <c r="B28" s="74" t="s">
@@ -7062,7 +7062,7 @@
       <c r="E28" s="69"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="156"/>
+      <c r="A29" s="140"/>
       <c r="B29" s="78" t="s">
         <v>57</v>
       </c>
@@ -7075,7 +7075,7 @@
       <c r="E29" s="68"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="153" t="s">
+      <c r="A30" s="155" t="s">
         <v>58</v>
       </c>
       <c r="B30" s="88" t="s">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C30" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B14/1000 + 1.575,HardpointsRr!C14/1000,HardpointsRr!D14/1000)&amp;"]"</f>
-        <v>[-0.022194 0.526395 0.155287]</v>
+        <v>[-0.022194 0.526395 0.180967]</v>
       </c>
       <c r="D30" s="12" t="s">
         <v>12</v>
@@ -7093,7 +7093,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="154"/>
+      <c r="A31" s="156"/>
       <c r="B31" s="89" t="s">
         <v>51</v>
       </c>
@@ -7109,7 +7109,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="155"/>
+      <c r="A32" s="157"/>
       <c r="B32" s="90" t="s">
         <v>12</v>
       </c>
@@ -7122,7 +7122,7 @@
       <c r="E32" s="70"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="146" t="s">
+      <c r="A33" s="138" t="s">
         <v>59</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -7140,7 +7140,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="147"/>
+      <c r="A34" s="139"/>
       <c r="B34" s="14" t="s">
         <v>61</v>
       </c>
@@ -7156,7 +7156,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="156"/>
+      <c r="A35" s="140"/>
       <c r="B35" s="19" t="s">
         <v>12</v>
       </c>
@@ -7300,7 +7300,7 @@
         <v>69</v>
       </c>
       <c r="B8" s="75"/>
-      <c r="C8" s="161">
+      <c r="C8" s="137">
         <f>1.979*2</f>
         <v>3.9580000000000002</v>
       </c>

</xml_diff>

<commit_message>
Suspension test rig optimisation and bug fixes
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC91F7D0-38BA-B946-A86E-9C35B31B7FC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F09127EB-0DDD-6E4F-BF95-EE21855C496C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="23260" windowHeight="12460" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12800" yWindow="1700" windowWidth="27000" windowHeight="16060" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Body" sheetId="1" r:id="rId1"/>
@@ -332,9 +332,6 @@
     <t>sPressureCentre</t>
   </si>
   <si>
-    <t>[-0.8 0 0.26]</t>
-  </si>
-  <si>
     <t>Spring</t>
   </si>
   <si>
@@ -575,7 +572,10 @@
     <t>[27 74 70]</t>
   </si>
   <si>
-    <t>[-0,823 0 0,315]</t>
+    <t>[-0.707 0 0.628]</t>
+  </si>
+  <si>
+    <t>[-0,8232 0 0,3583]</t>
   </si>
 </sst>
 </file>
@@ -1771,9 +1771,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2094,14 +2091,8 @@
     <xf numFmtId="165" fontId="3" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="3" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2120,6 +2111,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="58" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="63" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2142,6 +2139,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3350,11 +3350,11 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="119" t="s">
+      <c r="A5" s="118" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="74"/>
-      <c r="C5" s="77" t="s">
+      <c r="B5" s="73"/>
+      <c r="C5" s="76" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="12" t="s">
@@ -3365,11 +3365,11 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="119" t="s">
+      <c r="A6" s="118" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="75"/>
-      <c r="C6" s="76" t="s">
+      <c r="B6" s="74"/>
+      <c r="C6" s="75" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="15" t="s">
@@ -3380,11 +3380,11 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="119" t="s">
+      <c r="A7" s="118" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="75"/>
-      <c r="C7" s="76" t="s">
+      <c r="B7" s="74"/>
+      <c r="C7" s="75" t="s">
         <v>167</v>
       </c>
       <c r="D7" s="15" t="s">
@@ -3393,11 +3393,11 @@
       <c r="E7" s="16"/>
     </row>
     <row r="8" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="119" t="s">
+      <c r="A8" s="118" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="76" t="s">
+      <c r="B8" s="74"/>
+      <c r="C8" s="75" t="s">
         <v>19</v>
       </c>
       <c r="D8" s="15" t="s">
@@ -3408,11 +3408,11 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="119" t="s">
+      <c r="A9" s="118" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="75"/>
-      <c r="C9" s="76" t="s">
+      <c r="B9" s="74"/>
+      <c r="C9" s="75" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="15" t="s">
@@ -3423,11 +3423,11 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="119" t="s">
+      <c r="A10" s="118" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="75"/>
-      <c r="C10" s="76" t="s">
+      <c r="B10" s="74"/>
+      <c r="C10" s="75" t="s">
         <v>24</v>
       </c>
       <c r="D10" s="15" t="s">
@@ -3438,7 +3438,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="119" t="s">
+      <c r="A11" s="118" t="s">
         <v>25</v>
       </c>
       <c r="B11" s="14"/>
@@ -3454,10 +3454,10 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="119" t="s">
+      <c r="A12" s="118" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="75"/>
+      <c r="B12" s="74"/>
       <c r="C12" s="17">
         <f>HardpointsFr!C9*2/1000</f>
         <v>1.28</v>
@@ -3468,10 +3468,10 @@
       <c r="E12" s="16"/>
     </row>
     <row r="13" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="119" t="s">
+      <c r="A13" s="118" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="75"/>
+      <c r="B13" s="74"/>
       <c r="C13" s="17">
         <f>HardpointsRr!C9*2/1000</f>
         <v>1.2470640000000002</v>
@@ -3482,32 +3482,32 @@
       <c r="E13" s="18"/>
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="119" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="79"/>
-      <c r="C14" s="81">
+      <c r="A14" s="118" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="78"/>
+      <c r="C14" s="80">
         <v>255.07</v>
       </c>
-      <c r="D14" s="80" t="s">
+      <c r="D14" s="79" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="82" t="s">
+      <c r="E14" s="81" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="119" t="s">
+      <c r="A15" s="118" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="75"/>
-      <c r="C15" s="84" t="s">
-        <v>166</v>
-      </c>
-      <c r="D15" s="86" t="s">
+      <c r="B15" s="74"/>
+      <c r="C15" s="83" t="s">
+        <v>165</v>
+      </c>
+      <c r="D15" s="85" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="83" t="s">
+      <c r="E15" s="82" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3555,7 +3555,7 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -3566,7 +3566,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -3577,88 +3577,88 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="138" t="s">
+      <c r="A5" s="147" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="73" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="76" t="s">
         <v>89</v>
-      </c>
-      <c r="B5" s="74" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="77" t="s">
-        <v>90</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="139"/>
-      <c r="B6" s="94" t="s">
+      <c r="A6" s="148"/>
+      <c r="B6" s="93" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" s="94">
+        <v>78807.070000000007</v>
+      </c>
+      <c r="D6" s="95" t="s">
         <v>91</v>
       </c>
-      <c r="C6" s="95">
-        <v>78807.070000000007</v>
-      </c>
-      <c r="D6" s="96" t="s">
+      <c r="E6" s="96"/>
+    </row>
+    <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="157"/>
+      <c r="B7" s="77" t="s">
+        <v>143</v>
+      </c>
+      <c r="C7" s="20">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="29"/>
+    </row>
+    <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="147" t="s">
         <v>92</v>
       </c>
-      <c r="E6" s="97"/>
-    </row>
-    <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="140"/>
-      <c r="B7" s="78" t="s">
-        <v>144</v>
-      </c>
-      <c r="C7" s="20">
-        <v>1.6E-2</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="30"/>
-    </row>
-    <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="138" t="s">
-        <v>93</v>
-      </c>
-      <c r="B8" s="74" t="s">
+      <c r="B8" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="99" t="s">
-        <v>90</v>
+      <c r="C8" s="98" t="s">
+        <v>89</v>
       </c>
       <c r="D8" s="12"/>
       <c r="E8" s="28"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="139"/>
-      <c r="B9" s="94" t="s">
+      <c r="A9" s="148"/>
+      <c r="B9" s="93" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" s="97">
+        <v>56916.22</v>
+      </c>
+      <c r="D9" s="95" t="s">
         <v>91</v>
       </c>
-      <c r="C9" s="98">
-        <v>56916.22</v>
-      </c>
-      <c r="D9" s="96" t="s">
-        <v>92</v>
-      </c>
-      <c r="E9" s="97"/>
+      <c r="E9" s="96"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="140"/>
-      <c r="B10" s="78" t="s">
-        <v>144</v>
+      <c r="A10" s="157"/>
+      <c r="B10" s="77" t="s">
+        <v>143</v>
       </c>
       <c r="C10" s="20">
-        <v>1.7999999999999999E-2</v>
-      </c>
-      <c r="D10" s="87" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="30"/>
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="D10" s="86" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3707,8 +3707,8 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="102" t="s">
-        <v>157</v>
+      <c r="C2" s="101" t="s">
+        <v>156</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -3719,7 +3719,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -3730,196 +3730,196 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="138" t="s">
-        <v>89</v>
-      </c>
-      <c r="B5" s="74" t="s">
+      <c r="A5" s="147" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="77" t="s">
-        <v>159</v>
+      <c r="C5" s="76" t="s">
+        <v>158</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="139"/>
-      <c r="B6" s="94" t="s">
+      <c r="A6" s="148"/>
+      <c r="B6" s="93" t="s">
+        <v>93</v>
+      </c>
+      <c r="C6" s="130" t="s">
+        <v>93</v>
+      </c>
+      <c r="D6" s="95" t="s">
+        <v>91</v>
+      </c>
+      <c r="E6" s="131" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="148"/>
+      <c r="B7" s="74" t="s">
         <v>94</v>
-      </c>
-      <c r="C6" s="131" t="s">
-        <v>94</v>
-      </c>
-      <c r="D6" s="96" t="s">
-        <v>92</v>
-      </c>
-      <c r="E6" s="132" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="139"/>
-      <c r="B7" s="75" t="s">
-        <v>95</v>
       </c>
       <c r="C7" s="24">
         <v>100000</v>
       </c>
-      <c r="D7" s="86" t="s">
-        <v>92</v>
+      <c r="D7" s="85" t="s">
+        <v>91</v>
       </c>
       <c r="E7" s="18"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="139"/>
-      <c r="B8" s="75" t="s">
-        <v>96</v>
+      <c r="A8" s="148"/>
+      <c r="B8" s="74" t="s">
+        <v>95</v>
       </c>
       <c r="C8" s="24">
         <v>100000</v>
       </c>
-      <c r="D8" s="86" t="s">
-        <v>92</v>
+      <c r="D8" s="85" t="s">
+        <v>91</v>
       </c>
       <c r="E8" s="18"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="139"/>
-      <c r="B9" s="75" t="s">
-        <v>97</v>
+      <c r="A9" s="148"/>
+      <c r="B9" s="74" t="s">
+        <v>96</v>
       </c>
       <c r="C9" s="24">
         <v>150</v>
       </c>
-      <c r="D9" s="86" t="s">
-        <v>92</v>
+      <c r="D9" s="85" t="s">
+        <v>91</v>
       </c>
       <c r="E9" s="18"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="139"/>
-      <c r="B10" s="75" t="s">
-        <v>98</v>
+      <c r="A10" s="148"/>
+      <c r="B10" s="74" t="s">
+        <v>97</v>
       </c>
       <c r="C10" s="24">
         <v>150</v>
       </c>
-      <c r="D10" s="86" t="s">
-        <v>92</v>
+      <c r="D10" s="85" t="s">
+        <v>91</v>
       </c>
       <c r="E10" s="18"/>
     </row>
     <row r="11" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="140"/>
-      <c r="B11" s="78" t="s">
-        <v>99</v>
+      <c r="A11" s="157"/>
+      <c r="B11" s="77" t="s">
+        <v>98</v>
       </c>
       <c r="C11" s="26">
         <v>1E-4</v>
       </c>
-      <c r="D11" s="87" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="30"/>
+      <c r="D11" s="86" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="29"/>
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="138" t="s">
-        <v>93</v>
-      </c>
-      <c r="B12" s="74" t="s">
+      <c r="A12" s="147" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="77" t="s">
-        <v>159</v>
+      <c r="C12" s="76" t="s">
+        <v>158</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="28"/>
     </row>
     <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="139"/>
-      <c r="B13" s="94" t="s">
+      <c r="A13" s="148"/>
+      <c r="B13" s="93" t="s">
+        <v>93</v>
+      </c>
+      <c r="C13" s="130" t="s">
+        <v>93</v>
+      </c>
+      <c r="D13" s="100" t="s">
+        <v>91</v>
+      </c>
+      <c r="E13" s="131" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="148"/>
+      <c r="B14" s="74" t="s">
         <v>94</v>
-      </c>
-      <c r="C13" s="131" t="s">
-        <v>94</v>
-      </c>
-      <c r="D13" s="101" t="s">
-        <v>92</v>
-      </c>
-      <c r="E13" s="132" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="139"/>
-      <c r="B14" s="75" t="s">
-        <v>95</v>
       </c>
       <c r="C14" s="24">
         <v>100000</v>
       </c>
-      <c r="D14" s="101" t="s">
-        <v>92</v>
+      <c r="D14" s="100" t="s">
+        <v>91</v>
       </c>
       <c r="E14" s="18"/>
     </row>
     <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="139"/>
-      <c r="B15" s="75" t="s">
-        <v>96</v>
+      <c r="A15" s="148"/>
+      <c r="B15" s="74" t="s">
+        <v>95</v>
       </c>
       <c r="C15" s="24">
         <v>100000</v>
       </c>
-      <c r="D15" s="101" t="s">
-        <v>92</v>
+      <c r="D15" s="100" t="s">
+        <v>91</v>
       </c>
       <c r="E15" s="18"/>
     </row>
     <row r="16" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="139"/>
-      <c r="B16" s="75" t="s">
-        <v>97</v>
+      <c r="A16" s="148"/>
+      <c r="B16" s="74" t="s">
+        <v>96</v>
       </c>
       <c r="C16" s="24">
         <v>150</v>
       </c>
-      <c r="D16" s="101" t="s">
-        <v>92</v>
+      <c r="D16" s="100" t="s">
+        <v>91</v>
       </c>
       <c r="E16" s="18"/>
     </row>
     <row r="17" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="139"/>
-      <c r="B17" s="75" t="s">
-        <v>98</v>
+      <c r="A17" s="148"/>
+      <c r="B17" s="74" t="s">
+        <v>97</v>
       </c>
       <c r="C17" s="24">
         <v>150</v>
       </c>
-      <c r="D17" s="101" t="s">
-        <v>92</v>
+      <c r="D17" s="100" t="s">
+        <v>91</v>
       </c>
       <c r="E17" s="18"/>
     </row>
     <row r="18" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="140"/>
-      <c r="B18" s="78" t="s">
-        <v>99</v>
+      <c r="A18" s="157"/>
+      <c r="B18" s="77" t="s">
+        <v>98</v>
       </c>
       <c r="C18" s="26">
         <v>1E-4</v>
       </c>
-      <c r="D18" s="87" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" s="30"/>
+      <c r="D18" s="86" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3940,810 +3940,810 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="133">
+      <c r="A1" s="132">
         <v>-443.53</v>
       </c>
-      <c r="B1" s="133">
+      <c r="B1" s="132">
         <v>-3883.5949999999998</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="133">
+      <c r="A2" s="132">
         <v>-433.58</v>
       </c>
-      <c r="B2" s="133">
+      <c r="B2" s="132">
         <v>-3833.1889999999999</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="133">
+      <c r="A3" s="132">
         <v>-423.97</v>
       </c>
-      <c r="B3" s="133">
+      <c r="B3" s="132">
         <v>-3778.5659999999998</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="133">
+      <c r="A4" s="132">
         <v>-415</v>
       </c>
-      <c r="B4" s="133">
+      <c r="B4" s="132">
         <v>-3715.607</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="133">
+      <c r="A5" s="132">
         <v>-406.67</v>
       </c>
-      <c r="B5" s="133">
+      <c r="B5" s="132">
         <v>-3644.3130000000001</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="133">
+      <c r="A6" s="132">
         <v>-398.79</v>
       </c>
-      <c r="B6" s="133">
+      <c r="B6" s="132">
         <v>-3567.2330000000002</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="133">
+      <c r="A7" s="132">
         <v>-391.16</v>
       </c>
-      <c r="B7" s="133">
+      <c r="B7" s="132">
         <v>-3486.6219999999998</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="133">
+      <c r="A8" s="132">
         <v>-383.59</v>
       </c>
-      <c r="B8" s="133">
+      <c r="B8" s="132">
         <v>-3405.2269999999999</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="133">
+      <c r="A9" s="132">
         <v>-375.88</v>
       </c>
-      <c r="B9" s="133">
+      <c r="B9" s="132">
         <v>-3325.3029999999999</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="133">
+      <c r="A10" s="132">
         <v>-367.89</v>
       </c>
-      <c r="B10" s="133">
+      <c r="B10" s="132">
         <v>-3248.7130000000002</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="133">
+      <c r="A11" s="132">
         <v>-359.64</v>
       </c>
-      <c r="B11" s="133">
+      <c r="B11" s="132">
         <v>-3175.3589999999999</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="133">
+      <c r="A12" s="132">
         <v>-351.2</v>
       </c>
-      <c r="B12" s="133">
+      <c r="B12" s="132">
         <v>-3104.163</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="133">
+      <c r="A13" s="132">
         <v>-342.63</v>
       </c>
-      <c r="B13" s="133">
+      <c r="B13" s="132">
         <v>-3034.5360000000001</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="133">
+      <c r="A14" s="132">
         <v>-334</v>
       </c>
-      <c r="B14" s="133">
+      <c r="B14" s="132">
         <v>-2965.6930000000002</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" s="133">
+      <c r="A15" s="132">
         <v>-325.38</v>
       </c>
-      <c r="B15" s="133">
+      <c r="B15" s="132">
         <v>-2896.85</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="133">
+      <c r="A16" s="132">
         <v>-316.77</v>
       </c>
-      <c r="B16" s="133">
+      <c r="B16" s="132">
         <v>-2827.6149999999998</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="133">
+      <c r="A17" s="132">
         <v>-308.2</v>
       </c>
-      <c r="B17" s="133">
+      <c r="B17" s="132">
         <v>-2757.9879999999998</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="133">
+      <c r="A18" s="132">
         <v>-299.64999999999998</v>
       </c>
-      <c r="B18" s="133">
+      <c r="B18" s="132">
         <v>-2687.9690000000001</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="133">
+      <c r="A19" s="132">
         <v>-291.14</v>
       </c>
-      <c r="B19" s="133">
+      <c r="B19" s="132">
         <v>-2617.5569999999998</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="133">
+      <c r="A20" s="132">
         <v>-282.67</v>
       </c>
-      <c r="B20" s="133">
+      <c r="B20" s="132">
         <v>-2546.6550000000002</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="133">
+      <c r="A21" s="132">
         <v>-274.25</v>
       </c>
-      <c r="B21" s="133">
+      <c r="B21" s="132">
         <v>-2475.1640000000002</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="133">
+      <c r="A22" s="132">
         <v>-265.91000000000003</v>
       </c>
-      <c r="B22" s="133">
+      <c r="B22" s="132">
         <v>-2402.7910000000002</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="133">
+      <c r="A23" s="132">
         <v>-257.67</v>
       </c>
-      <c r="B23" s="133">
+      <c r="B23" s="132">
         <v>-2329.3389999999999</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" s="133">
+      <c r="A24" s="132">
         <v>-249.56</v>
       </c>
-      <c r="B24" s="133">
+      <c r="B24" s="132">
         <v>-2254.5149999999999</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25" s="133">
+      <c r="A25" s="132">
         <v>-241.62</v>
       </c>
-      <c r="B25" s="133">
+      <c r="B25" s="132">
         <v>-2178.2190000000001</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" s="133">
+      <c r="A26" s="132">
         <v>-233.85</v>
       </c>
-      <c r="B26" s="133">
+      <c r="B26" s="132">
         <v>-2100.06</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27" s="133">
+      <c r="A27" s="132">
         <v>-226.23</v>
       </c>
-      <c r="B27" s="133">
+      <c r="B27" s="132">
         <v>-2020.528</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A28" s="133">
+      <c r="A28" s="132">
         <v>-218.75</v>
       </c>
-      <c r="B28" s="133">
+      <c r="B28" s="132">
         <v>-1939.623</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A29" s="133">
+      <c r="A29" s="132">
         <v>-211.37</v>
       </c>
-      <c r="B29" s="133">
+      <c r="B29" s="132">
         <v>-1857.934</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A30" s="133">
+      <c r="A30" s="132">
         <v>-204.05</v>
       </c>
-      <c r="B30" s="133">
+      <c r="B30" s="132">
         <v>-1775.46</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A31" s="133">
+      <c r="A31" s="132">
         <v>-196.78</v>
       </c>
-      <c r="B31" s="133">
+      <c r="B31" s="132">
         <v>-1692.79</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A32" s="133">
+      <c r="A32" s="132">
         <v>-189.52</v>
       </c>
-      <c r="B32" s="133">
+      <c r="B32" s="132">
         <v>-1609.923</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A33" s="133">
+      <c r="A33" s="132">
         <v>-182.26</v>
       </c>
-      <c r="B33" s="133">
+      <c r="B33" s="132">
         <v>-1527.155</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A34" s="133">
+      <c r="A34" s="132">
         <v>-174.97</v>
       </c>
-      <c r="B34" s="133">
+      <c r="B34" s="132">
         <v>-1444.681</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A35" s="133">
+      <c r="A35" s="132">
         <v>-167.65</v>
       </c>
-      <c r="B35" s="133">
+      <c r="B35" s="132">
         <v>-1362.502</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A36" s="133">
+      <c r="A36" s="132">
         <v>-160.27000000000001</v>
       </c>
-      <c r="B36" s="133">
+      <c r="B36" s="132">
         <v>-1280.8119999999999</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A37" s="133">
+      <c r="A37" s="132">
         <v>-152.82</v>
       </c>
-      <c r="B37" s="133">
+      <c r="B37" s="132">
         <v>-1199.711</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A38" s="133">
+      <c r="A38" s="132">
         <v>-145.29</v>
       </c>
-      <c r="B38" s="133">
+      <c r="B38" s="132">
         <v>-1119.297</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A39" s="133">
+      <c r="A39" s="132">
         <v>-137.65</v>
       </c>
-      <c r="B39" s="133">
+      <c r="B39" s="132">
         <v>-1039.7650000000001</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A40" s="133">
+      <c r="A40" s="132">
         <v>-129.9</v>
       </c>
-      <c r="B40" s="133">
+      <c r="B40" s="132">
         <v>-961.31200000000001</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A41" s="133">
+      <c r="A41" s="132">
         <v>-122.02</v>
       </c>
-      <c r="B41" s="133">
+      <c r="B41" s="132">
         <v>-884.13300000000004</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" s="133">
+      <c r="A42" s="132">
         <v>-114.01</v>
       </c>
-      <c r="B42" s="133">
+      <c r="B42" s="132">
         <v>-808.32799999999997</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A43" s="133">
+      <c r="A43" s="132">
         <v>-105.84</v>
       </c>
-      <c r="B43" s="133">
+      <c r="B43" s="132">
         <v>-734.19</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A44" s="133">
+      <c r="A44" s="132">
         <v>-97.52</v>
       </c>
-      <c r="B44" s="133">
+      <c r="B44" s="132">
         <v>-661.71799999999996</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A45" s="133">
+      <c r="A45" s="132">
         <v>-89.05</v>
       </c>
-      <c r="B45" s="133">
+      <c r="B45" s="132">
         <v>-590.91399999999999</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A46" s="133">
+      <c r="A46" s="132">
         <v>-80.430000000000007</v>
       </c>
-      <c r="B46" s="133">
+      <c r="B46" s="132">
         <v>-521.67999999999995</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A47" s="133">
+      <c r="A47" s="132">
         <v>-71.680000000000007</v>
       </c>
-      <c r="B47" s="133">
+      <c r="B47" s="132">
         <v>-454.21</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A48" s="133">
+      <c r="A48" s="132">
         <v>-62.8</v>
       </c>
-      <c r="B48" s="133">
+      <c r="B48" s="132">
         <v>-388.113</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A49" s="133">
+      <c r="A49" s="132">
         <v>-53.8</v>
       </c>
-      <c r="B49" s="133">
+      <c r="B49" s="132">
         <v>-323.68299999999999</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A50" s="133">
+      <c r="A50" s="132">
         <v>-44.68</v>
       </c>
-      <c r="B50" s="133">
+      <c r="B50" s="132">
         <v>-260.92099999999999</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A51" s="133">
+      <c r="A51" s="132">
         <v>-35.409999999999997</v>
       </c>
-      <c r="B51" s="133">
+      <c r="B51" s="132">
         <v>-200.41399999999999</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A52" s="133">
+      <c r="A52" s="132">
         <v>-25.99</v>
       </c>
-      <c r="B52" s="133">
+      <c r="B52" s="132">
         <v>-142.26</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A53" s="133">
+      <c r="A53" s="132">
         <v>-16.38</v>
       </c>
-      <c r="B53" s="133">
+      <c r="B53" s="132">
         <v>-86.950999999999993</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A54" s="133">
+      <c r="A54" s="132">
         <v>-6.61</v>
       </c>
-      <c r="B54" s="133">
+      <c r="B54" s="132">
         <v>-34.387</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A55" s="133">
+      <c r="A55" s="132">
         <v>0</v>
       </c>
-      <c r="B55" s="133">
+      <c r="B55" s="132">
         <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A56" s="133">
+      <c r="A56" s="132">
         <v>3.23</v>
       </c>
-      <c r="B56" s="133">
+      <c r="B56" s="132">
         <v>16.803999999999998</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A57" s="133">
+      <c r="A57" s="132">
         <v>13.04</v>
       </c>
-      <c r="B57" s="133">
+      <c r="B57" s="132">
         <v>68.484999999999999</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A58" s="133">
+      <c r="A58" s="132">
         <v>22.71</v>
       </c>
-      <c r="B58" s="133">
+      <c r="B58" s="132">
         <v>122.42100000000001</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A59" s="133">
+      <c r="A59" s="132">
         <v>32.119999999999997</v>
       </c>
-      <c r="B59" s="133">
+      <c r="B59" s="132">
         <v>180.18199999999999</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A60" s="133">
+      <c r="A60" s="132">
         <v>41.25</v>
       </c>
-      <c r="B60" s="133">
+      <c r="B60" s="132">
         <v>242.25899999999999</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A61" s="133">
+      <c r="A61" s="132">
         <v>50.17</v>
       </c>
-      <c r="B61" s="133">
+      <c r="B61" s="132">
         <v>307.66899999999998</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A62" s="133">
+      <c r="A62" s="132">
         <v>58.93</v>
       </c>
-      <c r="B62" s="133">
+      <c r="B62" s="132">
         <v>375.33499999999998</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A63" s="133">
+      <c r="A63" s="132">
         <v>67.61</v>
       </c>
-      <c r="B63" s="133">
+      <c r="B63" s="132">
         <v>444.07900000000001</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A64" s="133">
+      <c r="A64" s="132">
         <v>76.28</v>
       </c>
-      <c r="B64" s="133">
+      <c r="B64" s="132">
         <v>512.92200000000003</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A65" s="133">
+      <c r="A65" s="132">
         <v>84.97</v>
       </c>
-      <c r="B65" s="133">
+      <c r="B65" s="132">
         <v>581.274</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A66" s="133">
+      <c r="A66" s="132">
         <v>93.66</v>
       </c>
-      <c r="B66" s="133">
+      <c r="B66" s="132">
         <v>649.33299999999997</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A67" s="133">
+      <c r="A67" s="132">
         <v>102.34</v>
       </c>
-      <c r="B67" s="133">
+      <c r="B67" s="132">
         <v>717.58699999999999</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A68" s="133">
+      <c r="A68" s="132">
         <v>110.99</v>
       </c>
-      <c r="B68" s="133">
+      <c r="B68" s="132">
         <v>786.23299999999995</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A69" s="133">
+      <c r="A69" s="132">
         <v>119.59</v>
       </c>
-      <c r="B69" s="133">
+      <c r="B69" s="132">
         <v>855.66399999999999</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A70" s="133">
+      <c r="A70" s="132">
         <v>128.15</v>
       </c>
-      <c r="B70" s="133">
+      <c r="B70" s="132">
         <v>925.68399999999997</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A71" s="133">
+      <c r="A71" s="132">
         <v>136.76</v>
       </c>
-      <c r="B71" s="133">
+      <c r="B71" s="132">
         <v>995.11500000000001</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A72" s="133">
+      <c r="A72" s="132">
         <v>145.5</v>
       </c>
-      <c r="B72" s="133">
+      <c r="B72" s="132">
         <v>1062.8789999999999</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A73" s="133">
+      <c r="A73" s="132">
         <v>154.46</v>
       </c>
-      <c r="B73" s="133">
+      <c r="B73" s="132">
         <v>1127.6030000000001</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A74" s="133">
+      <c r="A74" s="132">
         <v>163.72</v>
       </c>
-      <c r="B74" s="133">
+      <c r="B74" s="132">
         <v>1188.1099999999999</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A75" s="133">
+      <c r="A75" s="132">
         <v>173.35</v>
       </c>
-      <c r="B75" s="133">
+      <c r="B75" s="132">
         <v>1243.3209999999999</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A76" s="133">
+      <c r="A76" s="132">
         <v>183.3</v>
       </c>
-      <c r="B76" s="133">
+      <c r="B76" s="132">
         <v>1293.0409999999999</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A77" s="133">
+      <c r="A77" s="132">
         <v>193.53</v>
       </c>
-      <c r="B77" s="133">
+      <c r="B77" s="132">
         <v>1336.877</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A78" s="133">
+      <c r="A78" s="132">
         <v>204</v>
       </c>
-      <c r="B78" s="133">
+      <c r="B78" s="132">
         <v>1374.829</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A79" s="133">
+      <c r="A79" s="132">
         <v>214.66</v>
       </c>
-      <c r="B79" s="133">
+      <c r="B79" s="132">
         <v>1406.7</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A80" s="133">
+      <c r="A80" s="132">
         <v>225.46</v>
       </c>
-      <c r="B80" s="133">
+      <c r="B80" s="132">
         <v>1433.2760000000001</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A81" s="133">
+      <c r="A81" s="132">
         <v>236.35</v>
       </c>
-      <c r="B81" s="133">
+      <c r="B81" s="132">
         <v>1455.93</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A82" s="133">
+      <c r="A82" s="132">
         <v>247.31</v>
       </c>
-      <c r="B82" s="133">
+      <c r="B82" s="132">
         <v>1476.0329999999999</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A83" s="133">
+      <c r="A83" s="132">
         <v>258.27999999999997</v>
       </c>
-      <c r="B83" s="133">
+      <c r="B83" s="132">
         <v>1494.8620000000001</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A84" s="133">
+      <c r="A84" s="132">
         <v>269.26</v>
       </c>
-      <c r="B84" s="133">
+      <c r="B84" s="132">
         <v>1513.396</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A85" s="133">
+      <c r="A85" s="132">
         <v>280.23</v>
       </c>
-      <c r="B85" s="133">
+      <c r="B85" s="132">
         <v>1531.8330000000001</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A86" s="133">
+      <c r="A86" s="132">
         <v>291.19</v>
       </c>
-      <c r="B86" s="133">
+      <c r="B86" s="132">
         <v>1550.3679999999999</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A87" s="133">
+      <c r="A87" s="132">
         <v>302.14999999999998</v>
       </c>
-      <c r="B87" s="133">
+      <c r="B87" s="132">
         <v>1569.2940000000001</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A88" s="133">
+      <c r="A88" s="132">
         <v>313.10000000000002</v>
       </c>
-      <c r="B88" s="133">
+      <c r="B88" s="132">
         <v>1588.712</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A89" s="133">
+      <c r="A89" s="132">
         <v>324.05</v>
       </c>
-      <c r="B89" s="133">
+      <c r="B89" s="132">
         <v>1608.325</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A90" s="133">
+      <c r="A90" s="132">
         <v>335.01</v>
       </c>
-      <c r="B90" s="133">
+      <c r="B90" s="132">
         <v>1627.9380000000001</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A91" s="133">
+      <c r="A91" s="132">
         <v>345.96</v>
       </c>
-      <c r="B91" s="133">
+      <c r="B91" s="132">
         <v>1647.2570000000001</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A92" s="133">
+      <c r="A92" s="132">
         <v>356.92</v>
       </c>
-      <c r="B92" s="133">
+      <c r="B92" s="132">
         <v>1666.2819999999999</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A93" s="133">
+      <c r="A93" s="132">
         <v>367.88</v>
       </c>
-      <c r="B93" s="133">
+      <c r="B93" s="132">
         <v>1685.6010000000001</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A94" s="133">
+      <c r="A94" s="132">
         <v>378.83</v>
       </c>
-      <c r="B94" s="133">
+      <c r="B94" s="132">
         <v>1705.4110000000001</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A95" s="133">
+      <c r="A95" s="132">
         <v>389.75</v>
       </c>
-      <c r="B95" s="133">
+      <c r="B95" s="132">
         <v>1726.3969999999999</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A96" s="133">
+      <c r="A96" s="132">
         <v>400.65</v>
       </c>
-      <c r="B96" s="133">
+      <c r="B96" s="132">
         <v>1748.6579999999999</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A97" s="133">
+      <c r="A97" s="132">
         <v>411.52</v>
       </c>
-      <c r="B97" s="133">
+      <c r="B97" s="132">
         <v>1772.39</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A98" s="133">
+      <c r="A98" s="132">
         <v>422.35</v>
       </c>
-      <c r="B98" s="133">
+      <c r="B98" s="132">
         <v>1797.4949999999999</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A99" s="133">
+      <c r="A99" s="132">
         <v>433.15</v>
       </c>
-      <c r="B99" s="133">
+      <c r="B99" s="132">
         <v>1823.973</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A100" s="133">
+      <c r="A100" s="132">
         <v>443.91</v>
       </c>
-      <c r="B100" s="133">
+      <c r="B100" s="132">
         <v>1851.8240000000001</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A101" s="133">
+      <c r="A101" s="132">
         <v>454.66</v>
       </c>
-      <c r="B101" s="133">
+      <c r="B101" s="132">
         <v>1880.3610000000001</v>
       </c>
     </row>
@@ -4784,8 +4784,8 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="102" t="s">
-        <v>100</v>
+      <c r="C2" s="101" t="s">
+        <v>99</v>
       </c>
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
@@ -4795,8 +4795,8 @@
         <v>6</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="102" t="s">
-        <v>153</v>
+      <c r="C3" s="101" t="s">
+        <v>152</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
@@ -4806,145 +4806,145 @@
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="102" t="s">
-        <v>163</v>
+      <c r="C4" s="101" t="s">
+        <v>162</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="92" t="s">
+      <c r="A5" s="91" t="s">
+        <v>100</v>
+      </c>
+      <c r="B5" s="73"/>
+      <c r="C5" s="120" t="s">
+        <v>153</v>
+      </c>
+      <c r="D5" s="102" t="s">
         <v>101</v>
       </c>
-      <c r="B5" s="74"/>
-      <c r="C5" s="121" t="s">
-        <v>154</v>
-      </c>
-      <c r="D5" s="103" t="s">
+      <c r="E5" s="103" t="s">
         <v>102</v>
       </c>
-      <c r="E5" s="104" t="s">
+    </row>
+    <row r="6" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="91" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="92" t="s">
+      <c r="B6" s="73"/>
+      <c r="C6" s="99">
+        <v>10</v>
+      </c>
+      <c r="D6" s="102" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="28"/>
+    </row>
+    <row r="7" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="91" t="s">
         <v>104</v>
       </c>
-      <c r="B6" s="74"/>
-      <c r="C6" s="100">
-        <v>10</v>
-      </c>
-      <c r="D6" s="103" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="28"/>
-    </row>
-    <row r="7" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="92" t="s">
+      <c r="B7" s="73"/>
+      <c r="C7" s="99" t="s">
         <v>105</v>
       </c>
-      <c r="B7" s="74"/>
-      <c r="C7" s="100" t="s">
+      <c r="D7" s="102" t="s">
         <v>106</v>
       </c>
-      <c r="D7" s="103" t="s">
+      <c r="E7" s="28"/>
+    </row>
+    <row r="8" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="91" t="s">
         <v>107</v>
       </c>
-      <c r="E7" s="28"/>
-    </row>
-    <row r="8" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="92" t="s">
+      <c r="B8" s="73"/>
+      <c r="C8" s="104" t="s">
         <v>108</v>
       </c>
-      <c r="B8" s="74"/>
-      <c r="C8" s="105" t="s">
+      <c r="D8" s="102" t="s">
+        <v>101</v>
+      </c>
+      <c r="E8" s="28"/>
+    </row>
+    <row r="9" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="91" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="103" t="s">
-        <v>102</v>
-      </c>
-      <c r="E8" s="28"/>
-    </row>
-    <row r="9" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="92" t="s">
+      <c r="B9" s="73"/>
+      <c r="C9" s="99">
+        <v>25000</v>
+      </c>
+      <c r="D9" s="102"/>
+      <c r="E9" s="28"/>
+    </row>
+    <row r="10" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="91" t="s">
         <v>110</v>
       </c>
-      <c r="B9" s="74"/>
-      <c r="C9" s="100">
-        <v>25000</v>
-      </c>
-      <c r="D9" s="103"/>
-      <c r="E9" s="28"/>
-    </row>
-    <row r="10" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="92" t="s">
+      <c r="B10" s="73"/>
+      <c r="C10" s="99">
+        <v>0.01</v>
+      </c>
+      <c r="D10" s="102" t="s">
         <v>111</v>
       </c>
-      <c r="B10" s="74"/>
-      <c r="C10" s="100">
-        <v>0.01</v>
-      </c>
-      <c r="D10" s="103" t="s">
+      <c r="E10" s="103" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="104" t="s">
+    </row>
+    <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="147" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="138" t="s">
+      <c r="B11" s="105" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="106" t="s">
+        <v>147</v>
+      </c>
+      <c r="D11" s="90"/>
+      <c r="E11" s="70"/>
+    </row>
+    <row r="12" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="157"/>
+      <c r="B12" s="107" t="s">
         <v>114</v>
       </c>
-      <c r="B11" s="106" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="107" t="s">
-        <v>148</v>
-      </c>
-      <c r="D11" s="91"/>
-      <c r="E11" s="71"/>
-    </row>
-    <row r="12" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="140"/>
-      <c r="B12" s="108" t="s">
-        <v>115</v>
-      </c>
-      <c r="C12" s="109" t="s">
+      <c r="C12" s="108" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="110" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="111"/>
+      <c r="D12" s="109" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="110"/>
     </row>
     <row r="13" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="92" t="s">
+      <c r="A13" s="91" t="s">
+        <v>150</v>
+      </c>
+      <c r="B13" s="73"/>
+      <c r="C13" s="99" t="s">
+        <v>163</v>
+      </c>
+      <c r="D13" s="102"/>
+      <c r="E13" s="103" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="91" t="s">
         <v>151</v>
       </c>
-      <c r="B13" s="74"/>
-      <c r="C13" s="100" t="s">
+      <c r="B14" s="73"/>
+      <c r="C14" s="99" t="s">
         <v>164</v>
       </c>
-      <c r="D13" s="103"/>
-      <c r="E13" s="104" t="s">
+      <c r="D14" s="102"/>
+      <c r="E14" s="103"/>
+    </row>
+    <row r="18" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D18" s="135" t="s">
         <v>161</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="92" t="s">
-        <v>152</v>
-      </c>
-      <c r="B14" s="74"/>
-      <c r="C14" s="100" t="s">
-        <v>165</v>
-      </c>
-      <c r="D14" s="103"/>
-      <c r="E14" s="104"/>
-    </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D18" s="136" t="s">
-        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -4969,296 +4969,296 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="30" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="C1" s="30" t="s">
         <v>117</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="D1" s="30" t="s">
         <v>118</v>
       </c>
-      <c r="D1" s="31" t="s">
+    </row>
+    <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="31" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="32" t="s">
+      <c r="B2" s="32">
+        <v>200</v>
+      </c>
+      <c r="C2" s="33">
+        <v>203.34700000000001</v>
+      </c>
+      <c r="D2" s="33">
+        <v>126.35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="34" t="s">
         <v>120</v>
       </c>
-      <c r="B2" s="33">
-        <v>200</v>
-      </c>
-      <c r="C2" s="34">
-        <v>203.34700000000001</v>
-      </c>
-      <c r="D2" s="34">
+      <c r="B3" s="35">
+        <v>-200</v>
+      </c>
+      <c r="C3" s="36">
+        <v>225</v>
+      </c>
+      <c r="D3" s="36">
         <v>126.35</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="35" t="s">
+    <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="34" t="s">
         <v>121</v>
       </c>
-      <c r="B3" s="36">
-        <v>-200</v>
-      </c>
-      <c r="C3" s="37">
+      <c r="B4" s="35">
+        <v>11.946</v>
+      </c>
+      <c r="C4" s="36">
+        <v>587.82100000000003</v>
+      </c>
+      <c r="D4" s="36">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" s="35">
+        <v>148.751</v>
+      </c>
+      <c r="C5" s="36">
+        <v>207.047</v>
+      </c>
+      <c r="D5" s="36">
+        <v>321.79399999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="34" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" s="35">
+        <v>-184.72900000000001</v>
+      </c>
+      <c r="C6" s="36">
         <v>225</v>
       </c>
-      <c r="D3" s="37">
-        <v>126.35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="35" t="s">
-        <v>122</v>
-      </c>
-      <c r="B4" s="36">
-        <v>11.946</v>
-      </c>
-      <c r="C4" s="37">
-        <v>587.82100000000003</v>
-      </c>
-      <c r="D4" s="37">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="35" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="36">
-        <v>148.751</v>
-      </c>
-      <c r="C5" s="37">
-        <v>207.047</v>
-      </c>
-      <c r="D5" s="37">
-        <v>321.79399999999998</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="35" t="s">
+      <c r="D6" s="36">
+        <v>300.89400000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="B6" s="36">
-        <v>-184.72900000000001</v>
-      </c>
-      <c r="C6" s="37">
-        <v>225</v>
-      </c>
-      <c r="D6" s="37">
-        <v>300.89400000000001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="35" t="s">
+      <c r="B7" s="35">
+        <v>-12.932</v>
+      </c>
+      <c r="C7" s="36">
+        <v>518.67999999999995</v>
+      </c>
+      <c r="D7" s="36">
+        <v>374.39299999999997</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="34" t="s">
         <v>125</v>
       </c>
-      <c r="B7" s="36">
-        <v>-12.932</v>
-      </c>
-      <c r="C7" s="37">
-        <v>518.67999999999995</v>
-      </c>
-      <c r="D7" s="37">
-        <v>374.39299999999997</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="35" t="s">
+      <c r="B8" s="35">
+        <v>16.193999999999999</v>
+      </c>
+      <c r="C8" s="36">
+        <v>582.05899999999997</v>
+      </c>
+      <c r="D8" s="36">
+        <v>263.346</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="34" t="s">
         <v>126</v>
       </c>
-      <c r="B8" s="36">
-        <v>16.193999999999999</v>
-      </c>
-      <c r="C8" s="37">
-        <v>582.05899999999997</v>
-      </c>
-      <c r="D8" s="37">
-        <v>263.346</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="35" t="s">
+      <c r="B9" s="35">
+        <v>0</v>
+      </c>
+      <c r="C9" s="36">
+        <v>640</v>
+      </c>
+      <c r="D9" s="36">
+        <v>260.36099999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="B9" s="36">
+      <c r="B10" s="35">
+        <v>104.241</v>
+      </c>
+      <c r="C10" s="36">
+        <v>250</v>
+      </c>
+      <c r="D10" s="36">
+        <v>171.053</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="B11" s="35">
+        <v>85.097999999999999</v>
+      </c>
+      <c r="C11" s="36">
+        <v>575.40700000000004</v>
+      </c>
+      <c r="D11" s="36">
+        <v>188.44399999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="34" t="s">
+        <v>129</v>
+      </c>
+      <c r="B12" s="35">
+        <v>11.157</v>
+      </c>
+      <c r="C12" s="36">
+        <v>233.131</v>
+      </c>
+      <c r="D12" s="36">
+        <v>517.55100000000004</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="34" t="s">
+        <v>130</v>
+      </c>
+      <c r="B13" s="35">
+        <v>11.484999999999999</v>
+      </c>
+      <c r="C13" s="36">
+        <v>317.84199999999998</v>
+      </c>
+      <c r="D13" s="36">
+        <v>362.43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="34" t="s">
+        <v>131</v>
+      </c>
+      <c r="B14" s="35">
+        <v>11.821</v>
+      </c>
+      <c r="C14" s="36">
+        <v>550</v>
+      </c>
+      <c r="D14" s="36">
+        <v>178.70500000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="34" t="s">
+        <v>132</v>
+      </c>
+      <c r="B15" s="35">
+        <v>11.489000000000001</v>
+      </c>
+      <c r="C15" s="36">
+        <v>351.53699999999998</v>
+      </c>
+      <c r="D15" s="36">
+        <v>360.94299999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="34" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" s="35">
+        <v>11.558</v>
+      </c>
+      <c r="C16" s="36">
+        <v>244.43100000000001</v>
+      </c>
+      <c r="D16" s="36">
+        <v>328.19799999999998</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="34" t="s">
+        <v>134</v>
+      </c>
+      <c r="B17" s="35">
+        <v>20.965</v>
+      </c>
+      <c r="C17" s="36">
+        <v>262.85500000000002</v>
+      </c>
+      <c r="D17" s="36">
+        <v>101.35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="34" t="s">
+        <v>135</v>
+      </c>
+      <c r="B18" s="35">
+        <v>-23.5</v>
+      </c>
+      <c r="C18" s="36">
+        <v>262.85500000000002</v>
+      </c>
+      <c r="D18" s="36">
+        <v>101.51900000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="B19" s="35">
+        <v>11.526999999999999</v>
+      </c>
+      <c r="C19" s="36">
+        <v>292.24599999999998</v>
+      </c>
+      <c r="D19" s="36">
+        <v>342.81599999999997</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="34" t="s">
+        <v>137</v>
+      </c>
+      <c r="B20" s="35">
+        <v>104.241</v>
+      </c>
+      <c r="C20" s="36">
         <v>0</v>
       </c>
-      <c r="C9" s="37">
-        <v>640</v>
-      </c>
-      <c r="D9" s="37">
-        <v>260.36099999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="35" t="s">
-        <v>128</v>
-      </c>
-      <c r="B10" s="36">
-        <v>104.241</v>
-      </c>
-      <c r="C10" s="37">
-        <v>250</v>
-      </c>
-      <c r="D10" s="37">
+      <c r="D20" s="36">
         <v>171.053</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="35" t="s">
-        <v>129</v>
-      </c>
-      <c r="B11" s="36">
-        <v>85.097999999999999</v>
-      </c>
-      <c r="C11" s="37">
-        <v>575.40700000000004</v>
-      </c>
-      <c r="D11" s="37">
-        <v>188.44399999999999</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="35" t="s">
-        <v>130</v>
-      </c>
-      <c r="B12" s="36">
-        <v>11.157</v>
-      </c>
-      <c r="C12" s="37">
-        <v>233.131</v>
-      </c>
-      <c r="D12" s="37">
-        <v>517.55100000000004</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="35" t="s">
-        <v>131</v>
-      </c>
-      <c r="B13" s="36">
-        <v>11.484999999999999</v>
-      </c>
-      <c r="C13" s="37">
-        <v>317.84199999999998</v>
-      </c>
-      <c r="D13" s="37">
-        <v>362.43</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="35" t="s">
-        <v>132</v>
-      </c>
-      <c r="B14" s="36">
-        <v>11.821</v>
-      </c>
-      <c r="C14" s="37">
-        <v>550</v>
-      </c>
-      <c r="D14" s="37">
-        <v>178.70500000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="35" t="s">
-        <v>133</v>
-      </c>
-      <c r="B15" s="36">
-        <v>11.489000000000001</v>
-      </c>
-      <c r="C15" s="37">
-        <v>351.53699999999998</v>
-      </c>
-      <c r="D15" s="37">
-        <v>360.94299999999998</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="35" t="s">
-        <v>134</v>
-      </c>
-      <c r="B16" s="36">
-        <v>11.558</v>
-      </c>
-      <c r="C16" s="37">
-        <v>244.43100000000001</v>
-      </c>
-      <c r="D16" s="37">
-        <v>328.19799999999998</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="35" t="s">
-        <v>135</v>
-      </c>
-      <c r="B17" s="36">
-        <v>20.965</v>
-      </c>
-      <c r="C17" s="37">
-        <v>262.85500000000002</v>
-      </c>
-      <c r="D17" s="37">
-        <v>101.35</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="35" t="s">
-        <v>136</v>
-      </c>
-      <c r="B18" s="36">
-        <v>-23.5</v>
-      </c>
-      <c r="C18" s="37">
-        <v>262.85500000000002</v>
-      </c>
-      <c r="D18" s="37">
-        <v>101.51900000000001</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="35" t="s">
-        <v>137</v>
-      </c>
-      <c r="B19" s="36">
-        <v>11.526999999999999</v>
-      </c>
-      <c r="C19" s="37">
-        <v>292.24599999999998</v>
-      </c>
-      <c r="D19" s="37">
-        <v>342.81599999999997</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="35" t="s">
+    <row r="21" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="34" t="s">
         <v>138</v>
       </c>
-      <c r="B20" s="36">
-        <v>104.241</v>
-      </c>
-      <c r="C20" s="37">
+      <c r="B21" s="35">
+        <v>-324.96499999999997</v>
+      </c>
+      <c r="C21" s="36">
         <v>0</v>
       </c>
-      <c r="D20" s="37">
-        <v>171.053</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="35" t="s">
-        <v>139</v>
-      </c>
-      <c r="B21" s="36">
-        <v>-324.96499999999997</v>
-      </c>
-      <c r="C21" s="37">
-        <v>0</v>
-      </c>
-      <c r="D21" s="37">
+      <c r="D21" s="36">
         <v>533.79200000000003</v>
       </c>
     </row>
@@ -5285,268 +5285,268 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="30" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="C1" s="30" t="s">
         <v>117</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="D1" s="30" t="s">
         <v>118</v>
       </c>
-      <c r="D1" s="31" t="s">
+    </row>
+    <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="31" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="32" t="s">
+      <c r="B2" s="32">
+        <v>-1390</v>
+      </c>
+      <c r="C2" s="33">
+        <v>305</v>
+      </c>
+      <c r="D2" s="33">
+        <v>126.35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="34" t="s">
         <v>120</v>
       </c>
-      <c r="B2" s="33">
+      <c r="B3" s="35">
+        <v>-1830</v>
+      </c>
+      <c r="C3" s="36">
+        <v>270</v>
+      </c>
+      <c r="D3" s="36">
+        <v>126.35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="34" t="s">
+        <v>121</v>
+      </c>
+      <c r="B4" s="35">
+        <v>-1579.2370000000001</v>
+      </c>
+      <c r="C4" s="36">
+        <v>573.947</v>
+      </c>
+      <c r="D4" s="36">
+        <v>163.18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" s="35">
         <v>-1390</v>
       </c>
-      <c r="C2" s="34">
+      <c r="C5" s="36">
         <v>305</v>
       </c>
-      <c r="D2" s="34">
-        <v>126.35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="35" t="s">
-        <v>121</v>
-      </c>
-      <c r="B3" s="36">
+      <c r="D5" s="36">
+        <v>328.98099999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="34" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" s="35">
         <v>-1830</v>
       </c>
-      <c r="C3" s="37">
+      <c r="C6" s="36">
         <v>270</v>
       </c>
-      <c r="D3" s="37">
-        <v>126.35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="35" t="s">
-        <v>122</v>
-      </c>
-      <c r="B4" s="36">
-        <v>-1579.2370000000001</v>
-      </c>
-      <c r="C4" s="37">
-        <v>573.947</v>
-      </c>
-      <c r="D4" s="37">
-        <v>163.18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="35" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="36">
-        <v>-1390</v>
-      </c>
-      <c r="C5" s="37">
+      <c r="D6" s="36">
+        <v>354.47500000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="34" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" s="35">
+        <v>-1569.845</v>
+      </c>
+      <c r="C7" s="36">
+        <v>506.33</v>
+      </c>
+      <c r="D7" s="36">
+        <v>408.15100000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="B8" s="35">
+        <v>-1568.8710000000001</v>
+      </c>
+      <c r="C8" s="36">
+        <v>566.64200000000005</v>
+      </c>
+      <c r="D8" s="36">
+        <v>294.82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="34" t="s">
+        <v>126</v>
+      </c>
+      <c r="B9" s="35">
+        <v>-1574.5989999999999</v>
+      </c>
+      <c r="C9" s="36">
+        <v>623.53200000000004</v>
+      </c>
+      <c r="D9" s="36">
+        <v>286.04000000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="34" t="s">
+        <v>127</v>
+      </c>
+      <c r="B10" s="35">
+        <v>-1830</v>
+      </c>
+      <c r="C10" s="36">
+        <v>270</v>
+      </c>
+      <c r="D10" s="36">
+        <v>193.642</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="B11" s="35">
+        <v>-1675.904</v>
+      </c>
+      <c r="C11" s="36">
+        <v>576.73500000000001</v>
+      </c>
+      <c r="D11" s="36">
+        <v>251.011</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="34" t="s">
+        <v>129</v>
+      </c>
+      <c r="B12" s="35">
+        <v>-1395.9760000000001</v>
+      </c>
+      <c r="C12" s="36">
+        <v>283.399</v>
+      </c>
+      <c r="D12" s="36">
+        <v>436.10300000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="34" t="s">
+        <v>130</v>
+      </c>
+      <c r="B13" s="35">
+        <v>-1579.1110000000001</v>
+      </c>
+      <c r="C13" s="36">
+        <v>267.07299999999998</v>
+      </c>
+      <c r="D13" s="36">
+        <v>484.01</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="34" t="s">
+        <v>131</v>
+      </c>
+      <c r="B14" s="35">
+        <v>-1597.194</v>
+      </c>
+      <c r="C14" s="36">
+        <v>526.39499999999998</v>
+      </c>
+      <c r="D14" s="36">
+        <v>180.96700000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="34" t="s">
+        <v>132</v>
+      </c>
+      <c r="B15" s="35">
+        <v>-1664.6120000000001</v>
+      </c>
+      <c r="C15" s="36">
+        <v>349.04700000000003</v>
+      </c>
+      <c r="D15" s="36">
+        <v>403.92399999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="34" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" s="35">
+        <v>-1585.771</v>
+      </c>
+      <c r="C16" s="36">
+        <v>318.42700000000002</v>
+      </c>
+      <c r="D16" s="36">
+        <v>426.35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="34" t="s">
+        <v>134</v>
+      </c>
+      <c r="B17" s="35">
+        <v>-1830</v>
+      </c>
+      <c r="C17" s="36">
         <v>305</v>
       </c>
-      <c r="D5" s="37">
-        <v>328.98099999999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="35" t="s">
-        <v>124</v>
-      </c>
-      <c r="B6" s="36">
+      <c r="D17" s="36">
+        <v>401.35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="34" t="s">
+        <v>135</v>
+      </c>
+      <c r="B18" s="35">
         <v>-1830</v>
       </c>
-      <c r="C6" s="37">
-        <v>270</v>
-      </c>
-      <c r="D6" s="37">
-        <v>354.47500000000002</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="35" t="s">
-        <v>125</v>
-      </c>
-      <c r="B7" s="36">
-        <v>-1569.845</v>
-      </c>
-      <c r="C7" s="37">
-        <v>506.33</v>
-      </c>
-      <c r="D7" s="37">
-        <v>408.15100000000001</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="35" t="s">
-        <v>126</v>
-      </c>
-      <c r="B8" s="36">
-        <v>-1568.8710000000001</v>
-      </c>
-      <c r="C8" s="37">
-        <v>566.64200000000005</v>
-      </c>
-      <c r="D8" s="37">
-        <v>294.82</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="35" t="s">
-        <v>127</v>
-      </c>
-      <c r="B9" s="36">
-        <v>-1574.5989999999999</v>
-      </c>
-      <c r="C9" s="37">
-        <v>623.53200000000004</v>
-      </c>
-      <c r="D9" s="37">
-        <v>286.04000000000002</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="35" t="s">
-        <v>128</v>
-      </c>
-      <c r="B10" s="36">
-        <v>-1830</v>
-      </c>
-      <c r="C10" s="37">
-        <v>270</v>
-      </c>
-      <c r="D10" s="37">
-        <v>193.642</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="35" t="s">
-        <v>129</v>
-      </c>
-      <c r="B11" s="36">
-        <v>-1675.904</v>
-      </c>
-      <c r="C11" s="37">
-        <v>576.73500000000001</v>
-      </c>
-      <c r="D11" s="37">
-        <v>251.011</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="35" t="s">
-        <v>130</v>
-      </c>
-      <c r="B12" s="36">
-        <v>-1395.9760000000001</v>
-      </c>
-      <c r="C12" s="37">
-        <v>283.399</v>
-      </c>
-      <c r="D12" s="37">
-        <v>436.10300000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="35" t="s">
-        <v>131</v>
-      </c>
-      <c r="B13" s="36">
-        <v>-1579.1110000000001</v>
-      </c>
-      <c r="C13" s="37">
-        <v>267.07299999999998</v>
-      </c>
-      <c r="D13" s="37">
-        <v>484.01</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="35" t="s">
-        <v>132</v>
-      </c>
-      <c r="B14" s="36">
-        <v>-1597.194</v>
-      </c>
-      <c r="C14" s="37">
-        <v>526.39499999999998</v>
-      </c>
-      <c r="D14" s="37">
-        <v>180.96700000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="35" t="s">
-        <v>133</v>
-      </c>
-      <c r="B15" s="36">
-        <v>-1664.6120000000001</v>
-      </c>
-      <c r="C15" s="37">
-        <v>349.04700000000003</v>
-      </c>
-      <c r="D15" s="37">
-        <v>403.92399999999998</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="35" t="s">
-        <v>134</v>
-      </c>
-      <c r="B16" s="36">
-        <v>-1585.771</v>
-      </c>
-      <c r="C16" s="37">
-        <v>318.42700000000002</v>
-      </c>
-      <c r="D16" s="37">
-        <v>426.35</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="35" t="s">
-        <v>135</v>
-      </c>
-      <c r="B17" s="36">
-        <v>-1830</v>
-      </c>
-      <c r="C17" s="37">
+      <c r="C18" s="36">
         <v>305</v>
       </c>
-      <c r="D17" s="37">
-        <v>401.35</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="35" t="s">
+      <c r="D18" s="36">
+        <v>448.35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="34" t="s">
         <v>136</v>
       </c>
-      <c r="B18" s="36">
-        <v>-1830</v>
-      </c>
-      <c r="C18" s="37">
-        <v>305</v>
-      </c>
-      <c r="D18" s="37">
-        <v>448.35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="35" t="s">
-        <v>137</v>
-      </c>
-      <c r="B19" s="36">
+      <c r="B19" s="35">
         <v>-1600.4860000000001</v>
       </c>
-      <c r="C19" s="37">
+      <c r="C19" s="36">
         <v>287.56599999999997</v>
       </c>
-      <c r="D19" s="37">
+      <c r="D19" s="36">
         <v>463.988</v>
       </c>
     </row>
@@ -5623,24 +5623,24 @@
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="114"/>
-      <c r="C5" s="116" t="s">
-        <v>140</v>
-      </c>
-      <c r="D5" s="117" t="s">
+      <c r="B5" s="113"/>
+      <c r="C5" s="115" t="s">
+        <v>139</v>
+      </c>
+      <c r="D5" s="116" t="s">
         <v>64</v>
       </c>
-      <c r="E5" s="115"/>
+      <c r="E5" s="114"/>
     </row>
     <row r="6" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="78"/>
-      <c r="C6" s="85" t="s">
+      <c r="B6" s="77"/>
+      <c r="C6" s="84" t="s">
         <v>63</v>
       </c>
-      <c r="D6" s="87" t="s">
+      <c r="D6" s="86" t="s">
         <v>64</v>
       </c>
       <c r="E6" s="22"/>
@@ -5649,11 +5649,11 @@
       <c r="A7" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B7" s="78"/>
-      <c r="C7" s="85" t="s">
+      <c r="B7" s="77"/>
+      <c r="C7" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="D7" s="87" t="s">
+      <c r="D7" s="86" t="s">
         <v>64</v>
       </c>
       <c r="E7" s="22"/>
@@ -5700,7 +5700,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="102" t="s">
+      <c r="C2" s="101" t="s">
         <v>35</v>
       </c>
       <c r="D2" s="9"/>
@@ -5711,7 +5711,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="102" t="s">
+      <c r="C3" s="101" t="s">
         <v>36</v>
       </c>
       <c r="D3" s="9"/>
@@ -5722,17 +5722,17 @@
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="102" t="s">
+      <c r="C4" s="101" t="s">
         <v>37</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="144" t="s">
+      <c r="A5" s="141" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="74" t="s">
+      <c r="B5" s="73" t="s">
         <v>39</v>
       </c>
       <c r="C5" s="23" t="str">
@@ -5747,8 +5747,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="142"/>
-      <c r="B6" s="75" t="s">
+      <c r="A6" s="139"/>
+      <c r="B6" s="74" t="s">
         <v>41</v>
       </c>
       <c r="C6" s="24" t="str" cm="1">
@@ -5763,8 +5763,8 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="145"/>
-      <c r="B7" s="75" t="s">
+      <c r="A7" s="142"/>
+      <c r="B7" s="74" t="s">
         <v>42</v>
       </c>
       <c r="C7" s="24" t="str" cm="1">
@@ -5779,8 +5779,8 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="145"/>
-      <c r="B8" s="78" t="s">
+      <c r="A8" s="142"/>
+      <c r="B8" s="77" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="20">
@@ -5792,10 +5792,10 @@
       <c r="E8" s="22"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="146" t="s">
+      <c r="A9" s="143" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="74" t="s">
+      <c r="B9" s="73" t="s">
         <v>39</v>
       </c>
       <c r="C9" s="23" t="str" cm="1">
@@ -5810,8 +5810,8 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="143"/>
-      <c r="B10" s="75" t="s">
+      <c r="A10" s="140"/>
+      <c r="B10" s="74" t="s">
         <v>41</v>
       </c>
       <c r="C10" s="24" t="str" cm="1">
@@ -5826,8 +5826,8 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="143"/>
-      <c r="B11" s="75" t="s">
+      <c r="A11" s="140"/>
+      <c r="B11" s="74" t="s">
         <v>42</v>
       </c>
       <c r="C11" s="24" t="str" cm="1">
@@ -5842,8 +5842,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="142"/>
-      <c r="B12" s="78" t="s">
+      <c r="A12" s="139"/>
+      <c r="B12" s="77" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="20">
@@ -5857,10 +5857,10 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="147" t="s">
+      <c r="A13" s="144" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="74" t="s">
+      <c r="B13" s="73" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="23" t="str" cm="1">
@@ -5875,9 +5875,9 @@
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="145"/>
-      <c r="B14" s="75" t="s">
-        <v>149</v>
+      <c r="A14" s="142"/>
+      <c r="B14" s="74" t="s">
+        <v>148</v>
       </c>
       <c r="C14" s="24" t="str" cm="1">
         <f t="array" ref="C14">"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B9/1000,HardpointsFr!C9/1000,HardpointsFr!D9/1000)&amp;"]"</f>
@@ -5891,8 +5891,8 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="145"/>
-      <c r="B15" s="75" t="s">
+      <c r="A15" s="142"/>
+      <c r="B15" s="74" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="25">
@@ -5904,12 +5904,12 @@
       <c r="E15" s="18"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="148"/>
-      <c r="B16" s="75" t="s">
+      <c r="A16" s="145"/>
+      <c r="B16" s="74" t="s">
         <v>45</v>
       </c>
       <c r="C16" s="25">
-        <v>-0.5</v>
+        <v>-0.3</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>46</v>
@@ -5917,12 +5917,12 @@
       <c r="E16" s="16"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="143"/>
-      <c r="B17" s="75" t="s">
+      <c r="A17" s="140"/>
+      <c r="B17" s="74" t="s">
         <v>47</v>
       </c>
       <c r="C17" s="25">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>46</v>
@@ -5930,11 +5930,11 @@
       <c r="E17" s="16"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="143"/>
-      <c r="B18" s="75" t="s">
+      <c r="A18" s="140"/>
+      <c r="B18" s="74" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="112">
+      <c r="C18" s="111">
         <v>0.11</v>
       </c>
       <c r="D18" s="15" t="s">
@@ -5943,11 +5943,11 @@
       <c r="E18" s="16"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="143"/>
-      <c r="B19" s="75" t="s">
+      <c r="A19" s="140"/>
+      <c r="B19" s="74" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="112">
+      <c r="C19" s="111">
         <v>0.03</v>
       </c>
       <c r="D19" s="15" t="s">
@@ -5956,11 +5956,11 @@
       <c r="E19" s="16"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="142"/>
-      <c r="B20" s="78" t="s">
+      <c r="A20" s="139"/>
+      <c r="B20" s="77" t="s">
         <v>50</v>
       </c>
-      <c r="C20" s="113">
+      <c r="C20" s="112">
         <v>1.5</v>
       </c>
       <c r="D20" s="21" t="s">
@@ -5969,10 +5969,10 @@
       <c r="E20" s="22"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="141" t="s">
-        <v>143</v>
-      </c>
-      <c r="B21" s="74" t="s">
+      <c r="A21" s="138" t="s">
+        <v>142</v>
+      </c>
+      <c r="B21" s="73" t="s">
         <v>51</v>
       </c>
       <c r="C21" s="23" t="str" cm="1">
@@ -5987,7 +5987,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="143"/>
+      <c r="A22" s="140"/>
       <c r="B22" s="14" t="s">
         <v>42</v>
       </c>
@@ -6003,7 +6003,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="142"/>
+      <c r="A23" s="139"/>
       <c r="B23" s="19" t="s">
         <v>12</v>
       </c>
@@ -6016,10 +6016,10 @@
       <c r="E23" s="22"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="141" t="s">
+      <c r="A24" s="138" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="74" t="s">
+      <c r="B24" s="73" t="s">
         <v>53</v>
       </c>
       <c r="C24" s="23" t="str" cm="1">
@@ -6034,8 +6034,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="143"/>
-      <c r="B25" s="75" t="s">
+      <c r="A25" s="140"/>
+      <c r="B25" s="74" t="s">
         <v>54</v>
       </c>
       <c r="C25" s="24" t="str" cm="1">
@@ -6050,22 +6050,22 @@
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="149"/>
-      <c r="B26" s="79" t="s">
-        <v>147</v>
-      </c>
-      <c r="C26" s="125">
+      <c r="A26" s="146"/>
+      <c r="B26" s="78" t="s">
+        <v>146</v>
+      </c>
+      <c r="C26" s="124">
         <v>1.2</v>
       </c>
-      <c r="D26" s="126" t="s">
+      <c r="D26" s="125" t="s">
         <v>29</v>
       </c>
-      <c r="E26" s="82"/>
+      <c r="E26" s="81"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="142"/>
-      <c r="B27" s="78" t="s">
-        <v>146</v>
+      <c r="A27" s="139"/>
+      <c r="B27" s="77" t="s">
+        <v>145</v>
       </c>
       <c r="C27" s="20">
         <v>0.8</v>
@@ -6076,10 +6076,10 @@
       <c r="E27" s="22"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="141" t="s">
+      <c r="A28" s="138" t="s">
         <v>55</v>
       </c>
-      <c r="B28" s="74" t="s">
+      <c r="B28" s="73" t="s">
         <v>56</v>
       </c>
       <c r="C28" s="27">
@@ -6091,8 +6091,8 @@
       <c r="E28" s="13"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="142"/>
-      <c r="B29" s="78" t="s">
+      <c r="A29" s="139"/>
+      <c r="B29" s="77" t="s">
         <v>57</v>
       </c>
       <c r="C29" s="20">
@@ -6104,10 +6104,10 @@
       <c r="E29" s="22"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="141" t="s">
+      <c r="A30" s="138" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="88" t="s">
+      <c r="B30" s="87" t="s">
         <v>51</v>
       </c>
       <c r="C30" s="23" t="str" cm="1">
@@ -6122,8 +6122,8 @@
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="143"/>
-      <c r="B31" s="89" t="s">
+      <c r="A31" s="140"/>
+      <c r="B31" s="88" t="s">
         <v>42</v>
       </c>
       <c r="C31" s="24" t="str" cm="1">
@@ -6138,8 +6138,8 @@
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="142"/>
-      <c r="B32" s="90" t="s">
+      <c r="A32" s="139"/>
+      <c r="B32" s="89" t="s">
         <v>12</v>
       </c>
       <c r="C32" s="20">
@@ -6151,7 +6151,7 @@
       <c r="E32" s="22"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="141" t="s">
+      <c r="A33" s="138" t="s">
         <v>59</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -6169,7 +6169,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="143"/>
+      <c r="A34" s="140"/>
       <c r="B34" s="14" t="s">
         <v>61</v>
       </c>
@@ -6185,7 +6185,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="142"/>
+      <c r="A35" s="139"/>
       <c r="B35" s="19" t="s">
         <v>12</v>
       </c>
@@ -6278,10 +6278,10 @@
       <c r="E5" s="10"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="122" t="s">
+      <c r="A6" s="121" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="74"/>
+      <c r="B6" s="73"/>
       <c r="C6" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B19/1000,HardpointsFr!C19/1000,HardpointsFr!D19/1000)&amp;"]"</f>
         <v>[0.011527 0.292246 0.342816]</v>
@@ -6294,10 +6294,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="123" t="s">
+      <c r="A7" s="122" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="75"/>
+      <c r="B7" s="74"/>
       <c r="C7" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B17/1000,HardpointsFr!C17/1000,HardpointsFr!D17/1000)&amp;"]"</f>
         <v>[0.020965 0.262855 0.10135]</v>
@@ -6310,10 +6310,10 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="123" t="s">
+      <c r="A8" s="122" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="75"/>
+      <c r="B8" s="74"/>
       <c r="C8" s="24" t="str" cm="1">
         <f t="array" ref="C8">"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B18/1000,HardpointsFr!C18/1000,HardpointsFr!D18/1000)&amp;"]"</f>
         <v>[-0.0235 0.262855 0.101519]</v>
@@ -6326,25 +6326,25 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="123" t="s">
+      <c r="A9" s="122" t="s">
         <v>69</v>
       </c>
-      <c r="B9" s="75"/>
-      <c r="C9" s="134">
+      <c r="B9" s="74"/>
+      <c r="C9" s="133">
         <f>2.2813*2</f>
         <v>4.5625999999999998</v>
       </c>
-      <c r="D9" s="86" t="s">
-        <v>158</v>
+      <c r="D9" s="85" t="s">
+        <v>157</v>
       </c>
       <c r="E9" s="16"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="124" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="78"/>
-      <c r="C10" s="135">
+      <c r="A10" s="123" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="77"/>
+      <c r="C10" s="134">
         <v>0.7</v>
       </c>
       <c r="D10" s="21" t="s">
@@ -6426,13 +6426,13 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="138" t="s">
+      <c r="A5" s="147" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="74" t="s">
+      <c r="B5" s="73" t="s">
         <v>73</v>
       </c>
-      <c r="C5" s="41" t="str">
+      <c r="C5" s="40" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B20/1000,HardpointsFr!C20/1000,HardpointsFr!D20/1000)&amp;"]"</f>
         <v>[0.104241 0 0.171053]</v>
       </c>
@@ -6444,24 +6444,24 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="139"/>
-      <c r="B6" s="93" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="39">
+      <c r="A6" s="148"/>
+      <c r="B6" s="92" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="38">
         <v>0.87</v>
       </c>
-      <c r="D6" s="40" t="s">
+      <c r="D6" s="39" t="s">
         <v>29</v>
       </c>
       <c r="E6" s="18"/>
     </row>
     <row r="7" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="150"/>
-      <c r="B7" s="75" t="s">
+      <c r="A7" s="149"/>
+      <c r="B7" s="74" t="s">
         <v>74</v>
       </c>
-      <c r="C7" s="38">
+      <c r="C7" s="37">
         <v>50</v>
       </c>
       <c r="D7" s="15" t="s">
@@ -6470,26 +6470,26 @@
       <c r="E7" s="15"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="151" t="s">
+      <c r="A8" s="150" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="75" t="s">
+      <c r="B8" s="74" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="24">
         <v>0.5</v>
       </c>
-      <c r="D8" s="86" t="s">
+      <c r="D8" s="85" t="s">
         <v>29</v>
       </c>
       <c r="E8" s="16"/>
     </row>
     <row r="9" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="152"/>
-      <c r="B9" s="75" t="s">
+      <c r="A9" s="151"/>
+      <c r="B9" s="74" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="38" t="str">
+      <c r="C9" s="37" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B21/1000,HardpointsFr!C21/1000,HardpointsFr!D21/1000)&amp;"]"</f>
         <v>[-0.324965 0 0.533792]</v>
       </c>
@@ -6553,7 +6553,7 @@
         <v>35</v>
       </c>
       <c r="D2" s="9"/>
-      <c r="E2" s="53"/>
+      <c r="E2" s="52"/>
     </row>
     <row r="3" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -6564,68 +6564,68 @@
         <v>36</v>
       </c>
       <c r="D3" s="9"/>
-      <c r="E3" s="53"/>
+      <c r="E3" s="52"/>
     </row>
     <row r="4" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="102" t="s">
+      <c r="C4" s="101" t="s">
         <v>35</v>
       </c>
       <c r="D4" s="9"/>
-      <c r="E4" s="53"/>
+      <c r="E4" s="52"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="114"/>
-      <c r="C5" s="116" t="s">
-        <v>142</v>
-      </c>
-      <c r="D5" s="117" t="s">
+      <c r="B5" s="113"/>
+      <c r="C5" s="115" t="s">
+        <v>141</v>
+      </c>
+      <c r="D5" s="116" t="s">
         <v>64</v>
       </c>
-      <c r="E5" s="118"/>
+      <c r="E5" s="117"/>
     </row>
     <row r="6" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="78"/>
-      <c r="C6" s="85" t="s">
+      <c r="B6" s="77"/>
+      <c r="C6" s="84" t="s">
         <v>77</v>
       </c>
-      <c r="D6" s="87" t="s">
+      <c r="D6" s="86" t="s">
         <v>64</v>
       </c>
       <c r="E6" s="22"/>
     </row>
     <row r="7" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="153" t="s">
+      <c r="A7" s="152" t="s">
         <v>65</v>
       </c>
-      <c r="B7" s="127" t="s">
+      <c r="B7" s="126" t="s">
+        <v>154</v>
+      </c>
+      <c r="C7" s="127" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7" s="116"/>
+      <c r="E7" s="128"/>
+    </row>
+    <row r="8" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="153"/>
+      <c r="B8" s="126" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="115" t="s">
         <v>155</v>
       </c>
-      <c r="C7" s="128" t="s">
-        <v>65</v>
-      </c>
-      <c r="D7" s="117"/>
-      <c r="E7" s="129"/>
-    </row>
-    <row r="8" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="154"/>
-      <c r="B8" s="127" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="116" t="s">
-        <v>156</v>
-      </c>
-      <c r="D8" s="117"/>
-      <c r="E8" s="118"/>
+      <c r="D8" s="116"/>
+      <c r="E8" s="117"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6673,7 +6673,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="7"/>
-      <c r="C2" s="102" t="s">
+      <c r="C2" s="101" t="s">
         <v>35</v>
       </c>
       <c r="D2" s="9"/>
@@ -6684,7 +6684,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="102" t="s">
+      <c r="C3" s="101" t="s">
         <v>36</v>
       </c>
       <c r="D3" s="9"/>
@@ -6695,17 +6695,17 @@
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="102" t="s">
-        <v>141</v>
+      <c r="C4" s="101" t="s">
+        <v>140</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="153" t="s">
+      <c r="A5" s="152" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="74" t="s">
+      <c r="B5" s="73" t="s">
         <v>39</v>
       </c>
       <c r="C5" s="23" t="str">
@@ -6715,125 +6715,125 @@
       <c r="D5" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="54" t="s">
+      <c r="E5" s="53" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="158"/>
-      <c r="B6" s="75" t="s">
+      <c r="B6" s="74" t="s">
         <v>41</v>
       </c>
       <c r="C6" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B3/1000 +1.575,HardpointsRr!C3/1000,HardpointsRr!D3/1000)&amp;"]"</f>
         <v>[-0.255 0.27 0.12635]</v>
       </c>
-      <c r="D6" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="55" t="s">
+      <c r="D6" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="54" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="158"/>
-      <c r="B7" s="75" t="s">
+      <c r="B7" s="74" t="s">
         <v>42</v>
       </c>
       <c r="C7" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B4/1000 +1.575,HardpointsRr!C4/1000,HardpointsRr!D4/1000)&amp;"]"</f>
         <v>[-0.00423700000000005 0.573947 0.16318]</v>
       </c>
-      <c r="D7" s="46" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="56" t="s">
+      <c r="D7" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="55" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="154"/>
-      <c r="B8" s="78" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="48">
+      <c r="A8" s="153"/>
+      <c r="B8" s="77" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="47">
         <v>0.16500000000000001</v>
       </c>
-      <c r="D8" s="47" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="57"/>
+      <c r="D8" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="56"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="159" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="74" t="s">
+      <c r="B9" s="73" t="s">
         <v>39</v>
       </c>
       <c r="C9" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B5/1000 +1.575,HardpointsRr!C5/1000,HardpointsRr!D5/1000)&amp;"]"</f>
         <v>[0.185 0.305 0.328981]</v>
       </c>
-      <c r="D9" s="49" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="58" t="s">
+      <c r="D9" s="48" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="57" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="160"/>
-      <c r="B10" s="75" t="s">
+      <c r="B10" s="74" t="s">
         <v>41</v>
       </c>
       <c r="C10" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B6/1000 +1.575,HardpointsRr!C6/1000,HardpointsRr!D6/1000)&amp;"]"</f>
         <v>[-0.255 0.27 0.354475]</v>
       </c>
-      <c r="D10" s="52" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="59" t="s">
+      <c r="D10" s="51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="58" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="160"/>
-      <c r="B11" s="75" t="s">
+      <c r="B11" s="74" t="s">
         <v>42</v>
       </c>
       <c r="C11" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B7/1000 +1.575,HardpointsRr!C7/1000,HardpointsRr!D7/1000)&amp;"]"</f>
         <v>[0.00515500000000002 0.50633 0.408151]</v>
       </c>
-      <c r="D11" s="50" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="60" t="s">
+      <c r="D11" s="49" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="59" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="161"/>
-      <c r="B12" s="78" t="s">
+      <c r="B12" s="77" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="20">
         <v>0.12</v>
       </c>
-      <c r="D12" s="51" t="s">
+      <c r="D12" s="50" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="61" t="s">
+      <c r="E12" s="60" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="138" t="s">
+      <c r="A13" s="147" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="74" t="s">
+      <c r="B13" s="73" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="23" t="str">
@@ -6843,124 +6843,124 @@
       <c r="D13" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="54" t="s">
+      <c r="E13" s="53" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="139"/>
-      <c r="B14" s="75" t="s">
-        <v>149</v>
+      <c r="A14" s="148"/>
+      <c r="B14" s="74" t="s">
+        <v>148</v>
       </c>
       <c r="C14" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B9/1000 +1.575,HardpointsRr!C9/1000,HardpointsRr!D9/1000)&amp;"]"</f>
         <v>[0.000401000000000096 0.623532 0.28604]</v>
       </c>
-      <c r="D14" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="62" t="s">
+      <c r="D14" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="61" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="139"/>
-      <c r="B15" s="75" t="s">
+      <c r="A15" s="148"/>
+      <c r="B15" s="74" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="25">
         <v>1</v>
       </c>
-      <c r="D15" s="42" t="s">
+      <c r="D15" s="41" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="63"/>
+      <c r="E15" s="62"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="139"/>
-      <c r="B16" s="75" t="s">
+      <c r="A16" s="148"/>
+      <c r="B16" s="74" t="s">
         <v>45</v>
       </c>
       <c r="C16" s="25">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="61"/>
+      <c r="E16" s="60"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="139"/>
-      <c r="B17" s="75" t="s">
+      <c r="A17" s="148"/>
+      <c r="B17" s="74" t="s">
         <v>47</v>
       </c>
       <c r="C17" s="25">
-        <v>-1</v>
+        <v>-0.4</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="64"/>
+      <c r="E17" s="63"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="139"/>
-      <c r="B18" s="75" t="s">
+      <c r="A18" s="148"/>
+      <c r="B18" s="74" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="112">
+      <c r="C18" s="111">
         <v>0.11</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="64"/>
+      <c r="E18" s="63"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="139"/>
-      <c r="B19" s="75" t="s">
+      <c r="A19" s="148"/>
+      <c r="B19" s="74" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="112">
+      <c r="C19" s="111">
         <v>0.03</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="64"/>
+      <c r="E19" s="63"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="140"/>
-      <c r="B20" s="78" t="s">
+      <c r="A20" s="157"/>
+      <c r="B20" s="77" t="s">
         <v>50</v>
       </c>
-      <c r="C20" s="113">
+      <c r="C20" s="112">
         <v>1.5</v>
       </c>
       <c r="D20" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="65"/>
+      <c r="E20" s="64"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="138" t="s">
-        <v>143</v>
-      </c>
-      <c r="B21" s="74" t="s">
+      <c r="A21" s="147" t="s">
+        <v>142</v>
+      </c>
+      <c r="B21" s="73" t="s">
         <v>51</v>
       </c>
       <c r="C21" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B10/1000 +1.575,HardpointsRr!C10/1000,HardpointsRr!D10/1000)&amp;"]"</f>
         <v>[-0.255 0.27 0.193642]</v>
       </c>
-      <c r="D21" s="43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" s="66" t="s">
+      <c r="D21" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="65" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="139"/>
+      <c r="A22" s="148"/>
       <c r="B22" s="14" t="s">
         <v>42</v>
       </c>
@@ -6968,15 +6968,15 @@
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B11/1000 +1.575,HardpointsRr!C11/1000,HardpointsRr!D11/1000)&amp;"]"</f>
         <v>[-0.100904 0.576735 0.251011]</v>
       </c>
-      <c r="D22" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="E22" s="59" t="s">
+      <c r="D22" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" s="58" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="140"/>
+      <c r="A23" s="157"/>
       <c r="B23" s="19" t="s">
         <v>12</v>
       </c>
@@ -6986,29 +6986,29 @@
       <c r="D23" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E23" s="67"/>
+      <c r="E23" s="66"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="138" t="s">
+      <c r="A24" s="147" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="74" t="s">
+      <c r="B24" s="73" t="s">
         <v>53</v>
       </c>
       <c r="C24" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B12/1000 + 1.575,HardpointsRr!C12/1000,HardpointsRr!D12/1000)&amp;"]"</f>
         <v>[0.179024 0.283399 0.436103]</v>
       </c>
-      <c r="D24" s="43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E24" s="60" t="s">
+      <c r="D24" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="59" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="139"/>
-      <c r="B25" s="75" t="s">
+      <c r="A25" s="148"/>
+      <c r="B25" s="74" t="s">
         <v>54</v>
       </c>
       <c r="C25" s="23" t="str">
@@ -7018,25 +7018,25 @@
       <c r="D25" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E25" s="61" t="s">
+      <c r="E25" s="60" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="139"/>
-      <c r="B26" s="79" t="s">
+      <c r="A26" s="148"/>
+      <c r="B26" s="78" t="s">
+        <v>145</v>
+      </c>
+      <c r="C26" s="124">
+        <v>0.8</v>
+      </c>
+      <c r="D26" s="79"/>
+      <c r="E26" s="71"/>
+    </row>
+    <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="157"/>
+      <c r="B27" s="77" t="s">
         <v>146</v>
-      </c>
-      <c r="C26" s="125">
-        <v>0.8</v>
-      </c>
-      <c r="D26" s="80"/>
-      <c r="E26" s="72"/>
-    </row>
-    <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="140"/>
-      <c r="B27" s="78" t="s">
-        <v>147</v>
       </c>
       <c r="C27" s="20">
         <v>1.2</v>
@@ -7044,13 +7044,13 @@
       <c r="D27" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E27" s="68"/>
+      <c r="E27" s="67"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="138" t="s">
+      <c r="A28" s="147" t="s">
         <v>55</v>
       </c>
-      <c r="B28" s="74" t="s">
+      <c r="B28" s="73" t="s">
         <v>56</v>
       </c>
       <c r="C28" s="27">
@@ -7059,11 +7059,11 @@
       <c r="D28" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E28" s="69"/>
+      <c r="E28" s="68"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="140"/>
-      <c r="B29" s="78" t="s">
+      <c r="A29" s="157"/>
+      <c r="B29" s="77" t="s">
         <v>57</v>
       </c>
       <c r="C29" s="20">
@@ -7072,13 +7072,13 @@
       <c r="D29" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="E29" s="68"/>
+      <c r="E29" s="67"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="155" t="s">
+      <c r="A30" s="154" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="88" t="s">
+      <c r="B30" s="87" t="s">
         <v>42</v>
       </c>
       <c r="C30" s="23" t="str">
@@ -7088,29 +7088,29 @@
       <c r="D30" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E30" s="54" t="s">
+      <c r="E30" s="53" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="156"/>
-      <c r="B31" s="89" t="s">
+      <c r="A31" s="155"/>
+      <c r="B31" s="88" t="s">
         <v>51</v>
       </c>
       <c r="C31" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B15/1000 + 1.575,HardpointsRr!C15/1000,HardpointsRr!D15/1000)&amp;"]"</f>
         <v>[-0.089612 0.349047 0.403924]</v>
       </c>
-      <c r="D31" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="E31" s="59" t="s">
+      <c r="D31" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" s="58" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="157"/>
-      <c r="B32" s="90" t="s">
+      <c r="A32" s="156"/>
+      <c r="B32" s="89" t="s">
         <v>12</v>
       </c>
       <c r="C32" s="20">
@@ -7119,10 +7119,10 @@
       <c r="D32" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E32" s="70"/>
+      <c r="E32" s="69"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="138" t="s">
+      <c r="A33" s="147" t="s">
         <v>59</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -7135,12 +7135,12 @@
       <c r="D33" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E33" s="54" t="s">
+      <c r="E33" s="53" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="139"/>
+      <c r="A34" s="148"/>
       <c r="B34" s="14" t="s">
         <v>61</v>
       </c>
@@ -7148,15 +7148,15 @@
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B19/1000+ 1.575,HardpointsRr!C19/1000,HardpointsRr!D19/1000)&amp;"]"</f>
         <v>[-0.0254860000000001 0.287566 0.463988]</v>
       </c>
-      <c r="D34" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="E34" s="59" t="s">
+      <c r="D34" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" s="58" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="140"/>
+      <c r="A35" s="157"/>
       <c r="B35" s="19" t="s">
         <v>12</v>
       </c>
@@ -7166,7 +7166,7 @@
       <c r="D35" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="E35" s="70"/>
+      <c r="E35" s="69"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -7241,86 +7241,86 @@
         <v>8</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="102" t="s">
-        <v>150</v>
+      <c r="C4" s="101" t="s">
+        <v>149</v>
       </c>
       <c r="D4" s="9"/>
-      <c r="E4" s="71"/>
+      <c r="E4" s="70"/>
     </row>
     <row r="5" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="122" t="s">
+      <c r="A5" s="121" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="74"/>
+      <c r="B5" s="73"/>
       <c r="C5" s="23" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B19/1000+ 1.575,HardpointsRr!C19/1000,HardpointsRr!D19/1000)&amp;"]"</f>
         <v>[-0.0254860000000001 0.287566 0.463988]</v>
       </c>
-      <c r="D5" s="130" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="66" t="s">
+      <c r="D5" s="129" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="65" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="123" t="s">
+      <c r="A6" s="122" t="s">
         <v>51</v>
       </c>
-      <c r="B6" s="75"/>
+      <c r="B6" s="74"/>
       <c r="C6" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B17/1000+ 1.575,HardpointsRr!C17/1000,HardpointsRr!D17/1000)&amp;"]"</f>
         <v>[-0.255 0.305 0.40135]</v>
       </c>
-      <c r="D6" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="55" t="s">
+      <c r="D6" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="54" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="123" t="s">
+      <c r="A7" s="122" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="75"/>
+      <c r="B7" s="74"/>
       <c r="C7" s="24" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsRr!B18/1000 + 1.575,HardpointsRr!C18/1000,HardpointsRr!D18/1000)&amp;"]"</f>
         <v>[-0.255 0.305 0.44835]</v>
       </c>
-      <c r="D7" s="42" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="59" t="s">
+      <c r="D7" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="58" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="123" t="s">
+      <c r="A8" s="122" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="75"/>
-      <c r="C8" s="137">
+      <c r="B8" s="74"/>
+      <c r="C8" s="136">
         <f>1.979*2</f>
         <v>3.9580000000000002</v>
       </c>
-      <c r="D8" s="86" t="s">
-        <v>158</v>
-      </c>
-      <c r="E8" s="72"/>
+      <c r="D8" s="85" t="s">
+        <v>157</v>
+      </c>
+      <c r="E8" s="71"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="124" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="78"/>
+      <c r="A9" s="123" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="77"/>
       <c r="C9" s="20">
         <v>0.7</v>
       </c>
-      <c r="D9" s="44" t="s">
+      <c r="D9" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="73"/>
+      <c r="E9" s="72"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7394,10 +7394,10 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="120" t="s">
+      <c r="A5" s="119" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="74"/>
+      <c r="B5" s="73"/>
       <c r="C5" s="23">
         <v>-2.15</v>
       </c>
@@ -7405,10 +7405,10 @@
       <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="120" t="s">
+      <c r="A6" s="119" t="s">
         <v>81</v>
       </c>
-      <c r="B6" s="75"/>
+      <c r="B6" s="74"/>
       <c r="C6" s="24">
         <v>-1</v>
       </c>
@@ -7416,10 +7416,10 @@
       <c r="E6" s="18"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="120" t="s">
+      <c r="A7" s="119" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="75"/>
+      <c r="B7" s="74"/>
       <c r="C7" s="24">
         <v>1.2250000000000001</v>
       </c>
@@ -7429,10 +7429,10 @@
       <c r="E7" s="18"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="120" t="s">
-        <v>145</v>
-      </c>
-      <c r="B8" s="75"/>
+      <c r="A8" s="119" t="s">
+        <v>144</v>
+      </c>
+      <c r="B8" s="74"/>
       <c r="C8" s="24">
         <v>1.2</v>
       </c>
@@ -7442,12 +7442,12 @@
       <c r="E8" s="18"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="120" t="s">
+      <c r="A9" s="119" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="78"/>
-      <c r="C9" s="29" t="s">
-        <v>86</v>
+      <c r="B9" s="77"/>
+      <c r="C9" s="137" t="s">
+        <v>166</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>29</v>
@@ -7464,6 +7464,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009342B7EAA7728A4FA80A5CCAFE8D7EAF" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d037a5681ee6af0e7b5b5d0a2f99b20">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557458c-24b5-4c97-84ed-4c402655f54f" xmlns:ns3="72e3c584-9879-4b35-b9d8-6a248c93e240" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="966978c8b125399653e7c255ac8e342d" ns2:_="" ns3:_="">
     <xsd:import namespace="9557458c-24b5-4c97-84ed-4c402655f54f"/>
@@ -7724,27 +7744,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7761,23 +7780,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
-    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
A lot of bugfixes and balkans tracks, aero ggv diagram,
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F09127EB-0DDD-6E4F-BF95-EE21855C496C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1357B4F-C61A-0E4D-BD61-29CB543F16B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12800" yWindow="1700" windowWidth="27000" windowHeight="16060" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4580" yWindow="1880" windowWidth="34480" windowHeight="19400" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Body" sheetId="1" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="183">
   <si>
     <t>Category</t>
   </si>
@@ -560,22 +560,67 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
+    <t>1 steady state</t>
+  </si>
+  <si>
+    <t>1 combined</t>
+  </si>
+  <si>
+    <t>[27 74 70]</t>
+  </si>
+  <si>
+    <t>[-0.707 0 0.628]</t>
+  </si>
+  <si>
+    <t>[-0,8232 0 0,3583]</t>
+  </si>
+  <si>
     <t>MFEval</t>
   </si>
   <si>
-    <t>1 steady state</t>
-  </si>
-  <si>
-    <t>1 combined</t>
-  </si>
-  <si>
-    <t>[27 74 70]</t>
-  </si>
-  <si>
-    <t>[-0.707 0 0.628]</t>
-  </si>
-  <si>
-    <t>[-0,8232 0 0,3583]</t>
+    <t>aAxis</t>
+  </si>
+  <si>
+    <t>rad</t>
+  </si>
+  <si>
+    <t>FSAE</t>
+  </si>
+  <si>
+    <t>xRad</t>
+  </si>
+  <si>
+    <t>Pinion</t>
+  </si>
+  <si>
+    <t>Shaft_Upper</t>
+  </si>
+  <si>
+    <t>xLength</t>
+  </si>
+  <si>
+    <t>Shaft_Lower</t>
+  </si>
+  <si>
+    <t>Ratio_Table</t>
+  </si>
+  <si>
+    <t>[-3.1416 -2.8274 -2.5133 -2.1991 -1.8849 -1.5708 -1.2566 -0.94247 -0.62831 -0.31416 0 0.31416 0.62831 0.94247 1.2566 1.5708 1.8849 2.1991 2.5133 2.8274 3.1416]</t>
+  </si>
+  <si>
+    <t>[-0.042894 -0.038604 -0.034315 -0.030026 -0.025736 -0.021447 -0.017157 -0.012868 -0.0085787 -0.0042894 0 0.0042894 0.0085787 0.012868 0.017157 0.021447 0.025736 0.030026 0.034315 0.038604 0.042894]</t>
+  </si>
+  <si>
+    <t>aWheel</t>
+  </si>
+  <si>
+    <t>xRack</t>
+  </si>
+  <si>
+    <t>Rack Displacement - reference only</t>
+  </si>
+  <si>
+    <t>Wheel Angle - reference only</t>
   </si>
 </sst>
 </file>
@@ -700,7 +745,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="72">
+  <borders count="74">
     <border>
       <left/>
       <right/>
@@ -1683,11 +1728,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="162">
+  <cellXfs count="169">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2094,6 +2165,9 @@
     <xf numFmtId="49" fontId="3" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2155,6 +2229,24 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3385,7 +3477,7 @@
       </c>
       <c r="B7" s="74"/>
       <c r="C7" s="75" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>12</v>
@@ -3502,7 +3594,7 @@
       </c>
       <c r="B15" s="74"/>
       <c r="C15" s="83" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D15" s="85" t="s">
         <v>32</v>
@@ -3583,7 +3675,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="147" t="s">
+      <c r="A5" s="148" t="s">
         <v>88</v>
       </c>
       <c r="B5" s="73" t="s">
@@ -3596,7 +3688,7 @@
       <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="148"/>
+      <c r="A6" s="149"/>
       <c r="B6" s="93" t="s">
         <v>90</v>
       </c>
@@ -3609,7 +3701,7 @@
       <c r="E6" s="96"/>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="157"/>
+      <c r="A7" s="158"/>
       <c r="B7" s="77" t="s">
         <v>143</v>
       </c>
@@ -3622,7 +3714,7 @@
       <c r="E7" s="29"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="147" t="s">
+      <c r="A8" s="148" t="s">
         <v>92</v>
       </c>
       <c r="B8" s="73" t="s">
@@ -3635,7 +3727,7 @@
       <c r="E8" s="28"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="148"/>
+      <c r="A9" s="149"/>
       <c r="B9" s="93" t="s">
         <v>90</v>
       </c>
@@ -3648,7 +3740,7 @@
       <c r="E9" s="96"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="157"/>
+      <c r="A10" s="158"/>
       <c r="B10" s="77" t="s">
         <v>143</v>
       </c>
@@ -3736,7 +3828,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="147" t="s">
+      <c r="A5" s="148" t="s">
         <v>88</v>
       </c>
       <c r="B5" s="73" t="s">
@@ -3749,7 +3841,7 @@
       <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="148"/>
+      <c r="A6" s="149"/>
       <c r="B6" s="93" t="s">
         <v>93</v>
       </c>
@@ -3764,7 +3856,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="148"/>
+      <c r="A7" s="149"/>
       <c r="B7" s="74" t="s">
         <v>94</v>
       </c>
@@ -3777,7 +3869,7 @@
       <c r="E7" s="18"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="148"/>
+      <c r="A8" s="149"/>
       <c r="B8" s="74" t="s">
         <v>95</v>
       </c>
@@ -3790,7 +3882,7 @@
       <c r="E8" s="18"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="148"/>
+      <c r="A9" s="149"/>
       <c r="B9" s="74" t="s">
         <v>96</v>
       </c>
@@ -3803,7 +3895,7 @@
       <c r="E9" s="18"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="148"/>
+      <c r="A10" s="149"/>
       <c r="B10" s="74" t="s">
         <v>97</v>
       </c>
@@ -3816,7 +3908,7 @@
       <c r="E10" s="18"/>
     </row>
     <row r="11" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="157"/>
+      <c r="A11" s="158"/>
       <c r="B11" s="77" t="s">
         <v>98</v>
       </c>
@@ -3829,7 +3921,7 @@
       <c r="E11" s="29"/>
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="147" t="s">
+      <c r="A12" s="148" t="s">
         <v>92</v>
       </c>
       <c r="B12" s="73" t="s">
@@ -3842,7 +3934,7 @@
       <c r="E12" s="28"/>
     </row>
     <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="148"/>
+      <c r="A13" s="149"/>
       <c r="B13" s="93" t="s">
         <v>93</v>
       </c>
@@ -3857,7 +3949,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="148"/>
+      <c r="A14" s="149"/>
       <c r="B14" s="74" t="s">
         <v>94</v>
       </c>
@@ -3870,7 +3962,7 @@
       <c r="E14" s="18"/>
     </row>
     <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="148"/>
+      <c r="A15" s="149"/>
       <c r="B15" s="74" t="s">
         <v>95</v>
       </c>
@@ -3883,7 +3975,7 @@
       <c r="E15" s="18"/>
     </row>
     <row r="16" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="148"/>
+      <c r="A16" s="149"/>
       <c r="B16" s="74" t="s">
         <v>96</v>
       </c>
@@ -3896,7 +3988,7 @@
       <c r="E16" s="18"/>
     </row>
     <row r="17" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="148"/>
+      <c r="A17" s="149"/>
       <c r="B17" s="74" t="s">
         <v>97</v>
       </c>
@@ -3909,7 +4001,7 @@
       <c r="E17" s="18"/>
     </row>
     <row r="18" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="157"/>
+      <c r="A18" s="158"/>
       <c r="B18" s="77" t="s">
         <v>98</v>
       </c>
@@ -4807,7 +4899,7 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="101" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
@@ -4893,7 +4985,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="147" t="s">
+      <c r="A11" s="148" t="s">
         <v>113</v>
       </c>
       <c r="B11" s="105" t="s">
@@ -4906,7 +4998,7 @@
       <c r="E11" s="70"/>
     </row>
     <row r="12" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="157"/>
+      <c r="A12" s="158"/>
       <c r="B12" s="107" t="s">
         <v>114</v>
       </c>
@@ -4924,7 +5016,7 @@
       </c>
       <c r="B13" s="73"/>
       <c r="C13" s="99" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D13" s="102"/>
       <c r="E13" s="103" t="s">
@@ -4937,7 +5029,7 @@
       </c>
       <c r="B14" s="73"/>
       <c r="C14" s="99" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D14" s="102"/>
       <c r="E14" s="103"/>
@@ -5729,7 +5821,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="141" t="s">
+      <c r="A5" s="142" t="s">
         <v>38</v>
       </c>
       <c r="B5" s="73" t="s">
@@ -5747,7 +5839,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="139"/>
+      <c r="A6" s="140"/>
       <c r="B6" s="74" t="s">
         <v>41</v>
       </c>
@@ -5763,7 +5855,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="142"/>
+      <c r="A7" s="143"/>
       <c r="B7" s="74" t="s">
         <v>42</v>
       </c>
@@ -5779,7 +5871,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="142"/>
+      <c r="A8" s="143"/>
       <c r="B8" s="77" t="s">
         <v>12</v>
       </c>
@@ -5792,7 +5884,7 @@
       <c r="E8" s="22"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="143" t="s">
+      <c r="A9" s="144" t="s">
         <v>43</v>
       </c>
       <c r="B9" s="73" t="s">
@@ -5810,7 +5902,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="140"/>
+      <c r="A10" s="141"/>
       <c r="B10" s="74" t="s">
         <v>41</v>
       </c>
@@ -5826,7 +5918,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="140"/>
+      <c r="A11" s="141"/>
       <c r="B11" s="74" t="s">
         <v>42</v>
       </c>
@@ -5842,7 +5934,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="139"/>
+      <c r="A12" s="140"/>
       <c r="B12" s="77" t="s">
         <v>12</v>
       </c>
@@ -5857,7 +5949,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="144" t="s">
+      <c r="A13" s="145" t="s">
         <v>44</v>
       </c>
       <c r="B13" s="73" t="s">
@@ -5875,7 +5967,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="142"/>
+      <c r="A14" s="143"/>
       <c r="B14" s="74" t="s">
         <v>148</v>
       </c>
@@ -5891,7 +5983,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="142"/>
+      <c r="A15" s="143"/>
       <c r="B15" s="74" t="s">
         <v>12</v>
       </c>
@@ -5904,7 +5996,7 @@
       <c r="E15" s="18"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="145"/>
+      <c r="A16" s="146"/>
       <c r="B16" s="74" t="s">
         <v>45</v>
       </c>
@@ -5917,7 +6009,7 @@
       <c r="E16" s="16"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="140"/>
+      <c r="A17" s="141"/>
       <c r="B17" s="74" t="s">
         <v>47</v>
       </c>
@@ -5930,7 +6022,7 @@
       <c r="E17" s="16"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="140"/>
+      <c r="A18" s="141"/>
       <c r="B18" s="74" t="s">
         <v>48</v>
       </c>
@@ -5943,7 +6035,7 @@
       <c r="E18" s="16"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="140"/>
+      <c r="A19" s="141"/>
       <c r="B19" s="74" t="s">
         <v>49</v>
       </c>
@@ -5956,7 +6048,7 @@
       <c r="E19" s="16"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="139"/>
+      <c r="A20" s="140"/>
       <c r="B20" s="77" t="s">
         <v>50</v>
       </c>
@@ -5969,7 +6061,7 @@
       <c r="E20" s="22"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="138" t="s">
+      <c r="A21" s="139" t="s">
         <v>142</v>
       </c>
       <c r="B21" s="73" t="s">
@@ -5987,7 +6079,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="140"/>
+      <c r="A22" s="141"/>
       <c r="B22" s="14" t="s">
         <v>42</v>
       </c>
@@ -6003,7 +6095,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="139"/>
+      <c r="A23" s="140"/>
       <c r="B23" s="19" t="s">
         <v>12</v>
       </c>
@@ -6016,7 +6108,7 @@
       <c r="E23" s="22"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="138" t="s">
+      <c r="A24" s="139" t="s">
         <v>52</v>
       </c>
       <c r="B24" s="73" t="s">
@@ -6034,7 +6126,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="140"/>
+      <c r="A25" s="141"/>
       <c r="B25" s="74" t="s">
         <v>54</v>
       </c>
@@ -6050,7 +6142,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="146"/>
+      <c r="A26" s="147"/>
       <c r="B26" s="78" t="s">
         <v>146</v>
       </c>
@@ -6063,7 +6155,7 @@
       <c r="E26" s="81"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="139"/>
+      <c r="A27" s="140"/>
       <c r="B27" s="77" t="s">
         <v>145</v>
       </c>
@@ -6076,7 +6168,7 @@
       <c r="E27" s="22"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="138" t="s">
+      <c r="A28" s="139" t="s">
         <v>55</v>
       </c>
       <c r="B28" s="73" t="s">
@@ -6091,7 +6183,7 @@
       <c r="E28" s="13"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="139"/>
+      <c r="A29" s="140"/>
       <c r="B29" s="77" t="s">
         <v>57</v>
       </c>
@@ -6104,7 +6196,7 @@
       <c r="E29" s="22"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="138" t="s">
+      <c r="A30" s="139" t="s">
         <v>58</v>
       </c>
       <c r="B30" s="87" t="s">
@@ -6122,7 +6214,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="140"/>
+      <c r="A31" s="141"/>
       <c r="B31" s="88" t="s">
         <v>42</v>
       </c>
@@ -6138,7 +6230,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="139"/>
+      <c r="A32" s="140"/>
       <c r="B32" s="89" t="s">
         <v>12</v>
       </c>
@@ -6151,7 +6243,7 @@
       <c r="E32" s="22"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="138" t="s">
+      <c r="A33" s="139" t="s">
         <v>59</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -6169,7 +6261,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="140"/>
+      <c r="A34" s="141"/>
       <c r="B34" s="14" t="s">
         <v>61</v>
       </c>
@@ -6185,7 +6277,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="139"/>
+      <c r="A35" s="140"/>
       <c r="B35" s="19" t="s">
         <v>12</v>
       </c>
@@ -6363,7 +6455,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" style="1" customWidth="1"/>
@@ -6426,7 +6518,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="147" t="s">
+      <c r="A5" s="148" t="s">
         <v>72</v>
       </c>
       <c r="B5" s="73" t="s">
@@ -6444,7 +6536,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="148"/>
+      <c r="A6" s="149"/>
       <c r="B6" s="92" t="s">
         <v>12</v>
       </c>
@@ -6457,7 +6549,7 @@
       <c r="E6" s="18"/>
     </row>
     <row r="7" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="149"/>
+      <c r="A7" s="150"/>
       <c r="B7" s="74" t="s">
         <v>74</v>
       </c>
@@ -6470,40 +6562,185 @@
       <c r="E7" s="15"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="150" t="s">
+      <c r="A8" s="151" t="s">
         <v>76</v>
       </c>
       <c r="B8" s="74" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="24">
+        <v>168</v>
+      </c>
+      <c r="C8" s="37">
+        <v>0.72919999999999996</v>
+      </c>
+      <c r="D8" s="85" t="s">
+        <v>169</v>
+      </c>
+      <c r="E8" s="41"/>
+    </row>
+    <row r="9" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="163"/>
+      <c r="B9" s="74" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="164" t="s">
+        <v>170</v>
+      </c>
+      <c r="D9" s="15"/>
+      <c r="E9" s="41"/>
+    </row>
+    <row r="10" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="163"/>
+      <c r="B10" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="24">
         <v>0.5</v>
       </c>
-      <c r="D8" s="85" t="s">
+      <c r="D10" s="85" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="16"/>
-    </row>
-    <row r="9" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="151"/>
-      <c r="B9" s="74" t="s">
+      <c r="E10" s="16"/>
+    </row>
+    <row r="11" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="152"/>
+      <c r="B11" s="74" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="37" t="str">
+      <c r="C11" s="37" t="str">
         <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B21/1000,HardpointsFr!C21/1000,HardpointsFr!D21/1000)&amp;"]"</f>
         <v>[-0.324965 0 0.533792]</v>
       </c>
-      <c r="D9" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="15" t="s">
+      <c r="D11" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="15" t="s">
         <v>40</v>
       </c>
     </row>
+    <row r="12" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="165" t="s">
+        <v>172</v>
+      </c>
+      <c r="B12" s="74" t="s">
+        <v>171</v>
+      </c>
+      <c r="C12" s="37">
+        <v>1.2732E-2</v>
+      </c>
+      <c r="D12" s="85" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="41"/>
+    </row>
+    <row r="13" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="163"/>
+      <c r="B13" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="164">
+        <v>0.05</v>
+      </c>
+      <c r="D13" s="85" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" s="41"/>
+    </row>
+    <row r="14" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="166"/>
+      <c r="B14" s="74" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="24" t="str">
+        <f>"["&amp;_xlfn.TEXTJOIN(" ",TRUE,HardpointsFr!B20/1000 - SIN(C8) * C12, 0, HardpointsFr!D20/1000-C8*C12)&amp;"]"</f>
+        <v>[0.0957580085717026 0 0.1617688256]</v>
+      </c>
+      <c r="D14" s="85" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="16"/>
+    </row>
+    <row r="15" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="167" t="s">
+        <v>173</v>
+      </c>
+      <c r="B15" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="37">
+        <v>0.2</v>
+      </c>
+      <c r="D15" s="85" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="15"/>
+    </row>
+    <row r="16" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="152"/>
+      <c r="B16" s="74" t="s">
+        <v>174</v>
+      </c>
+      <c r="C16" s="37">
+        <f>SQRT(SUMXMY2(HardpointsFr!B20:D20,HardpointsFr!B21:D21))/1000/2</f>
+        <v>0.28097925748932073</v>
+      </c>
+      <c r="D16" s="85" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="15"/>
+    </row>
+    <row r="17" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="138" t="s">
+        <v>175</v>
+      </c>
+      <c r="B17" s="74" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="37">
+        <v>0.2</v>
+      </c>
+      <c r="D17" s="85" t="s">
+        <v>29</v>
+      </c>
+      <c r="E17" s="15"/>
+    </row>
+    <row r="18" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="165" t="s">
+        <v>176</v>
+      </c>
+      <c r="B18" s="74" t="s">
+        <v>179</v>
+      </c>
+      <c r="C18" s="168" t="s">
+        <v>177</v>
+      </c>
+      <c r="D18" s="85" t="s">
+        <v>169</v>
+      </c>
+      <c r="E18" s="85" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="152"/>
+      <c r="B19" s="74" t="s">
+        <v>180</v>
+      </c>
+      <c r="C19" s="168" t="s">
+        <v>178</v>
+      </c>
+      <c r="D19" s="85" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>181</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="5">
+    <mergeCell ref="A18:A19"/>
     <mergeCell ref="A5:A7"/>
-    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="A15:A16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -6604,7 +6841,7 @@
       <c r="E6" s="22"/>
     </row>
     <row r="7" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="152" t="s">
+      <c r="A7" s="153" t="s">
         <v>65</v>
       </c>
       <c r="B7" s="126" t="s">
@@ -6617,7 +6854,7 @@
       <c r="E7" s="128"/>
     </row>
     <row r="8" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="153"/>
+      <c r="A8" s="154"/>
       <c r="B8" s="126" t="s">
         <v>8</v>
       </c>
@@ -6702,7 +6939,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="152" t="s">
+      <c r="A5" s="153" t="s">
         <v>38</v>
       </c>
       <c r="B5" s="73" t="s">
@@ -6720,7 +6957,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" s="1" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="158"/>
+      <c r="A6" s="159"/>
       <c r="B6" s="74" t="s">
         <v>41</v>
       </c>
@@ -6736,7 +6973,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="158"/>
+      <c r="A7" s="159"/>
       <c r="B7" s="74" t="s">
         <v>42</v>
       </c>
@@ -6752,7 +6989,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="153"/>
+      <c r="A8" s="154"/>
       <c r="B8" s="77" t="s">
         <v>12</v>
       </c>
@@ -6765,7 +7002,7 @@
       <c r="E8" s="56"/>
     </row>
     <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="159" t="s">
+      <c r="A9" s="160" t="s">
         <v>43</v>
       </c>
       <c r="B9" s="73" t="s">
@@ -6783,7 +7020,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="160"/>
+      <c r="A10" s="161"/>
       <c r="B10" s="74" t="s">
         <v>41</v>
       </c>
@@ -6799,7 +7036,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="160"/>
+      <c r="A11" s="161"/>
       <c r="B11" s="74" t="s">
         <v>42</v>
       </c>
@@ -6815,7 +7052,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="161"/>
+      <c r="A12" s="162"/>
       <c r="B12" s="77" t="s">
         <v>12</v>
       </c>
@@ -6830,7 +7067,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="147" t="s">
+      <c r="A13" s="148" t="s">
         <v>44</v>
       </c>
       <c r="B13" s="73" t="s">
@@ -6848,7 +7085,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="148"/>
+      <c r="A14" s="149"/>
       <c r="B14" s="74" t="s">
         <v>148</v>
       </c>
@@ -6864,7 +7101,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="148"/>
+      <c r="A15" s="149"/>
       <c r="B15" s="74" t="s">
         <v>12</v>
       </c>
@@ -6877,7 +7114,7 @@
       <c r="E15" s="62"/>
     </row>
     <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="148"/>
+      <c r="A16" s="149"/>
       <c r="B16" s="74" t="s">
         <v>45</v>
       </c>
@@ -6890,7 +7127,7 @@
       <c r="E16" s="60"/>
     </row>
     <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="148"/>
+      <c r="A17" s="149"/>
       <c r="B17" s="74" t="s">
         <v>47</v>
       </c>
@@ -6903,7 +7140,7 @@
       <c r="E17" s="63"/>
     </row>
     <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="148"/>
+      <c r="A18" s="149"/>
       <c r="B18" s="74" t="s">
         <v>48</v>
       </c>
@@ -6916,7 +7153,7 @@
       <c r="E18" s="63"/>
     </row>
     <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="148"/>
+      <c r="A19" s="149"/>
       <c r="B19" s="74" t="s">
         <v>49</v>
       </c>
@@ -6929,7 +7166,7 @@
       <c r="E19" s="63"/>
     </row>
     <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="157"/>
+      <c r="A20" s="158"/>
       <c r="B20" s="77" t="s">
         <v>50</v>
       </c>
@@ -6942,7 +7179,7 @@
       <c r="E20" s="64"/>
     </row>
     <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="147" t="s">
+      <c r="A21" s="148" t="s">
         <v>142</v>
       </c>
       <c r="B21" s="73" t="s">
@@ -6960,7 +7197,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="148"/>
+      <c r="A22" s="149"/>
       <c r="B22" s="14" t="s">
         <v>42</v>
       </c>
@@ -6976,7 +7213,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="157"/>
+      <c r="A23" s="158"/>
       <c r="B23" s="19" t="s">
         <v>12</v>
       </c>
@@ -6989,7 +7226,7 @@
       <c r="E23" s="66"/>
     </row>
     <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="147" t="s">
+      <c r="A24" s="148" t="s">
         <v>52</v>
       </c>
       <c r="B24" s="73" t="s">
@@ -7007,7 +7244,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="148"/>
+      <c r="A25" s="149"/>
       <c r="B25" s="74" t="s">
         <v>54</v>
       </c>
@@ -7023,7 +7260,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="148"/>
+      <c r="A26" s="149"/>
       <c r="B26" s="78" t="s">
         <v>145</v>
       </c>
@@ -7034,7 +7271,7 @@
       <c r="E26" s="71"/>
     </row>
     <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="157"/>
+      <c r="A27" s="158"/>
       <c r="B27" s="77" t="s">
         <v>146</v>
       </c>
@@ -7047,7 +7284,7 @@
       <c r="E27" s="67"/>
     </row>
     <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="147" t="s">
+      <c r="A28" s="148" t="s">
         <v>55</v>
       </c>
       <c r="B28" s="73" t="s">
@@ -7062,7 +7299,7 @@
       <c r="E28" s="68"/>
     </row>
     <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="157"/>
+      <c r="A29" s="158"/>
       <c r="B29" s="77" t="s">
         <v>57</v>
       </c>
@@ -7075,7 +7312,7 @@
       <c r="E29" s="67"/>
     </row>
     <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="154" t="s">
+      <c r="A30" s="155" t="s">
         <v>58</v>
       </c>
       <c r="B30" s="87" t="s">
@@ -7093,7 +7330,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="155"/>
+      <c r="A31" s="156"/>
       <c r="B31" s="88" t="s">
         <v>51</v>
       </c>
@@ -7109,7 +7346,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="156"/>
+      <c r="A32" s="157"/>
       <c r="B32" s="89" t="s">
         <v>12</v>
       </c>
@@ -7122,7 +7359,7 @@
       <c r="E32" s="69"/>
     </row>
     <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="147" t="s">
+      <c r="A33" s="148" t="s">
         <v>59</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -7140,7 +7377,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="148"/>
+      <c r="A34" s="149"/>
       <c r="B34" s="14" t="s">
         <v>61</v>
       </c>
@@ -7156,7 +7393,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="157"/>
+      <c r="A35" s="158"/>
       <c r="B35" s="19" t="s">
         <v>12</v>
       </c>
@@ -7399,7 +7636,7 @@
       </c>
       <c r="B5" s="73"/>
       <c r="C5" s="23">
-        <v>-2.15</v>
+        <v>-2.48</v>
       </c>
       <c r="D5" s="12"/>
       <c r="E5" s="28"/>
@@ -7410,7 +7647,7 @@
       </c>
       <c r="B6" s="74"/>
       <c r="C6" s="24">
-        <v>-1</v>
+        <v>1.08</v>
       </c>
       <c r="D6" s="15"/>
       <c r="E6" s="18"/>
@@ -7447,7 +7684,7 @@
       </c>
       <c r="B9" s="77"/>
       <c r="C9" s="137" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>29</v>
@@ -7464,26 +7701,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009342B7EAA7728A4FA80A5CCAFE8D7EAF" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d037a5681ee6af0e7b5b5d0a2f99b20">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557458c-24b5-4c97-84ed-4c402655f54f" xmlns:ns3="72e3c584-9879-4b35-b9d8-6a248c93e240" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="966978c8b125399653e7c255ac8e342d" ns2:_="" ns3:_="">
     <xsd:import namespace="9557458c-24b5-4c97-84ed-4c402655f54f"/>
@@ -7744,10 +7961,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7764,20 +8012,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
-    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Better tire model and Balkans tracks
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="13_ncr:1_{A1357B4F-C61A-0E4D-BD61-29CB543F16B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40916596-B1F0-4DBB-A9DC-9DF1CABA6375}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98642FD4-5D90-E44C-ADEF-D223C164BEEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4580" yWindow="1880" windowWidth="34480" windowHeight="19400" firstSheet="4" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3920" yWindow="1880" windowWidth="34480" windowHeight="19400" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Body" sheetId="1" r:id="rId1"/>
@@ -485,9 +485,6 @@
     <t>tirFile</t>
   </si>
   <si>
-    <t>which('Hoosier_R20B_20p5x7_R13_7in_12psi.tir')</t>
-  </si>
-  <si>
     <t>fileName</t>
   </si>
   <si>
@@ -621,6 +618,9 @@
   </si>
   <si>
     <t>Steer Wheel</t>
+  </si>
+  <si>
+    <t>which('Hoosier_R20B_20p5x7_R13_7in.tir')</t>
   </si>
 </sst>
 </file>
@@ -632,7 +632,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -2180,6 +2180,30 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="58" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2207,18 +2231,6 @@
     <xf numFmtId="0" fontId="2" fillId="11" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2249,18 +2261,6 @@
     <xf numFmtId="49" fontId="2" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="22" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3395,18 +3395,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5" style="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="47.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.85546875" style="1"/>
+    <col min="4" max="4" width="9.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="47.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3421,7 +3421,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.1" customHeight="1">
+    <row r="2" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -3432,7 +3432,7 @@
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" ht="14.1" customHeight="1">
+    <row r="3" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -3443,7 +3443,7 @@
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="4" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -3454,7 +3454,7 @@
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="5" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="118" t="s">
         <v>10</v>
       </c>
@@ -3469,7 +3469,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15" customHeight="1" thickBot="1">
+    <row r="6" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="118" t="s">
         <v>14</v>
       </c>
@@ -3484,7 +3484,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15" customHeight="1" thickBot="1">
+    <row r="7" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="118" t="s">
         <v>17</v>
       </c>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="E7" s="16"/>
     </row>
-    <row r="8" spans="1:5" ht="15" customHeight="1" thickBot="1">
+    <row r="8" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="118" t="s">
         <v>19</v>
       </c>
@@ -3512,7 +3512,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15" customHeight="1" thickBot="1">
+    <row r="9" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="118" t="s">
         <v>22</v>
       </c>
@@ -3527,7 +3527,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15" customHeight="1" thickBot="1">
+    <row r="10" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="118" t="s">
         <v>24</v>
       </c>
@@ -3542,7 +3542,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15.95" thickBot="1">
+    <row r="11" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="118" t="s">
         <v>26</v>
       </c>
@@ -3558,7 +3558,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
+    <row r="12" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="118" t="s">
         <v>28</v>
       </c>
@@ -3572,7 +3572,7 @@
       </c>
       <c r="E12" s="16"/>
     </row>
-    <row r="13" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
+    <row r="13" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="118" t="s">
         <v>29</v>
       </c>
@@ -3586,7 +3586,7 @@
       </c>
       <c r="E13" s="18"/>
     </row>
-    <row r="14" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
+    <row r="14" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="118" t="s">
         <v>12</v>
       </c>
@@ -3601,7 +3601,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="13.5" customHeight="1">
+    <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="118" t="s">
         <v>32</v>
       </c>
@@ -3628,18 +3628,18 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="42.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="14.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="42.5" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3654,7 +3654,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.1" customHeight="1">
+    <row r="2" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -3665,7 +3665,7 @@
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" ht="14.1" customHeight="1">
+    <row r="3" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -3676,7 +3676,7 @@
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="4" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -3687,8 +3687,8 @@
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" ht="14.1" customHeight="1">
-      <c r="A5" s="143" t="s">
+    <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="155" t="s">
         <v>118</v>
       </c>
       <c r="B5" s="73" t="s">
@@ -3700,8 +3700,8 @@
       <c r="D5" s="12"/>
       <c r="E5" s="28"/>
     </row>
-    <row r="6" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A6" s="144"/>
+    <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="156"/>
       <c r="B6" s="93" t="s">
         <v>120</v>
       </c>
@@ -3713,8 +3713,8 @@
       </c>
       <c r="E6" s="96"/>
     </row>
-    <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A7" s="159"/>
+    <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="167"/>
       <c r="B7" s="77" t="s">
         <v>122</v>
       </c>
@@ -3726,8 +3726,8 @@
       </c>
       <c r="E7" s="29"/>
     </row>
-    <row r="8" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A8" s="143" t="s">
+    <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="155" t="s">
         <v>123</v>
       </c>
       <c r="B8" s="73" t="s">
@@ -3739,8 +3739,8 @@
       <c r="D8" s="12"/>
       <c r="E8" s="28"/>
     </row>
-    <row r="9" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A9" s="144"/>
+    <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="156"/>
       <c r="B9" s="93" t="s">
         <v>120</v>
       </c>
@@ -3752,8 +3752,8 @@
       </c>
       <c r="E9" s="96"/>
     </row>
-    <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A10" s="159"/>
+    <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="167"/>
       <c r="B10" s="77" t="s">
         <v>122</v>
       </c>
@@ -3781,18 +3781,18 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:E18"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="42.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="14.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="42.5" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3807,7 +3807,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.1" customHeight="1">
+    <row r="2" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -3818,7 +3818,7 @@
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" ht="14.1" customHeight="1">
+    <row r="3" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -3829,7 +3829,7 @@
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="4" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -3840,8 +3840,8 @@
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" ht="14.1" customHeight="1">
-      <c r="A5" s="143" t="s">
+    <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="155" t="s">
         <v>118</v>
       </c>
       <c r="B5" s="73" t="s">
@@ -3853,8 +3853,8 @@
       <c r="D5" s="12"/>
       <c r="E5" s="28"/>
     </row>
-    <row r="6" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A6" s="144"/>
+    <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="156"/>
       <c r="B6" s="93" t="s">
         <v>126</v>
       </c>
@@ -3868,8 +3868,8 @@
         <v>127</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A7" s="144"/>
+    <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="156"/>
       <c r="B7" s="74" t="s">
         <v>128</v>
       </c>
@@ -3881,8 +3881,8 @@
       </c>
       <c r="E7" s="18"/>
     </row>
-    <row r="8" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A8" s="144"/>
+    <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="156"/>
       <c r="B8" s="74" t="s">
         <v>129</v>
       </c>
@@ -3894,8 +3894,8 @@
       </c>
       <c r="E8" s="18"/>
     </row>
-    <row r="9" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A9" s="144"/>
+    <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="156"/>
       <c r="B9" s="74" t="s">
         <v>130</v>
       </c>
@@ -3907,8 +3907,8 @@
       </c>
       <c r="E9" s="18"/>
     </row>
-    <row r="10" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A10" s="144"/>
+    <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="156"/>
       <c r="B10" s="74" t="s">
         <v>131</v>
       </c>
@@ -3920,8 +3920,8 @@
       </c>
       <c r="E10" s="18"/>
     </row>
-    <row r="11" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A11" s="159"/>
+    <row r="11" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="167"/>
       <c r="B11" s="77" t="s">
         <v>132</v>
       </c>
@@ -3933,8 +3933,8 @@
       </c>
       <c r="E11" s="29"/>
     </row>
-    <row r="12" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A12" s="143" t="s">
+    <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="155" t="s">
         <v>123</v>
       </c>
       <c r="B12" s="73" t="s">
@@ -3946,8 +3946,8 @@
       <c r="D12" s="12"/>
       <c r="E12" s="28"/>
     </row>
-    <row r="13" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A13" s="144"/>
+    <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="156"/>
       <c r="B13" s="93" t="s">
         <v>126</v>
       </c>
@@ -3961,8 +3961,8 @@
         <v>127</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A14" s="144"/>
+    <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="156"/>
       <c r="B14" s="74" t="s">
         <v>128</v>
       </c>
@@ -3974,8 +3974,8 @@
       </c>
       <c r="E14" s="18"/>
     </row>
-    <row r="15" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A15" s="144"/>
+    <row r="15" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="156"/>
       <c r="B15" s="74" t="s">
         <v>129</v>
       </c>
@@ -3987,8 +3987,8 @@
       </c>
       <c r="E15" s="18"/>
     </row>
-    <row r="16" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A16" s="144"/>
+    <row r="16" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="156"/>
       <c r="B16" s="74" t="s">
         <v>130</v>
       </c>
@@ -4000,8 +4000,8 @@
       </c>
       <c r="E16" s="18"/>
     </row>
-    <row r="17" spans="1:5" ht="13.5" customHeight="1">
-      <c r="A17" s="144"/>
+    <row r="17" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="156"/>
       <c r="B17" s="74" t="s">
         <v>131</v>
       </c>
@@ -4013,8 +4013,8 @@
       </c>
       <c r="E17" s="18"/>
     </row>
-    <row r="18" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A18" s="159"/>
+    <row r="18" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="167"/>
       <c r="B18" s="77" t="s">
         <v>132</v>
       </c>
@@ -4042,9 +4042,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CD2A3BA-06BE-A64D-A72B-9CFCF024C1FD}">
   <dimension ref="A1:B101"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="132">
         <v>-443.53</v>
       </c>
@@ -4052,7 +4052,7 @@
         <v>-3883.5949999999998</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="132">
         <v>-433.58</v>
       </c>
@@ -4060,7 +4060,7 @@
         <v>-3833.1889999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="132">
         <v>-423.97</v>
       </c>
@@ -4068,7 +4068,7 @@
         <v>-3778.5659999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="132">
         <v>-415</v>
       </c>
@@ -4076,7 +4076,7 @@
         <v>-3715.607</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="132">
         <v>-406.67</v>
       </c>
@@ -4084,7 +4084,7 @@
         <v>-3644.3130000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="132">
         <v>-398.79</v>
       </c>
@@ -4092,7 +4092,7 @@
         <v>-3567.2330000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="132">
         <v>-391.16</v>
       </c>
@@ -4100,7 +4100,7 @@
         <v>-3486.6219999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="132">
         <v>-383.59</v>
       </c>
@@ -4108,7 +4108,7 @@
         <v>-3405.2269999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="132">
         <v>-375.88</v>
       </c>
@@ -4116,7 +4116,7 @@
         <v>-3325.3029999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="132">
         <v>-367.89</v>
       </c>
@@ -4124,7 +4124,7 @@
         <v>-3248.7130000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="132">
         <v>-359.64</v>
       </c>
@@ -4132,7 +4132,7 @@
         <v>-3175.3589999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="132">
         <v>-351.2</v>
       </c>
@@ -4140,7 +4140,7 @@
         <v>-3104.163</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="132">
         <v>-342.63</v>
       </c>
@@ -4148,7 +4148,7 @@
         <v>-3034.5360000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="132">
         <v>-334</v>
       </c>
@@ -4156,7 +4156,7 @@
         <v>-2965.6930000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="132">
         <v>-325.38</v>
       </c>
@@ -4164,7 +4164,7 @@
         <v>-2896.85</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="132">
         <v>-316.77</v>
       </c>
@@ -4172,7 +4172,7 @@
         <v>-2827.6149999999998</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="132">
         <v>-308.2</v>
       </c>
@@ -4180,7 +4180,7 @@
         <v>-2757.9879999999998</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="132">
         <v>-299.64999999999998</v>
       </c>
@@ -4188,7 +4188,7 @@
         <v>-2687.9690000000001</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="132">
         <v>-291.14</v>
       </c>
@@ -4196,7 +4196,7 @@
         <v>-2617.5569999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="132">
         <v>-282.67</v>
       </c>
@@ -4204,7 +4204,7 @@
         <v>-2546.6550000000002</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="132">
         <v>-274.25</v>
       </c>
@@ -4212,7 +4212,7 @@
         <v>-2475.1640000000002</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="132">
         <v>-265.91000000000003</v>
       </c>
@@ -4220,7 +4220,7 @@
         <v>-2402.7910000000002</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="132">
         <v>-257.67</v>
       </c>
@@ -4228,7 +4228,7 @@
         <v>-2329.3389999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="132">
         <v>-249.56</v>
       </c>
@@ -4236,7 +4236,7 @@
         <v>-2254.5149999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="132">
         <v>-241.62</v>
       </c>
@@ -4244,7 +4244,7 @@
         <v>-2178.2190000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="132">
         <v>-233.85</v>
       </c>
@@ -4252,7 +4252,7 @@
         <v>-2100.06</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="132">
         <v>-226.23</v>
       </c>
@@ -4260,7 +4260,7 @@
         <v>-2020.528</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="132">
         <v>-218.75</v>
       </c>
@@ -4268,7 +4268,7 @@
         <v>-1939.623</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="132">
         <v>-211.37</v>
       </c>
@@ -4276,7 +4276,7 @@
         <v>-1857.934</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="132">
         <v>-204.05</v>
       </c>
@@ -4284,7 +4284,7 @@
         <v>-1775.46</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="132">
         <v>-196.78</v>
       </c>
@@ -4292,7 +4292,7 @@
         <v>-1692.79</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="132">
         <v>-189.52</v>
       </c>
@@ -4300,7 +4300,7 @@
         <v>-1609.923</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="132">
         <v>-182.26</v>
       </c>
@@ -4308,7 +4308,7 @@
         <v>-1527.155</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="132">
         <v>-174.97</v>
       </c>
@@ -4316,7 +4316,7 @@
         <v>-1444.681</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="132">
         <v>-167.65</v>
       </c>
@@ -4324,7 +4324,7 @@
         <v>-1362.502</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="132">
         <v>-160.27000000000001</v>
       </c>
@@ -4332,7 +4332,7 @@
         <v>-1280.8119999999999</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" s="132">
         <v>-152.82</v>
       </c>
@@ -4340,7 +4340,7 @@
         <v>-1199.711</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="132">
         <v>-145.29</v>
       </c>
@@ -4348,7 +4348,7 @@
         <v>-1119.297</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="132">
         <v>-137.65</v>
       </c>
@@ -4356,7 +4356,7 @@
         <v>-1039.7650000000001</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" s="132">
         <v>-129.9</v>
       </c>
@@ -4364,7 +4364,7 @@
         <v>-961.31200000000001</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="132">
         <v>-122.02</v>
       </c>
@@ -4372,7 +4372,7 @@
         <v>-884.13300000000004</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" s="132">
         <v>-114.01</v>
       </c>
@@ -4380,7 +4380,7 @@
         <v>-808.32799999999997</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" s="132">
         <v>-105.84</v>
       </c>
@@ -4388,7 +4388,7 @@
         <v>-734.19</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" s="132">
         <v>-97.52</v>
       </c>
@@ -4396,7 +4396,7 @@
         <v>-661.71799999999996</v>
       </c>
     </row>
-    <row r="45" spans="1:2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" s="132">
         <v>-89.05</v>
       </c>
@@ -4404,7 +4404,7 @@
         <v>-590.91399999999999</v>
       </c>
     </row>
-    <row r="46" spans="1:2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="132">
         <v>-80.430000000000007</v>
       </c>
@@ -4412,7 +4412,7 @@
         <v>-521.67999999999995</v>
       </c>
     </row>
-    <row r="47" spans="1:2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="132">
         <v>-71.680000000000007</v>
       </c>
@@ -4420,7 +4420,7 @@
         <v>-454.21</v>
       </c>
     </row>
-    <row r="48" spans="1:2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="132">
         <v>-62.8</v>
       </c>
@@ -4428,7 +4428,7 @@
         <v>-388.113</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="132">
         <v>-53.8</v>
       </c>
@@ -4436,7 +4436,7 @@
         <v>-323.68299999999999</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="132">
         <v>-44.68</v>
       </c>
@@ -4444,7 +4444,7 @@
         <v>-260.92099999999999</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" s="132">
         <v>-35.409999999999997</v>
       </c>
@@ -4452,7 +4452,7 @@
         <v>-200.41399999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="132">
         <v>-25.99</v>
       </c>
@@ -4460,7 +4460,7 @@
         <v>-142.26</v>
       </c>
     </row>
-    <row r="53" spans="1:2">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" s="132">
         <v>-16.38</v>
       </c>
@@ -4468,7 +4468,7 @@
         <v>-86.950999999999993</v>
       </c>
     </row>
-    <row r="54" spans="1:2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" s="132">
         <v>-6.61</v>
       </c>
@@ -4476,7 +4476,7 @@
         <v>-34.387</v>
       </c>
     </row>
-    <row r="55" spans="1:2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" s="132">
         <v>0</v>
       </c>
@@ -4484,7 +4484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:2">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" s="132">
         <v>3.23</v>
       </c>
@@ -4492,7 +4492,7 @@
         <v>16.803999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:2">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" s="132">
         <v>13.04</v>
       </c>
@@ -4500,7 +4500,7 @@
         <v>68.484999999999999</v>
       </c>
     </row>
-    <row r="58" spans="1:2">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" s="132">
         <v>22.71</v>
       </c>
@@ -4508,7 +4508,7 @@
         <v>122.42100000000001</v>
       </c>
     </row>
-    <row r="59" spans="1:2">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" s="132">
         <v>32.119999999999997</v>
       </c>
@@ -4516,7 +4516,7 @@
         <v>180.18199999999999</v>
       </c>
     </row>
-    <row r="60" spans="1:2">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" s="132">
         <v>41.25</v>
       </c>
@@ -4524,7 +4524,7 @@
         <v>242.25899999999999</v>
       </c>
     </row>
-    <row r="61" spans="1:2">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" s="132">
         <v>50.17</v>
       </c>
@@ -4532,7 +4532,7 @@
         <v>307.66899999999998</v>
       </c>
     </row>
-    <row r="62" spans="1:2">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" s="132">
         <v>58.93</v>
       </c>
@@ -4540,7 +4540,7 @@
         <v>375.33499999999998</v>
       </c>
     </row>
-    <row r="63" spans="1:2">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" s="132">
         <v>67.61</v>
       </c>
@@ -4548,7 +4548,7 @@
         <v>444.07900000000001</v>
       </c>
     </row>
-    <row r="64" spans="1:2">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" s="132">
         <v>76.28</v>
       </c>
@@ -4556,7 +4556,7 @@
         <v>512.92200000000003</v>
       </c>
     </row>
-    <row r="65" spans="1:2">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" s="132">
         <v>84.97</v>
       </c>
@@ -4564,7 +4564,7 @@
         <v>581.274</v>
       </c>
     </row>
-    <row r="66" spans="1:2">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" s="132">
         <v>93.66</v>
       </c>
@@ -4572,7 +4572,7 @@
         <v>649.33299999999997</v>
       </c>
     </row>
-    <row r="67" spans="1:2">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" s="132">
         <v>102.34</v>
       </c>
@@ -4580,7 +4580,7 @@
         <v>717.58699999999999</v>
       </c>
     </row>
-    <row r="68" spans="1:2">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" s="132">
         <v>110.99</v>
       </c>
@@ -4588,7 +4588,7 @@
         <v>786.23299999999995</v>
       </c>
     </row>
-    <row r="69" spans="1:2">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" s="132">
         <v>119.59</v>
       </c>
@@ -4596,7 +4596,7 @@
         <v>855.66399999999999</v>
       </c>
     </row>
-    <row r="70" spans="1:2">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" s="132">
         <v>128.15</v>
       </c>
@@ -4604,7 +4604,7 @@
         <v>925.68399999999997</v>
       </c>
     </row>
-    <row r="71" spans="1:2">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" s="132">
         <v>136.76</v>
       </c>
@@ -4612,7 +4612,7 @@
         <v>995.11500000000001</v>
       </c>
     </row>
-    <row r="72" spans="1:2">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" s="132">
         <v>145.5</v>
       </c>
@@ -4620,7 +4620,7 @@
         <v>1062.8789999999999</v>
       </c>
     </row>
-    <row r="73" spans="1:2">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" s="132">
         <v>154.46</v>
       </c>
@@ -4628,7 +4628,7 @@
         <v>1127.6030000000001</v>
       </c>
     </row>
-    <row r="74" spans="1:2">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A74" s="132">
         <v>163.72</v>
       </c>
@@ -4636,7 +4636,7 @@
         <v>1188.1099999999999</v>
       </c>
     </row>
-    <row r="75" spans="1:2">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A75" s="132">
         <v>173.35</v>
       </c>
@@ -4644,7 +4644,7 @@
         <v>1243.3209999999999</v>
       </c>
     </row>
-    <row r="76" spans="1:2">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A76" s="132">
         <v>183.3</v>
       </c>
@@ -4652,7 +4652,7 @@
         <v>1293.0409999999999</v>
       </c>
     </row>
-    <row r="77" spans="1:2">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A77" s="132">
         <v>193.53</v>
       </c>
@@ -4660,7 +4660,7 @@
         <v>1336.877</v>
       </c>
     </row>
-    <row r="78" spans="1:2">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A78" s="132">
         <v>204</v>
       </c>
@@ -4668,7 +4668,7 @@
         <v>1374.829</v>
       </c>
     </row>
-    <row r="79" spans="1:2">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A79" s="132">
         <v>214.66</v>
       </c>
@@ -4676,7 +4676,7 @@
         <v>1406.7</v>
       </c>
     </row>
-    <row r="80" spans="1:2">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A80" s="132">
         <v>225.46</v>
       </c>
@@ -4684,7 +4684,7 @@
         <v>1433.2760000000001</v>
       </c>
     </row>
-    <row r="81" spans="1:2">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A81" s="132">
         <v>236.35</v>
       </c>
@@ -4692,7 +4692,7 @@
         <v>1455.93</v>
       </c>
     </row>
-    <row r="82" spans="1:2">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A82" s="132">
         <v>247.31</v>
       </c>
@@ -4700,7 +4700,7 @@
         <v>1476.0329999999999</v>
       </c>
     </row>
-    <row r="83" spans="1:2">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A83" s="132">
         <v>258.27999999999997</v>
       </c>
@@ -4708,7 +4708,7 @@
         <v>1494.8620000000001</v>
       </c>
     </row>
-    <row r="84" spans="1:2">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A84" s="132">
         <v>269.26</v>
       </c>
@@ -4716,7 +4716,7 @@
         <v>1513.396</v>
       </c>
     </row>
-    <row r="85" spans="1:2">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A85" s="132">
         <v>280.23</v>
       </c>
@@ -4724,7 +4724,7 @@
         <v>1531.8330000000001</v>
       </c>
     </row>
-    <row r="86" spans="1:2">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A86" s="132">
         <v>291.19</v>
       </c>
@@ -4732,7 +4732,7 @@
         <v>1550.3679999999999</v>
       </c>
     </row>
-    <row r="87" spans="1:2">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A87" s="132">
         <v>302.14999999999998</v>
       </c>
@@ -4740,7 +4740,7 @@
         <v>1569.2940000000001</v>
       </c>
     </row>
-    <row r="88" spans="1:2">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A88" s="132">
         <v>313.10000000000002</v>
       </c>
@@ -4748,7 +4748,7 @@
         <v>1588.712</v>
       </c>
     </row>
-    <row r="89" spans="1:2">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A89" s="132">
         <v>324.05</v>
       </c>
@@ -4756,7 +4756,7 @@
         <v>1608.325</v>
       </c>
     </row>
-    <row r="90" spans="1:2">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A90" s="132">
         <v>335.01</v>
       </c>
@@ -4764,7 +4764,7 @@
         <v>1627.9380000000001</v>
       </c>
     </row>
-    <row r="91" spans="1:2">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A91" s="132">
         <v>345.96</v>
       </c>
@@ -4772,7 +4772,7 @@
         <v>1647.2570000000001</v>
       </c>
     </row>
-    <row r="92" spans="1:2">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A92" s="132">
         <v>356.92</v>
       </c>
@@ -4780,7 +4780,7 @@
         <v>1666.2819999999999</v>
       </c>
     </row>
-    <row r="93" spans="1:2">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A93" s="132">
         <v>367.88</v>
       </c>
@@ -4788,7 +4788,7 @@
         <v>1685.6010000000001</v>
       </c>
     </row>
-    <row r="94" spans="1:2">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" s="132">
         <v>378.83</v>
       </c>
@@ -4796,7 +4796,7 @@
         <v>1705.4110000000001</v>
       </c>
     </row>
-    <row r="95" spans="1:2">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" s="132">
         <v>389.75</v>
       </c>
@@ -4804,7 +4804,7 @@
         <v>1726.3969999999999</v>
       </c>
     </row>
-    <row r="96" spans="1:2">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" s="132">
         <v>400.65</v>
       </c>
@@ -4812,7 +4812,7 @@
         <v>1748.6579999999999</v>
       </c>
     </row>
-    <row r="97" spans="1:2">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" s="132">
         <v>411.52</v>
       </c>
@@ -4820,7 +4820,7 @@
         <v>1772.39</v>
       </c>
     </row>
-    <row r="98" spans="1:2">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A98" s="132">
         <v>422.35</v>
       </c>
@@ -4828,7 +4828,7 @@
         <v>1797.4949999999999</v>
       </c>
     </row>
-    <row r="99" spans="1:2">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A99" s="132">
         <v>433.15</v>
       </c>
@@ -4836,7 +4836,7 @@
         <v>1823.973</v>
       </c>
     </row>
-    <row r="100" spans="1:2">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A100" s="132">
         <v>443.91</v>
       </c>
@@ -4844,7 +4844,7 @@
         <v>1851.8240000000001</v>
       </c>
     </row>
-    <row r="101" spans="1:2">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A101" s="132">
         <v>454.66</v>
       </c>
@@ -4860,16 +4860,16 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF15C171-B68F-9245-AAB8-281BA0072F89}">
   <dimension ref="A1:E18"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.28515625" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" customWidth="1"/>
-    <col min="3" max="3" width="39.140625" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
-    <col min="5" max="5" width="73.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.33203125" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+    <col min="3" max="3" width="39.1640625" customWidth="1"/>
+    <col min="4" max="4" width="12.5" customWidth="1"/>
+    <col min="5" max="5" width="73.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.95" thickBot="1">
+    <row r="1" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -4884,7 +4884,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.95" thickBot="1">
+    <row r="2" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -4895,7 +4895,7 @@
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" ht="15.95" thickBot="1">
+    <row r="3" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -4906,7 +4906,7 @@
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" ht="15.95" thickBot="1">
+    <row r="4" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -4917,24 +4917,24 @@
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" ht="17.100000000000001" thickBot="1">
+    <row r="5" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="91" t="s">
         <v>136</v>
       </c>
       <c r="B5" s="73"/>
       <c r="C5" s="120" t="s">
+        <v>182</v>
+      </c>
+      <c r="D5" s="102" t="s">
         <v>137</v>
       </c>
-      <c r="D5" s="102" t="s">
+      <c r="E5" s="103" t="s">
         <v>138</v>
       </c>
-      <c r="E5" s="103" t="s">
+    </row>
+    <row r="6" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="91" t="s">
         <v>139</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="17.100000000000001" thickBot="1">
-      <c r="A6" s="91" t="s">
-        <v>140</v>
       </c>
       <c r="B6" s="73"/>
       <c r="C6" s="99">
@@ -4945,35 +4945,35 @@
       </c>
       <c r="E6" s="28"/>
     </row>
-    <row r="7" spans="1:5" ht="17.100000000000001" thickBot="1">
+    <row r="7" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="91" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B7" s="73"/>
       <c r="C7" s="99" t="s">
+        <v>141</v>
+      </c>
+      <c r="D7" s="102" t="s">
         <v>142</v>
       </c>
-      <c r="D7" s="102" t="s">
+      <c r="E7" s="28"/>
+    </row>
+    <row r="8" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="91" t="s">
         <v>143</v>
-      </c>
-      <c r="E7" s="28"/>
-    </row>
-    <row r="8" spans="1:5" ht="17.100000000000001" thickBot="1">
-      <c r="A8" s="91" t="s">
-        <v>144</v>
       </c>
       <c r="B8" s="73"/>
       <c r="C8" s="104" t="s">
+        <v>144</v>
+      </c>
+      <c r="D8" s="102" t="s">
+        <v>137</v>
+      </c>
+      <c r="E8" s="28"/>
+    </row>
+    <row r="9" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="91" t="s">
         <v>145</v>
-      </c>
-      <c r="D8" s="102" t="s">
-        <v>138</v>
-      </c>
-      <c r="E8" s="28"/>
-    </row>
-    <row r="9" spans="1:5" ht="17.100000000000001" thickBot="1">
-      <c r="A9" s="91" t="s">
-        <v>146</v>
       </c>
       <c r="B9" s="73"/>
       <c r="C9" s="99">
@@ -4982,38 +4982,38 @@
       <c r="D9" s="102"/>
       <c r="E9" s="28"/>
     </row>
-    <row r="10" spans="1:5" ht="17.100000000000001" thickBot="1">
+    <row r="10" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="91" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B10" s="73"/>
       <c r="C10" s="99">
         <v>0.01</v>
       </c>
       <c r="D10" s="102" t="s">
+        <v>147</v>
+      </c>
+      <c r="E10" s="103" t="s">
         <v>148</v>
       </c>
-      <c r="E10" s="103" t="s">
+    </row>
+    <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="155" t="s">
         <v>149</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="17.100000000000001" customHeight="1">
-      <c r="A11" s="143" t="s">
-        <v>150</v>
       </c>
       <c r="B11" s="105" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="106" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D11" s="90"/>
       <c r="E11" s="70"/>
     </row>
-    <row r="12" spans="1:5" ht="15.95" thickBot="1">
-      <c r="A12" s="159"/>
+    <row r="12" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="167"/>
       <c r="B12" s="107" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C12" s="108" t="s">
         <v>11</v>
@@ -5023,33 +5023,33 @@
       </c>
       <c r="E12" s="110"/>
     </row>
-    <row r="13" spans="1:5" ht="17.100000000000001" thickBot="1">
+    <row r="13" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="91" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B13" s="73"/>
       <c r="C13" s="99" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D13" s="102"/>
       <c r="E13" s="103" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="91" t="s">
         <v>155</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="15.95">
-      <c r="A14" s="91" t="s">
-        <v>156</v>
       </c>
       <c r="B14" s="73"/>
       <c r="C14" s="99" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D14" s="102"/>
       <c r="E14" s="103"/>
     </row>
-    <row r="18" spans="4:4">
+    <row r="18" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D18" s="135" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -5066,30 +5066,30 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultColWidth="16.28515625" defaultRowHeight="15.6" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="15.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" style="1" customWidth="1"/>
-    <col min="2" max="5" width="16.28515625" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="16.28515625" style="1"/>
+    <col min="1" max="1" width="28.5" style="1" customWidth="1"/>
+    <col min="2" max="5" width="16.33203125" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="16.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13.35" customHeight="1">
+    <row r="1" spans="1:5" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B1" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="C1" s="30" t="s">
         <v>160</v>
       </c>
-      <c r="C1" s="30" t="s">
+      <c r="D1" s="30" t="s">
         <v>161</v>
       </c>
-      <c r="D1" s="30" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="31" t="s">
         <v>162</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="13.35" customHeight="1">
-      <c r="A2" s="31" t="s">
-        <v>163</v>
       </c>
       <c r="B2" s="32">
         <v>200</v>
@@ -5101,9 +5101,9 @@
         <v>76.349999999999994</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="12.95" customHeight="1">
+    <row r="3" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="34" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B3" s="35">
         <v>-196</v>
@@ -5115,9 +5115,9 @@
         <v>76.349999999999994</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="12.95" customHeight="1">
+    <row r="4" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="34" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B4" s="35">
         <v>11.981999999999999</v>
@@ -5129,9 +5129,9 @@
         <v>152.5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="12.95" customHeight="1">
+    <row r="5" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="34" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B5" s="35">
         <v>152.88200000000001</v>
@@ -5143,9 +5143,9 @@
         <v>271.78199999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="12.95" customHeight="1">
+    <row r="6" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="34" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B6" s="35">
         <v>-180.72900000000001</v>
@@ -5157,9 +5157,9 @@
         <v>250.89400000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="12.95" customHeight="1">
+    <row r="7" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="34" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B7" s="35">
         <v>-12.087</v>
@@ -5171,38 +5171,38 @@
         <v>381.5</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="12.95" customHeight="1">
+    <row r="8" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="34" t="s">
+        <v>168</v>
+      </c>
+      <c r="B8" s="141">
+        <v>16.809999999999999</v>
+      </c>
+      <c r="C8" s="142">
+        <v>582.16999999999996</v>
+      </c>
+      <c r="D8" s="142">
+        <v>281.08999999999997</v>
+      </c>
+      <c r="E8" s="143"/>
+    </row>
+    <row r="9" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="B8" s="164">
-        <v>16.809999999999999</v>
-      </c>
-      <c r="C8" s="165">
-        <v>582.16999999999996</v>
-      </c>
-      <c r="D8" s="165">
-        <v>281.08999999999997</v>
-      </c>
-      <c r="E8" s="166"/>
-    </row>
-    <row r="9" spans="1:5" ht="12.95" customHeight="1">
-      <c r="A9" s="34" t="s">
+      <c r="B9" s="141">
+        <v>0</v>
+      </c>
+      <c r="C9" s="142">
+        <v>640</v>
+      </c>
+      <c r="D9" s="142">
+        <v>266.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="34" t="s">
         <v>170</v>
-      </c>
-      <c r="B9" s="164">
-        <v>0</v>
-      </c>
-      <c r="C9" s="165">
-        <v>640</v>
-      </c>
-      <c r="D9" s="165">
-        <v>266.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="12.95" customHeight="1">
-      <c r="A10" s="34" t="s">
-        <v>171</v>
       </c>
       <c r="B10" s="35">
         <v>105.45399999999999</v>
@@ -5214,9 +5214,9 @@
         <v>126.39700000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="12.95" customHeight="1">
+    <row r="11" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="34" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B11" s="35">
         <v>86.251999999999995</v>
@@ -5228,9 +5228,9 @@
         <v>206.5</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="12.95" customHeight="1">
+    <row r="12" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="34" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B12" s="35">
         <v>7.8460000000000001</v>
@@ -5242,9 +5242,9 @@
         <v>468.06400000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="12.95" customHeight="1">
+    <row r="13" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="34" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B13" s="35">
         <v>9.5190000000000001</v>
@@ -5256,9 +5256,9 @@
         <v>312.06599999999997</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="13.5" customHeight="1">
+    <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="34" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B14" s="35">
         <v>11.606999999999999</v>
@@ -5270,9 +5270,9 @@
         <v>173.935</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="12.95" customHeight="1">
+    <row r="15" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B15" s="35">
         <v>9.5399999999999991</v>
@@ -5284,9 +5284,9 @@
         <v>310.57900000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="12.95" customHeight="1">
+    <row r="16" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="34" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B16" s="35">
         <v>9.9</v>
@@ -5298,9 +5298,9 @@
         <v>277.83600000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="12.95" customHeight="1">
+    <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="34" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B17" s="35">
         <v>-7</v>
@@ -5312,9 +5312,9 @@
         <v>51.518999999999998</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="12.95" customHeight="1">
+    <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="34" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B18" s="35">
         <v>-67.747</v>
@@ -5326,9 +5326,9 @@
         <v>51.353999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="12.95" customHeight="1">
+    <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="34" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B19" s="35">
         <v>9.74</v>
@@ -5340,9 +5340,9 @@
         <v>292.45299999999997</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="12.95" customHeight="1">
+    <row r="20" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="34" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B20" s="35">
         <v>105.45399999999999</v>
@@ -5354,17 +5354,17 @@
         <v>126.39700000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="12.95" customHeight="1">
+    <row r="21" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="34" t="s">
-        <v>182</v>
-      </c>
-      <c r="B21" s="164">
+        <v>181</v>
+      </c>
+      <c r="B21" s="141">
         <v>-324.96499999999997</v>
       </c>
-      <c r="C21" s="165">
+      <c r="C21" s="142">
         <v>0</v>
       </c>
-      <c r="D21" s="165">
+      <c r="D21" s="142">
         <v>533.79200000000003</v>
       </c>
     </row>
@@ -5383,30 +5383,30 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultColWidth="16.28515625" defaultRowHeight="15.6" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="15.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.42578125" style="1" customWidth="1"/>
-    <col min="2" max="5" width="16.28515625" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="16.28515625" style="1"/>
+    <col min="1" max="1" width="31.5" style="1" customWidth="1"/>
+    <col min="2" max="5" width="16.33203125" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="16.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="13.35" customHeight="1">
+    <row r="1" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B1" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="C1" s="30" t="s">
         <v>160</v>
       </c>
-      <c r="C1" s="30" t="s">
+      <c r="D1" s="30" t="s">
         <v>161</v>
       </c>
-      <c r="D1" s="30" t="s">
+    </row>
+    <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="31" t="s">
         <v>162</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="13.35" customHeight="1">
-      <c r="A2" s="31" t="s">
-        <v>163</v>
       </c>
       <c r="B2" s="32">
         <v>-1390</v>
@@ -5418,9 +5418,9 @@
         <v>111.35</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="12.95" customHeight="1">
+    <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="34" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B3" s="35">
         <v>-1830</v>
@@ -5432,9 +5432,9 @@
         <v>111.35</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="12.95" customHeight="1">
+    <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="34" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B4" s="35">
         <v>-1579.278</v>
@@ -5446,9 +5446,9 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="12.95" customHeight="1">
+    <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="34" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B5" s="35">
         <v>-1390</v>
@@ -5460,9 +5460,9 @@
         <v>313.98099999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="12.95" customHeight="1">
+    <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="34" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B6" s="35">
         <v>-1830</v>
@@ -5474,9 +5474,9 @@
         <v>339.47500000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="12.95" customHeight="1">
+    <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="34" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B7" s="35">
         <v>-1570.7049999999999</v>
@@ -5488,37 +5488,37 @@
         <v>389.5</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="12.95" customHeight="1">
+    <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="34" t="s">
+        <v>168</v>
+      </c>
+      <c r="B8" s="141">
+        <v>-1569.287</v>
+      </c>
+      <c r="C8" s="142">
+        <v>568.86300000000006</v>
+      </c>
+      <c r="D8" s="142">
+        <v>272.678</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="B8" s="164">
-        <v>-1569.287</v>
-      </c>
-      <c r="C8" s="165">
-        <v>568.86300000000006</v>
-      </c>
-      <c r="D8" s="165">
-        <v>272.678</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="12.95" customHeight="1">
-      <c r="A9" s="34" t="s">
+      <c r="B9" s="141">
+        <v>-1575</v>
+      </c>
+      <c r="C9" s="142">
+        <v>625</v>
+      </c>
+      <c r="D9" s="142">
+        <v>266.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="34" t="s">
         <v>170</v>
-      </c>
-      <c r="B9" s="164">
-        <v>-1575</v>
-      </c>
-      <c r="C9" s="165">
-        <v>625</v>
-      </c>
-      <c r="D9" s="165">
-        <v>266.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="12.95" customHeight="1">
-      <c r="A10" s="34" t="s">
-        <v>171</v>
       </c>
       <c r="B10" s="35">
         <v>-1830</v>
@@ -5530,9 +5530,9 @@
         <v>178.642</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="12.95" customHeight="1">
+    <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="34" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B11" s="35">
         <v>-1676.222</v>
@@ -5544,9 +5544,9 @@
         <v>231.5</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="12.95" customHeight="1">
+    <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="34" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B12" s="35">
         <v>-1398.8620000000001</v>
@@ -5558,9 +5558,9 @@
         <v>421.80700000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="12.95" customHeight="1">
+    <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="34" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B13" s="35">
         <v>-1582.4280000000001</v>
@@ -5572,9 +5572,9 @@
         <v>466.95600000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="12.95" customHeight="1">
+    <row r="14" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="34" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B14" s="35">
         <v>-1598.432</v>
@@ -5586,9 +5586,9 @@
         <v>164.11600000000001</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="12.95" customHeight="1">
+    <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B15" s="35">
         <v>-1663.0229999999999</v>
@@ -5600,9 +5600,9 @@
         <v>387.30799999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="12.95" customHeight="1">
+    <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="34" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B16" s="35">
         <v>-1585.771</v>
@@ -5614,9 +5614,9 @@
         <v>411.35</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="12.95" customHeight="1">
+    <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="34" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B17" s="35">
         <v>-1830</v>
@@ -5628,9 +5628,9 @@
         <v>444.35</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="12.95" customHeight="1">
+    <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="34" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B18" s="35">
         <v>-1830</v>
@@ -5642,9 +5642,9 @@
         <v>386.35</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="12.95" customHeight="1">
+    <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="34" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B19" s="35">
         <v>-1602.577</v>
@@ -5668,18 +5668,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="37.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="6.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="50.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="24.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="37.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="50.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5696,7 +5696,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.1" customHeight="1">
+    <row r="2" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -5705,7 +5705,7 @@
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" ht="14.1" customHeight="1">
+    <row r="3" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -5714,7 +5714,7 @@
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="4" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -5725,7 +5725,7 @@
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="5" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>37</v>
       </c>
@@ -5738,7 +5738,7 @@
       </c>
       <c r="E5" s="114"/>
     </row>
-    <row r="6" spans="1:5" ht="14.45" customHeight="1" thickBot="1">
+    <row r="6" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>40</v>
       </c>
@@ -5751,7 +5751,7 @@
       </c>
       <c r="E6" s="22"/>
     </row>
-    <row r="7" spans="1:5" ht="14.45" customHeight="1" thickBot="1">
+    <row r="7" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>42</v>
       </c>
@@ -5776,15 +5776,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23B3B35C-CB70-D641-97B1-CD6FD7CCE140}">
   <dimension ref="A1:E35"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" customWidth="1"/>
-    <col min="5" max="5" width="50.28515625" customWidth="1"/>
+    <col min="3" max="3" width="33.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="50.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1">
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5801,7 +5801,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="1" customFormat="1" ht="14.1" customHeight="1" thickBot="1">
+    <row r="2" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -5812,7 +5812,7 @@
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" s="1" customFormat="1" ht="14.1" customHeight="1" thickBot="1">
+    <row r="3" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -5823,7 +5823,7 @@
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" s="1" customFormat="1" ht="14.1" customHeight="1" thickBot="1">
+    <row r="4" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -5834,8 +5834,8 @@
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" s="1" customFormat="1" ht="14.1" customHeight="1">
-      <c r="A5" s="151" t="s">
+    <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="147" t="s">
         <v>45</v>
       </c>
       <c r="B5" s="73" t="s">
@@ -5852,8 +5852,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1">
-      <c r="A6" s="167"/>
+    <row r="6" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="145"/>
       <c r="B6" s="74" t="s">
         <v>48</v>
       </c>
@@ -5868,8 +5868,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1">
-      <c r="A7" s="168"/>
+    <row r="7" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="148"/>
       <c r="B7" s="74" t="s">
         <v>49</v>
       </c>
@@ -5884,8 +5884,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="1" customFormat="1" ht="14.1" customHeight="1" thickBot="1">
-      <c r="A8" s="168"/>
+    <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="148"/>
       <c r="B8" s="77" t="s">
         <v>12</v>
       </c>
@@ -5897,8 +5897,8 @@
       </c>
       <c r="E8" s="22"/>
     </row>
-    <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A9" s="152" t="s">
+    <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="149" t="s">
         <v>50</v>
       </c>
       <c r="B9" s="73" t="s">
@@ -5915,8 +5915,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A10" s="169"/>
+    <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="146"/>
       <c r="B10" s="74" t="s">
         <v>48</v>
       </c>
@@ -5931,8 +5931,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A11" s="169"/>
+    <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="146"/>
       <c r="B11" s="74" t="s">
         <v>49</v>
       </c>
@@ -5947,8 +5947,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A12" s="167"/>
+    <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="145"/>
       <c r="B12" s="77" t="s">
         <v>12</v>
       </c>
@@ -5962,8 +5962,8 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A13" s="153" t="s">
+    <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="150" t="s">
         <v>51</v>
       </c>
       <c r="B13" s="73" t="s">
@@ -5980,8 +5980,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A14" s="168"/>
+    <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="148"/>
       <c r="B14" s="74" t="s">
         <v>52</v>
       </c>
@@ -5996,8 +5996,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A15" s="168"/>
+    <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="148"/>
       <c r="B15" s="74" t="s">
         <v>12</v>
       </c>
@@ -6009,8 +6009,8 @@
       </c>
       <c r="E15" s="18"/>
     </row>
-    <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A16" s="170"/>
+    <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="151"/>
       <c r="B16" s="74" t="s">
         <v>53</v>
       </c>
@@ -6022,8 +6022,8 @@
       </c>
       <c r="E16" s="16"/>
     </row>
-    <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A17" s="169"/>
+    <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="146"/>
       <c r="B17" s="74" t="s">
         <v>55</v>
       </c>
@@ -6035,8 +6035,8 @@
       </c>
       <c r="E17" s="16"/>
     </row>
-    <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A18" s="169"/>
+    <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="146"/>
       <c r="B18" s="74" t="s">
         <v>56</v>
       </c>
@@ -6048,8 +6048,8 @@
       </c>
       <c r="E18" s="16"/>
     </row>
-    <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A19" s="169"/>
+    <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="146"/>
       <c r="B19" s="74" t="s">
         <v>57</v>
       </c>
@@ -6061,8 +6061,8 @@
       </c>
       <c r="E19" s="16"/>
     </row>
-    <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A20" s="167"/>
+    <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="145"/>
       <c r="B20" s="77" t="s">
         <v>58</v>
       </c>
@@ -6074,8 +6074,8 @@
       </c>
       <c r="E20" s="22"/>
     </row>
-    <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A21" s="150" t="s">
+    <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="144" t="s">
         <v>59</v>
       </c>
       <c r="B21" s="73" t="s">
@@ -6092,8 +6092,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A22" s="169"/>
+    <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="146"/>
       <c r="B22" s="14" t="s">
         <v>49</v>
       </c>
@@ -6108,8 +6108,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A23" s="167"/>
+    <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="145"/>
       <c r="B23" s="19" t="s">
         <v>12</v>
       </c>
@@ -6121,8 +6121,8 @@
       </c>
       <c r="E23" s="22"/>
     </row>
-    <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A24" s="150" t="s">
+    <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="144" t="s">
         <v>61</v>
       </c>
       <c r="B24" s="73" t="s">
@@ -6139,8 +6139,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A25" s="169"/>
+    <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="146"/>
       <c r="B25" s="74" t="s">
         <v>63</v>
       </c>
@@ -6155,8 +6155,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A26" s="171"/>
+    <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="152"/>
       <c r="B26" s="78" t="s">
         <v>64</v>
       </c>
@@ -6168,8 +6168,8 @@
       </c>
       <c r="E26" s="81"/>
     </row>
-    <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A27" s="167"/>
+    <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="145"/>
       <c r="B27" s="77" t="s">
         <v>65</v>
       </c>
@@ -6181,8 +6181,8 @@
       </c>
       <c r="E27" s="22"/>
     </row>
-    <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A28" s="150" t="s">
+    <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="144" t="s">
         <v>66</v>
       </c>
       <c r="B28" s="73" t="s">
@@ -6196,8 +6196,8 @@
       </c>
       <c r="E28" s="13"/>
     </row>
-    <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A29" s="167"/>
+    <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="145"/>
       <c r="B29" s="77" t="s">
         <v>68</v>
       </c>
@@ -6209,8 +6209,8 @@
       </c>
       <c r="E29" s="22"/>
     </row>
-    <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A30" s="150" t="s">
+    <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="144" t="s">
         <v>69</v>
       </c>
       <c r="B30" s="87" t="s">
@@ -6227,8 +6227,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A31" s="169"/>
+    <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="146"/>
       <c r="B31" s="88" t="s">
         <v>49</v>
       </c>
@@ -6243,8 +6243,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A32" s="167"/>
+    <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="145"/>
       <c r="B32" s="89" t="s">
         <v>12</v>
       </c>
@@ -6256,8 +6256,8 @@
       </c>
       <c r="E32" s="22"/>
     </row>
-    <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A33" s="150" t="s">
+    <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="144" t="s">
         <v>70</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -6274,8 +6274,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A34" s="169"/>
+    <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="146"/>
       <c r="B34" s="14" t="s">
         <v>72</v>
       </c>
@@ -6290,8 +6290,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A35" s="167"/>
+    <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="145"/>
       <c r="B35" s="19" t="s">
         <v>12</v>
       </c>
@@ -6321,19 +6321,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="37.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="50.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="14.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="37.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="50.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="76.349999999999994" customHeight="1"/>
-    <row r="2" spans="1:5" ht="15" customHeight="1">
+    <row r="1" spans="1:5" ht="76.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -6350,7 +6350,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="14.1" customHeight="1">
+    <row r="3" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
@@ -6361,7 +6361,7 @@
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" ht="14.1" customHeight="1">
+    <row r="4" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>6</v>
       </c>
@@ -6372,7 +6372,7 @@
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="5" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>8</v>
       </c>
@@ -6383,7 +6383,7 @@
       <c r="D5" s="9"/>
       <c r="E5" s="10"/>
     </row>
-    <row r="6" spans="1:5" ht="13.5" customHeight="1">
+    <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="121" t="s">
         <v>75</v>
       </c>
@@ -6399,7 +6399,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="13.5" customHeight="1">
+    <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="122" t="s">
         <v>60</v>
       </c>
@@ -6415,7 +6415,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="13.5" customHeight="1">
+    <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="122" t="s">
         <v>49</v>
       </c>
@@ -6431,7 +6431,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="13.5" customHeight="1">
+    <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="122" t="s">
         <v>76</v>
       </c>
@@ -6445,7 +6445,7 @@
       </c>
       <c r="E9" s="16"/>
     </row>
-    <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
+    <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="123" t="s">
         <v>12</v>
       </c>
@@ -6470,18 +6470,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="50.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="14.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="50.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -6498,7 +6498,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.1" customHeight="1">
+    <row r="2" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -6509,7 +6509,7 @@
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" ht="14.1" customHeight="1">
+    <row r="3" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -6520,7 +6520,7 @@
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="4" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -6531,8 +6531,8 @@
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" ht="14.1" customHeight="1">
-      <c r="A5" s="143" t="s">
+    <row r="5" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="155" t="s">
         <v>80</v>
       </c>
       <c r="B5" s="73" t="s">
@@ -6549,8 +6549,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="14.1" customHeight="1">
-      <c r="A6" s="144"/>
+    <row r="6" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="156"/>
       <c r="B6" s="92" t="s">
         <v>12</v>
       </c>
@@ -6562,8 +6562,8 @@
       </c>
       <c r="E6" s="18"/>
     </row>
-    <row r="7" spans="1:5" ht="14.1" customHeight="1">
-      <c r="A7" s="145"/>
+    <row r="7" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="157"/>
       <c r="B7" s="74" t="s">
         <v>82</v>
       </c>
@@ -6575,8 +6575,8 @@
       </c>
       <c r="E7" s="15"/>
     </row>
-    <row r="8" spans="1:5" ht="14.1" customHeight="1">
-      <c r="A8" s="146" t="s">
+    <row r="8" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="158" t="s">
         <v>84</v>
       </c>
       <c r="B8" s="74" t="s">
@@ -6590,8 +6590,8 @@
       </c>
       <c r="E8" s="41"/>
     </row>
-    <row r="9" spans="1:5" ht="14.1" customHeight="1">
-      <c r="A9" s="147"/>
+    <row r="9" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="159"/>
       <c r="B9" s="74" t="s">
         <v>8</v>
       </c>
@@ -6601,8 +6601,8 @@
       <c r="D9" s="15"/>
       <c r="E9" s="41"/>
     </row>
-    <row r="10" spans="1:5" ht="14.1" customHeight="1">
-      <c r="A10" s="147"/>
+    <row r="10" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="159"/>
       <c r="B10" s="74" t="s">
         <v>12</v>
       </c>
@@ -6614,8 +6614,8 @@
       </c>
       <c r="E10" s="16"/>
     </row>
-    <row r="11" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
-      <c r="A11" s="142"/>
+    <row r="11" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="154"/>
       <c r="B11" s="74" t="s">
         <v>81</v>
       </c>
@@ -6630,8 +6630,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="14.45" customHeight="1">
-      <c r="A12" s="141" t="s">
+    <row r="12" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="153" t="s">
         <v>88</v>
       </c>
       <c r="B12" s="74" t="s">
@@ -6645,8 +6645,8 @@
       </c>
       <c r="E12" s="41"/>
     </row>
-    <row r="13" spans="1:5" ht="14.45" customHeight="1">
-      <c r="A13" s="147"/>
+    <row r="13" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="159"/>
       <c r="B13" s="74" t="s">
         <v>12</v>
       </c>
@@ -6658,8 +6658,8 @@
       </c>
       <c r="E13" s="41"/>
     </row>
-    <row r="14" spans="1:5" ht="14.45" customHeight="1">
-      <c r="A14" s="148"/>
+    <row r="14" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="160"/>
       <c r="B14" s="74" t="s">
         <v>81</v>
       </c>
@@ -6672,8 +6672,8 @@
       </c>
       <c r="E14" s="16"/>
     </row>
-    <row r="15" spans="1:5" ht="14.45" customHeight="1">
-      <c r="A15" s="149" t="s">
+    <row r="15" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="161" t="s">
         <v>90</v>
       </c>
       <c r="B15" s="74" t="s">
@@ -6687,8 +6687,8 @@
       </c>
       <c r="E15" s="15"/>
     </row>
-    <row r="16" spans="1:5" ht="14.45" customHeight="1" thickBot="1">
-      <c r="A16" s="142"/>
+    <row r="16" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="154"/>
       <c r="B16" s="74" t="s">
         <v>91</v>
       </c>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="E16" s="15"/>
     </row>
-    <row r="17" spans="1:5" ht="14.45" customHeight="1" thickBot="1">
+    <row r="17" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="138" t="s">
         <v>92</v>
       </c>
@@ -6716,8 +6716,8 @@
       </c>
       <c r="E17" s="15"/>
     </row>
-    <row r="18" spans="1:5" ht="14.1" customHeight="1">
-      <c r="A18" s="141" t="s">
+    <row r="18" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="153" t="s">
         <v>93</v>
       </c>
       <c r="B18" s="74" t="s">
@@ -6733,8 +6733,8 @@
         <v>96</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="14.45" customHeight="1" thickBot="1">
-      <c r="A19" s="142"/>
+    <row r="19" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="154"/>
       <c r="B19" s="74" t="s">
         <v>97</v>
       </c>
@@ -6767,18 +6767,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="37.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="50.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="14.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="37.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="50.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1" thickBot="1">
+    <row r="1" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -6795,7 +6795,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="2" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -6806,7 +6806,7 @@
       <c r="D2" s="9"/>
       <c r="E2" s="52"/>
     </row>
-    <row r="3" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="3" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -6817,7 +6817,7 @@
       <c r="D3" s="9"/>
       <c r="E3" s="52"/>
     </row>
-    <row r="4" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="4" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -6828,7 +6828,7 @@
       <c r="D4" s="9"/>
       <c r="E4" s="52"/>
     </row>
-    <row r="5" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="5" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>37</v>
       </c>
@@ -6841,7 +6841,7 @@
       </c>
       <c r="E5" s="117"/>
     </row>
-    <row r="6" spans="1:5" ht="14.45" customHeight="1" thickBot="1">
+    <row r="6" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>40</v>
       </c>
@@ -6854,8 +6854,8 @@
       </c>
       <c r="E6" s="22"/>
     </row>
-    <row r="7" spans="1:5" ht="14.45" customHeight="1" thickBot="1">
-      <c r="A7" s="154" t="s">
+    <row r="7" spans="1:5" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="162" t="s">
         <v>42</v>
       </c>
       <c r="B7" s="126" t="s">
@@ -6867,8 +6867,8 @@
       <c r="D7" s="116"/>
       <c r="E7" s="128"/>
     </row>
-    <row r="8" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
-      <c r="A8" s="155"/>
+    <row r="8" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="163"/>
       <c r="B8" s="126" t="s">
         <v>8</v>
       </c>
@@ -6893,16 +6893,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E45A869-B0F3-7240-9246-177BC72F43B2}">
   <dimension ref="A1:E35"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.28515625" customWidth="1"/>
-    <col min="5" max="5" width="50.28515625" customWidth="1"/>
+    <col min="3" max="3" width="38.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="50.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1">
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -6919,7 +6919,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="1" customFormat="1" ht="14.1" customHeight="1" thickBot="1">
+    <row r="2" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -6930,7 +6930,7 @@
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" s="1" customFormat="1" ht="14.1" customHeight="1" thickBot="1">
+    <row r="3" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -6941,7 +6941,7 @@
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" s="1" customFormat="1" ht="14.1" customHeight="1" thickBot="1">
+    <row r="4" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -6952,8 +6952,8 @@
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" s="1" customFormat="1" ht="14.1" customHeight="1" thickBot="1">
-      <c r="A5" s="154" t="s">
+    <row r="5" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="162" t="s">
         <v>45</v>
       </c>
       <c r="B5" s="73" t="s">
@@ -6970,8 +6970,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="1" customFormat="1" ht="15.95" thickBot="1">
-      <c r="A6" s="160"/>
+    <row r="6" spans="1:5" s="1" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="168"/>
       <c r="B6" s="74" t="s">
         <v>48</v>
       </c>
@@ -6986,8 +6986,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:5" s="1" customFormat="1">
-      <c r="A7" s="160"/>
+    <row r="7" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="168"/>
       <c r="B7" s="74" t="s">
         <v>49</v>
       </c>
@@ -7002,8 +7002,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="1" customFormat="1" ht="14.1" customHeight="1" thickBot="1">
-      <c r="A8" s="155"/>
+    <row r="8" spans="1:5" s="1" customFormat="1" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="163"/>
       <c r="B8" s="77" t="s">
         <v>12</v>
       </c>
@@ -7015,8 +7015,8 @@
       </c>
       <c r="E8" s="56"/>
     </row>
-    <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A9" s="161" t="s">
+    <row r="9" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="169" t="s">
         <v>50</v>
       </c>
       <c r="B9" s="73" t="s">
@@ -7033,8 +7033,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A10" s="162"/>
+    <row r="10" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="170"/>
       <c r="B10" s="74" t="s">
         <v>48</v>
       </c>
@@ -7049,8 +7049,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A11" s="162"/>
+    <row r="11" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="170"/>
       <c r="B11" s="74" t="s">
         <v>49</v>
       </c>
@@ -7065,8 +7065,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A12" s="163"/>
+    <row r="12" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="171"/>
       <c r="B12" s="77" t="s">
         <v>12</v>
       </c>
@@ -7080,8 +7080,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A13" s="143" t="s">
+    <row r="13" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="155" t="s">
         <v>51</v>
       </c>
       <c r="B13" s="73" t="s">
@@ -7098,8 +7098,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A14" s="144"/>
+    <row r="14" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="156"/>
       <c r="B14" s="74" t="s">
         <v>52</v>
       </c>
@@ -7114,8 +7114,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A15" s="144"/>
+    <row r="15" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="156"/>
       <c r="B15" s="74" t="s">
         <v>12</v>
       </c>
@@ -7127,8 +7127,8 @@
       </c>
       <c r="E15" s="62"/>
     </row>
-    <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A16" s="144"/>
+    <row r="16" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="156"/>
       <c r="B16" s="74" t="s">
         <v>53</v>
       </c>
@@ -7140,8 +7140,8 @@
       </c>
       <c r="E16" s="60"/>
     </row>
-    <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A17" s="144"/>
+    <row r="17" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="156"/>
       <c r="B17" s="74" t="s">
         <v>55</v>
       </c>
@@ -7153,8 +7153,8 @@
       </c>
       <c r="E17" s="63"/>
     </row>
-    <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A18" s="144"/>
+    <row r="18" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="156"/>
       <c r="B18" s="74" t="s">
         <v>56</v>
       </c>
@@ -7166,8 +7166,8 @@
       </c>
       <c r="E18" s="63"/>
     </row>
-    <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A19" s="144"/>
+    <row r="19" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="156"/>
       <c r="B19" s="74" t="s">
         <v>57</v>
       </c>
@@ -7179,8 +7179,8 @@
       </c>
       <c r="E19" s="63"/>
     </row>
-    <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A20" s="159"/>
+    <row r="20" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="167"/>
       <c r="B20" s="77" t="s">
         <v>58</v>
       </c>
@@ -7192,8 +7192,8 @@
       </c>
       <c r="E20" s="64"/>
     </row>
-    <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A21" s="143" t="s">
+    <row r="21" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="155" t="s">
         <v>59</v>
       </c>
       <c r="B21" s="73" t="s">
@@ -7210,8 +7210,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A22" s="144"/>
+    <row r="22" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="156"/>
       <c r="B22" s="14" t="s">
         <v>49</v>
       </c>
@@ -7226,8 +7226,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A23" s="159"/>
+    <row r="23" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="167"/>
       <c r="B23" s="19" t="s">
         <v>12</v>
       </c>
@@ -7239,8 +7239,8 @@
       </c>
       <c r="E23" s="66"/>
     </row>
-    <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A24" s="143" t="s">
+    <row r="24" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="155" t="s">
         <v>61</v>
       </c>
       <c r="B24" s="73" t="s">
@@ -7257,8 +7257,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A25" s="144"/>
+    <row r="25" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="156"/>
       <c r="B25" s="74" t="s">
         <v>63</v>
       </c>
@@ -7273,8 +7273,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A26" s="144"/>
+    <row r="26" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="156"/>
       <c r="B26" s="78" t="s">
         <v>65</v>
       </c>
@@ -7284,8 +7284,8 @@
       <c r="D26" s="79"/>
       <c r="E26" s="71"/>
     </row>
-    <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A27" s="159"/>
+    <row r="27" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="167"/>
       <c r="B27" s="77" t="s">
         <v>64</v>
       </c>
@@ -7297,8 +7297,8 @@
       </c>
       <c r="E27" s="67"/>
     </row>
-    <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A28" s="143" t="s">
+    <row r="28" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="155" t="s">
         <v>66</v>
       </c>
       <c r="B28" s="73" t="s">
@@ -7312,8 +7312,8 @@
       </c>
       <c r="E28" s="68"/>
     </row>
-    <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A29" s="159"/>
+    <row r="29" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="167"/>
       <c r="B29" s="77" t="s">
         <v>68</v>
       </c>
@@ -7325,8 +7325,8 @@
       </c>
       <c r="E29" s="67"/>
     </row>
-    <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A30" s="156" t="s">
+    <row r="30" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="164" t="s">
         <v>69</v>
       </c>
       <c r="B30" s="87" t="s">
@@ -7343,8 +7343,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A31" s="157"/>
+    <row r="31" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="165"/>
       <c r="B31" s="88" t="s">
         <v>60</v>
       </c>
@@ -7359,8 +7359,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A32" s="158"/>
+    <row r="32" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="166"/>
       <c r="B32" s="89" t="s">
         <v>12</v>
       </c>
@@ -7372,8 +7372,8 @@
       </c>
       <c r="E32" s="69"/>
     </row>
-    <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A33" s="143" t="s">
+    <row r="33" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="155" t="s">
         <v>70</v>
       </c>
       <c r="B33" s="11" t="s">
@@ -7390,8 +7390,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A34" s="144"/>
+    <row r="34" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="156"/>
       <c r="B34" s="14" t="s">
         <v>72</v>
       </c>
@@ -7406,8 +7406,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A35" s="159"/>
+    <row r="35" spans="1:5" s="1" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="167"/>
       <c r="B35" s="19" t="s">
         <v>12</v>
       </c>
@@ -7437,18 +7437,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="37.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="50.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="14.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="37.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="50.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -7465,7 +7465,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.1" customHeight="1">
+    <row r="2" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -7476,7 +7476,7 @@
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" ht="15" customHeight="1">
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -7487,7 +7487,7 @@
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" ht="15" customHeight="1" thickBot="1">
+    <row r="4" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -7498,7 +7498,7 @@
       <c r="D4" s="9"/>
       <c r="E4" s="70"/>
     </row>
-    <row r="5" spans="1:5" ht="13.5" customHeight="1">
+    <row r="5" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="121" t="s">
         <v>75</v>
       </c>
@@ -7514,7 +7514,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="13.5" customHeight="1">
+    <row r="6" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="122" t="s">
         <v>60</v>
       </c>
@@ -7530,7 +7530,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="13.5" customHeight="1">
+    <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="122" t="s">
         <v>49</v>
       </c>
@@ -7546,7 +7546,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="13.5" customHeight="1">
+    <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="122" t="s">
         <v>76</v>
       </c>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="E8" s="71"/>
     </row>
-    <row r="9" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
+    <row r="9" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="123" t="s">
         <v>12</v>
       </c>
@@ -7585,18 +7585,18 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="42.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.85546875" style="1"/>
+    <col min="1" max="1" width="14.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="42.5" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -7611,7 +7611,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.1" customHeight="1">
+    <row r="2" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -7622,7 +7622,7 @@
       <c r="D2" s="9"/>
       <c r="E2" s="10"/>
     </row>
-    <row r="3" spans="1:5" ht="14.1" customHeight="1">
+    <row r="3" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -7633,7 +7633,7 @@
       <c r="D3" s="9"/>
       <c r="E3" s="10"/>
     </row>
-    <row r="4" spans="1:5" ht="14.1" customHeight="1" thickBot="1">
+    <row r="4" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -7644,7 +7644,7 @@
       <c r="D4" s="9"/>
       <c r="E4" s="10"/>
     </row>
-    <row r="5" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
+    <row r="5" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="119" t="s">
         <v>108</v>
       </c>
@@ -7655,7 +7655,7 @@
       <c r="D5" s="12"/>
       <c r="E5" s="28"/>
     </row>
-    <row r="6" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
+    <row r="6" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="119" t="s">
         <v>109</v>
       </c>
@@ -7666,7 +7666,7 @@
       <c r="D6" s="15"/>
       <c r="E6" s="18"/>
     </row>
-    <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
+    <row r="7" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="119" t="s">
         <v>110</v>
       </c>
@@ -7679,7 +7679,7 @@
       </c>
       <c r="E7" s="18"/>
     </row>
-    <row r="8" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
+    <row r="8" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="119" t="s">
         <v>112</v>
       </c>
@@ -7692,7 +7692,7 @@
       </c>
       <c r="E8" s="18"/>
     </row>
-    <row r="9" spans="1:5" ht="13.5" customHeight="1" thickBot="1">
+    <row r="9" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="119" t="s">
         <v>114</v>
       </c>
@@ -7715,26 +7715,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009342B7EAA7728A4FA80A5CCAFE8D7EAF" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d037a5681ee6af0e7b5b5d0a2f99b20">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557458c-24b5-4c97-84ed-4c402655f54f" xmlns:ns3="72e3c584-9879-4b35-b9d8-6a248c93e240" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="966978c8b125399653e7c255ac8e342d" ns2:_="" ns3:_="">
     <xsd:import namespace="9557458c-24b5-4c97-84ed-4c402655f54f"/>
@@ -7995,14 +7975,60 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DD7EDCD-D7E5-429F-A499-76DDCD78D8B8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added - GGV sweep scripts - tire model plots scripts - improved tire model
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Chassis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/Vehicle_Model/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88977B5A-C91C-694E-AF6E-1D5B901CEA81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32436DAD-AE86-834A-96B0-C055C3929EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3920" yWindow="1880" windowWidth="34480" windowHeight="19400" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="184">
   <si>
     <t>Category</t>
   </si>
@@ -542,85 +542,88 @@
     <t>Slip</t>
   </si>
   <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Z</t>
+  </si>
+  <si>
+    <t>LowerWishbone  Front Pickup</t>
+  </si>
+  <si>
+    <t>LowerWishbone Rear Pickup</t>
+  </si>
+  <si>
+    <t>LowerWishbone Outboard</t>
+  </si>
+  <si>
+    <t>UpperWishbone Front Pickup</t>
+  </si>
+  <si>
+    <t>UpperWishbone Rear Pickup</t>
+  </si>
+  <si>
+    <t>UpperWishbone Outboard</t>
+  </si>
+  <si>
+    <t>Upright CoG</t>
+  </si>
+  <si>
+    <t>Wheel Center</t>
+  </si>
+  <si>
+    <t>trackrod Inboard</t>
+  </si>
+  <si>
+    <t>trackrod Outboard</t>
+  </si>
+  <si>
+    <t>Shock Chassis Mount</t>
+  </si>
+  <si>
+    <t>Shock Bottom</t>
+  </si>
+  <si>
+    <t>Pushrod Outboard</t>
+  </si>
+  <si>
+    <t>Pushrod Inboard</t>
+  </si>
+  <si>
+    <t>BC Pivot</t>
+  </si>
+  <si>
+    <t>ARB Cantilever Start</t>
+  </si>
+  <si>
+    <t>ARB Cantilever End</t>
+  </si>
+  <si>
+    <t>ARB to Bellcrank</t>
+  </si>
+  <si>
+    <t>Steer Rack</t>
+  </si>
+  <si>
+    <t>Steer Wheel</t>
+  </si>
+  <si>
+    <t>2 combined+turnslip</t>
+  </si>
+  <si>
     <t>1 combined</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>Z</t>
-  </si>
-  <si>
-    <t>LowerWishbone  Front Pickup</t>
-  </si>
-  <si>
-    <t>LowerWishbone Rear Pickup</t>
-  </si>
-  <si>
-    <t>LowerWishbone Outboard</t>
-  </si>
-  <si>
-    <t>UpperWishbone Front Pickup</t>
-  </si>
-  <si>
-    <t>UpperWishbone Rear Pickup</t>
-  </si>
-  <si>
-    <t>UpperWishbone Outboard</t>
-  </si>
-  <si>
-    <t>Upright CoG</t>
-  </si>
-  <si>
-    <t>Wheel Center</t>
-  </si>
-  <si>
-    <t>trackrod Inboard</t>
-  </si>
-  <si>
-    <t>trackrod Outboard</t>
-  </si>
-  <si>
-    <t>Shock Chassis Mount</t>
-  </si>
-  <si>
-    <t>Shock Bottom</t>
-  </si>
-  <si>
-    <t>Pushrod Outboard</t>
-  </si>
-  <si>
-    <t>Pushrod Inboard</t>
-  </si>
-  <si>
-    <t>BC Pivot</t>
-  </si>
-  <si>
-    <t>ARB Cantilever Start</t>
-  </si>
-  <si>
-    <t>ARB Cantilever End</t>
-  </si>
-  <si>
-    <t>ARB to Bellcrank</t>
-  </si>
-  <si>
-    <t>Steer Rack</t>
-  </si>
-  <si>
-    <t>Steer Wheel</t>
-  </si>
-  <si>
-    <t>which('Hoosier_R20B_20p5x7_R13_7in_12psi.tir')</t>
+    <t>which('Hoosier_R20B_20p5x7_R13_7in_v2.tir')</t>
   </si>
 </sst>
 </file>
@@ -4923,7 +4926,7 @@
       </c>
       <c r="B5" s="73"/>
       <c r="C5" s="120" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D5" s="102" t="s">
         <v>137</v>
@@ -5042,14 +5045,16 @@
       </c>
       <c r="B14" s="73"/>
       <c r="C14" s="99" t="s">
-        <v>156</v>
+        <v>182</v>
       </c>
       <c r="D14" s="102"/>
-      <c r="E14" s="103"/>
+      <c r="E14" s="103" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="18" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D18" s="135" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -5075,21 +5080,21 @@
   <sheetData>
     <row r="1" spans="1:5" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="30" t="s">
+        <v>157</v>
+      </c>
+      <c r="B1" s="30" t="s">
         <v>158</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="C1" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="C1" s="30" t="s">
+      <c r="D1" s="30" t="s">
         <v>160</v>
-      </c>
-      <c r="D1" s="30" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B2" s="32">
         <v>200</v>
@@ -5103,7 +5108,7 @@
     </row>
     <row r="3" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="34" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B3" s="35">
         <v>-196</v>
@@ -5117,7 +5122,7 @@
     </row>
     <row r="4" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="34" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B4" s="35">
         <v>11.981999999999999</v>
@@ -5131,7 +5136,7 @@
     </row>
     <row r="5" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="34" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B5" s="35">
         <v>152.88200000000001</v>
@@ -5145,7 +5150,7 @@
     </row>
     <row r="6" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="34" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B6" s="35">
         <v>-180.72900000000001</v>
@@ -5159,7 +5164,7 @@
     </row>
     <row r="7" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="34" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B7" s="35">
         <v>-12.087</v>
@@ -5173,7 +5178,7 @@
     </row>
     <row r="8" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="34" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B8" s="141">
         <v>16.809999999999999</v>
@@ -5188,7 +5193,7 @@
     </row>
     <row r="9" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="34" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B9" s="141">
         <v>0</v>
@@ -5202,7 +5207,7 @@
     </row>
     <row r="10" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="34" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B10" s="35">
         <v>105.45399999999999</v>
@@ -5216,7 +5221,7 @@
     </row>
     <row r="11" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="34" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B11" s="35">
         <v>86.251999999999995</v>
@@ -5230,7 +5235,7 @@
     </row>
     <row r="12" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="34" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B12" s="35">
         <v>7.8460000000000001</v>
@@ -5244,7 +5249,7 @@
     </row>
     <row r="13" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="34" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B13" s="35">
         <v>9.5190000000000001</v>
@@ -5258,7 +5263,7 @@
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="34" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B14" s="35">
         <v>11.606999999999999</v>
@@ -5272,7 +5277,7 @@
     </row>
     <row r="15" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="34" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B15" s="35">
         <v>9.5399999999999991</v>
@@ -5286,7 +5291,7 @@
     </row>
     <row r="16" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B16" s="35">
         <v>9.9</v>
@@ -5300,7 +5305,7 @@
     </row>
     <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="34" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B17" s="35">
         <v>-7</v>
@@ -5314,7 +5319,7 @@
     </row>
     <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="34" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B18" s="35">
         <v>-67.747</v>
@@ -5328,7 +5333,7 @@
     </row>
     <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="34" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B19" s="35">
         <v>9.74</v>
@@ -5342,7 +5347,7 @@
     </row>
     <row r="20" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="34" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B20" s="35">
         <v>105.45399999999999</v>
@@ -5356,7 +5361,7 @@
     </row>
     <row r="21" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="34" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B21" s="141">
         <v>-324.96499999999997</v>
@@ -5392,21 +5397,21 @@
   <sheetData>
     <row r="1" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="30" t="s">
+        <v>157</v>
+      </c>
+      <c r="B1" s="30" t="s">
         <v>158</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="C1" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="C1" s="30" t="s">
+      <c r="D1" s="30" t="s">
         <v>160</v>
-      </c>
-      <c r="D1" s="30" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B2" s="32">
         <v>-1390</v>
@@ -5420,7 +5425,7 @@
     </row>
     <row r="3" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="34" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B3" s="35">
         <v>-1830</v>
@@ -5434,7 +5439,7 @@
     </row>
     <row r="4" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="34" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B4" s="35">
         <v>-1579.278</v>
@@ -5448,7 +5453,7 @@
     </row>
     <row r="5" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="34" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B5" s="35">
         <v>-1390</v>
@@ -5462,7 +5467,7 @@
     </row>
     <row r="6" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="34" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B6" s="35">
         <v>-1830</v>
@@ -5476,7 +5481,7 @@
     </row>
     <row r="7" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="34" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B7" s="35">
         <v>-1570.7049999999999</v>
@@ -5490,7 +5495,7 @@
     </row>
     <row r="8" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="34" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B8" s="141">
         <v>-1569.287</v>
@@ -5504,7 +5509,7 @@
     </row>
     <row r="9" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="34" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B9" s="141">
         <v>-1575</v>
@@ -5518,7 +5523,7 @@
     </row>
     <row r="10" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="34" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B10" s="35">
         <v>-1830</v>
@@ -5532,7 +5537,7 @@
     </row>
     <row r="11" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="34" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B11" s="35">
         <v>-1676.222</v>
@@ -5546,7 +5551,7 @@
     </row>
     <row r="12" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="34" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B12" s="35">
         <v>-1398.8620000000001</v>
@@ -5560,7 +5565,7 @@
     </row>
     <row r="13" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="34" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B13" s="35">
         <v>-1582.4280000000001</v>
@@ -5574,7 +5579,7 @@
     </row>
     <row r="14" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="34" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B14" s="35">
         <v>-1598.432</v>
@@ -5588,7 +5593,7 @@
     </row>
     <row r="15" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="34" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B15" s="35">
         <v>-1663.0229999999999</v>
@@ -5602,7 +5607,7 @@
     </row>
     <row r="16" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="34" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B16" s="35">
         <v>-1585.771</v>
@@ -5616,7 +5621,7 @@
     </row>
     <row r="17" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="34" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B17" s="35">
         <v>-1830</v>
@@ -5630,7 +5635,7 @@
     </row>
     <row r="18" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="34" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B18" s="35">
         <v>-1830</v>
@@ -5644,7 +5649,7 @@
     </row>
     <row r="19" spans="1:4" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="34" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B19" s="35">
         <v>-1602.577</v>
@@ -7715,26 +7720,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009342B7EAA7728A4FA80A5CCAFE8D7EAF" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d037a5681ee6af0e7b5b5d0a2f99b20">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9557458c-24b5-4c97-84ed-4c402655f54f" xmlns:ns3="72e3c584-9879-4b35-b9d8-6a248c93e240" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="966978c8b125399653e7c255ac8e342d" ns2:_="" ns3:_="">
     <xsd:import namespace="9557458c-24b5-4c97-84ed-4c402655f54f"/>
@@ -7995,10 +7980,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
+    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8015,20 +8031,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{725057E1-111A-4671-B2A8-840A9FE9E195}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23C60B87-FF36-4F0E-B782-0EC386590CC0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="9557458c-24b5-4c97-84ed-4c402655f54f"/>
-    <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>